<commit_message>
v2: topic heat model, overview ranking, 7-day grids, update_heat.py
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="帖子与来源" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="话题热度" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,14 +429,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
@@ -1561,6 +1562,510 @@
       <c r="G32" t="n">
         <v>496</v>
       </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>马斯克：No more AI, SI</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/elonmusk/status/2106665679361618173</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>超级智能 SI · 🦉猫头鹰</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>马斯克：It always was（猫头鹰封面）</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/elonmusk/status/2106672522771272121</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>超级智能 SI · 🦉猫头鹰</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>blockchainbob：OWL 是 10M+ runner</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/blockchainbob/status/2108158782010540282</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>超级智能 SI · 🦉猫头鹰</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Super Inu 回撤 &gt;70%</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/LEEJETJET/status/2107363707663851645</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>超级智能 SI · 🦉猫头鹰</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>OWL 聪明钱买入 · $1.3M</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/PeepRadars/status/2108201749873869220</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>超级智能 SI · 🦉猫头鹰</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>复制盘墓地：Owl -74.6%</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/Ldger_Logic/status/2107864245903688129</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>超级智能 SI · 🦉猫头鹰</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>新闻：MemeBitcoin 量子破解游戏</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/i/trending/2107444605931122925</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>量子 / AI 破解私钥 · 地堡</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>新闻：Pollak 在 Token2049 讲 memestocks</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/i/trending/2107892114243670355</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>股票 meme · 代币化美股</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>STONK 快照 $150M</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/LordWinty/status/2107833485301785000</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>股票 meme · 代币化美股</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>STONK vs PUMP 收入对比</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/merccuu/status/2107708461966369176</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>股票 meme · 代币化美股</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>新闻：Murad 预测 meme 超越比特币</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/i/trending/2108211927600300533</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>股票 meme · 代币化美股</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ZCAT 快照 $49.68M</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/LordWinty/status/2108331717727584352</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>持币分红盘 · ZCAT/BATON</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>BATON 第二腿</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/uncsnipes/status/2108289033051005224</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>持币分红盘 · ZCAT/BATON</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>新闻：Cake Wallet 创始人买 MCAT</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/i/trending/2107557735109713954</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>持币分红盘 · ZCAT/BATON</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>新闻：ZEC 回调与 ZCAT</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/i/trending/2107332169756712972</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>持币分红盘 · ZCAT/BATON</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>ANSEM 第 90 天：$142.3M</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/folashade_aduke/status/2108306839230357742</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ANSEM · SOL 老龙头</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>新闻：ANSEM 社区分歧</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/i/trending/2107375013032792464</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ANSEM · SOL 老龙头</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>新闻：首笔原子 L1→L2</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/i/trending/2107378801793445978</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>以太坊近况 · Glamsterdam</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>新闻：BEARISH 迁回以太坊</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/i/trending/2108295762803302646</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>以太坊近况 · Glamsterdam</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>新闻：Tom Lee 预测</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/i/trending/2107515726969856078</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>以太坊近况 · Glamsterdam</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>EtherWorld：Glamsterdam 上 Sepolia</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/ether_world/status/2107510399436538071</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>以太坊近况 · Glamsterdam</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>币安人生：致 CZ</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/digishahed/status/2108101740809904251</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>BSC 中文盘 · 币安人生</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>币安人生 ATH $900M / 龙虾 $310M</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/0xkitty69/status/2107177206199865466</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>BSC 中文盘 · 币安人生</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>新闻：LAPTOP 崩盘报告</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/i/trending/2107922838963335273</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LAPTOP · 亨特·拜登盘</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1595,7 +2100,673 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>排名</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>话题</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>状态</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>热度</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>趋势</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>龙头</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>结论</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>10-03 帖数</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>10-04 帖数</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>10-05 帖数</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>10-06 帖数</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>10-07 帖数</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>10-08 帖数</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>10-09 帖数</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Starlink 印度 · Ambani</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>91</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>↑</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>10/8 起从 ~100 条/天暴涨到 2.9 万条，国家级政治热度最高，但没有币 → 只当注意力风向，不追盘</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>93</v>
+      </c>
+      <c r="I2" t="n">
+        <v>154</v>
+      </c>
+      <c r="J2" t="n">
+        <v>158</v>
+      </c>
+      <c r="K2" t="n">
+        <v>107</v>
+      </c>
+      <c r="L2" t="n">
+        <v>8270</v>
+      </c>
+      <c r="M2" t="n">
+        <v>28953</v>
+      </c>
+      <c r="N2" t="n">
+        <v>29483</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Grok Bot · “花生钱雇天才”</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>78</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>↑</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>马斯克本周第一主推，讨论量一周 3 倍，但链上还没看到公认龙头 → 关注 BOT / Peanut 联动盘</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>6297</v>
+      </c>
+      <c r="I3" t="n">
+        <v>7496</v>
+      </c>
+      <c r="J3" t="n">
+        <v>6023</v>
+      </c>
+      <c r="K3" t="n">
+        <v>6485</v>
+      </c>
+      <c r="L3" t="n">
+        <v>12939</v>
+      </c>
+      <c r="M3" t="n">
+        <v>20107</v>
+      </c>
+      <c r="N3" t="n">
+        <v>18942</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>量子 / AI 破解私钥 · 地堡</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>65</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>↑</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>QUANTUM</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>讨论量 3 天翻 2.6 倍，真催化剂，但链上 14+ 同名盘、无龙头 → 等某盘站稳 1M + 大号转发</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>2410</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2468</v>
+      </c>
+      <c r="J4" t="n">
+        <v>2448</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2412</v>
+      </c>
+      <c r="L4" t="n">
+        <v>3816</v>
+      </c>
+      <c r="M4" t="n">
+        <v>6388</v>
+      </c>
+      <c r="N4" t="n">
+        <v>6442</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>股票 meme · 代币化美股</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>41</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>↓</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>STONK</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Base 创始人 Token2049 站台 memestocks，有收入支撑；但讨论量 10/5 见顶后回落 → 龙头 STONK 低吸，不追 Base 小盘</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>4484</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4215</v>
+      </c>
+      <c r="J5" t="n">
+        <v>6827</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3662</v>
+      </c>
+      <c r="L5" t="n">
+        <v>4273</v>
+      </c>
+      <c r="M5" t="n">
+        <v>3697</v>
+      </c>
+      <c r="N5" t="n">
+        <v>3540</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>超级智能 SI · 🦉猫头鹰</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>40</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>↓</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>叙事最正（马斯克亲口改名 AI→SI + 发猫头鹰封面），但龙头 SI 已从 ~$68M 回撤到 $24–31M，讨论 10/5 见顶后降温 → 等二次点火</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>976</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2744</v>
+      </c>
+      <c r="J6" t="n">
+        <v>3065</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1323</v>
+      </c>
+      <c r="L6" t="n">
+        <v>638</v>
+      </c>
+      <c r="M6" t="n">
+        <v>694</v>
+      </c>
+      <c r="N6" t="n">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>持币分红盘 · ZCAT/BATON</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>40</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>↑</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ZCAT</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>“持币吃 ZEC/PUMP/XMR 分红”玩法稳步升温，ZCAT 约 $50M 稳，BATON 走第二腿 → 最健康的一条线</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>910</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1410</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1630</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1788</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1338</v>
+      </c>
+      <c r="M7" t="n">
+        <v>2110</v>
+      </c>
+      <c r="N7" t="n">
+        <v>2047</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ANSEM · SOL 老龙头</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>39</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>ANSEM</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>$142M、15 万持有人，讨论平稳略降 → 大盘情绪锚，不是新机会</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>1459</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2068</v>
+      </c>
+      <c r="J8" t="n">
+        <v>2071</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2221</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2084</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1930</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1933</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BSC 中文盘 · 币安人生</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>33</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>币安人生</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>讨论量 10/3 后持续下降、刷屏号多 → 冷却，暂不参与</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>951</v>
+      </c>
+      <c r="I9" t="n">
+        <v>810</v>
+      </c>
+      <c r="J9" t="n">
+        <v>529</v>
+      </c>
+      <c r="K9" t="n">
+        <v>491</v>
+      </c>
+      <c r="L9" t="n">
+        <v>351</v>
+      </c>
+      <c r="M9" t="n">
+        <v>355</v>
+      </c>
+      <c r="N9" t="n">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>以太坊近况 · Glamsterdam</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>26</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>↓</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>技术/宏观新闻多（Glamsterdam 测试网、首笔原子 L1→L2、Abstract 关停），ETH ~$2,700 横盘，meme 热度低 → 只看 BURR 迁移</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>462</v>
+      </c>
+      <c r="I10" t="n">
+        <v>623</v>
+      </c>
+      <c r="J10" t="n">
+        <v>944</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1721</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1734</v>
+      </c>
+      <c r="M10" t="n">
+        <v>1119</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>LAPTOP · 亨特·拜登盘</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>26</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>↑</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>LAPTOP</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>政治名人盘，曾 1 小时 -98%，10/7 报告后小反弹，但讨论多为刷票机器人 → 回避</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>51</v>
+      </c>
+      <c r="I11" t="n">
+        <v>35</v>
+      </c>
+      <c r="J11" t="n">
+        <v>34</v>
+      </c>
+      <c r="K11" t="n">
+        <v>64</v>
+      </c>
+      <c r="L11" t="n">
+        <v>595</v>
+      </c>
+      <c r="M11" t="n">
+        <v>449</v>
+      </c>
+      <c r="N11" t="n">
+        <v>395</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
v3: 24h view, GMGN-verified CAs, live Dexscreener prices, refresh_tokens.py, prune dead coins
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="帖子与来源" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="话题热度" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="代币" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2504,7 +2505,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>QUANTUM</t>
+          <t>QI</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2558,7 +2559,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>PQC</t>
+          <t>BNKR</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2882,7 +2883,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2969,4 +2970,1722 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>话题</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>周期</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>角色</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>代币</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>链</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>状态</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>市值$</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>1h%</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>24h%</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>流动性$</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>叙事</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>GMGN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>超级智能 SI · 🦉猫头鹰</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>龙头</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>DEW9dSN6QpWyNthphCpMmAbZP1Q4cEKR9xQXAri98WDP</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>25053627</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="J2" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="K2" t="n">
+        <v>807857</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Super Inu：马斯克“SI 超级智能”梗龙头，ATH ~$69M，现在 ~$25M 横盘。</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/DEW9dSN6QpWyNthphCpMmAbZP1Q4cEKR9xQXAri98WDP</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>超级智能 SI · 🦉猫头鹰</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>9aqmJjCnnMQv42TXLk921ceUkN35nea2QP969n1caqjj</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>1390791</v>
+      </c>
+      <c r="I3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J3" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="K3" t="n">
+        <v>162747</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Super Intelligence：同名二号 SI，9/30 上线，百万级市值。</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/9aqmJjCnnMQv42TXLk921ceUkN35nea2QP969n1caqjj</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>超级智能 SI · 🦉猫头鹰</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>OWL</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>68AGsjomsgTtiTaDhF6XGCeVJDnFeh415ngYYgVxGzns</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>958179</v>
+      </c>
+      <c r="I4" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="J4" t="n">
+        <v>174.4</v>
+      </c>
+      <c r="K4" t="n">
+        <v>114575</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Superintelligence Owl：马斯克“It always was”猫头鹰封面吉祥物盘，24h 反弹 +170%。</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/68AGsjomsgTtiTaDhF6XGCeVJDnFeh415ngYYgVxGzns</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>超级智能 SI · 🦉猫头鹰</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>OWLNIGHT</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>CmCHvr99aXrLDQB7jAtFtsBwg3DnXqq4spcTEMt7pump</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>496700</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="J5" t="n">
+        <v>16466.4</v>
+      </c>
+      <c r="K5" t="n">
+        <v>67994</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Owl Nighter：10/09 新猫头鹰盘，1.6 万持有人，24h 暴涨后回落一半。</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/CmCHvr99aXrLDQB7jAtFtsBwg3DnXqq4spcTEMt7pump</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>超级智能 SI · 🦉猫头鹰</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Ap7R5jTGxFCZEbkFc3WNMiN3ru6nkPkn3Co5p6tbpump</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>22569</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>325.3</v>
+      </c>
+      <c r="K6" t="n">
+        <v>13654</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Superintelligence（2024 老盘复活）：小市值同名盘，流动性薄。</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/Ap7R5jTGxFCZEbkFc3WNMiN3ru6nkPkn3Co5p6tbpump</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>超级智能 SI · 🦉猫头鹰</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>SI276</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>HMYd9tosnUXuNHmq7pXmoePRVBLBBjA3JBfydq6upump</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>1809264</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-7.1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>308.3</v>
+      </c>
+      <c r="K7" t="n">
+        <v>125983</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Super Intelligence SI276：GMGN 自动发现的新 SI 同名盘（&lt;72h），~$1.8M，叙事待人工核实。</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/HMYd9tosnUXuNHmq7pXmoePRVBLBBjA3JBfydq6upump</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>量子 / AI 破解私钥</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>龙头</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>QI</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>8TiMkgvsrat9tM2esko8zVTt99LZLpefUM4SnZaziXaQ</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>812217</v>
+      </c>
+      <c r="I8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J8" t="n">
+        <v>27479.9</v>
+      </c>
+      <c r="K8" t="n">
+        <v>85932</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Quantum Inu：10/09 新盘，量子狗，量子赛道当前市值最大的纯 meme，24h 涨幅上万 %。</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/8TiMkgvsrat9tM2esko8zVTt99LZLpefUM4SnZaziXaQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>量子 / AI 破解私钥</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>BUNKER</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>8NCievmJCg2d9Vc2TWgz2HkE6ANeSX7kwvdq5AL7pump</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>947145</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>-14</v>
+      </c>
+      <c r="K9" t="n">
+        <v>135165</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>BunkerCoin（bunkercoin.io）：toly 2024 愚人节“短波电台区块链”论文的老梗盘，1 月上线，ATH ~$9.8M，量子恐慌让“地堡”梗回流。</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/8NCievmJCg2d9Vc2TWgz2HkE6ANeSX7kwvdq5AL7pump</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>量子 / AI 破解私钥</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>QCAT</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>GmsAcJAFKEtAXDoRUroaQP5GBdmPcGwA2sRdC9Mbpump</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>27809</v>
+      </c>
+      <c r="I10" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J10" t="n">
+        <v>861.7</v>
+      </c>
+      <c r="K10" t="n">
+        <v>11859</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Quantum Cat：10/09 新量子猫，小盘高波动，捆绑 ~15%，只当彩票。</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/GmsAcJAFKEtAXDoRUroaQP5GBdmPcGwA2sRdC9Mbpump</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>股票 meme · 代币化美股</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>龙头</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>STONK</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>6GmAFSYs4gk3FDao5FzzySQpPZaWsa4rUJHacpMpUNgx</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>123040661</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4</v>
+      </c>
+      <c r="J11" t="n">
+        <v>-10.9</v>
+      </c>
+      <c r="K11" t="n">
+        <v>283015</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>StonkFun 发射台币：股票 meme 龙头，30 天收入 ~$28–31M，市值 ~$1.2 亿。</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/6GmAFSYs4gk3FDao5FzzySQpPZaWsa4rUJHacpMpUNgx</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>股票 meme · 代币化美股</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>PONS</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>robinhood</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0x39dbed3a2bd333467115de45665cc57f813c4571</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>350199860</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-0.9</v>
+      </c>
+      <c r="J12" t="n">
+        <v>-13.7</v>
+      </c>
+      <c r="K12" t="n">
+        <v>2808685</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Robinhood Chain 发射台币 Pons：10 万持有人，股票链 meme 的庄家盘。</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/robinhood/token/0x39dbed3a2bd333467115de45665cc57f813c4571</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>股票 meme · 代币化美股</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>BLUECHIP</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0xb200000000000000000000cfbdf64a8706a94a01</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>6937854</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="J13" t="n">
+        <v>-0.9</v>
+      </c>
+      <c r="K13" t="n">
+        <v>337144</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Base 股票 meme：Jesse Pollak Token2049 幻灯片点名。</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/base/token/0xb200000000000000000000cfbdf64a8706a94a01</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>股票 meme · 代币化美股</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>IPOD</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0xa6af0cea8fbc93e1eccc00f1fdd9a0bba251fee1</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>1316058</v>
+      </c>
+      <c r="I14" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="J14" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="K14" t="n">
+        <v>269520</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Base 苹果股票梗 iPod，Jesse 幻灯片点名。</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/base/token/0xa6af0cea8fbc93e1eccc00f1fdd9a0bba251fee1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>股票 meme · 代币化美股</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>DGUY</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0xe34356dcd3d7bb991248f322e4ec31b5d60bc54e</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>661512</v>
+      </c>
+      <c r="I15" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="J15" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="K15" t="n">
+        <v>94074</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Delivery Guy：Base 股票 meme，Jesse 幻灯片点名。</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/base/token/0xe34356dcd3d7bb991248f322e4ec31b5d60bc54e</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>股票 meme · 代币化美股</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>TEMU</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0x3c573bdd88008c94f025e5023212f28e5f39744c</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>339588</v>
+      </c>
+      <c r="I16" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="J16" t="n">
+        <v>4</v>
+      </c>
+      <c r="K16" t="n">
+        <v>65757</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>TEMU on Base：Jesse 幻灯片点名的拼多多梗。</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/base/token/0x3c573bdd88008c94f025e5023212f28e5f39744c</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>持币分红盘 · ZCAT/BATON</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>龙头</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>ZCAT</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>43239149</v>
+      </c>
+      <c r="I17" t="n">
+        <v>-2.6</v>
+      </c>
+      <c r="J17" t="n">
+        <v>-6.7</v>
+      </c>
+      <c r="K17" t="n">
+        <v>1074363</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Anonymous Cat：3% 交易税自动换 ZEC 分红给持有人，分红盘龙头。</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>持币分红盘 · ZCAT/BATON</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>BATON</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>12843686</v>
+      </c>
+      <c r="I18" t="n">
+        <v>-3</v>
+      </c>
+      <c r="J18" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="K18" t="n">
+        <v>752065</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>baton：分红 PUMP 的分红盘，ATH ~$19M，回调后第二腿。</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>持币分红盘 · ZCAT/BATON</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MCAT</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>187585</v>
+      </c>
+      <c r="I19" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="J19" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="K19" t="n">
+        <v>39682</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Addicted Cat：分红门罗币 XMR，Cake Wallet 创始人买入。</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ANSEM · SOL 老龙头</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>龙头</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ANSEM</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>140249094</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K20" t="n">
+        <v>2350060</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>The Black Bull：Ansem 本人梗的 SOL 老龙头，15 万持有人，前十持仓 ~65% 偏集中。</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>以太坊近况 · Glamsterdam</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>龙头</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>367308060</v>
+      </c>
+      <c r="I21" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="J21" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="K21" t="n">
+        <v>11116240</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>SPX6900：Murad 舞台喊“meme 将超越比特币”的 ETH 主网 meme 龙头。</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/eth/token/0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BSC 中文盘 · 币安人生</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>龙头</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>币安人生</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>bsc</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>548460940</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J22" t="n">
+        <v>-2.6</v>
+      </c>
+      <c r="K22" t="n">
+        <v>8401363</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>币安人生：何一推文带火的 BSC 中文 meme 龙头，ATH ~$9 亿，现 ~$5.5 亿。</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/bsc/token/0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BSC 中文盘 · 币安人生</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>龙虾</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>bsc</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>0xeccbb861c0dda7efd964010085488b69317e4444</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>43133249</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J23" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2041758</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>龙虾：币安中文号推文出圈的中文盘，ATH ~$3.1 亿，现 ~$4300 万。注意今天有同名高仿盘。</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/bsc/token/0xeccbb861c0dda7efd964010085488b69317e4444</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>LAPTOP · 亨特·拜登盘</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>龙头</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>LAPTOP</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>0xb095274743941e953c746f9c228da9c18bb6ec29</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>75239810</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J24" t="n">
+        <v>-7.2</v>
+      </c>
+      <c r="K24" t="n">
+        <v>659750</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Hunter Biden 本人发的“笔记本电脑”梗币，前十持仓 ~91% 极度集中。</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/base/token/0xb095274743941e953c746f9c228da9c18bb6ec29</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>后量子地堡 · BNKR/PQC</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>龙头</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>BNKR</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>5YfBLGhU7k5YDcfMUjNmftv7crbZCHoh2shScZVXnbKo</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>191225</v>
+      </c>
+      <c r="I25" t="n">
+        <v>-6.3</v>
+      </c>
+      <c r="J25" t="n">
+        <v>6330.7</v>
+      </c>
+      <c r="K25" t="n">
+        <v>39607</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>pqc.market 官方发的“首个带后量子（哈希签名）证明的 Solana meme”，10/09 13:18 悉尼上线，当天最高 ~$420K。</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/5YfBLGhU7k5YDcfMUjNmftv7crbZCHoh2shScZVXnbKo</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>后量子地堡 · BNKR/PQC</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>PQC</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>1396724</v>
+      </c>
+      <c r="I26" t="n">
+        <v>-6.9</v>
+      </c>
+      <c r="J26" t="n">
+        <v>809.6</v>
+      </c>
+      <c r="K26" t="n">
+        <v>142524</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>pqc.market 平台币：后量子发射台，10/08 上线，24h 成交 ~$7.7M，BNKR 的母盘。</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>后量子地堡 · BNKR/PQC</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>BUNKER</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2WNiZqRefcndEA9c1T6A1bdie31pbBGdFQpyR52h9TWr</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>124547</v>
+      </c>
+      <c r="I27" t="n">
+        <v>64.59999999999999</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1778.7</v>
+      </c>
+      <c r="K27" t="n">
+        <v>29428</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>bunker.markets：蹭“地堡”热度的同名盘，10/08 晚上线，24h +2000%，机器人/捆绑占比高。</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/2WNiZqRefcndEA9c1T6A1bdie31pbBGdFQpyR52h9TWr</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>后量子地堡 · BNKR/PQC</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>PQC</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>3ZwW1DmGH9qfLM23c2ZVmtVP1PBPrC1Tgc14v4YRTC91</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>61337</v>
+      </c>
+      <c r="I28" t="n">
+        <v>213.7</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1989.6</v>
+      </c>
+      <c r="K28" t="n">
+        <v>18451</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Post Quantum Cat：10/09 在 pqc.market 上发的量子猫，小盘，只当彩票。</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/3ZwW1DmGH9qfLM23c2ZVmtVP1PBPrC1Tgc14v4YRTC91</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId27"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
tokens 10/12 16:11 radar
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -3166,16 +3166,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>23110232</v>
+        <v>23806138</v>
       </c>
       <c r="I2" t="n">
-        <v>-4.7</v>
+        <v>3.2</v>
       </c>
       <c r="J2" t="n">
-        <v>-16.5</v>
+        <v>-17</v>
       </c>
       <c r="K2" t="n">
-        <v>874724</v>
+        <v>878760</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -3225,16 +3225,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1445249</v>
+        <v>1513519</v>
       </c>
       <c r="I3" t="n">
-        <v>7.8</v>
+        <v>5.4</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="K3" t="n">
-        <v>168941</v>
+        <v>174851</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -3284,16 +3284,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>852422</v>
+        <v>838512</v>
       </c>
       <c r="I4" t="n">
-        <v>9</v>
+        <v>8.1</v>
       </c>
       <c r="J4" t="n">
-        <v>33</v>
+        <v>30.6</v>
       </c>
       <c r="K4" t="n">
-        <v>108799</v>
+        <v>108400</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -3343,16 +3343,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>24393</v>
+        <v>24841</v>
       </c>
       <c r="I5" t="n">
-        <v>11.1</v>
+        <v>13.2</v>
       </c>
       <c r="J5" t="n">
-        <v>21.4</v>
+        <v>29.9</v>
       </c>
       <c r="K5" t="n">
-        <v>14741</v>
+        <v>14884</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -3402,16 +3402,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1337015</v>
+        <v>1340057</v>
       </c>
       <c r="I6" t="n">
-        <v>-10.5</v>
+        <v>-8.1</v>
       </c>
       <c r="J6" t="n">
-        <v>55.7</v>
+        <v>57.1</v>
       </c>
       <c r="K6" t="n">
-        <v>114926</v>
+        <v>114455</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -3461,16 +3461,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>43840</v>
+        <v>43636</v>
       </c>
       <c r="I7" t="n">
-        <v>-1.8</v>
+        <v>-1.6</v>
       </c>
       <c r="J7" t="n">
-        <v>-31.6</v>
+        <v>-55.7</v>
       </c>
       <c r="K7" t="n">
-        <v>17081</v>
+        <v>17024</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -3520,16 +3520,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>1689743</v>
+        <v>1657515</v>
       </c>
       <c r="I8" t="n">
-        <v>10.1</v>
+        <v>-2.3</v>
       </c>
       <c r="J8" t="n">
-        <v>-36.8</v>
+        <v>-38</v>
       </c>
       <c r="K8" t="n">
-        <v>164964</v>
+        <v>165141</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -3579,16 +3579,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>50481</v>
+        <v>42328</v>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>-4.3</v>
       </c>
       <c r="J9" t="n">
-        <v>-65</v>
+        <v>-71.3</v>
       </c>
       <c r="K9" t="n">
-        <v>20497</v>
+        <v>18507</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -3638,16 +3638,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>148659</v>
+        <v>148280</v>
       </c>
       <c r="I10" t="n">
-        <v>20.9</v>
+        <v>38.1</v>
       </c>
       <c r="J10" t="n">
-        <v>-56.3</v>
+        <v>-60.9</v>
       </c>
       <c r="K10" t="n">
-        <v>53044</v>
+        <v>52937</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -3697,16 +3697,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>3346199</v>
+        <v>3359771</v>
       </c>
       <c r="I11" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="J11" t="n">
-        <v>23.1</v>
+        <v>23.4</v>
       </c>
       <c r="K11" t="n">
-        <v>159935</v>
+        <v>160436</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -3756,16 +3756,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>121678176</v>
+        <v>121717155</v>
       </c>
       <c r="I12" t="n">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="J12" t="n">
-        <v>4.8</v>
+        <v>3.8</v>
       </c>
       <c r="K12" t="n">
-        <v>249411</v>
+        <v>248858</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -3815,16 +3815,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>354210840</v>
+        <v>357071250</v>
       </c>
       <c r="I13" t="n">
-        <v>2.2</v>
+        <v>2.7</v>
       </c>
       <c r="J13" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="K13" t="n">
-        <v>2800832</v>
+        <v>2825790</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -3874,16 +3874,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>7337236</v>
+        <v>7282780</v>
       </c>
       <c r="I14" t="n">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="J14" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="K14" t="n">
-        <v>345821</v>
+        <v>343386</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -3933,16 +3933,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1229600</v>
+        <v>1236772</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.1</v>
+        <v>0.7</v>
       </c>
       <c r="J15" t="n">
-        <v>-1.9</v>
+        <v>-1.3</v>
       </c>
       <c r="K15" t="n">
-        <v>266768</v>
+        <v>267127</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -3992,16 +3992,16 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>1033036</v>
+        <v>1031373</v>
       </c>
       <c r="I16" t="n">
-        <v>3.5</v>
+        <v>6.2</v>
       </c>
       <c r="J16" t="n">
-        <v>69.90000000000001</v>
+        <v>69.7</v>
       </c>
       <c r="K16" t="n">
-        <v>121410</v>
+        <v>121597</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -4051,16 +4051,16 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>323461</v>
+        <v>331142</v>
       </c>
       <c r="I17" t="n">
-        <v>-0.5</v>
+        <v>2.3</v>
       </c>
       <c r="J17" t="n">
-        <v>23.7</v>
+        <v>25.6</v>
       </c>
       <c r="K17" t="n">
-        <v>62986</v>
+        <v>64016</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -4110,16 +4110,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>54274568</v>
+        <v>52637035</v>
       </c>
       <c r="I18" t="n">
-        <v>8.199999999999999</v>
+        <v>4.8</v>
       </c>
       <c r="J18" t="n">
-        <v>23.9</v>
+        <v>21.5</v>
       </c>
       <c r="K18" t="n">
-        <v>1263866</v>
+        <v>1264971</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -4169,16 +4169,16 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>16982471</v>
+        <v>17303305</v>
       </c>
       <c r="I19" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="J19" t="n">
-        <v>31.8</v>
+        <v>30.5</v>
       </c>
       <c r="K19" t="n">
-        <v>886315</v>
+        <v>901973</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -4231,10 +4231,10 @@
         <v>120985</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.4</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>-9.4</v>
+        <v>-17</v>
       </c>
       <c r="K20" t="n">
         <v>31064</v>
@@ -4287,16 +4287,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>42622</v>
+        <v>46436</v>
       </c>
       <c r="I21" t="n">
-        <v>-4.8</v>
+        <v>16.3</v>
       </c>
       <c r="J21" t="n">
-        <v>1.2</v>
+        <v>-2.1</v>
       </c>
       <c r="K21" t="n">
-        <v>17172</v>
+        <v>17811</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -4346,16 +4346,16 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>148325758</v>
+        <v>149095791</v>
       </c>
       <c r="I22" t="n">
-        <v>0.1</v>
+        <v>-1.4</v>
       </c>
       <c r="J22" t="n">
-        <v>13.5</v>
+        <v>14.1</v>
       </c>
       <c r="K22" t="n">
-        <v>2454217</v>
+        <v>2458400</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -4405,16 +4405,16 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>390001570</v>
+        <v>389210880</v>
       </c>
       <c r="I23" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="J23" t="n">
-        <v>6</v>
+        <v>5.2</v>
       </c>
       <c r="K23" t="n">
-        <v>11593453</v>
+        <v>11607446</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -4464,16 +4464,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>615917270</v>
+        <v>609784910</v>
       </c>
       <c r="I24" t="n">
-        <v>-0.6</v>
+        <v>-1.9</v>
       </c>
       <c r="J24" t="n">
-        <v>9.199999999999999</v>
+        <v>7.7</v>
       </c>
       <c r="K24" t="n">
-        <v>8983759</v>
+        <v>8942347</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -4523,16 +4523,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>42105277</v>
+        <v>42004343</v>
       </c>
       <c r="I25" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="J25" t="n">
-        <v>-5.5</v>
+        <v>-5.8</v>
       </c>
       <c r="K25" t="n">
-        <v>2040036</v>
+        <v>2037865</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -4582,16 +4582,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>314802</v>
+        <v>305236</v>
       </c>
       <c r="I26" t="n">
-        <v>-6.4</v>
+        <v>-18.5</v>
       </c>
       <c r="J26" t="n">
-        <v>-13.4</v>
+        <v>-16.9</v>
       </c>
       <c r="K26" t="n">
-        <v>55579</v>
+        <v>54738</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -4641,16 +4641,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>174911</v>
+        <v>173735</v>
       </c>
       <c r="I27" t="n">
-        <v>5.4</v>
+        <v>4.4</v>
       </c>
       <c r="J27" t="n">
-        <v>-33.3</v>
+        <v>-37.9</v>
       </c>
       <c r="K27" t="n">
-        <v>41659</v>
+        <v>41530</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -4700,16 +4700,16 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>74886812</v>
+        <v>74785959</v>
       </c>
       <c r="I28" t="n">
-        <v>-0.3</v>
+        <v>-0.8</v>
       </c>
       <c r="J28" t="n">
-        <v>-1.7</v>
+        <v>-2.8</v>
       </c>
       <c r="K28" t="n">
-        <v>254591</v>
+        <v>251558</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -4759,16 +4759,16 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>358047</v>
+        <v>342315</v>
       </c>
       <c r="I29" t="n">
-        <v>14.2</v>
+        <v>0.3</v>
       </c>
       <c r="J29" t="n">
-        <v>-22.7</v>
+        <v>-35.1</v>
       </c>
       <c r="K29" t="n">
-        <v>71762</v>
+        <v>70641</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -4818,16 +4818,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>242434</v>
+        <v>230487</v>
       </c>
       <c r="I30" t="n">
-        <v>33.4</v>
+        <v>23.5</v>
       </c>
       <c r="J30" t="n">
-        <v>97.40000000000001</v>
+        <v>111</v>
       </c>
       <c r="K30" t="n">
-        <v>43658</v>
+        <v>42766</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
radar silent 10/12 16:14
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -2348,7 +2348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2365,6 +2365,9 @@
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2438,6 +2441,21 @@
           <t>10-09 帖数</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>10-10 帖数</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>10-11 帖数</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>10-12 帖数</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -2492,6 +2510,9 @@
       <c r="N2" t="n">
         <v>30080</v>
       </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -2499,7 +2520,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Grok Bot · 整家公司由 AI 组成</t>
+          <t>量子 / AI 破解私钥</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2508,7 +2529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -2517,35 +2538,38 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>QI</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>马斯克本周第一主推，讨论量一周 3 倍，但链上只有 &lt;$60K 的小盘，没有像样龙头 → 只盯叙事，不追盘</t>
+          <t>讨论量 3 天翻 2.6 倍；旧龙头 QUANTUM 已归零删除，新龙头 Quantum Inu ~$80 万。地堡/后量子玩法已拆成独立 24h 话题</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>6297</v>
+        <v>2410</v>
       </c>
       <c r="I3" t="n">
-        <v>7496</v>
+        <v>2468</v>
       </c>
       <c r="J3" t="n">
-        <v>6023</v>
+        <v>2448</v>
       </c>
       <c r="K3" t="n">
-        <v>6485</v>
+        <v>2412</v>
       </c>
       <c r="L3" t="n">
-        <v>12939</v>
+        <v>3816</v>
       </c>
       <c r="M3" t="n">
-        <v>20083</v>
+        <v>6372</v>
       </c>
       <c r="N3" t="n">
-        <v>17798</v>
-      </c>
+        <v>6619</v>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -2553,7 +2577,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>量子 / AI 破解私钥</t>
+          <t>Grok Bot · 整家公司由 AI 组成</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2562,43 +2586,52 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>↑</t>
+          <t>→</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>QI</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>讨论量 3 天翻 2.6 倍；旧龙头 QUANTUM 已归零删除，新龙头 Quantum Inu ~$80 万。地堡/后量子玩法已拆成独立 24h 话题</t>
+          <t>10/12：马斯克再推 Cybercab 内 Grok @Bot（已核实，~45万浏览）；链上仍无像样龙头 → 盯叙事不追盘</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2410</v>
+        <v>6297</v>
       </c>
       <c r="I4" t="n">
-        <v>2468</v>
+        <v>7496</v>
       </c>
       <c r="J4" t="n">
-        <v>2448</v>
+        <v>6023</v>
       </c>
       <c r="K4" t="n">
-        <v>2412</v>
+        <v>9131</v>
       </c>
       <c r="L4" t="n">
-        <v>3816</v>
+        <v>17994</v>
       </c>
       <c r="M4" t="n">
-        <v>6372</v>
+        <v>24942</v>
       </c>
       <c r="N4" t="n">
-        <v>6619</v>
+        <v>18413</v>
+      </c>
+      <c r="O4" t="n">
+        <v>18427</v>
+      </c>
+      <c r="P4" t="n">
+        <v>18577</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>18931</v>
       </c>
     </row>
     <row r="5">
@@ -2607,7 +2640,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>后量子地堡 · BNKR/PQC</t>
+          <t>股票 meme · 代币化美股</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2616,44 +2649,47 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>↑</t>
+          <t>↓</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>PQC</t>
+          <t>STONK</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>量子恐慌的第一个“产品化”玩法：pqc.market 发射台 + 官方 BNKR。X 讨论 2 天翻 4 倍，但 BNKR 已从 $420K 回撤到 ~$180K，PQC 是母盘</t>
+          <t>Base 创始人 Token2049 站台 memestocks，有收入支撑；但讨论量 10/5 见顶后回落 → 龙头 STONK 低吸，不追 Base 小盘</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>392</v>
+        <v>4484</v>
       </c>
       <c r="I5" t="n">
-        <v>243</v>
+        <v>4215</v>
       </c>
       <c r="J5" t="n">
-        <v>303</v>
+        <v>6827</v>
       </c>
       <c r="K5" t="n">
-        <v>324</v>
+        <v>3662</v>
       </c>
       <c r="L5" t="n">
-        <v>223</v>
+        <v>4273</v>
       </c>
       <c r="M5" t="n">
-        <v>1132</v>
+        <v>3694</v>
       </c>
       <c r="N5" t="n">
-        <v>1950</v>
-      </c>
+        <v>3672</v>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -2661,7 +2697,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>股票 meme · 代币化美股</t>
+          <t>持币分红盘 · ZCAT/BATON</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2670,44 +2706,47 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>↑</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>STONK</t>
+          <t>ZCAT</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Base 创始人 Token2049 站台 memestocks，有收入支撑；但讨论量 10/5 见顶后回落 → 龙头 STONK 低吸，不追 Base 小盘</t>
+          <t>“持币吃 ZEC/PUMP/XMR 分红”玩法稳步升温，ZCAT 约 $50M 稳，BATON 走第二腿 → 最健康的一条线</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>4484</v>
+        <v>910</v>
       </c>
       <c r="I6" t="n">
-        <v>4215</v>
+        <v>1410</v>
       </c>
       <c r="J6" t="n">
-        <v>6827</v>
+        <v>1630</v>
       </c>
       <c r="K6" t="n">
-        <v>3662</v>
+        <v>1788</v>
       </c>
       <c r="L6" t="n">
-        <v>4273</v>
+        <v>1338</v>
       </c>
       <c r="M6" t="n">
-        <v>3694</v>
+        <v>2103</v>
       </c>
       <c r="N6" t="n">
-        <v>3672</v>
-      </c>
+        <v>2047</v>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2715,7 +2754,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>持币分红盘 · ZCAT/BATON</t>
+          <t>ANSEM · SOL 老龙头</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2728,40 +2767,43 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>↑</t>
+          <t>→</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>ZCAT</t>
+          <t>ANSEM</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>“持币吃 ZEC/PUMP/XMR 分红”玩法稳步升温，ZCAT 约 $50M 稳，BATON 走第二腿 → 最健康的一条线</t>
+          <t>$142M、15 万持有人，讨论平稳略降 → 大盘情绪锚，不是新机会</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>910</v>
+        <v>1459</v>
       </c>
       <c r="I7" t="n">
-        <v>1410</v>
+        <v>2068</v>
       </c>
       <c r="J7" t="n">
-        <v>1630</v>
+        <v>2071</v>
       </c>
       <c r="K7" t="n">
-        <v>1788</v>
+        <v>2221</v>
       </c>
       <c r="L7" t="n">
-        <v>1338</v>
+        <v>2084</v>
       </c>
       <c r="M7" t="n">
-        <v>2103</v>
+        <v>1930</v>
       </c>
       <c r="N7" t="n">
-        <v>2047</v>
-      </c>
+        <v>2009</v>
+      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2769,7 +2811,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ANSEM · SOL 老龙头</t>
+          <t>超级智能 SI · 🦉猫头鹰</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2778,44 +2820,47 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>→</t>
+          <t>↓</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>ANSEM</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>$142M、15 万持有人，讨论平稳略降 → 大盘情绪锚，不是新机会</t>
+          <t>10/10 新增：Salesforce CEO Benioff 官宣 AIForce 改名 SIForce（原帖 35 万浏览，已核实），SI 叙事再获大公司背书；但龙头 Super Inu 6h 仍 -11%、约 $22M，市场暂未反应 → 等二次点火</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>1459</v>
+        <v>976</v>
       </c>
       <c r="I8" t="n">
-        <v>2068</v>
+        <v>2744</v>
       </c>
       <c r="J8" t="n">
-        <v>2071</v>
+        <v>3065</v>
       </c>
       <c r="K8" t="n">
-        <v>2221</v>
+        <v>1323</v>
       </c>
       <c r="L8" t="n">
-        <v>2084</v>
+        <v>638</v>
       </c>
       <c r="M8" t="n">
-        <v>1930</v>
+        <v>692</v>
       </c>
       <c r="N8" t="n">
-        <v>2009</v>
-      </c>
+        <v>663</v>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -2823,7 +2868,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>超级智能 SI · 🦉猫头鹰</t>
+          <t>BSC 中文盘 · 币安人生</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2832,44 +2877,47 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>→</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>币安人生</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>10/10 新增：Salesforce CEO Benioff 官宣 AIForce 改名 SIForce（原帖 35 万浏览，已核实），SI 叙事再获大公司背书；但龙头 Super Inu 6h 仍 -11%、约 $22M，市场暂未反应 → 等二次点火</t>
+          <t>讨论量 10/3 后持续下降、刷屏号多 → 冷却，暂不参与</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>976</v>
+        <v>951</v>
       </c>
       <c r="I9" t="n">
-        <v>2744</v>
+        <v>810</v>
       </c>
       <c r="J9" t="n">
-        <v>3065</v>
+        <v>529</v>
       </c>
       <c r="K9" t="n">
-        <v>1323</v>
+        <v>491</v>
       </c>
       <c r="L9" t="n">
-        <v>638</v>
+        <v>351</v>
       </c>
       <c r="M9" t="n">
-        <v>692</v>
+        <v>354</v>
       </c>
       <c r="N9" t="n">
-        <v>663</v>
-      </c>
+        <v>579</v>
+      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -2877,7 +2925,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BSC 中文盘 · 币安人生</t>
+          <t>以太坊近况 · Glamsterdam</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2886,44 +2934,47 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>→</t>
+          <t>↓</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>币安人生</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>讨论量 10/3 后持续下降、刷屏号多 → 冷却，暂不参与</t>
+          <t>技术/宏观新闻多（Glamsterdam 测试网、首笔原子 L1→L2、Abstract 关停），ETH ~$2,700 横盘，meme 热度低 → 只看 BURR 迁移</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>951</v>
+        <v>462</v>
       </c>
       <c r="I10" t="n">
-        <v>810</v>
+        <v>623</v>
       </c>
       <c r="J10" t="n">
-        <v>529</v>
+        <v>944</v>
       </c>
       <c r="K10" t="n">
-        <v>491</v>
+        <v>1721</v>
       </c>
       <c r="L10" t="n">
-        <v>351</v>
+        <v>1734</v>
       </c>
       <c r="M10" t="n">
-        <v>354</v>
+        <v>1117</v>
       </c>
       <c r="N10" t="n">
-        <v>579</v>
-      </c>
+        <v>1123</v>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -2931,7 +2982,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>以太坊近况 · Glamsterdam</t>
+          <t>LAPTOP · 亨特·拜登盘</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2940,44 +2991,47 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>↑</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>LAPTOP</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>技术/宏观新闻多（Glamsterdam 测试网、首笔原子 L1→L2、Abstract 关停），ETH ~$2,700 横盘，meme 热度低 → 只看 BURR 迁移</t>
+          <t>政治名人盘，曾 1 小时 -98%，10/7 报告后小反弹，但讨论多为刷票机器人 → 回避</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>462</v>
+        <v>51</v>
       </c>
       <c r="I11" t="n">
-        <v>623</v>
+        <v>35</v>
       </c>
       <c r="J11" t="n">
-        <v>944</v>
+        <v>34</v>
       </c>
       <c r="K11" t="n">
-        <v>1721</v>
+        <v>64</v>
       </c>
       <c r="L11" t="n">
-        <v>1734</v>
+        <v>595</v>
       </c>
       <c r="M11" t="n">
-        <v>1117</v>
+        <v>448</v>
       </c>
       <c r="N11" t="n">
-        <v>1123</v>
-      </c>
+        <v>384</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2985,7 +3039,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LAPTOP · 亨特·拜登盘</t>
+          <t>后量子地堡 · BNKR/PQC</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2998,39 +3052,48 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>↑</t>
+          <t>↓</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>LAPTOP</t>
+          <t>PQC</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>政治名人盘，曾 1 小时 -98%，10/7 报告后小反弹，但讨论多为刷票机器人 → 回避</t>
+          <t>量子恐慌的第一个“产品化”玩法：pqc.market 发射台 + 官方 BNKR。X 讨论 2 天翻 4 倍，但 BNKR 已从 $420K 回撤到 ~$180K，PQC 是母盘</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>51</v>
+        <v>392</v>
       </c>
       <c r="I12" t="n">
-        <v>35</v>
+        <v>243</v>
       </c>
       <c r="J12" t="n">
-        <v>34</v>
+        <v>303</v>
       </c>
       <c r="K12" t="n">
-        <v>64</v>
+        <v>282</v>
       </c>
       <c r="L12" t="n">
-        <v>595</v>
+        <v>564</v>
       </c>
       <c r="M12" t="n">
-        <v>448</v>
+        <v>1588</v>
       </c>
       <c r="N12" t="n">
-        <v>384</v>
+        <v>1463</v>
+      </c>
+      <c r="O12" t="n">
+        <v>728</v>
+      </c>
+      <c r="P12" t="n">
+        <v>587</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>590</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
radar silent 10/12 16:54
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -3107,7 +3107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M33"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3229,16 +3229,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>23160414</v>
+        <v>23808968</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.9</v>
+        <v>0.2</v>
       </c>
       <c r="J2" t="n">
-        <v>-18.2</v>
+        <v>-17.4</v>
       </c>
       <c r="K2" t="n">
-        <v>883582</v>
+        <v>883569</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -3288,16 +3288,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1583092</v>
+        <v>1782736</v>
       </c>
       <c r="I3" t="n">
-        <v>13.9</v>
+        <v>26.3</v>
       </c>
       <c r="J3" t="n">
-        <v>9.1</v>
+        <v>28.1</v>
       </c>
       <c r="K3" t="n">
-        <v>178438</v>
+        <v>189843</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -3347,16 +3347,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>833265</v>
+        <v>848364</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.3</v>
+        <v>3.7</v>
       </c>
       <c r="J4" t="n">
-        <v>28.3</v>
+        <v>31</v>
       </c>
       <c r="K4" t="n">
-        <v>108129</v>
+        <v>108401</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -3406,16 +3406,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>26178</v>
+        <v>25019</v>
       </c>
       <c r="I5" t="n">
-        <v>18.6</v>
+        <v>2.6</v>
       </c>
       <c r="J5" t="n">
-        <v>39.7</v>
+        <v>33</v>
       </c>
       <c r="K5" t="n">
-        <v>15250</v>
+        <v>14939</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -3465,16 +3465,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1264364</v>
+        <v>1246987</v>
       </c>
       <c r="I6" t="n">
-        <v>-8.300000000000001</v>
+        <v>-8.1</v>
       </c>
       <c r="J6" t="n">
-        <v>51.9</v>
+        <v>50.2</v>
       </c>
       <c r="K6" t="n">
-        <v>110744</v>
+        <v>110772</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -3524,16 +3524,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>32444</v>
+        <v>32590</v>
       </c>
       <c r="I7" t="n">
-        <v>-26.5</v>
+        <v>-25.7</v>
       </c>
       <c r="J7" t="n">
-        <v>-75.8</v>
+        <v>-70.40000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>13974</v>
+        <v>14132</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -3583,16 +3583,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>110242</v>
+        <v>101710</v>
       </c>
       <c r="I8" t="n">
-        <v>1.7</v>
+        <v>-32.7</v>
       </c>
       <c r="J8" t="n">
-        <v>918.4</v>
+        <v>839.6</v>
       </c>
       <c r="K8" t="n">
-        <v>34736</v>
+        <v>33357</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -3642,16 +3642,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1559467</v>
+        <v>1556596</v>
       </c>
       <c r="I9" t="n">
-        <v>-10.1</v>
+        <v>-9</v>
       </c>
       <c r="J9" t="n">
         <v>-32.4</v>
       </c>
       <c r="K9" t="n">
-        <v>152429</v>
+        <v>152526</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -3701,16 +3701,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>42781</v>
+        <v>42043</v>
       </c>
       <c r="I10" t="n">
-        <v>-16.8</v>
+        <v>-18.9</v>
       </c>
       <c r="J10" t="n">
-        <v>-70.2</v>
+        <v>-70.7</v>
       </c>
       <c r="K10" t="n">
-        <v>18590</v>
+        <v>18396</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -3760,16 +3760,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>136972</v>
+        <v>147827</v>
       </c>
       <c r="I11" t="n">
-        <v>0.6</v>
+        <v>-4.8</v>
       </c>
       <c r="J11" t="n">
-        <v>-60.5</v>
+        <v>-54.6</v>
       </c>
       <c r="K11" t="n">
-        <v>51212</v>
+        <v>53235</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -3819,16 +3819,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3355044</v>
+        <v>3368951</v>
       </c>
       <c r="I12" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="J12" t="n">
-        <v>22.8</v>
+        <v>24</v>
       </c>
       <c r="K12" t="n">
-        <v>159870</v>
+        <v>160568</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -3878,16 +3878,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>52881</v>
+        <v>70049</v>
       </c>
       <c r="I13" t="n">
-        <v>32.2</v>
+        <v>71.2</v>
       </c>
       <c r="J13" t="n">
-        <v>849</v>
+        <v>1157.1</v>
       </c>
       <c r="K13" t="n">
-        <v>25054</v>
+        <v>28713</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -3937,16 +3937,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>123957184</v>
+        <v>124243718</v>
       </c>
       <c r="I14" t="n">
-        <v>2.2</v>
+        <v>1.8</v>
       </c>
       <c r="J14" t="n">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="K14" t="n">
-        <v>251640</v>
+        <v>252591</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -3996,16 +3996,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>354209360</v>
+        <v>353515370</v>
       </c>
       <c r="I15" t="n">
         <v>0.4</v>
       </c>
       <c r="J15" t="n">
-        <v>0.2</v>
+        <v>-0.1</v>
       </c>
       <c r="K15" t="n">
-        <v>2822421</v>
+        <v>2826212</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -4055,16 +4055,16 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>7266863</v>
+        <v>7277985</v>
       </c>
       <c r="I16" t="n">
-        <v>-6.4</v>
+        <v>-0.9</v>
       </c>
       <c r="J16" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="K16" t="n">
-        <v>342957</v>
+        <v>342914</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -4114,16 +4114,16 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>1236772</v>
+        <v>1239050</v>
       </c>
       <c r="I17" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="J17" t="n">
-        <v>-1.3</v>
+        <v>-1.1</v>
       </c>
       <c r="K17" t="n">
-        <v>267127</v>
+        <v>266857</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -4173,16 +4173,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>1016121</v>
+        <v>998947</v>
       </c>
       <c r="I18" t="n">
-        <v>-0.2</v>
+        <v>-3.3</v>
       </c>
       <c r="J18" t="n">
-        <v>65.40000000000001</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="K18" t="n">
-        <v>120438</v>
+        <v>119793</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -4232,16 +4232,16 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>331142</v>
+        <v>329110</v>
       </c>
       <c r="I19" t="n">
-        <v>2.4</v>
+        <v>1.7</v>
       </c>
       <c r="J19" t="n">
-        <v>25.2</v>
+        <v>24.5</v>
       </c>
       <c r="K19" t="n">
-        <v>64016</v>
+        <v>63800</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -4257,7 +4257,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>股票 meme · 代币化美股</t>
+          <t>持币分红盘 · ZCAT/BATON</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -4267,12 +4267,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>SCLAUDIA</t>
+          <t>ZCAT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -4282,7 +4282,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>8u6kqPWo694jKgEq4Nd5UynbVBnEhuLXMgnjGGMPpump</t>
+          <t>HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -4291,25 +4291,25 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>128540</v>
+        <v>54816284</v>
       </c>
       <c r="I20" t="n">
-        <v>4071.6</v>
+        <v>1</v>
       </c>
       <c r="J20" t="n">
-        <v>4071.6</v>
+        <v>26.3</v>
       </c>
       <c r="K20" t="n">
-        <v>33930</v>
+        <v>1266396</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Stonks Claudia（10/12 16:35 悉尼上线），名字命中「股票」关键词；叙事待人工核实。</t>
+          <t>Anonymous Cat：3% 交易税自动换 ZEC 分红给持有人，分红盘龙头。</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/8u6kqPWo694jKgEq4Nd5UynbVBnEhuLXMgnjGGMPpump</t>
+          <t>https://gmgn.ai/sol/token/HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
         </is>
       </c>
     </row>
@@ -4326,12 +4326,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ZCAT</t>
+          <t>BATON</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
+          <t>Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -4350,25 +4350,25 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>51237143</v>
+        <v>19024842</v>
       </c>
       <c r="I21" t="n">
-        <v>1.2</v>
+        <v>13.2</v>
       </c>
       <c r="J21" t="n">
-        <v>12.9</v>
+        <v>47.1</v>
       </c>
       <c r="K21" t="n">
-        <v>1226660</v>
+        <v>938716</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Anonymous Cat：3% 交易税自动换 ZEC 分红给持有人，分红盘龙头。</t>
+          <t>baton：分红 PUMP 的分红盘，ATH ~$19M，回调后第二腿。</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
+          <t>https://gmgn.ai/sol/token/Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
         </is>
       </c>
     </row>
@@ -4390,7 +4390,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>BATON</t>
+          <t>MCAT</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
+          <t>H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -4409,25 +4409,25 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>17572699</v>
+        <v>128432</v>
       </c>
       <c r="I22" t="n">
-        <v>2.9</v>
+        <v>6.2</v>
       </c>
       <c r="J22" t="n">
-        <v>37</v>
+        <v>-12.5</v>
       </c>
       <c r="K22" t="n">
-        <v>902270</v>
+        <v>32636</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>baton：分红 PUMP 的分红盘，ATH ~$19M，回调后第二腿。</t>
+          <t>Addicted Cat：分红门罗币 XMR，Cake Wallet 创始人买入。</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
+          <t>https://gmgn.ai/sol/token/H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
         </is>
       </c>
     </row>
@@ -4449,7 +4449,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>MCAT</t>
+          <t>FACTORY</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -4459,7 +4459,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
+          <t>7536qC4LEs3W2GtSKbhVGNJSiRfuXJhKVthxsgfkpump</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -4468,32 +4468,32 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>128432</v>
+        <v>47774</v>
       </c>
       <c r="I23" t="n">
-        <v>6.2</v>
+        <v>12.1</v>
       </c>
       <c r="J23" t="n">
-        <v>-12.5</v>
+        <v>-15.9</v>
       </c>
       <c r="K23" t="n">
-        <v>32636</v>
+        <v>18323</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Addicted Cat：分红门罗币 XMR，Cake Wallet 创始人买入。</t>
+          <t>🆕 GMGN 自动发现：Baton Factory（10/10 22:26 悉尼上线），名字命中「持币分红盘」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
+          <t>https://gmgn.ai/sol/token/7536qC4LEs3W2GtSKbhVGNJSiRfuXJhKVthxsgfkpump</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>持币分红盘 · ZCAT/BATON</t>
+          <t>ANSEM · SOL 老龙头</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4503,12 +4503,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>FACTORY</t>
+          <t>ANSEM</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -4518,7 +4518,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>7536qC4LEs3W2GtSKbhVGNJSiRfuXJhKVthxsgfkpump</t>
+          <t>9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -4527,32 +4527,32 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>44953</v>
+        <v>147114272</v>
       </c>
       <c r="I24" t="n">
-        <v>8.199999999999999</v>
+        <v>-1</v>
       </c>
       <c r="J24" t="n">
-        <v>-11.9</v>
+        <v>12.7</v>
       </c>
       <c r="K24" t="n">
-        <v>17636</v>
+        <v>2439624</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Baton Factory（10/10 22:26 悉尼上线），名字命中「持币分红盘」关键词；叙事待人工核实。</t>
+          <t>The Black Bull：Ansem 本人梗的 SOL 老龙头，15 万持有人，前十持仓 ~65% 偏集中。</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/7536qC4LEs3W2GtSKbhVGNJSiRfuXJhKVthxsgfkpump</t>
+          <t>https://gmgn.ai/sol/token/9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ANSEM · SOL 老龙头</t>
+          <t>以太坊近况 · Glamsterdam</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4567,17 +4567,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>ANSEM</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
+          <t>0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -4586,32 +4586,32 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>146987478</v>
+        <v>384153350</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.4</v>
+        <v>-0.5</v>
       </c>
       <c r="J25" t="n">
-        <v>12.8</v>
+        <v>3.6</v>
       </c>
       <c r="K25" t="n">
-        <v>2433857</v>
+        <v>11514103</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>The Black Bull：Ansem 本人梗的 SOL 老龙头，15 万持有人，前十持仓 ~65% 偏集中。</t>
+          <t>SPX6900：Murad 舞台喊“meme 将超越比特币”的 ETH 主网 meme 龙头。</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
+          <t>https://gmgn.ai/eth/token/0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>以太坊近况 · Glamsterdam</t>
+          <t>BSC 中文盘 · 币安人生</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4626,17 +4626,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>币安人生</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>eth</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
+          <t>0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -4645,25 +4645,25 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>384661770</v>
+        <v>612313770</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.9</v>
+        <v>-0.6</v>
       </c>
       <c r="J26" t="n">
-        <v>3.7</v>
+        <v>7.8</v>
       </c>
       <c r="K26" t="n">
-        <v>11516521</v>
+        <v>8955281</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>SPX6900：Murad 舞台喊“meme 将超越比特币”的 ETH 主网 meme 龙头。</t>
+          <t>币安人生：何一推文带火的 BSC 中文 meme 龙头，ATH ~$9 亿，现 ~$5.5 亿。</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/eth/token/0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
+          <t>https://gmgn.ai/bsc/token/0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
         </is>
       </c>
     </row>
@@ -4680,12 +4680,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>币安人生</t>
+          <t>龙虾</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
+          <t>0xeccbb861c0dda7efd964010085488b69317e4444</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -4704,25 +4704,25 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>608071390</v>
+        <v>41352174</v>
       </c>
       <c r="I27" t="n">
-        <v>-1.7</v>
+        <v>-1.8</v>
       </c>
       <c r="J27" t="n">
-        <v>7</v>
+        <v>-7.8</v>
       </c>
       <c r="K27" t="n">
-        <v>8912577</v>
+        <v>2020384</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>币安人生：何一推文带火的 BSC 中文 meme 龙头，ATH ~$9 亿，现 ~$5.5 亿。</t>
+          <t>龙虾：币安中文号推文出圈的中文盘，ATH ~$3.1 亿，现 ~$4300 万。注意今天有同名高仿盘。</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
+          <t>https://gmgn.ai/bsc/token/0xeccbb861c0dda7efd964010085488b69317e4444</t>
         </is>
       </c>
     </row>
@@ -4744,7 +4744,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>龙虾</t>
+          <t>币安圣羊</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -4754,7 +4754,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0xeccbb861c0dda7efd964010085488b69317e4444</t>
+          <t>0xcc4cc7ebaab40aa19317027b63e584333f697777</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -4763,25 +4763,25 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>41306591</v>
+        <v>303323</v>
       </c>
       <c r="I28" t="n">
-        <v>-1.9</v>
+        <v>-3.8</v>
       </c>
       <c r="J28" t="n">
-        <v>-7.7</v>
+        <v>-17.2</v>
       </c>
       <c r="K28" t="n">
-        <v>2017901</v>
+        <v>54486</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>龙虾：币安中文号推文出圈的中文盘，ATH ~$3.1 亿，现 ~$4300 万。注意今天有同名高仿盘。</t>
+          <t>🆕 GMGN 自动发现：币安圣羊（10/10 04:20 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0xeccbb861c0dda7efd964010085488b69317e4444</t>
+          <t>https://gmgn.ai/bsc/token/0xcc4cc7ebaab40aa19317027b63e584333f697777</t>
         </is>
       </c>
     </row>
@@ -4803,7 +4803,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>币安圣羊</t>
+          <t>币安人</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -4813,7 +4813,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0xcc4cc7ebaab40aa19317027b63e584333f697777</t>
+          <t>0x2c2d4298548ae585c224714555f18abde7367777</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -4822,32 +4822,32 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>303323</v>
+        <v>175791</v>
       </c>
       <c r="I29" t="n">
-        <v>-6.4</v>
+        <v>1.6</v>
       </c>
       <c r="J29" t="n">
-        <v>-17.6</v>
+        <v>-31.8</v>
       </c>
       <c r="K29" t="n">
-        <v>54486</v>
+        <v>41746</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：币安圣羊（10/10 04:20 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：Binance Man（10/10 22:33 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0xcc4cc7ebaab40aa19317027b63e584333f697777</t>
+          <t>https://gmgn.ai/bsc/token/0x2c2d4298548ae585c224714555f18abde7367777</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BSC 中文盘 · 币安人生</t>
+          <t>LAPTOP · 亨特·拜登盘</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4857,22 +4857,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>币安人</t>
+          <t>LAPTOP</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>bsc</t>
+          <t>base</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>0x2c2d4298548ae585c224714555f18abde7367777</t>
+          <t>0xb095274743941e953c746f9c228da9c18bb6ec29</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -4881,32 +4881,32 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>174241</v>
+        <v>74984117</v>
       </c>
       <c r="I30" t="n">
-        <v>2.5</v>
+        <v>-0.2</v>
       </c>
       <c r="J30" t="n">
-        <v>-32.8</v>
+        <v>-1.9</v>
       </c>
       <c r="K30" t="n">
-        <v>41510</v>
+        <v>254521</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Binance Man（10/10 22:33 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
+          <t>Hunter Biden 本人发的“笔记本电脑”梗币，前十持仓 ~91% 极度集中。</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x2c2d4298548ae585c224714555f18abde7367777</t>
+          <t>https://gmgn.ai/base/token/0xb095274743941e953c746f9c228da9c18bb6ec29</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>LAPTOP · 亨特·拜登盘</t>
+          <t>后量子地堡 · BNKR/PQC</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4921,17 +4921,17 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>LAPTOP</t>
+          <t>PQC</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0xb095274743941e953c746f9c228da9c18bb6ec29</t>
+          <t>7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -4940,25 +4940,25 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>75307374</v>
+        <v>343803</v>
       </c>
       <c r="I31" t="n">
-        <v>-0.1</v>
+        <v>-3.2</v>
       </c>
       <c r="J31" t="n">
-        <v>-1.2</v>
+        <v>-18.9</v>
       </c>
       <c r="K31" t="n">
-        <v>254789</v>
+        <v>70320</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Hunter Biden 本人发的“笔记本电脑”梗币，前十持仓 ~91% 极度集中。</t>
+          <t>pqc.market 平台币：后量子发射台，10/08 上线，24h 成交 ~$7.7M，BNKR 的母盘。</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/base/token/0xb095274743941e953c746f9c228da9c18bb6ec29</t>
+          <t>https://gmgn.ai/sol/token/7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
         </is>
       </c>
     </row>
@@ -4975,12 +4975,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>PQC</t>
+          <t>BUNKER</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -4990,7 +4990,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
+          <t>BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -4999,82 +4999,23 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>333671</v>
+        <v>218519</v>
       </c>
       <c r="I32" t="n">
-        <v>-5.2</v>
+        <v>16.2</v>
       </c>
       <c r="J32" t="n">
-        <v>-25</v>
+        <v>113.4</v>
       </c>
       <c r="K32" t="n">
-        <v>69558</v>
+        <v>41301</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>pqc.market 平台币：后量子发射台，10/08 上线，24h 成交 ~$7.7M，BNKR 的母盘。</t>
+          <t>🆕 GMGN 自动发现：Bunker Mode（10/10 10:14 悉尼上线），名字命中「后量子地堡」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
-        <is>
-          <t>https://gmgn.ai/sol/token/7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>后量子地堡 · BNKR/PQC</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>大周期</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>beta</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>BUNKER</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>sol</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>alive</t>
-        </is>
-      </c>
-      <c r="H33" t="n">
-        <v>216072</v>
-      </c>
-      <c r="I33" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="J33" t="n">
-        <v>109</v>
-      </c>
-      <c r="K33" t="n">
-        <v>40920</v>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>🆕 GMGN 自动发现：Bunker Mode（10/10 10:14 悉尼上线），名字命中「后量子地堡」关键词；叙事待人工核实。</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>https://gmgn.ai/sol/token/BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
         </is>
@@ -5113,7 +5054,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
radar silent 10/12 18:30
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -3274,7 +3274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M34"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3396,16 +3396,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>23850152</v>
+        <v>23809616</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.3</v>
+        <v>-1.9</v>
       </c>
       <c r="J2" t="n">
-        <v>-18.2</v>
+        <v>-21</v>
       </c>
       <c r="K2" t="n">
-        <v>867212</v>
+        <v>866780</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -3455,16 +3455,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1665576</v>
+        <v>1623613</v>
       </c>
       <c r="I3" t="n">
-        <v>-1.4</v>
+        <v>-0.4</v>
       </c>
       <c r="J3" t="n">
-        <v>14.2</v>
+        <v>20.5</v>
       </c>
       <c r="K3" t="n">
-        <v>183205</v>
+        <v>180026</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -3514,16 +3514,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>952353</v>
+        <v>925933</v>
       </c>
       <c r="I4" t="n">
-        <v>16</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>54.2</v>
+        <v>49.5</v>
       </c>
       <c r="K4" t="n">
-        <v>115023</v>
+        <v>113813</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>22351</v>
+        <v>22341</v>
       </c>
       <c r="I5" t="n">
-        <v>-13.8</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>60.2</v>
+        <v>69.7</v>
       </c>
       <c r="K5" t="n">
-        <v>14079</v>
+        <v>14057</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -3632,16 +3632,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1119663</v>
+        <v>1106702</v>
       </c>
       <c r="I6" t="n">
-        <v>-11.2</v>
+        <v>-3.1</v>
       </c>
       <c r="J6" t="n">
-        <v>46.4</v>
+        <v>41.3</v>
       </c>
       <c r="K6" t="n">
-        <v>104899</v>
+        <v>104151</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -3691,16 +3691,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>28191</v>
+        <v>34989</v>
       </c>
       <c r="I7" t="n">
-        <v>-10.5</v>
+        <v>12.2</v>
       </c>
       <c r="J7" t="n">
-        <v>-77.90000000000001</v>
+        <v>-60.6</v>
       </c>
       <c r="K7" t="n">
-        <v>12811</v>
+        <v>14731</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -3750,16 +3750,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>65082</v>
+        <v>65766</v>
       </c>
       <c r="I8" t="n">
-        <v>-32.2</v>
+        <v>-30.3</v>
       </c>
       <c r="J8" t="n">
-        <v>501.2</v>
+        <v>507.5</v>
       </c>
       <c r="K8" t="n">
-        <v>26636</v>
+        <v>26943</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -3809,16 +3809,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1517583</v>
+        <v>1504491</v>
       </c>
       <c r="I9" t="n">
-        <v>-2.9</v>
+        <v>-3</v>
       </c>
       <c r="J9" t="n">
-        <v>-23.6</v>
+        <v>-20.4</v>
       </c>
       <c r="K9" t="n">
-        <v>166479</v>
+        <v>165341</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -3868,16 +3868,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>43531</v>
+        <v>43410</v>
       </c>
       <c r="I10" t="n">
-        <v>3.2</v>
+        <v>1.4</v>
       </c>
       <c r="J10" t="n">
-        <v>-67.7</v>
+        <v>-66.90000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>18808</v>
+        <v>18754</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -3927,16 +3927,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>243112</v>
+        <v>243714</v>
       </c>
       <c r="I11" t="n">
-        <v>31.7</v>
+        <v>18.4</v>
       </c>
       <c r="J11" t="n">
-        <v>-21.6</v>
+        <v>-14.6</v>
       </c>
       <c r="K11" t="n">
-        <v>67319</v>
+        <v>67342</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -3986,16 +3986,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3356229</v>
+        <v>3393849</v>
       </c>
       <c r="I12" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="J12" t="n">
-        <v>23.3</v>
+        <v>23.6</v>
       </c>
       <c r="K12" t="n">
-        <v>160912</v>
+        <v>161030</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -4045,16 +4045,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>54021</v>
+        <v>61999</v>
       </c>
       <c r="I13" t="n">
-        <v>-34.7</v>
+        <v>-50.6</v>
       </c>
       <c r="J13" t="n">
-        <v>869.5</v>
+        <v>1012.7</v>
       </c>
       <c r="K13" t="n">
-        <v>25429</v>
+        <v>27245</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -4104,16 +4104,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>127951141</v>
+        <v>128548675</v>
       </c>
       <c r="I14" t="n">
-        <v>2.2</v>
+        <v>3.9</v>
       </c>
       <c r="J14" t="n">
-        <v>12.2</v>
+        <v>13.2</v>
       </c>
       <c r="K14" t="n">
-        <v>258081</v>
+        <v>259141</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -4163,16 +4163,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>350156470</v>
+        <v>353358480</v>
       </c>
       <c r="I15" t="n">
-        <v>0.5</v>
+        <v>1.9</v>
       </c>
       <c r="J15" t="n">
-        <v>-1.3</v>
+        <v>-0.4</v>
       </c>
       <c r="K15" t="n">
-        <v>2774763</v>
+        <v>2777066</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -4222,16 +4222,16 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>7013930</v>
+        <v>7028681</v>
       </c>
       <c r="I16" t="n">
-        <v>-3</v>
+        <v>-2.4</v>
       </c>
       <c r="J16" t="n">
-        <v>-2.5</v>
+        <v>-2.3</v>
       </c>
       <c r="K16" t="n">
-        <v>335777</v>
+        <v>335807</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -4281,16 +4281,16 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>1228114</v>
+        <v>1230158</v>
       </c>
       <c r="I17" t="n">
-        <v>-0.6</v>
+        <v>-0.4</v>
       </c>
       <c r="J17" t="n">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>266622</v>
+        <v>267017</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -4340,16 +4340,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>1110817</v>
+        <v>1077803</v>
       </c>
       <c r="I18" t="n">
-        <v>14.1</v>
+        <v>8.5</v>
       </c>
       <c r="J18" t="n">
-        <v>84.59999999999999</v>
+        <v>80.2</v>
       </c>
       <c r="K18" t="n">
-        <v>126748</v>
+        <v>124818</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -4399,16 +4399,16 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>333102</v>
+        <v>335496</v>
       </c>
       <c r="I19" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="J19" t="n">
-        <v>23</v>
+        <v>23.9</v>
       </c>
       <c r="K19" t="n">
-        <v>63953</v>
+        <v>64430</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -4458,16 +4458,16 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>54172649</v>
+        <v>53671386</v>
       </c>
       <c r="I20" t="n">
-        <v>0.6</v>
+        <v>3.8</v>
       </c>
       <c r="J20" t="n">
-        <v>24.6</v>
+        <v>20.1</v>
       </c>
       <c r="K20" t="n">
-        <v>1255004</v>
+        <v>1230000</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -4517,16 +4517,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>17762205</v>
+        <v>18060805</v>
       </c>
       <c r="I21" t="n">
-        <v>-4.9</v>
+        <v>-8.5</v>
       </c>
       <c r="J21" t="n">
-        <v>37</v>
+        <v>43.1</v>
       </c>
       <c r="K21" t="n">
-        <v>904020</v>
+        <v>908016</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -4582,7 +4582,7 @@
         <v>-0.1</v>
       </c>
       <c r="J22" t="n">
-        <v>-14.3</v>
+        <v>-8</v>
       </c>
       <c r="K22" t="n">
         <v>32520</v>
@@ -4635,16 +4635,16 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>67229</v>
+        <v>66069</v>
       </c>
       <c r="I23" t="n">
-        <v>37.7</v>
+        <v>36.1</v>
       </c>
       <c r="J23" t="n">
-        <v>29.5</v>
+        <v>38.6</v>
       </c>
       <c r="K23" t="n">
-        <v>22305</v>
+        <v>22244</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -4694,16 +4694,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>147590901</v>
+        <v>146988055</v>
       </c>
       <c r="I24" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="J24" t="n">
-        <v>13.1</v>
+        <v>12.7</v>
       </c>
       <c r="K24" t="n">
-        <v>2442552</v>
+        <v>2439437</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -4753,16 +4753,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>383787310</v>
+        <v>383332590</v>
       </c>
       <c r="I25" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="J25" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="K25" t="n">
-        <v>11541496</v>
+        <v>11527606</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -4812,16 +4812,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>607765110</v>
+        <v>602672280</v>
       </c>
       <c r="I26" t="n">
-        <v>0.5</v>
+        <v>-0.3</v>
       </c>
       <c r="J26" t="n">
-        <v>7.5</v>
+        <v>6.6</v>
       </c>
       <c r="K26" t="n">
-        <v>8940535</v>
+        <v>8895695</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -4871,16 +4871,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>41410753</v>
+        <v>41396449</v>
       </c>
       <c r="I27" t="n">
-        <v>-1.9</v>
+        <v>-0.3</v>
       </c>
       <c r="J27" t="n">
-        <v>-10</v>
+        <v>-9.9</v>
       </c>
       <c r="K27" t="n">
-        <v>2027760</v>
+        <v>2025493</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -4930,16 +4930,16 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>281920</v>
+        <v>280646</v>
       </c>
       <c r="I28" t="n">
-        <v>-0.9</v>
+        <v>-1.3</v>
       </c>
       <c r="J28" t="n">
-        <v>-1.4</v>
+        <v>-7</v>
       </c>
       <c r="K28" t="n">
-        <v>52547</v>
+        <v>52517</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -4989,16 +4989,16 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>167591</v>
+        <v>168419</v>
       </c>
       <c r="I29" t="n">
-        <v>-3.4</v>
+        <v>-3</v>
       </c>
       <c r="J29" t="n">
-        <v>-45.2</v>
+        <v>-40.7</v>
       </c>
       <c r="K29" t="n">
-        <v>41028</v>
+        <v>40894</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -5051,13 +5051,13 @@
         <v>75404470</v>
       </c>
       <c r="I30" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="J30" t="n">
         <v>0.7</v>
       </c>
       <c r="K30" t="n">
-        <v>253580</v>
+        <v>253319</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -5107,16 +5107,16 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>354706</v>
+        <v>348196</v>
       </c>
       <c r="I31" t="n">
-        <v>8</v>
+        <v>12.7</v>
       </c>
       <c r="J31" t="n">
-        <v>-22.6</v>
+        <v>-25.4</v>
       </c>
       <c r="K31" t="n">
-        <v>71958</v>
+        <v>71150</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -5166,16 +5166,16 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>184479</v>
+        <v>178865</v>
       </c>
       <c r="I32" t="n">
-        <v>-7.2</v>
+        <v>-3.4</v>
       </c>
       <c r="J32" t="n">
-        <v>89.3</v>
+        <v>84.5</v>
       </c>
       <c r="K32" t="n">
-        <v>37860</v>
+        <v>37195</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -5225,16 +5225,16 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>450487</v>
+        <v>422642</v>
       </c>
       <c r="I33" t="n">
         <v>-31.7</v>
       </c>
       <c r="J33" t="n">
-        <v>13122.8</v>
+        <v>12305.5</v>
       </c>
       <c r="K33" t="n">
-        <v>89731</v>
+        <v>92071</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -5284,16 +5284,16 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>10830</v>
+        <v>10444</v>
       </c>
       <c r="I34" t="n">
-        <v>-45.8</v>
+        <v>-41</v>
       </c>
       <c r="J34" t="n">
-        <v>219.5</v>
+        <v>208.1</v>
       </c>
       <c r="K34" t="n">
-        <v>13506</v>
+        <v>12296</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -5303,6 +5303,65 @@
       <c r="M34" s="2" t="inlineStr">
         <is>
           <t>https://gmgn.ai/sol/token/72WTP6f1k2dLpgW576Wkt3ZQY793sbLTxshZwrctpump</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Solamians · Solana 官方插画里的“国籍”</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Solamians</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>677hfbabdMDpv6GVagJ6FoDSvEr2hLJJKzr83TFsySQG</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>315686</v>
+      </c>
+      <c r="I35" t="n">
+        <v>111867980.9</v>
+      </c>
+      <c r="J35" t="n">
+        <v>111867980.9</v>
+      </c>
+      <c r="K35" t="n">
+        <v>65065</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>🆕 GMGN 自动发现：Solamians（10/12 17:36 悉尼上线），名字命中「Solamians」关键词；叙事待人工核实。</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/677hfbabdMDpv6GVagJ6FoDSvEr2hLJJKzr83TFsySQG</t>
         </is>
       </c>
     </row>
@@ -5341,6 +5400,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId34"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
radar 10/12 19:05 slopcaesar
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2375,6 +2375,111 @@
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>@Devon8zzh 原视频帖</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/Devon8zzh/status/2109507158790545903</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>@pmarca 转发记录</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/pmarca/status/2109527802194342355</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>@pmarca 10/11 转发 Devon 前作</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/pmarca/status/2109398097285861513</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>社区告知 Devon 手续费已划给他</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/solanashaka/status/2109532284848373933</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Devon：还在研究怎么领</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/Devon8zzh/status/2109548421078233180</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2447,6 +2552,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId74"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2458,7 +2568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2807,7 +2917,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>股票 meme · 代币化美股</t>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2816,47 +2926,47 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>↑</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>STONK</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Base 创始人 Token2049 站台 memestocks，有收入支撑；但讨论量 10/5 见顶后回落 → 龙头 STONK 低吸，不追 Base 小盘</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>4484</v>
-      </c>
-      <c r="I6" t="n">
-        <v>4215</v>
-      </c>
-      <c r="J6" t="n">
-        <v>6827</v>
-      </c>
+          <t>10/12：a16z 创始人 Marc Andreessen（@pmarca，660 万粉）转发 AI 创作者 @Devon8zzh 的 6 分钟 AI 短片《Slop Caesar》（已核实，他 10/11 也转过 Devon 的另一条）。社区盘 CAESAR 从 ~$1.4 万冲到 ATH ~$29 万后回到 ~$20 万；创作者尚未公开站台或领取手续费，讨论量已从峰值回落 → 观望，等创作者认领</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="n">
-        <v>3662</v>
+        <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>4273</v>
+        <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>3694</v>
+        <v>1</v>
       </c>
       <c r="N6" t="n">
-        <v>3672</v>
-      </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="O6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>424</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2864,7 +2974,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>持币分红盘 · ZCAT/BATON</t>
+          <t>股票 meme · 代币化美股</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2873,43 +2983,43 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>↑</t>
+          <t>↓</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>ZCAT</t>
+          <t>STONK</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>“持币吃 ZEC/PUMP/XMR 分红”玩法稳步升温，ZCAT 约 $50M 稳，BATON 走第二腿 → 最健康的一条线</t>
+          <t>Base 创始人 Token2049 站台 memestocks，有收入支撑；但讨论量 10/5 见顶后回落 → 龙头 STONK 低吸，不追 Base 小盘</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>910</v>
+        <v>4484</v>
       </c>
       <c r="I7" t="n">
-        <v>1410</v>
+        <v>4215</v>
       </c>
       <c r="J7" t="n">
-        <v>1630</v>
+        <v>6827</v>
       </c>
       <c r="K7" t="n">
-        <v>1788</v>
+        <v>3662</v>
       </c>
       <c r="L7" t="n">
-        <v>1338</v>
+        <v>4273</v>
       </c>
       <c r="M7" t="n">
-        <v>2103</v>
+        <v>3694</v>
       </c>
       <c r="N7" t="n">
-        <v>2047</v>
+        <v>3672</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
@@ -2921,7 +3031,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ANSEM · SOL 老龙头</t>
+          <t>持币分红盘 · ZCAT/BATON</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2934,39 +3044,39 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>→</t>
+          <t>↑</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>ANSEM</t>
+          <t>ZCAT</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>$142M、15 万持有人，讨论平稳略降 → 大盘情绪锚，不是新机会</t>
+          <t>“持币吃 ZEC/PUMP/XMR 分红”玩法稳步升温，ZCAT 约 $50M 稳，BATON 走第二腿 → 最健康的一条线</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>1459</v>
+        <v>910</v>
       </c>
       <c r="I8" t="n">
-        <v>2068</v>
+        <v>1410</v>
       </c>
       <c r="J8" t="n">
-        <v>2071</v>
+        <v>1630</v>
       </c>
       <c r="K8" t="n">
-        <v>2221</v>
+        <v>1788</v>
       </c>
       <c r="L8" t="n">
-        <v>2084</v>
+        <v>1338</v>
       </c>
       <c r="M8" t="n">
-        <v>1930</v>
+        <v>2103</v>
       </c>
       <c r="N8" t="n">
-        <v>2009</v>
+        <v>2047</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
@@ -2978,7 +3088,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>超级智能 SI · 🦉猫头鹰</t>
+          <t>ANSEM · SOL 老龙头</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2987,43 +3097,43 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>→</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>ANSEM</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>10/10 新增：Salesforce CEO Benioff 官宣 AIForce 改名 SIForce（原帖 35 万浏览，已核实），SI 叙事再获大公司背书；但龙头 Super Inu 6h 仍 -11%、约 $22M，市场暂未反应 → 等二次点火</t>
+          <t>$142M、15 万持有人，讨论平稳略降 → 大盘情绪锚，不是新机会</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>976</v>
+        <v>1459</v>
       </c>
       <c r="I9" t="n">
-        <v>2744</v>
+        <v>2068</v>
       </c>
       <c r="J9" t="n">
-        <v>3065</v>
+        <v>2071</v>
       </c>
       <c r="K9" t="n">
-        <v>1323</v>
+        <v>2221</v>
       </c>
       <c r="L9" t="n">
-        <v>638</v>
+        <v>2084</v>
       </c>
       <c r="M9" t="n">
-        <v>692</v>
+        <v>1930</v>
       </c>
       <c r="N9" t="n">
-        <v>663</v>
+        <v>2009</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
@@ -3035,7 +3145,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BSC 中文盘 · 币安人生</t>
+          <t>超级智能 SI · 🦉猫头鹰</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3044,43 +3154,43 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>→</t>
+          <t>↓</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>币安人生</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>讨论量 10/3 后持续下降、刷屏号多 → 冷却，暂不参与</t>
+          <t>10/10 新增：Salesforce CEO Benioff 官宣 AIForce 改名 SIForce（原帖 35 万浏览，已核实），SI 叙事再获大公司背书；但龙头 Super Inu 6h 仍 -11%、约 $22M，市场暂未反应 → 等二次点火</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>951</v>
+        <v>976</v>
       </c>
       <c r="I10" t="n">
-        <v>810</v>
+        <v>2744</v>
       </c>
       <c r="J10" t="n">
-        <v>529</v>
+        <v>3065</v>
       </c>
       <c r="K10" t="n">
-        <v>491</v>
+        <v>1323</v>
       </c>
       <c r="L10" t="n">
-        <v>351</v>
+        <v>638</v>
       </c>
       <c r="M10" t="n">
-        <v>354</v>
+        <v>692</v>
       </c>
       <c r="N10" t="n">
-        <v>579</v>
+        <v>663</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
@@ -3092,7 +3202,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>以太坊近况 · Glamsterdam</t>
+          <t>BSC 中文盘 · 币安人生</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3101,43 +3211,43 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>→</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>币安人生</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>技术/宏观新闻多（Glamsterdam 测试网、首笔原子 L1→L2、Abstract 关停），ETH ~$2,700 横盘，meme 热度低 → 只看 BURR 迁移</t>
+          <t>讨论量 10/3 后持续下降、刷屏号多 → 冷却，暂不参与</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>462</v>
+        <v>951</v>
       </c>
       <c r="I11" t="n">
-        <v>623</v>
+        <v>810</v>
       </c>
       <c r="J11" t="n">
-        <v>944</v>
+        <v>529</v>
       </c>
       <c r="K11" t="n">
-        <v>1721</v>
+        <v>491</v>
       </c>
       <c r="L11" t="n">
-        <v>1734</v>
+        <v>351</v>
       </c>
       <c r="M11" t="n">
-        <v>1117</v>
+        <v>354</v>
       </c>
       <c r="N11" t="n">
-        <v>1123</v>
+        <v>579</v>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
@@ -3149,7 +3259,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LAPTOP · 亨特·拜登盘</t>
+          <t>以太坊近况 · Glamsterdam</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -3158,43 +3268,43 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>↑</t>
+          <t>↓</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>LAPTOP</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>政治名人盘，曾 1 小时 -98%，10/7 报告后小反弹，但讨论多为刷票机器人 → 回避</t>
+          <t>技术/宏观新闻多（Glamsterdam 测试网、首笔原子 L1→L2、Abstract 关停），ETH ~$2,700 横盘，meme 热度低 → 只看 BURR 迁移</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>51</v>
+        <v>462</v>
       </c>
       <c r="I12" t="n">
-        <v>35</v>
+        <v>623</v>
       </c>
       <c r="J12" t="n">
-        <v>34</v>
+        <v>944</v>
       </c>
       <c r="K12" t="n">
-        <v>64</v>
+        <v>1721</v>
       </c>
       <c r="L12" t="n">
-        <v>595</v>
+        <v>1734</v>
       </c>
       <c r="M12" t="n">
-        <v>448</v>
+        <v>1117</v>
       </c>
       <c r="N12" t="n">
-        <v>384</v>
+        <v>1123</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
@@ -3206,7 +3316,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>后量子地堡 · BNKR/PQC</t>
+          <t>LAPTOP · 亨特·拜登盘</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3219,47 +3329,104 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
+          <t>↑</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>LAPTOP</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>政治名人盘，曾 1 小时 -98%，10/7 报告后小反弹，但讨论多为刷票机器人 → 回避</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>51</v>
+      </c>
+      <c r="I13" t="n">
+        <v>35</v>
+      </c>
+      <c r="J13" t="n">
+        <v>34</v>
+      </c>
+      <c r="K13" t="n">
+        <v>64</v>
+      </c>
+      <c r="L13" t="n">
+        <v>595</v>
+      </c>
+      <c r="M13" t="n">
+        <v>448</v>
+      </c>
+      <c r="N13" t="n">
+        <v>384</v>
+      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>后量子地堡 · BNKR/PQC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>25</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
           <t>↓</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>PQC</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>量子恐慌的第一个“产品化”玩法：pqc.market 发射台 + 官方 BNKR。X 讨论 2 天翻 4 倍，但 BNKR 已从 $420K 回撤到 ~$180K，PQC 是母盘</t>
         </is>
       </c>
-      <c r="H13" t="n">
+      <c r="H14" t="n">
         <v>392</v>
       </c>
-      <c r="I13" t="n">
+      <c r="I14" t="n">
         <v>243</v>
       </c>
-      <c r="J13" t="n">
+      <c r="J14" t="n">
         <v>303</v>
       </c>
-      <c r="K13" t="n">
+      <c r="K14" t="n">
         <v>282</v>
       </c>
-      <c r="L13" t="n">
+      <c r="L14" t="n">
         <v>564</v>
       </c>
-      <c r="M13" t="n">
+      <c r="M14" t="n">
         <v>1588</v>
       </c>
-      <c r="N13" t="n">
+      <c r="N14" t="n">
         <v>1463</v>
       </c>
-      <c r="O13" t="n">
+      <c r="O14" t="n">
         <v>728</v>
       </c>
-      <c r="P13" t="n">
+      <c r="P14" t="n">
         <v>587</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="Q14" t="n">
         <v>590</v>
       </c>
     </row>
@@ -3396,16 +3563,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>24651152</v>
+        <v>24406060</v>
       </c>
       <c r="I2" t="n">
-        <v>4.4</v>
+        <v>2.6</v>
       </c>
       <c r="J2" t="n">
-        <v>-17.1</v>
+        <v>-17.9</v>
       </c>
       <c r="K2" t="n">
-        <v>863316</v>
+        <v>869165</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -3455,16 +3622,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1569509</v>
+        <v>1568357</v>
       </c>
       <c r="I3" t="n">
-        <v>-6.5</v>
+        <v>-5.2</v>
       </c>
       <c r="J3" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="K3" t="n">
-        <v>176734</v>
+        <v>176459</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -3514,16 +3681,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>910720</v>
+        <v>903269</v>
       </c>
       <c r="I4" t="n">
-        <v>3.7</v>
+        <v>-0.9</v>
       </c>
       <c r="J4" t="n">
-        <v>47.1</v>
+        <v>45.9</v>
       </c>
       <c r="K4" t="n">
-        <v>112926</v>
+        <v>111821</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -3576,7 +3743,7 @@
         <v>20976</v>
       </c>
       <c r="I5" t="n">
-        <v>-8.300000000000001</v>
+        <v>-7.3</v>
       </c>
       <c r="J5" t="n">
         <v>36.2</v>
@@ -3632,16 +3799,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1068337</v>
+        <v>1073102</v>
       </c>
       <c r="I6" t="n">
-        <v>-3.6</v>
+        <v>-5.8</v>
       </c>
       <c r="J6" t="n">
-        <v>39.3</v>
+        <v>39.9</v>
       </c>
       <c r="K6" t="n">
-        <v>102248</v>
+        <v>102301</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -3691,16 +3858,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>32526</v>
+        <v>33002</v>
       </c>
       <c r="I7" t="n">
-        <v>23.1</v>
+        <v>26.1</v>
       </c>
       <c r="J7" t="n">
-        <v>-66.5</v>
+        <v>-66</v>
       </c>
       <c r="K7" t="n">
-        <v>14181</v>
+        <v>14174</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -3750,16 +3917,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>35610</v>
+        <v>47601</v>
       </c>
       <c r="I8" t="n">
-        <v>-59.3</v>
+        <v>-45.7</v>
       </c>
       <c r="J8" t="n">
-        <v>229</v>
+        <v>339.7</v>
       </c>
       <c r="K8" t="n">
-        <v>19908</v>
+        <v>22948</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -3809,16 +3976,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1484490</v>
+        <v>1462023</v>
       </c>
       <c r="I9" t="n">
-        <v>-4.1</v>
+        <v>-3.4</v>
       </c>
       <c r="J9" t="n">
-        <v>-20.8</v>
+        <v>-22</v>
       </c>
       <c r="K9" t="n">
-        <v>160029</v>
+        <v>159329</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -3927,16 +4094,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>212310</v>
+        <v>210216</v>
       </c>
       <c r="I11" t="n">
-        <v>-3.4</v>
+        <v>-4.4</v>
       </c>
       <c r="J11" t="n">
-        <v>-29.3</v>
+        <v>-29.9</v>
       </c>
       <c r="K11" t="n">
-        <v>62100</v>
+        <v>61962</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -3986,16 +4153,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3389721</v>
+        <v>3351981</v>
       </c>
       <c r="I12" t="n">
-        <v>0.3</v>
+        <v>-0.8</v>
       </c>
       <c r="J12" t="n">
-        <v>23.3</v>
+        <v>21.9</v>
       </c>
       <c r="K12" t="n">
-        <v>160657</v>
+        <v>160417</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -4045,16 +4212,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>51324</v>
+        <v>49661</v>
       </c>
       <c r="I13" t="n">
-        <v>-19.7</v>
+        <v>-16.5</v>
       </c>
       <c r="J13" t="n">
-        <v>821.1</v>
+        <v>791.2</v>
       </c>
       <c r="K13" t="n">
-        <v>24897</v>
+        <v>24404</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -4104,16 +4271,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>129731541</v>
+        <v>129718319</v>
       </c>
       <c r="I14" t="n">
-        <v>2.6</v>
+        <v>2.3</v>
       </c>
       <c r="J14" t="n">
         <v>15.3</v>
       </c>
       <c r="K14" t="n">
-        <v>262960</v>
+        <v>262013</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -4163,16 +4330,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>352497040</v>
+        <v>351591160</v>
       </c>
       <c r="I15" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="J15" t="n">
-        <v>-0.6</v>
+        <v>-0.8</v>
       </c>
       <c r="K15" t="n">
-        <v>2770202</v>
+        <v>2767567</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -4222,13 +4389,13 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>7010749</v>
+        <v>6988053</v>
       </c>
       <c r="I16" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="J16" t="n">
-        <v>-2.7</v>
+        <v>-3</v>
       </c>
       <c r="K16" t="n">
         <v>335807</v>
@@ -4340,16 +4507,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>1010340</v>
+        <v>983287</v>
       </c>
       <c r="I18" t="n">
-        <v>-9.300000000000001</v>
+        <v>-11.7</v>
       </c>
       <c r="J18" t="n">
-        <v>70.40000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="K18" t="n">
-        <v>120040</v>
+        <v>119626</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -4458,13 +4625,13 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>54833499</v>
+        <v>54687431</v>
       </c>
       <c r="I20" t="n">
-        <v>4.7</v>
+        <v>4.4</v>
       </c>
       <c r="J20" t="n">
-        <v>28.2</v>
+        <v>27.8</v>
       </c>
       <c r="K20" t="n">
         <v>1257285</v>
@@ -4517,16 +4684,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>17745248</v>
+        <v>17701862</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.2</v>
+        <v>-1.5</v>
       </c>
       <c r="J21" t="n">
-        <v>32.6</v>
+        <v>32.3</v>
       </c>
       <c r="K21" t="n">
-        <v>901720</v>
+        <v>901505</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -4694,16 +4861,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>144571</v>
+        <v>180364</v>
       </c>
       <c r="I24" t="n">
-        <v>4568.9</v>
+        <v>5724.8</v>
       </c>
       <c r="J24" t="n">
-        <v>4568.9</v>
+        <v>5724.8</v>
       </c>
       <c r="K24" t="n">
-        <v>35993</v>
+        <v>40092</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -4753,16 +4920,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>146194316</v>
+        <v>145895487</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.6</v>
+        <v>-0.5</v>
       </c>
       <c r="J25" t="n">
-        <v>11.9</v>
+        <v>11.7</v>
       </c>
       <c r="K25" t="n">
-        <v>2430480</v>
+        <v>2424210</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -4812,16 +4979,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>383092120</v>
+        <v>381892100</v>
       </c>
       <c r="I26" t="n">
-        <v>0.1</v>
+        <v>-0.3</v>
       </c>
       <c r="J26" t="n">
-        <v>3</v>
+        <v>2.6</v>
       </c>
       <c r="K26" t="n">
-        <v>11490358</v>
+        <v>11460436</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -4871,16 +5038,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>595328650</v>
+        <v>595118710</v>
       </c>
       <c r="I27" t="n">
-        <v>-1.2</v>
+        <v>-1</v>
       </c>
       <c r="J27" t="n">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="K27" t="n">
-        <v>8827146</v>
+        <v>8822080</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -4930,16 +5097,16 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>41207691</v>
+        <v>41040954</v>
       </c>
       <c r="I28" t="n">
         <v>-0.4</v>
       </c>
       <c r="J28" t="n">
-        <v>-8.6</v>
+        <v>-9</v>
       </c>
       <c r="K28" t="n">
-        <v>2017067</v>
+        <v>2013115</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -4989,16 +5156,16 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>281000</v>
+        <v>276738</v>
       </c>
       <c r="I29" t="n">
-        <v>-0.6</v>
+        <v>-2.1</v>
       </c>
       <c r="J29" t="n">
-        <v>-12.5</v>
+        <v>-13.8</v>
       </c>
       <c r="K29" t="n">
-        <v>52516</v>
+        <v>52047</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -5048,16 +5215,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>162185</v>
+        <v>157773</v>
       </c>
       <c r="I30" t="n">
-        <v>-4.7</v>
+        <v>-7.3</v>
       </c>
       <c r="J30" t="n">
-        <v>-33.8</v>
+        <v>-35.6</v>
       </c>
       <c r="K30" t="n">
-        <v>40096</v>
+        <v>39528</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -5107,16 +5274,16 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>75303746</v>
+        <v>75182083</v>
       </c>
       <c r="I31" t="n">
-        <v>0.9</v>
+        <v>-0.2</v>
       </c>
       <c r="J31" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="K31" t="n">
-        <v>253618</v>
+        <v>253640</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -5166,16 +5333,16 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>322359</v>
+        <v>325717</v>
       </c>
       <c r="I32" t="n">
-        <v>-4.3</v>
+        <v>-4.2</v>
       </c>
       <c r="J32" t="n">
-        <v>-21.4</v>
+        <v>-20.6</v>
       </c>
       <c r="K32" t="n">
-        <v>68176</v>
+        <v>68115</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -5225,16 +5392,16 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>177605</v>
+        <v>177132</v>
       </c>
       <c r="I33" t="n">
-        <v>-4.4</v>
+        <v>-3.9</v>
       </c>
       <c r="J33" t="n">
-        <v>95</v>
+        <v>94.5</v>
       </c>
       <c r="K33" t="n">
-        <v>37027</v>
+        <v>36892</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -5284,16 +5451,16 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>413950</v>
+        <v>378491</v>
       </c>
       <c r="I34" t="n">
-        <v>-21.7</v>
+        <v>-20.8</v>
       </c>
       <c r="J34" t="n">
-        <v>12050.4</v>
+        <v>11009.6</v>
       </c>
       <c r="K34" t="n">
-        <v>79397</v>
+        <v>72277</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -5343,16 +5510,16 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>293853</v>
+        <v>277202</v>
       </c>
       <c r="I35" t="n">
-        <v>-42.7</v>
+        <v>-6.8</v>
       </c>
       <c r="J35" t="n">
-        <v>104131051.6</v>
+        <v>98230656.3</v>
       </c>
       <c r="K35" t="n">
-        <v>71114</v>
+        <v>66169</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
radar 10/12 19:08 slopcaesar coin
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -2935,7 +2935,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAESAR</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -3441,7 +3441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M35"/>
+  <dimension ref="A1:M36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3563,16 +3563,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>24406060</v>
+        <v>24569467</v>
       </c>
       <c r="I2" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="J2" t="n">
-        <v>-17.9</v>
+        <v>-17.4</v>
       </c>
       <c r="K2" t="n">
-        <v>869165</v>
+        <v>867856</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -3622,16 +3622,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1568357</v>
+        <v>1569687</v>
       </c>
       <c r="I3" t="n">
-        <v>-5.2</v>
+        <v>-4.9</v>
       </c>
       <c r="J3" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="K3" t="n">
-        <v>176459</v>
+        <v>176363</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -3681,16 +3681,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>903269</v>
+        <v>857043</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.9</v>
+        <v>-8</v>
       </c>
       <c r="J4" t="n">
-        <v>45.9</v>
+        <v>38.4</v>
       </c>
       <c r="K4" t="n">
-        <v>111821</v>
+        <v>109529</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -3740,16 +3740,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>20976</v>
+        <v>20814</v>
       </c>
       <c r="I5" t="n">
-        <v>-7.3</v>
+        <v>-8</v>
       </c>
       <c r="J5" t="n">
-        <v>36.2</v>
+        <v>35.2</v>
       </c>
       <c r="K5" t="n">
-        <v>13645</v>
+        <v>13603</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -3799,16 +3799,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1073102</v>
+        <v>1068341</v>
       </c>
       <c r="I6" t="n">
-        <v>-5.8</v>
+        <v>-4.6</v>
       </c>
       <c r="J6" t="n">
-        <v>39.9</v>
+        <v>39.3</v>
       </c>
       <c r="K6" t="n">
-        <v>102301</v>
+        <v>102032</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -3858,16 +3858,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>33002</v>
+        <v>32429</v>
       </c>
       <c r="I7" t="n">
-        <v>26.1</v>
+        <v>23.6</v>
       </c>
       <c r="J7" t="n">
-        <v>-66</v>
+        <v>-66.59999999999999</v>
       </c>
       <c r="K7" t="n">
-        <v>14174</v>
+        <v>14140</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -3917,16 +3917,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>47601</v>
+        <v>48516</v>
       </c>
       <c r="I8" t="n">
-        <v>-45.7</v>
+        <v>-44.8</v>
       </c>
       <c r="J8" t="n">
-        <v>339.7</v>
+        <v>348.2</v>
       </c>
       <c r="K8" t="n">
-        <v>22948</v>
+        <v>23194</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -3976,16 +3976,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1462023</v>
+        <v>1479568</v>
       </c>
       <c r="I9" t="n">
-        <v>-3.4</v>
+        <v>-1.3</v>
       </c>
       <c r="J9" t="n">
-        <v>-22</v>
+        <v>-21.1</v>
       </c>
       <c r="K9" t="n">
-        <v>159329</v>
+        <v>159396</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -4038,7 +4038,7 @@
         <v>42621</v>
       </c>
       <c r="I10" t="n">
-        <v>1.5</v>
+        <v>3.9</v>
       </c>
       <c r="J10" t="n">
         <v>-64</v>
@@ -4094,16 +4094,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>210216</v>
+        <v>211019</v>
       </c>
       <c r="I11" t="n">
-        <v>-4.4</v>
+        <v>-4.3</v>
       </c>
       <c r="J11" t="n">
-        <v>-29.9</v>
+        <v>-29.7</v>
       </c>
       <c r="K11" t="n">
-        <v>61962</v>
+        <v>61824</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -4153,16 +4153,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3351981</v>
+        <v>3383824</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.8</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>21.9</v>
+        <v>23.1</v>
       </c>
       <c r="K12" t="n">
-        <v>160417</v>
+        <v>160422</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -4212,16 +4212,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>49661</v>
+        <v>49464</v>
       </c>
       <c r="I13" t="n">
-        <v>-16.5</v>
+        <v>-7.2</v>
       </c>
       <c r="J13" t="n">
-        <v>791.2</v>
+        <v>787.7</v>
       </c>
       <c r="K13" t="n">
-        <v>24404</v>
+        <v>24401</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -4271,16 +4271,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>129718319</v>
+        <v>128968245</v>
       </c>
       <c r="I14" t="n">
-        <v>2.3</v>
+        <v>-0.1</v>
       </c>
       <c r="J14" t="n">
-        <v>15.3</v>
+        <v>14.6</v>
       </c>
       <c r="K14" t="n">
-        <v>262013</v>
+        <v>260988</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -4330,16 +4330,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>351591160</v>
+        <v>351908700</v>
       </c>
       <c r="I15" t="n">
         <v>0.3</v>
       </c>
       <c r="J15" t="n">
-        <v>-0.8</v>
+        <v>-0.7</v>
       </c>
       <c r="K15" t="n">
-        <v>2767567</v>
+        <v>2767061</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -4389,13 +4389,13 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>6988053</v>
+        <v>7013383</v>
       </c>
       <c r="I16" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="J16" t="n">
-        <v>-3</v>
+        <v>-2.7</v>
       </c>
       <c r="K16" t="n">
         <v>335807</v>
@@ -4507,16 +4507,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>983287</v>
+        <v>979765</v>
       </c>
       <c r="I18" t="n">
-        <v>-11.7</v>
+        <v>-12.8</v>
       </c>
       <c r="J18" t="n">
-        <v>65.8</v>
+        <v>65.2</v>
       </c>
       <c r="K18" t="n">
-        <v>119626</v>
+        <v>118475</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -4566,16 +4566,16 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>325387</v>
+        <v>324056</v>
       </c>
       <c r="I19" t="n">
-        <v>-1.3</v>
+        <v>-1.7</v>
       </c>
       <c r="J19" t="n">
-        <v>19.7</v>
+        <v>19.2</v>
       </c>
       <c r="K19" t="n">
-        <v>63074</v>
+        <v>62884</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -4625,16 +4625,16 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>54687431</v>
+        <v>53033976</v>
       </c>
       <c r="I20" t="n">
-        <v>4.4</v>
+        <v>1.1</v>
       </c>
       <c r="J20" t="n">
-        <v>27.8</v>
+        <v>24</v>
       </c>
       <c r="K20" t="n">
-        <v>1257285</v>
+        <v>1255482</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -4684,16 +4684,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>17701862</v>
+        <v>17702785</v>
       </c>
       <c r="I21" t="n">
-        <v>-1.5</v>
+        <v>-0.8</v>
       </c>
       <c r="J21" t="n">
         <v>32.3</v>
       </c>
       <c r="K21" t="n">
-        <v>901505</v>
+        <v>897087</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -4805,7 +4805,7 @@
         <v>59111</v>
       </c>
       <c r="I23" t="n">
-        <v>-8.6</v>
+        <v>-10.8</v>
       </c>
       <c r="J23" t="n">
         <v>17.8</v>
@@ -4861,16 +4861,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>180364</v>
+        <v>183745</v>
       </c>
       <c r="I24" t="n">
-        <v>5724.8</v>
+        <v>5834</v>
       </c>
       <c r="J24" t="n">
-        <v>5724.8</v>
+        <v>5834</v>
       </c>
       <c r="K24" t="n">
-        <v>40092</v>
+        <v>41059</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -4920,16 +4920,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>145895487</v>
+        <v>145817583</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.5</v>
+        <v>-0.8</v>
       </c>
       <c r="J25" t="n">
         <v>11.7</v>
       </c>
       <c r="K25" t="n">
-        <v>2424210</v>
+        <v>2424998</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -4979,16 +4979,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>381892100</v>
+        <v>380721530</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.3</v>
+        <v>-0.6</v>
       </c>
       <c r="J26" t="n">
-        <v>2.6</v>
+        <v>2.3</v>
       </c>
       <c r="K26" t="n">
-        <v>11460436</v>
+        <v>11459917</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -5038,16 +5038,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>595118710</v>
+        <v>595017660</v>
       </c>
       <c r="I27" t="n">
-        <v>-1</v>
+        <v>-1.2</v>
       </c>
       <c r="J27" t="n">
         <v>4.4</v>
       </c>
       <c r="K27" t="n">
-        <v>8822080</v>
+        <v>8821210</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -5097,16 +5097,16 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>41040954</v>
+        <v>41081106</v>
       </c>
       <c r="I28" t="n">
-        <v>-0.4</v>
+        <v>-0.6</v>
       </c>
       <c r="J28" t="n">
-        <v>-9</v>
+        <v>-8.9</v>
       </c>
       <c r="K28" t="n">
-        <v>2013115</v>
+        <v>2013910</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -5156,7 +5156,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>276738</v>
+        <v>276853</v>
       </c>
       <c r="I29" t="n">
         <v>-2.1</v>
@@ -5165,7 +5165,7 @@
         <v>-13.8</v>
       </c>
       <c r="K29" t="n">
-        <v>52047</v>
+        <v>52061</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -5215,16 +5215,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>157773</v>
+        <v>157573</v>
       </c>
       <c r="I30" t="n">
-        <v>-7.3</v>
+        <v>-7.4</v>
       </c>
       <c r="J30" t="n">
         <v>-35.6</v>
       </c>
       <c r="K30" t="n">
-        <v>39528</v>
+        <v>39500</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -5283,7 +5283,7 @@
         <v>0.4</v>
       </c>
       <c r="K31" t="n">
-        <v>253640</v>
+        <v>253654</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -5333,16 +5333,16 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>325717</v>
+        <v>325120</v>
       </c>
       <c r="I32" t="n">
-        <v>-4.2</v>
+        <v>-4.3</v>
       </c>
       <c r="J32" t="n">
-        <v>-20.6</v>
+        <v>-20.7</v>
       </c>
       <c r="K32" t="n">
-        <v>68115</v>
+        <v>68154</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -5392,16 +5392,16 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>177132</v>
+        <v>176522</v>
       </c>
       <c r="I33" t="n">
-        <v>-3.9</v>
+        <v>-4.2</v>
       </c>
       <c r="J33" t="n">
-        <v>94.5</v>
+        <v>93.8</v>
       </c>
       <c r="K33" t="n">
-        <v>36892</v>
+        <v>36846</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -5451,16 +5451,16 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>378491</v>
+        <v>369642</v>
       </c>
       <c r="I34" t="n">
-        <v>-20.8</v>
+        <v>-20.9</v>
       </c>
       <c r="J34" t="n">
-        <v>11009.6</v>
+        <v>10749.8</v>
       </c>
       <c r="K34" t="n">
-        <v>72277</v>
+        <v>73115</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -5510,16 +5510,16 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>277202</v>
+        <v>272236</v>
       </c>
       <c r="I35" t="n">
-        <v>-6.8</v>
+        <v>-22.5</v>
       </c>
       <c r="J35" t="n">
-        <v>98230656.3</v>
+        <v>96470888.40000001</v>
       </c>
       <c r="K35" t="n">
-        <v>66169</v>
+        <v>66027</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -5529,6 +5529,65 @@
       <c r="M35" s="2" t="inlineStr">
         <is>
           <t>https://gmgn.ai/sol/token/677hfbabdMDpv6GVagJ6FoDSvEr2hLJJKzr83TFsySQG</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>龙头</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>CAESAR</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>183682</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J36" t="n">
+        <v>4744.5</v>
+      </c>
+      <c r="K36" t="n">
+        <v>37362</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>pmarca 转发的 AI 短片《Slop Caesar》社区盘（转发已核实，pmarca 没提币）。开发者已清仓、批量发币地址；机器人约 66%；创作者 Devon 未认领手续费。</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
         </is>
       </c>
     </row>
@@ -5568,6 +5627,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId35"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
radar silent 10/12 19:18
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2480,6 +2480,48 @@
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr"/>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Devon：比我一年存的还多（引用 1.2 万手续费帖）</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/Devon8zzh/status/2109555248457228716</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr"/>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>社区帖：CAESAR 手续费约 1.2 万美元待领（未核实）</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/TheRealM0nkii/status/2109555562946150806</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2557,6 +2599,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2940,7 +2984,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10/12：a16z 创始人 Marc Andreessen（@pmarca，660 万粉）转发 AI 创作者 @Devon8zzh 的 6 分钟 AI 短片《Slop Caesar》（已核实，他 10/11 也转过 Devon 的另一条）。社区盘 CAESAR 从 ~$1.4 万冲到 ATH ~$29 万后回到 ~$20 万；创作者尚未公开站台或领取手续费，讨论量已从峰值回落 → 观望，等创作者认领</t>
+          <t>10/12：a16z 创始人 Marc Andreessen（@pmarca）转发 AI 创作者 @Devon8zzh 的 AI 短片《Slop Caesar》（已核实）。19:00 后 Devon 连发十几条回应社区：引用“CAESAR 盘已为你攒了约 1.2 万美元手续费”的帖子说“比我一年存的还多”、“够做 8 支虾视频”，但仍说“等我搞明白怎么领”，截至 19:15 未见领取或明确认领某个 CA（1.2 万这个数字来自社区账号，未核实）。帖子浏览仅千级，热度没有新一轮放大 → 继续观望，等他真正领取手续费或点名 CA</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -3441,7 +3485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3563,16 +3607,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>24569467</v>
+        <v>24451521</v>
       </c>
       <c r="I2" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="J2" t="n">
-        <v>-17.4</v>
+        <v>-19.9</v>
       </c>
       <c r="K2" t="n">
-        <v>867856</v>
+        <v>866265</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -3622,16 +3666,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1569687</v>
+        <v>1568560</v>
       </c>
       <c r="I3" t="n">
-        <v>-4.9</v>
+        <v>-6.7</v>
       </c>
       <c r="J3" t="n">
-        <v>11.6</v>
+        <v>13.2</v>
       </c>
       <c r="K3" t="n">
-        <v>176363</v>
+        <v>177156</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -3681,16 +3725,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>857043</v>
+        <v>840812</v>
       </c>
       <c r="I4" t="n">
-        <v>-8</v>
+        <v>-12.2</v>
       </c>
       <c r="J4" t="n">
-        <v>38.4</v>
+        <v>32.3</v>
       </c>
       <c r="K4" t="n">
-        <v>109529</v>
+        <v>107868</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -3740,16 +3784,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>20814</v>
+        <v>20995</v>
       </c>
       <c r="I5" t="n">
-        <v>-8</v>
+        <v>-6.8</v>
       </c>
       <c r="J5" t="n">
-        <v>35.2</v>
+        <v>56.6</v>
       </c>
       <c r="K5" t="n">
-        <v>13603</v>
+        <v>13661</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -3799,16 +3843,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1068341</v>
+        <v>1073123</v>
       </c>
       <c r="I6" t="n">
-        <v>-4.6</v>
+        <v>-4.1</v>
       </c>
       <c r="J6" t="n">
-        <v>39.3</v>
+        <v>29</v>
       </c>
       <c r="K6" t="n">
-        <v>102032</v>
+        <v>102154</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -3858,16 +3902,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>32429</v>
+        <v>32903</v>
       </c>
       <c r="I7" t="n">
-        <v>23.6</v>
+        <v>15.5</v>
       </c>
       <c r="J7" t="n">
-        <v>-66.59999999999999</v>
+        <v>-64.3</v>
       </c>
       <c r="K7" t="n">
-        <v>14140</v>
+        <v>14149</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -3917,16 +3961,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>48516</v>
+        <v>39390</v>
       </c>
       <c r="I8" t="n">
-        <v>-44.8</v>
+        <v>-42.6</v>
       </c>
       <c r="J8" t="n">
-        <v>348.2</v>
+        <v>263.9</v>
       </c>
       <c r="K8" t="n">
-        <v>23194</v>
+        <v>20880</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -3976,16 +4020,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1479568</v>
+        <v>1464975</v>
       </c>
       <c r="I9" t="n">
-        <v>-1.3</v>
+        <v>-3.4</v>
       </c>
       <c r="J9" t="n">
-        <v>-21.1</v>
+        <v>-25.5</v>
       </c>
       <c r="K9" t="n">
-        <v>159396</v>
+        <v>158597</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -4035,16 +4079,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>42621</v>
+        <v>41773</v>
       </c>
       <c r="I10" t="n">
-        <v>3.9</v>
+        <v>-4</v>
       </c>
       <c r="J10" t="n">
-        <v>-64</v>
+        <v>-65.09999999999999</v>
       </c>
       <c r="K10" t="n">
-        <v>18488</v>
+        <v>18162</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -4094,16 +4138,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>211019</v>
+        <v>182568</v>
       </c>
       <c r="I11" t="n">
-        <v>-4.3</v>
+        <v>-24.7</v>
       </c>
       <c r="J11" t="n">
-        <v>-29.7</v>
+        <v>-35.2</v>
       </c>
       <c r="K11" t="n">
-        <v>61824</v>
+        <v>57814</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -4153,16 +4197,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3383824</v>
+        <v>3356812</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>-0.8</v>
       </c>
       <c r="J12" t="n">
-        <v>23.1</v>
+        <v>21.9</v>
       </c>
       <c r="K12" t="n">
-        <v>160422</v>
+        <v>160189</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -4212,16 +4256,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>49464</v>
+        <v>64446</v>
       </c>
       <c r="I13" t="n">
-        <v>-7.2</v>
+        <v>19.4</v>
       </c>
       <c r="J13" t="n">
-        <v>787.7</v>
+        <v>1056.6</v>
       </c>
       <c r="K13" t="n">
-        <v>24401</v>
+        <v>27793</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -4271,16 +4315,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>128968245</v>
+        <v>128089786</v>
       </c>
       <c r="I14" t="n">
-        <v>-0.1</v>
+        <v>0.5</v>
       </c>
       <c r="J14" t="n">
-        <v>14.6</v>
+        <v>14.7</v>
       </c>
       <c r="K14" t="n">
-        <v>260988</v>
+        <v>260597</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -4330,16 +4374,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>351908700</v>
+        <v>351323140</v>
       </c>
       <c r="I15" t="n">
         <v>0.3</v>
       </c>
       <c r="J15" t="n">
-        <v>-0.7</v>
+        <v>-1</v>
       </c>
       <c r="K15" t="n">
-        <v>2767061</v>
+        <v>2759036</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -4389,16 +4433,16 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>7013383</v>
+        <v>7018125</v>
       </c>
       <c r="I16" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="J16" t="n">
-        <v>-2.7</v>
+        <v>-1.9</v>
       </c>
       <c r="K16" t="n">
-        <v>335807</v>
+        <v>335938</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -4448,16 +4492,16 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>1250227</v>
+        <v>1251334</v>
       </c>
       <c r="I17" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="J17" t="n">
         <v>1.6</v>
       </c>
       <c r="K17" t="n">
-        <v>268298</v>
+        <v>268100</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -4507,16 +4551,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>979765</v>
+        <v>980736</v>
       </c>
       <c r="I18" t="n">
-        <v>-12.8</v>
+        <v>-10.1</v>
       </c>
       <c r="J18" t="n">
-        <v>65.2</v>
+        <v>65.8</v>
       </c>
       <c r="K18" t="n">
-        <v>118475</v>
+        <v>118493</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -4566,16 +4610,16 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>324056</v>
+        <v>318565</v>
       </c>
       <c r="I19" t="n">
-        <v>-1.7</v>
+        <v>-4.4</v>
       </c>
       <c r="J19" t="n">
-        <v>19.2</v>
+        <v>17.2</v>
       </c>
       <c r="K19" t="n">
-        <v>62884</v>
+        <v>62873</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -4625,16 +4669,16 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>53033976</v>
+        <v>51909286</v>
       </c>
       <c r="I20" t="n">
-        <v>1.1</v>
+        <v>-1.1</v>
       </c>
       <c r="J20" t="n">
-        <v>24</v>
+        <v>21.6</v>
       </c>
       <c r="K20" t="n">
-        <v>1255482</v>
+        <v>1221593</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -4684,16 +4728,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>17702785</v>
+        <v>16874304</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.8</v>
+        <v>-5</v>
       </c>
       <c r="J21" t="n">
-        <v>32.3</v>
+        <v>24.6</v>
       </c>
       <c r="K21" t="n">
-        <v>897087</v>
+        <v>876035</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -4802,16 +4846,16 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>59111</v>
+        <v>58138</v>
       </c>
       <c r="I23" t="n">
-        <v>-10.8</v>
+        <v>-10.4</v>
       </c>
       <c r="J23" t="n">
-        <v>17.8</v>
+        <v>20.1</v>
       </c>
       <c r="K23" t="n">
-        <v>20685</v>
+        <v>20392</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -4861,16 +4905,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>183745</v>
+        <v>210074</v>
       </c>
       <c r="I24" t="n">
-        <v>5834</v>
+        <v>6684.2</v>
       </c>
       <c r="J24" t="n">
-        <v>5834</v>
+        <v>6684.2</v>
       </c>
       <c r="K24" t="n">
-        <v>41059</v>
+        <v>47709</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -4920,16 +4964,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>145817583</v>
+        <v>145207357</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.8</v>
+        <v>-1</v>
       </c>
       <c r="J25" t="n">
-        <v>11.7</v>
+        <v>10.7</v>
       </c>
       <c r="K25" t="n">
-        <v>2424998</v>
+        <v>2414841</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -4979,16 +5023,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>380721530</v>
+        <v>378963730</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.6</v>
+        <v>-1.3</v>
       </c>
       <c r="J26" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="K26" t="n">
-        <v>11459917</v>
+        <v>11420540</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -5038,16 +5082,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>595017660</v>
+        <v>593208070</v>
       </c>
       <c r="I27" t="n">
-        <v>-1.2</v>
+        <v>-2.3</v>
       </c>
       <c r="J27" t="n">
-        <v>4.4</v>
+        <v>4.1</v>
       </c>
       <c r="K27" t="n">
-        <v>8821210</v>
+        <v>8803078</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -5097,16 +5141,16 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>41081106</v>
+        <v>41016387</v>
       </c>
       <c r="I28" t="n">
-        <v>-0.6</v>
+        <v>-0.2</v>
       </c>
       <c r="J28" t="n">
-        <v>-8.9</v>
+        <v>-6.9</v>
       </c>
       <c r="K28" t="n">
-        <v>2013910</v>
+        <v>2010500</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -5156,16 +5200,16 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>276853</v>
+        <v>267320</v>
       </c>
       <c r="I29" t="n">
-        <v>-2.1</v>
+        <v>-4.9</v>
       </c>
       <c r="J29" t="n">
-        <v>-13.8</v>
+        <v>-16.9</v>
       </c>
       <c r="K29" t="n">
-        <v>52061</v>
+        <v>51158</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -5215,16 +5259,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>157573</v>
+        <v>151241</v>
       </c>
       <c r="I30" t="n">
-        <v>-7.4</v>
+        <v>-10.7</v>
       </c>
       <c r="J30" t="n">
-        <v>-35.6</v>
+        <v>-38.7</v>
       </c>
       <c r="K30" t="n">
-        <v>39500</v>
+        <v>38677</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -5240,7 +5284,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>LAPTOP · 亨特·拜登盘</t>
+          <t>BSC 中文盘 · 币安人生</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5250,22 +5294,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>LAPTOP</t>
+          <t>Binance Angels</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0xb095274743941e953c746f9c228da9c18bb6ec29</t>
+          <t>0x62bb38c83afeb82e8f468d122b1b9051b6167777</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -5274,32 +5318,32 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>75182083</v>
+        <v>65272</v>
       </c>
       <c r="I31" t="n">
-        <v>-0.2</v>
+        <v>1370.5</v>
       </c>
       <c r="J31" t="n">
-        <v>0.4</v>
+        <v>1224.1</v>
       </c>
       <c r="K31" t="n">
-        <v>253654</v>
+        <v>24260</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Hunter Biden 本人发的“笔记本电脑”梗币，前十持仓 ~91% 极度集中。</t>
+          <t>🆕 GMGN 自动发现：QQ:945497833（10/12 19:12 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/base/token/0xb095274743941e953c746f9c228da9c18bb6ec29</t>
+          <t>https://gmgn.ai/bsc/token/0x62bb38c83afeb82e8f468d122b1b9051b6167777</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>后量子地堡 · BNKR/PQC</t>
+          <t>LAPTOP · 亨特·拜登盘</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5314,17 +5358,17 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>PQC</t>
+          <t>LAPTOP</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>base</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
+          <t>0xb095274743941e953c746f9c228da9c18bb6ec29</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -5333,25 +5377,25 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>325120</v>
+        <v>75502860</v>
       </c>
       <c r="I32" t="n">
-        <v>-4.3</v>
+        <v>0.1</v>
       </c>
       <c r="J32" t="n">
-        <v>-20.7</v>
+        <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>68154</v>
+        <v>253855</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>pqc.market 平台币：后量子发射台，10/08 上线，24h 成交 ~$7.7M，BNKR 的母盘。</t>
+          <t>Hunter Biden 本人发的“笔记本电脑”梗币，前十持仓 ~91% 极度集中。</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
+          <t>https://gmgn.ai/base/token/0xb095274743941e953c746f9c228da9c18bb6ec29</t>
         </is>
       </c>
     </row>
@@ -5368,12 +5412,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>BUNKER</t>
+          <t>PQC</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -5383,7 +5427,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
+          <t>7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -5392,47 +5436,47 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>176522</v>
+        <v>328000</v>
       </c>
       <c r="I33" t="n">
-        <v>-4.2</v>
+        <v>-8.9</v>
       </c>
       <c r="J33" t="n">
-        <v>93.8</v>
+        <v>-23.9</v>
       </c>
       <c r="K33" t="n">
-        <v>36846</v>
+        <v>68746</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Bunker Mode（10/10 10:14 悉尼上线），名字命中「后量子地堡」关键词；叙事待人工核实。</t>
+          <t>pqc.market 平台币：后量子发射台，10/08 上线，24h 成交 ~$7.7M，BNKR 的母盘。</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
+          <t>https://gmgn.ai/sol/token/7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Solamians · Solana 官方插画里的“国籍”</t>
+          <t>后量子地堡 · BNKR/PQC</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>24小时</t>
+          <t>大周期</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Solamians</t>
+          <t>BUNKER</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -5442,7 +5486,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>8ZP5CzbPL1fmP8dn1GEmLd8xw1JdudUF5Dk7EpLxpump</t>
+          <t>BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -5451,25 +5495,25 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>369642</v>
+        <v>176635</v>
       </c>
       <c r="I34" t="n">
-        <v>-20.9</v>
+        <v>-4.2</v>
       </c>
       <c r="J34" t="n">
-        <v>10749.8</v>
+        <v>98.2</v>
       </c>
       <c r="K34" t="n">
-        <v>73115</v>
+        <v>36789</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Solana 官方 Breakpoint 指南护照插画写着 Nationality: Solamian（已核实原图）。10/12 13:09 创建，ATH ~$910K，机器人成交约 57%。</t>
+          <t>🆕 GMGN 自动发现：Bunker Mode（10/10 10:14 悉尼上线），名字命中「后量子地堡」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/8ZP5CzbPL1fmP8dn1GEmLd8xw1JdudUF5Dk7EpLxpump</t>
+          <t>https://gmgn.ai/sol/token/BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5530,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -5501,7 +5545,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>677hfbabdMDpv6GVagJ6FoDSvEr2hLJJKzr83TFsySQG</t>
+          <t>8ZP5CzbPL1fmP8dn1GEmLd8xw1JdudUF5Dk7EpLxpump</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -5510,84 +5554,202 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>272236</v>
+        <v>375533</v>
       </c>
       <c r="I35" t="n">
-        <v>-22.5</v>
+        <v>-13.1</v>
       </c>
       <c r="J35" t="n">
-        <v>96470888.40000001</v>
+        <v>10922.8</v>
       </c>
       <c r="K35" t="n">
-        <v>66027</v>
+        <v>73037</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Solamians（10/12 17:36 悉尼上线），名字命中「Solamians」关键词；叙事待人工核实。</t>
+          <t>Solana 官方 Breakpoint 指南护照插画写着 Nationality: Solamian（已核实原图）。10/12 13:09 创建，ATH ~$910K，机器人成交约 57%。</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/677hfbabdMDpv6GVagJ6FoDSvEr2hLJJKzr83TFsySQG</t>
+          <t>https://gmgn.ai/sol/token/8ZP5CzbPL1fmP8dn1GEmLd8xw1JdudUF5Dk7EpLxpump</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>Solamians · Solana 官方插画里的“国籍”</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Solamians</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>677hfbabdMDpv6GVagJ6FoDSvEr2hLJJKzr83TFsySQG</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>250724</v>
+      </c>
+      <c r="I36" t="n">
+        <v>-37.8</v>
+      </c>
+      <c r="J36" t="n">
+        <v>88847642.8</v>
+      </c>
+      <c r="K36" t="n">
+        <v>66226</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>🆕 GMGN 自动发现：Solamians（10/12 17:36 悉尼上线），名字命中「Solamians」关键词；叙事待人工核实。</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/677hfbabdMDpv6GVagJ6FoDSvEr2hLJJKzr83TFsySQG</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>24小时</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>龙头</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>CAESAR</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>sol</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>alive</t>
         </is>
       </c>
-      <c r="H36" t="n">
-        <v>183682</v>
-      </c>
-      <c r="I36" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="J36" t="n">
-        <v>4744.5</v>
-      </c>
-      <c r="K36" t="n">
-        <v>37362</v>
-      </c>
-      <c r="L36" t="inlineStr">
+      <c r="H37" t="n">
+        <v>218088</v>
+      </c>
+      <c r="I37" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="J37" t="n">
+        <v>5651.9</v>
+      </c>
+      <c r="K37" t="n">
+        <v>41982</v>
+      </c>
+      <c r="L37" t="inlineStr">
         <is>
           <t>pmarca 转发的 AI 短片《Slop Caesar》社区盘（转发已核实，pmarca 没提币）。开发者已清仓、批量发币地址；机器人约 66%；创作者 Devon 未认领手续费。</t>
         </is>
       </c>
-      <c r="M36" s="2" t="inlineStr">
+      <c r="M37" s="2" t="inlineStr">
         <is>
           <t>https://gmgn.ai/sol/token/EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>CAESAR</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>EUTas4zV2UYrfCqEsPXFvuX5uhexwUuzDCCBkptih3MS</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H38" t="n">
+        <v>92225</v>
+      </c>
+      <c r="I38" t="n">
+        <v>88.3</v>
+      </c>
+      <c r="J38" t="n">
+        <v>862.5</v>
+      </c>
+      <c r="K38" t="n">
+        <v>62316</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>🆕 GMGN 自动发现：Slop Caesar（10/12 17:50 悉尼上线），名字命中「Slop」关键词；叙事待人工核实。</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/EUTas4zV2UYrfCqEsPXFvuX5uhexwUuzDCCBkptih3MS</t>
         </is>
       </c>
     </row>
@@ -5628,6 +5790,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
radar 10/12 19:31 caesar fee claim
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2522,6 +2522,69 @@
       </c>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Devon 贴出 CA（19:24）</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/Devon8zzh/status/2109560849610522736</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr"/>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Devon：108.07 SOL（19:26）</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/Devon8zzh/status/2109561327723458614</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr"/>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Devon 截图 I found the button</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/Devon8zzh/status/2109561610268553597</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2601,6 +2664,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId79"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2984,7 +3050,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10/12：a16z 创始人 Marc Andreessen（@pmarca）转发 AI 创作者 @Devon8zzh 的 AI 短片《Slop Caesar》（已核实）。19:00 后 Devon 连发十几条回应社区：引用“CAESAR 盘已为你攒了约 1.2 万美元手续费”的帖子说“比我一年存的还多”、“够做 8 支虾视频”，但仍说“等我搞明白怎么领”，截至 19:15 未见领取或明确认领某个 CA（1.2 万这个数字来自社区账号，未核实）。帖子浏览仅千级，热度没有新一轮放大 → 继续观望，等他真正领取手续费或点名 CA</t>
+          <t>10/12：pmarca 转发 AI 创作者 @Devon8zzh 的《Slop Caesar》（已核实）。19:24 Devon 本人发帖贴出 EaqX… CA 并问“Is this right?”，19:26 问“108.07 SOL 算多吗”，截图显示“I found the button”（自称已领手续费，X 原帖已核实）；GMGN 显示 EaqX 盘 100% 创作者分成指向 GitHub 账号 devonmvfisher 且已领取（GitHub 号与 X 号是否同一人未核实，但该号有 passage 仓库）。截图同时显示有人在私信教他喊单、“先别领其他盘”。讨论量在降（14 点档 244 帖 → 15 点档 148 → 19:00–19:30 约 51），19:30 盘子约 $164K、1h -3%，市场暂未反应</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -5685,7 +5751,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>pmarca 转发的 AI 短片《Slop Caesar》社区盘（转发已核实，pmarca 没提币）。开发者已清仓、批量发币地址；机器人约 66%；创作者 Devon 未认领手续费。</t>
+          <t>pmarca 转发的《Slop Caesar》社区盘。19:24 Devon 本人贴出此 CA，自称已领约 108 SOL 手续费（GMGN：分成 100% 给 devonmvfisher，已领取）。原开发者已清仓、批量发币地址；机器人约 62%。</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">

</xml_diff>

<commit_message>
radar silent 10/12 19:55 gta6 cyberleek
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2585,6 +2585,111 @@
       </c>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr"/>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Kotaku：泄露者 3000 万市值威胁（引用 10/10 原文）</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>https://kotaku.com/gta-6-leaker-threatens-rockstar-with-doomsday-scenario-if-meme-coin-hits-30-million-2000743779</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr"/>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Yahoo Finance：CYBERLEEK 24h 涨 273%</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/markets/crypto/articles/solana-meme-coin-tied-gta-150454094.html</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr"/>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Dotesports：8 月提走约 25 万美元手续费</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>https://dotesports.com/gta/news/cyberleek-gta-6-full-build-ultimatum</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr"/>
+      <c r="B84" t="inlineStr"/>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Seeking Alpha 推文</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/SeekingAlpha/status/2109436393017807208</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr"/>
+      <c r="B85" t="inlineStr"/>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>@robtmb1：泄露视频里的 Dacity Coin（未核实）</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/robtmb1/status/2109241600002118071</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2667,6 +2772,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId84"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2678,7 +2788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2970,7 +3080,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Solamians · Solana 官方插画里的“国籍”</t>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2979,7 +3089,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -2988,37 +3098,37 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Solamians</t>
+          <t>CYBERLEEK</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>10/12 新梗：Solana 官方 Breakpoint 指南插画护照上写着 Republic of Solami / Sola / Nationality: Solamian（已核实原图）。但这是 9/29 就发布的旧插画被重新挖出，不是新消息；官方和大号未下场，龙头已从高点回撤约 3 成 → 观望不追</t>
+          <t>10/10 泄露者 Cyberleek 在自家网站发《The Offer》：CYBERLEEK 市值到 3000 万美元就放出 GTA 6 完整剧情版，Take-Two 出实体光盘并公开道歉可免（已核实：Kotaku、Yahoo Finance、Dotesports、Tom's Hardware 均引用原文；我未直接打开其网站）。完整版是否真的存在无法核实。币 10/11 冲到约 $8M 后回落，10/12 19:50 约 $2.9M、24h -53%；讨论量从 10/11 晚高峰约 600 帖/小时降到约 170。属于已发酵两天的旧叙事，未推送，只观察。</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>663</v>
       </c>
       <c r="L5" t="n">
-        <v>1</v>
+        <v>685</v>
       </c>
       <c r="M5" t="n">
-        <v>1</v>
+        <v>7520</v>
       </c>
       <c r="N5" t="n">
-        <v>1</v>
+        <v>4595</v>
       </c>
       <c r="O5" t="n">
-        <v>1</v>
+        <v>4765</v>
       </c>
       <c r="P5" t="n">
-        <v>1</v>
+        <v>6928</v>
       </c>
       <c r="Q5" t="n">
-        <v>854</v>
+        <v>6205</v>
       </c>
     </row>
     <row r="6">
@@ -3027,7 +3137,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+          <t>Solamians · Solana 官方插画里的“国籍”</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3036,7 +3146,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -3045,12 +3155,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>CAESAR</t>
+          <t>Solamians</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10/12：pmarca 转发 AI 创作者 @Devon8zzh 的《Slop Caesar》（已核实）。19:24 Devon 本人发帖贴出 EaqX… CA 并问“Is this right?”，19:26 问“108.07 SOL 算多吗”，截图显示“I found the button”（自称已领手续费，X 原帖已核实）；GMGN 显示 EaqX 盘 100% 创作者分成指向 GitHub 账号 devonmvfisher 且已领取（GitHub 号与 X 号是否同一人未核实，但该号有 passage 仓库）。截图同时显示有人在私信教他喊单、“先别领其他盘”。讨论量在降（17 点档 244 帖 → 18 点档 148 → 19:00–19:30 约 51），19:30 盘子约 $164K、1h -3%，市场暂未反应</t>
+          <t>10/12 新梗：Solana 官方 Breakpoint 指南插画护照上写着 Republic of Solami / Sola / Nationality: Solamian（已核实原图）。但这是 9/29 就发布的旧插画被重新挖出，不是新消息；官方和大号未下场，龙头已从高点回撤约 3 成 → 观望不追</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -3075,7 +3185,7 @@
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>424</v>
+        <v>854</v>
       </c>
     </row>
     <row r="7">
@@ -3084,7 +3194,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>股票 meme · 代币化美股</t>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3093,47 +3203,47 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>↑</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>STONK</t>
+          <t>CAESAR</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Base 创始人 Token2049 站台 memestocks，有收入支撑；但讨论量 10/5 见顶后回落 → 龙头 STONK 低吸，不追 Base 小盘</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>4484</v>
-      </c>
-      <c r="I7" t="n">
-        <v>4215</v>
-      </c>
-      <c r="J7" t="n">
-        <v>6827</v>
-      </c>
+          <t>10/12：pmarca 转发 AI 创作者 @Devon8zzh 的《Slop Caesar》（已核实）。19:24 Devon 本人发帖贴出 EaqX… CA 并问“Is this right?”，19:26 问“108.07 SOL 算多吗”，截图显示“I found the button”（自称已领手续费，X 原帖已核实）；GMGN 显示 EaqX 盘 100% 创作者分成指向 GitHub 账号 devonmvfisher 且已领取（GitHub 号与 X 号是否同一人未核实，但该号有 passage 仓库）。截图同时显示有人在私信教他喊单、“先别领其他盘”。讨论量在降（17 点档 244 帖 → 18 点档 148 → 19:00–19:30 约 51），19:30 盘子约 $164K、1h -3%，市场暂未反应</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
-        <v>3662</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>4273</v>
+        <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>3694</v>
+        <v>1</v>
       </c>
       <c r="N7" t="n">
-        <v>3672</v>
-      </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>424</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -3141,7 +3251,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>持币分红盘 · ZCAT/BATON</t>
+          <t>股票 meme · 代币化美股</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3150,43 +3260,43 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>↑</t>
+          <t>↓</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>ZCAT</t>
+          <t>STONK</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>“持币吃 ZEC/PUMP/XMR 分红”玩法稳步升温，ZCAT 约 $50M 稳，BATON 走第二腿 → 最健康的一条线</t>
+          <t>Base 创始人 Token2049 站台 memestocks，有收入支撑；但讨论量 10/5 见顶后回落 → 龙头 STONK 低吸，不追 Base 小盘</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>910</v>
+        <v>4484</v>
       </c>
       <c r="I8" t="n">
-        <v>1410</v>
+        <v>4215</v>
       </c>
       <c r="J8" t="n">
-        <v>1630</v>
+        <v>6827</v>
       </c>
       <c r="K8" t="n">
-        <v>1788</v>
+        <v>3662</v>
       </c>
       <c r="L8" t="n">
-        <v>1338</v>
+        <v>4273</v>
       </c>
       <c r="M8" t="n">
-        <v>2103</v>
+        <v>3694</v>
       </c>
       <c r="N8" t="n">
-        <v>2047</v>
+        <v>3672</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
@@ -3198,7 +3308,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ANSEM · SOL 老龙头</t>
+          <t>持币分红盘 · ZCAT/BATON</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -3211,39 +3321,39 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>→</t>
+          <t>↑</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ANSEM</t>
+          <t>ZCAT</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>$142M、15 万持有人，讨论平稳略降 → 大盘情绪锚，不是新机会</t>
+          <t>“持币吃 ZEC/PUMP/XMR 分红”玩法稳步升温，ZCAT 约 $50M 稳，BATON 走第二腿 → 最健康的一条线</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1459</v>
+        <v>910</v>
       </c>
       <c r="I9" t="n">
-        <v>2068</v>
+        <v>1410</v>
       </c>
       <c r="J9" t="n">
-        <v>2071</v>
+        <v>1630</v>
       </c>
       <c r="K9" t="n">
-        <v>2221</v>
+        <v>1788</v>
       </c>
       <c r="L9" t="n">
-        <v>2084</v>
+        <v>1338</v>
       </c>
       <c r="M9" t="n">
-        <v>1930</v>
+        <v>2103</v>
       </c>
       <c r="N9" t="n">
-        <v>2009</v>
+        <v>2047</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
@@ -3255,7 +3365,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>超级智能 SI · 🦉猫头鹰</t>
+          <t>ANSEM · SOL 老龙头</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3264,43 +3374,43 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>→</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>ANSEM</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>10/10 新增：Salesforce CEO Benioff 官宣 AIForce 改名 SIForce（原帖 35 万浏览，已核实），SI 叙事再获大公司背书；但龙头 Super Inu 6h 仍 -11%、约 $22M，市场暂未反应 → 等二次点火</t>
+          <t>$142M、15 万持有人，讨论平稳略降 → 大盘情绪锚，不是新机会</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>976</v>
+        <v>1459</v>
       </c>
       <c r="I10" t="n">
-        <v>2744</v>
+        <v>2068</v>
       </c>
       <c r="J10" t="n">
-        <v>3065</v>
+        <v>2071</v>
       </c>
       <c r="K10" t="n">
-        <v>1323</v>
+        <v>2221</v>
       </c>
       <c r="L10" t="n">
-        <v>638</v>
+        <v>2084</v>
       </c>
       <c r="M10" t="n">
-        <v>692</v>
+        <v>1930</v>
       </c>
       <c r="N10" t="n">
-        <v>663</v>
+        <v>2009</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
@@ -3312,7 +3422,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BSC 中文盘 · 币安人生</t>
+          <t>超级智能 SI · 🦉猫头鹰</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3321,43 +3431,43 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>→</t>
+          <t>↓</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>币安人生</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>讨论量 10/3 后持续下降、刷屏号多 → 冷却，暂不参与</t>
+          <t>10/10 新增：Salesforce CEO Benioff 官宣 AIForce 改名 SIForce（原帖 35 万浏览，已核实），SI 叙事再获大公司背书；但龙头 Super Inu 6h 仍 -11%、约 $22M，市场暂未反应 → 等二次点火</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>951</v>
+        <v>976</v>
       </c>
       <c r="I11" t="n">
-        <v>810</v>
+        <v>2744</v>
       </c>
       <c r="J11" t="n">
-        <v>529</v>
+        <v>3065</v>
       </c>
       <c r="K11" t="n">
-        <v>491</v>
+        <v>1323</v>
       </c>
       <c r="L11" t="n">
-        <v>351</v>
+        <v>638</v>
       </c>
       <c r="M11" t="n">
-        <v>354</v>
+        <v>692</v>
       </c>
       <c r="N11" t="n">
-        <v>579</v>
+        <v>663</v>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
@@ -3369,7 +3479,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>以太坊近况 · Glamsterdam</t>
+          <t>BSC 中文盘 · 币安人生</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -3378,43 +3488,43 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>→</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>币安人生</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>技术/宏观新闻多（Glamsterdam 测试网、首笔原子 L1→L2、Abstract 关停），ETH ~$2,700 横盘，meme 热度低 → 只看 BURR 迁移</t>
+          <t>讨论量 10/3 后持续下降、刷屏号多 → 冷却，暂不参与</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>462</v>
+        <v>951</v>
       </c>
       <c r="I12" t="n">
-        <v>623</v>
+        <v>810</v>
       </c>
       <c r="J12" t="n">
-        <v>944</v>
+        <v>529</v>
       </c>
       <c r="K12" t="n">
-        <v>1721</v>
+        <v>491</v>
       </c>
       <c r="L12" t="n">
-        <v>1734</v>
+        <v>351</v>
       </c>
       <c r="M12" t="n">
-        <v>1117</v>
+        <v>354</v>
       </c>
       <c r="N12" t="n">
-        <v>1123</v>
+        <v>579</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
@@ -3426,7 +3536,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>LAPTOP · 亨特·拜登盘</t>
+          <t>以太坊近况 · Glamsterdam</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3435,43 +3545,43 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>↑</t>
+          <t>↓</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>LAPTOP</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>政治名人盘，曾 1 小时 -98%，10/7 报告后小反弹，但讨论多为刷票机器人 → 回避</t>
+          <t>技术/宏观新闻多（Glamsterdam 测试网、首笔原子 L1→L2、Abstract 关停），ETH ~$2,700 横盘，meme 热度低 → 只看 BURR 迁移</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>51</v>
+        <v>462</v>
       </c>
       <c r="I13" t="n">
-        <v>35</v>
+        <v>623</v>
       </c>
       <c r="J13" t="n">
-        <v>34</v>
+        <v>944</v>
       </c>
       <c r="K13" t="n">
-        <v>64</v>
+        <v>1721</v>
       </c>
       <c r="L13" t="n">
-        <v>595</v>
+        <v>1734</v>
       </c>
       <c r="M13" t="n">
-        <v>448</v>
+        <v>1117</v>
       </c>
       <c r="N13" t="n">
-        <v>384</v>
+        <v>1123</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
@@ -3483,7 +3593,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>后量子地堡 · BNKR/PQC</t>
+          <t>LAPTOP · 亨特·拜登盘</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -3496,47 +3606,104 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>↑</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>LAPTOP</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>政治名人盘，曾 1 小时 -98%，10/7 报告后小反弹，但讨论多为刷票机器人 → 回避</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>51</v>
+      </c>
+      <c r="I14" t="n">
+        <v>35</v>
+      </c>
+      <c r="J14" t="n">
+        <v>34</v>
+      </c>
+      <c r="K14" t="n">
+        <v>64</v>
+      </c>
+      <c r="L14" t="n">
+        <v>595</v>
+      </c>
+      <c r="M14" t="n">
+        <v>448</v>
+      </c>
+      <c r="N14" t="n">
+        <v>384</v>
+      </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>后量子地堡 · BNKR/PQC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>25</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
           <t>↓</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>PQC</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>量子恐慌的第一个“产品化”玩法：pqc.market 发射台 + 官方 BNKR。X 讨论 2 天翻 4 倍，但 BNKR 已从 $420K 回撤到 ~$180K，PQC 是母盘</t>
         </is>
       </c>
-      <c r="H14" t="n">
+      <c r="H15" t="n">
         <v>392</v>
       </c>
-      <c r="I14" t="n">
+      <c r="I15" t="n">
         <v>243</v>
       </c>
-      <c r="J14" t="n">
+      <c r="J15" t="n">
         <v>303</v>
       </c>
-      <c r="K14" t="n">
+      <c r="K15" t="n">
         <v>282</v>
       </c>
-      <c r="L14" t="n">
+      <c r="L15" t="n">
         <v>564</v>
       </c>
-      <c r="M14" t="n">
+      <c r="M15" t="n">
         <v>1588</v>
       </c>
-      <c r="N14" t="n">
+      <c r="N15" t="n">
         <v>1463</v>
       </c>
-      <c r="O14" t="n">
+      <c r="O15" t="n">
         <v>728</v>
       </c>
-      <c r="P14" t="n">
+      <c r="P15" t="n">
         <v>587</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="Q15" t="n">
         <v>590</v>
       </c>
     </row>
@@ -3551,7 +3718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3673,16 +3840,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>24507339</v>
+        <v>24530555</v>
       </c>
       <c r="I2" t="n">
-        <v>4.8</v>
+        <v>0.3</v>
       </c>
       <c r="J2" t="n">
-        <v>-19.7</v>
+        <v>-19.2</v>
       </c>
       <c r="K2" t="n">
-        <v>858196</v>
+        <v>863330</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -3732,16 +3899,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1525887</v>
+        <v>1550137</v>
       </c>
       <c r="I3" t="n">
-        <v>-10</v>
+        <v>-2.4</v>
       </c>
       <c r="J3" t="n">
-        <v>10.1</v>
+        <v>11.8</v>
       </c>
       <c r="K3" t="n">
-        <v>173505</v>
+        <v>175626</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -3791,16 +3958,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>783502</v>
+        <v>774852</v>
       </c>
       <c r="I4" t="n">
-        <v>-16.2</v>
+        <v>-22.3</v>
       </c>
       <c r="J4" t="n">
-        <v>23.3</v>
+        <v>1.7</v>
       </c>
       <c r="K4" t="n">
-        <v>104675</v>
+        <v>106121</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -3850,16 +4017,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>20852</v>
+        <v>20784</v>
       </c>
       <c r="I5" t="n">
-        <v>-6.7</v>
+        <v>0.1</v>
       </c>
       <c r="J5" t="n">
-        <v>55.5</v>
+        <v>38.3</v>
       </c>
       <c r="K5" t="n">
-        <v>13587</v>
+        <v>13564</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -3909,16 +4076,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1072943</v>
+        <v>1093507</v>
       </c>
       <c r="I6" t="n">
-        <v>-3.8</v>
+        <v>2.2</v>
       </c>
       <c r="J6" t="n">
-        <v>29</v>
+        <v>12.9</v>
       </c>
       <c r="K6" t="n">
-        <v>102019</v>
+        <v>103148</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -3968,16 +4135,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>33406</v>
+        <v>31849</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.8</v>
+        <v>-6</v>
       </c>
       <c r="J7" t="n">
-        <v>-63.8</v>
+        <v>-63.1</v>
       </c>
       <c r="K7" t="n">
-        <v>14253</v>
+        <v>13993</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -4027,16 +4194,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>50877</v>
+        <v>40239</v>
       </c>
       <c r="I8" t="n">
-        <v>-17.7</v>
+        <v>-25.8</v>
       </c>
       <c r="J8" t="n">
-        <v>370</v>
+        <v>23.9</v>
       </c>
       <c r="K8" t="n">
-        <v>23857</v>
+        <v>20980</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -4086,16 +4253,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1465568</v>
+        <v>1470386</v>
       </c>
       <c r="I9" t="n">
-        <v>-3.1</v>
+        <v>-2.9</v>
       </c>
       <c r="J9" t="n">
-        <v>-25.5</v>
+        <v>-24.6</v>
       </c>
       <c r="K9" t="n">
-        <v>158108</v>
+        <v>169663</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -4145,16 +4312,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>41773</v>
+        <v>40724</v>
       </c>
       <c r="I10" t="n">
-        <v>-3.8</v>
+        <v>-7.9</v>
       </c>
       <c r="J10" t="n">
-        <v>-65.09999999999999</v>
+        <v>-64.40000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>18162</v>
+        <v>18002</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -4204,16 +4371,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>179020</v>
+        <v>196453</v>
       </c>
       <c r="I11" t="n">
-        <v>-26.4</v>
+        <v>-6.4</v>
       </c>
       <c r="J11" t="n">
-        <v>-36.5</v>
+        <v>-29.7</v>
       </c>
       <c r="K11" t="n">
-        <v>57118</v>
+        <v>59976</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -4263,16 +4430,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3387978</v>
+        <v>3357369</v>
       </c>
       <c r="I12" t="n">
         <v>-0.1</v>
       </c>
       <c r="J12" t="n">
-        <v>23</v>
+        <v>22.9</v>
       </c>
       <c r="K12" t="n">
-        <v>160074</v>
+        <v>160259</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -4322,16 +4489,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>69021</v>
+        <v>74954</v>
       </c>
       <c r="I13" t="n">
-        <v>25.8</v>
+        <v>38.3</v>
       </c>
       <c r="J13" t="n">
-        <v>1138.7</v>
+        <v>1245.2</v>
       </c>
       <c r="K13" t="n">
-        <v>28836</v>
+        <v>30017</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -4381,16 +4548,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>127425188</v>
+        <v>127190615</v>
       </c>
       <c r="I14" t="n">
-        <v>-2</v>
+        <v>-2.2</v>
       </c>
       <c r="J14" t="n">
-        <v>14.1</v>
+        <v>14.4</v>
       </c>
       <c r="K14" t="n">
-        <v>257973</v>
+        <v>250581</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -4440,16 +4607,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>350227760</v>
+        <v>351937300</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.7</v>
+        <v>-0.1</v>
       </c>
       <c r="J15" t="n">
-        <v>-1.3</v>
+        <v>-1.7</v>
       </c>
       <c r="K15" t="n">
-        <v>2759823</v>
+        <v>2765230</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -4499,16 +4666,16 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>7011639</v>
+        <v>7018112</v>
       </c>
       <c r="I16" t="n">
-        <v>0.2</v>
+        <v>-0.2</v>
       </c>
       <c r="J16" t="n">
-        <v>-2</v>
+        <v>-2.3</v>
       </c>
       <c r="K16" t="n">
-        <v>335196</v>
+        <v>335785</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -4561,13 +4728,13 @@
         <v>1251334</v>
       </c>
       <c r="I17" t="n">
-        <v>1.7</v>
+        <v>1.1</v>
       </c>
       <c r="J17" t="n">
         <v>1.6</v>
       </c>
       <c r="K17" t="n">
-        <v>268100</v>
+        <v>265951</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -4617,16 +4784,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>979001</v>
+        <v>971006</v>
       </c>
       <c r="I18" t="n">
-        <v>-10.1</v>
+        <v>-3.9</v>
       </c>
       <c r="J18" t="n">
-        <v>65.5</v>
+        <v>61.1</v>
       </c>
       <c r="K18" t="n">
-        <v>118427</v>
+        <v>117861</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -4676,16 +4843,16 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>318565</v>
+        <v>318672</v>
       </c>
       <c r="I19" t="n">
-        <v>-5.9</v>
+        <v>-1.1</v>
       </c>
       <c r="J19" t="n">
-        <v>17.2</v>
+        <v>18.1</v>
       </c>
       <c r="K19" t="n">
-        <v>62873</v>
+        <v>62729</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -4735,16 +4902,16 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>54011786</v>
+        <v>53659760</v>
       </c>
       <c r="I20" t="n">
-        <v>0.7</v>
+        <v>1.5</v>
       </c>
       <c r="J20" t="n">
-        <v>26.6</v>
+        <v>26.3</v>
       </c>
       <c r="K20" t="n">
-        <v>1243945</v>
+        <v>1217809</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -4794,16 +4961,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>16858440</v>
+        <v>17051086</v>
       </c>
       <c r="I21" t="n">
-        <v>-7.7</v>
+        <v>-4.6</v>
       </c>
       <c r="J21" t="n">
-        <v>24.5</v>
+        <v>28</v>
       </c>
       <c r="K21" t="n">
-        <v>874192</v>
+        <v>880901</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -4853,16 +5020,16 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>131540</v>
+        <v>120691</v>
       </c>
       <c r="I22" t="n">
-        <v>2.5</v>
+        <v>-7.3</v>
       </c>
       <c r="J22" t="n">
-        <v>-5.9</v>
+        <v>-12.7</v>
       </c>
       <c r="K22" t="n">
-        <v>32975</v>
+        <v>31072</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -4912,16 +5079,16 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>58892</v>
+        <v>56395</v>
       </c>
       <c r="I23" t="n">
-        <v>-11.1</v>
+        <v>-2.6</v>
       </c>
       <c r="J23" t="n">
-        <v>21.6</v>
+        <v>15.8</v>
       </c>
       <c r="K23" t="n">
-        <v>20714</v>
+        <v>20171</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -4971,16 +5138,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>209765</v>
+        <v>340021</v>
       </c>
       <c r="I24" t="n">
-        <v>6674.3</v>
+        <v>219.2</v>
       </c>
       <c r="J24" t="n">
-        <v>6674.3</v>
+        <v>10880.8</v>
       </c>
       <c r="K24" t="n">
-        <v>51799</v>
+        <v>74176</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -5030,16 +5197,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>145432730</v>
+        <v>145066958</v>
       </c>
       <c r="I25" t="n">
-        <v>-1</v>
+        <v>-0.9</v>
       </c>
       <c r="J25" t="n">
-        <v>10.9</v>
+        <v>8.6</v>
       </c>
       <c r="K25" t="n">
-        <v>2413935</v>
+        <v>2416336</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -5089,16 +5256,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>379128960</v>
+        <v>379160510</v>
       </c>
       <c r="I26" t="n">
         <v>-1.1</v>
       </c>
       <c r="J26" t="n">
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
       <c r="K26" t="n">
-        <v>11420540</v>
+        <v>11427436</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -5148,16 +5315,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>592815770</v>
+        <v>598372970</v>
       </c>
       <c r="I27" t="n">
-        <v>-1.7</v>
+        <v>0.3</v>
       </c>
       <c r="J27" t="n">
-        <v>4</v>
+        <v>5.2</v>
       </c>
       <c r="K27" t="n">
-        <v>8798645</v>
+        <v>8804694</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -5207,16 +5374,16 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>41018448</v>
+        <v>41307631</v>
       </c>
       <c r="I28" t="n">
-        <v>-0.9</v>
+        <v>-0.1</v>
       </c>
       <c r="J28" t="n">
-        <v>-6.9</v>
+        <v>-7.3</v>
       </c>
       <c r="K28" t="n">
-        <v>2010968</v>
+        <v>2017762</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -5266,16 +5433,16 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>245766</v>
+        <v>253063</v>
       </c>
       <c r="I29" t="n">
-        <v>-12.5</v>
+        <v>-9.9</v>
       </c>
       <c r="J29" t="n">
-        <v>-23.6</v>
+        <v>-21.6</v>
       </c>
       <c r="K29" t="n">
-        <v>49035</v>
+        <v>49747</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -5325,16 +5492,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>140403</v>
+        <v>146810</v>
       </c>
       <c r="I30" t="n">
-        <v>-17.3</v>
+        <v>-10.9</v>
       </c>
       <c r="J30" t="n">
-        <v>-43.1</v>
+        <v>-39.1</v>
       </c>
       <c r="K30" t="n">
-        <v>37266</v>
+        <v>38114</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -5384,16 +5551,16 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>47023</v>
+        <v>64185</v>
       </c>
       <c r="I31" t="n">
-        <v>959.4</v>
+        <v>844.7</v>
       </c>
       <c r="J31" t="n">
-        <v>853.9</v>
+        <v>1188.2</v>
       </c>
       <c r="K31" t="n">
-        <v>20615</v>
+        <v>24175</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -5443,16 +5610,16 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>75468242</v>
+        <v>75400413</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="J32" t="n">
-        <v>-0.1</v>
+        <v>-0.5</v>
       </c>
       <c r="K32" t="n">
-        <v>254170</v>
+        <v>253806</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -5502,16 +5669,16 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>330267</v>
+        <v>318645</v>
       </c>
       <c r="I33" t="n">
-        <v>-8.300000000000001</v>
+        <v>-4.8</v>
       </c>
       <c r="J33" t="n">
-        <v>-23.4</v>
+        <v>-31.1</v>
       </c>
       <c r="K33" t="n">
-        <v>68280</v>
+        <v>67321</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -5561,16 +5728,16 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>176509</v>
+        <v>175374</v>
       </c>
       <c r="I34" t="n">
-        <v>-4.1</v>
+        <v>-1.5</v>
       </c>
       <c r="J34" t="n">
-        <v>98.09999999999999</v>
+        <v>98.5</v>
       </c>
       <c r="K34" t="n">
-        <v>36782</v>
+        <v>36659</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -5620,16 +5787,16 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>421364</v>
+        <v>364175</v>
       </c>
       <c r="I35" t="n">
-        <v>-0.6</v>
+        <v>-11.7</v>
       </c>
       <c r="J35" t="n">
-        <v>12268</v>
+        <v>10589.4</v>
       </c>
       <c r="K35" t="n">
-        <v>71326</v>
+        <v>68212</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -5645,7 +5812,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Solamians · Solana 官方插画里的“国籍”</t>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5655,12 +5822,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Solamians</t>
+          <t>CAESAR</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -5670,7 +5837,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>677hfbabdMDpv6GVagJ6FoDSvEr2hLJJKzr83TFsySQG</t>
+          <t>EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -5679,32 +5846,32 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>302753</v>
+        <v>98991</v>
       </c>
       <c r="I36" t="n">
-        <v>-17</v>
+        <v>-61.1</v>
       </c>
       <c r="J36" t="n">
-        <v>107284986</v>
+        <v>2510.8</v>
       </c>
       <c r="K36" t="n">
-        <v>72445</v>
+        <v>26868</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Solamians（10/12 17:36 悉尼上线），名字命中「Solamians」关键词；叙事待人工核实。</t>
+          <t>pmarca 转发的《Slop Caesar》社区盘。19:24 Devon 本人贴出此 CA，自称已领约 108 SOL 手续费（GMGN：分成 100% 给 devonmvfisher，已领取）。原开发者已清仓、批量发币地址；机器人约 62%。</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/677hfbabdMDpv6GVagJ6FoDSvEr2hLJJKzr83TFsySQG</t>
+          <t>https://gmgn.ai/sol/token/EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -5719,7 +5886,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>CAESAR</t>
+          <t>CYBERLEEK</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -5729,7 +5896,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
+          <t>ApZuxdpzMrbEYTGEzeY9afh5pj9d6qPRJCTgQYiipbKg</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -5738,32 +5905,32 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>164539</v>
+        <v>2758058</v>
       </c>
       <c r="I37" t="n">
-        <v>-2.2</v>
+        <v>-0.6</v>
       </c>
       <c r="J37" t="n">
-        <v>4239.6</v>
+        <v>-55.6</v>
       </c>
       <c r="K37" t="n">
-        <v>35818</v>
+        <v>934715</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>pmarca 转发的《Slop Caesar》社区盘。19:24 Devon 本人贴出此 CA，自称已领约 108 SOL 手续费（GMGN：分成 100% 给 devonmvfisher，已领取）。原开发者已清仓、批量发币地址；机器人约 62%。</t>
+          <t>GTA 6 泄露者的币，10/10 喊出 3000 万市值放完整版。8 月曾提款后崩盘，24h -53%。</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
+          <t>https://gmgn.ai/sol/token/ApZuxdpzMrbEYTGEzeY9afh5pj9d6qPRJCTgQYiipbKg</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -5778,7 +5945,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>CAESAR</t>
+          <t>Dacity</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -5788,7 +5955,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>EUTas4zV2UYrfCqEsPXFvuX5uhexwUuzDCCBkptih3MS</t>
+          <t>nxPqZ4F7ux8Vph5NFu25rEP6Kx9Gr1U6Fmj36Rjpump</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -5797,25 +5964,84 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>84973</v>
+        <v>145173</v>
       </c>
       <c r="I38" t="n">
-        <v>76.59999999999999</v>
+        <v>5.5</v>
       </c>
       <c r="J38" t="n">
-        <v>786.8</v>
+        <v>4157.3</v>
       </c>
       <c r="K38" t="n">
-        <v>59580</v>
+        <v>35381</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Slop Caesar（10/12 17:50 悉尼上线），名字命中「Slop」关键词；叙事待人工核实。</t>
+          <t>据称出现在泄露视频里的游戏内币（未核实），ATH 回撤 88%，机器人多。</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/EUTas4zV2UYrfCqEsPXFvuX5uhexwUuzDCCBkptih3MS</t>
+          <t>https://gmgn.ai/sol/token/nxPqZ4F7ux8Vph5NFu25rEP6Kx9Gr1U6Fmj36Rjpump</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>CYBERLEEK</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>6zGNMJemLTGCHm3exz8ns5k1pq9XeKxrBc19Y5pqpump</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>758296837</v>
+      </c>
+      <c r="I39" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J39" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="K39" t="n">
+        <v>2440539</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>🆕 GMGN 自动发现：CYBERLEEK（10/11 01:51 悉尼上线），名字命中「GTA」关键词；叙事待人工核实。</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/6zGNMJemLTGCHm3exz8ns5k1pq9XeKxrBc19Y5pqpump</t>
         </is>
       </c>
     </row>
@@ -5858,6 +6084,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId38"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
radar 10/12 19:58 drop fake cyberleek clone
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -3718,7 +3718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5983,65 +5983,6 @@
       <c r="M38" s="2" t="inlineStr">
         <is>
           <t>https://gmgn.ai/sol/token/nxPqZ4F7ux8Vph5NFu25rEP6Kx9Gr1U6Fmj36Rjpump</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>24小时</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>beta</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>CYBERLEEK</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>sol</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>6zGNMJemLTGCHm3exz8ns5k1pq9XeKxrBc19Y5pqpump</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>alive</t>
-        </is>
-      </c>
-      <c r="H39" t="n">
-        <v>758296837</v>
-      </c>
-      <c r="I39" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="J39" t="n">
-        <v>60.3</v>
-      </c>
-      <c r="K39" t="n">
-        <v>2440539</v>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>🆕 GMGN 自动发现：CYBERLEEK（10/11 01:51 悉尼上线），名字命中「GTA」关键词；叙事待人工核实。</t>
-        </is>
-      </c>
-      <c r="M39" s="2" t="inlineStr">
-        <is>
-          <t>https://gmgn.ai/sol/token/6zGNMJemLTGCHm3exz8ns5k1pq9XeKxrBc19Y5pqpump</t>
         </is>
       </c>
     </row>
@@ -6084,7 +6025,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId38"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
radar silent 10/12 20:15
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:G86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2591,17 +2591,17 @@
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Kotaku：泄露者 3000 万市值威胁（引用 10/10 原文）</t>
+          <t>Devon 确认领取手续费 19:59</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>https://kotaku.com/gta-6-leaker-threatens-rockstar-with-doomsday-scenario-if-meme-coin-hits-30-million-2000743779</t>
+          <t>https://x.com/Devon8zzh/status/2109569560009679193</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
@@ -2612,12 +2612,12 @@
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Yahoo Finance：CYBERLEEK 24h 涨 273%</t>
+          <t>Kotaku：泄露者 3000 万市值威胁（引用 10/10 原文）</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>https://finance.yahoo.com/markets/crypto/articles/solana-meme-coin-tied-gta-150454094.html</t>
+          <t>https://kotaku.com/gta-6-leaker-threatens-rockstar-with-doomsday-scenario-if-meme-coin-hits-30-million-2000743779</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -2633,12 +2633,12 @@
       <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Dotesports：8 月提走约 25 万美元手续费</t>
+          <t>Yahoo Finance：CYBERLEEK 24h 涨 273%</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>https://dotesports.com/gta/news/cyberleek-gta-6-full-build-ultimatum</t>
+          <t>https://finance.yahoo.com/markets/crypto/articles/solana-meme-coin-tied-gta-150454094.html</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -2654,12 +2654,12 @@
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Seeking Alpha 推文</t>
+          <t>Dotesports：8 月提走约 25 万美元手续费</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/SeekingAlpha/status/2109436393017807208</t>
+          <t>https://dotesports.com/gta/news/cyberleek-gta-6-full-build-ultimatum</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -2675,12 +2675,12 @@
       <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr">
         <is>
-          <t>@robtmb1：泄露视频里的 Dacity Coin（未核实）</t>
+          <t>Seeking Alpha 推文</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/robtmb1/status/2109241600002118071</t>
+          <t>https://x.com/SeekingAlpha/status/2109436393017807208</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -2690,6 +2690,27 @@
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr"/>
+      <c r="B86" t="inlineStr"/>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>@robtmb1：泄露视频里的 Dacity Coin（未核实）</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/robtmb1/status/2109241600002118071</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2777,6 +2798,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId85"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3217,7 +3239,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>10/12：pmarca 转发 AI 创作者 @Devon8zzh 的《Slop Caesar》（已核实）。19:24 Devon 本人发帖贴出 EaqX… CA 并问“Is this right?”，19:26 问“108.07 SOL 算多吗”，截图显示“I found the button”（自称已领手续费，X 原帖已核实）；GMGN 显示 EaqX 盘 100% 创作者分成指向 GitHub 账号 devonmvfisher 且已领取（GitHub 号与 X 号是否同一人未核实，但该号有 passage 仓库）。截图同时显示有人在私信教他喊单、“先别领其他盘”。讨论量在降（17 点档 244 帖 → 18 点档 148 → 19:00–19:30 约 51），19:30 盘子约 $164K、1h -3%，市场暂未反应</t>
+          <t>10/12：pmarca 转发 AI 创作者 @Devon8zzh 的《Slop Caesar》（已核实）。19:24 Devon 本人发帖贴出 EaqX… CA 并问“Is this right?”，19:26 问“108.07 SOL 算多吗”，截图显示“I found the button”（自称已领手续费，X 原帖已核实）；GMGN 显示 EaqX 盘 100% 创作者分成指向 GitHub 账号 devonmvfisher 且已领取（GitHub 号与 X 号是否同一人未核实，但该号有 passage 仓库）。截图同时显示有人在私信教他喊单、“先别领其他盘”。讨论量在降（17 点档 244 帖 → 18 点档 148 → 19:00–19:30 约 51），19:30 盘子约 $164K、1h -3%，市场暂未反应；19:59 Devon 再发帖确认已领创作者手续费、称“不是喊单”，钱用来做更多视频（X 原帖已核实），并在做 8 分钟新片（19/52 场景）。但 20:10 盘子约 $114K、1h -42%，市场没买账 → 继续观望</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -3840,16 +3862,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>24530555</v>
+        <v>24585230</v>
       </c>
       <c r="I2" t="n">
-        <v>0.3</v>
+        <v>-0.3</v>
       </c>
       <c r="J2" t="n">
-        <v>-19.2</v>
+        <v>-21.6</v>
       </c>
       <c r="K2" t="n">
-        <v>863330</v>
+        <v>862331</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -3899,16 +3921,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1550137</v>
+        <v>1848785</v>
       </c>
       <c r="I3" t="n">
-        <v>-2.4</v>
+        <v>17.7</v>
       </c>
       <c r="J3" t="n">
-        <v>11.8</v>
+        <v>41.9</v>
       </c>
       <c r="K3" t="n">
-        <v>175626</v>
+        <v>190997</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -3958,16 +3980,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>774852</v>
+        <v>771925</v>
       </c>
       <c r="I4" t="n">
-        <v>-22.3</v>
+        <v>-7.4</v>
       </c>
       <c r="J4" t="n">
-        <v>1.7</v>
+        <v>13.2</v>
       </c>
       <c r="K4" t="n">
-        <v>106121</v>
+        <v>103280</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -4017,16 +4039,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>20784</v>
+        <v>20690</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1</v>
+        <v>-1.5</v>
       </c>
       <c r="J5" t="n">
-        <v>38.3</v>
+        <v>37.7</v>
       </c>
       <c r="K5" t="n">
-        <v>13564</v>
+        <v>13533</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -4076,16 +4098,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1093507</v>
+        <v>1213732</v>
       </c>
       <c r="I6" t="n">
-        <v>2.2</v>
+        <v>11.3</v>
       </c>
       <c r="J6" t="n">
-        <v>12.9</v>
+        <v>24.1</v>
       </c>
       <c r="K6" t="n">
-        <v>103148</v>
+        <v>108780</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -4135,16 +4157,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>31849</v>
+        <v>31853</v>
       </c>
       <c r="I7" t="n">
-        <v>-6</v>
+        <v>-1.8</v>
       </c>
       <c r="J7" t="n">
-        <v>-63.1</v>
+        <v>-60.4</v>
       </c>
       <c r="K7" t="n">
-        <v>13993</v>
+        <v>13800</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -4194,16 +4216,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>40239</v>
+        <v>39126</v>
       </c>
       <c r="I8" t="n">
-        <v>-25.8</v>
+        <v>20.4</v>
       </c>
       <c r="J8" t="n">
-        <v>23.9</v>
+        <v>-12.7</v>
       </c>
       <c r="K8" t="n">
-        <v>20980</v>
+        <v>20825</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -4253,16 +4275,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1470386</v>
+        <v>1415926</v>
       </c>
       <c r="I9" t="n">
-        <v>-2.9</v>
+        <v>-3.3</v>
       </c>
       <c r="J9" t="n">
-        <v>-24.6</v>
+        <v>-25.7</v>
       </c>
       <c r="K9" t="n">
-        <v>169663</v>
+        <v>179514</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -4312,16 +4334,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>40724</v>
+        <v>41905</v>
       </c>
       <c r="I10" t="n">
-        <v>-7.9</v>
+        <v>0.5</v>
       </c>
       <c r="J10" t="n">
-        <v>-64.40000000000001</v>
+        <v>-61.7</v>
       </c>
       <c r="K10" t="n">
-        <v>18002</v>
+        <v>18277</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -4371,16 +4393,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>196453</v>
+        <v>201200</v>
       </c>
       <c r="I11" t="n">
-        <v>-6.4</v>
+        <v>6</v>
       </c>
       <c r="J11" t="n">
-        <v>-29.7</v>
+        <v>-30.6</v>
       </c>
       <c r="K11" t="n">
-        <v>59976</v>
+        <v>61542</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -4430,16 +4452,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3357369</v>
+        <v>3379665</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.1</v>
+        <v>0.4</v>
       </c>
       <c r="J12" t="n">
-        <v>22.9</v>
+        <v>23.2</v>
       </c>
       <c r="K12" t="n">
-        <v>160259</v>
+        <v>159946</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -4489,16 +4511,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>74954</v>
+        <v>82546</v>
       </c>
       <c r="I13" t="n">
-        <v>38.3</v>
+        <v>58.9</v>
       </c>
       <c r="J13" t="n">
-        <v>1245.2</v>
+        <v>1381.4</v>
       </c>
       <c r="K13" t="n">
-        <v>30017</v>
+        <v>31477</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -4548,16 +4570,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>127190615</v>
+        <v>128100951</v>
       </c>
       <c r="I14" t="n">
-        <v>-2.2</v>
+        <v>-0.5</v>
       </c>
       <c r="J14" t="n">
         <v>14.4</v>
       </c>
       <c r="K14" t="n">
-        <v>250581</v>
+        <v>251417</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -4607,16 +4629,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>351937300</v>
+        <v>351584250</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.1</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>-1.7</v>
+        <v>-1.3</v>
       </c>
       <c r="K15" t="n">
-        <v>2765230</v>
+        <v>2765335</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -4666,16 +4688,16 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>7018112</v>
+        <v>7028292</v>
       </c>
       <c r="I16" t="n">
-        <v>-0.2</v>
+        <v>0.6</v>
       </c>
       <c r="J16" t="n">
-        <v>-2.3</v>
+        <v>-2.2</v>
       </c>
       <c r="K16" t="n">
-        <v>335785</v>
+        <v>335731</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -4728,7 +4750,7 @@
         <v>1251334</v>
       </c>
       <c r="I17" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
         <v>1.6</v>
@@ -4784,16 +4806,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>971006</v>
+        <v>977693</v>
       </c>
       <c r="I18" t="n">
-        <v>-3.9</v>
+        <v>-0.1</v>
       </c>
       <c r="J18" t="n">
-        <v>61.1</v>
+        <v>63.4</v>
       </c>
       <c r="K18" t="n">
-        <v>117861</v>
+        <v>117578</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -4843,13 +4865,13 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>318672</v>
+        <v>318033</v>
       </c>
       <c r="I19" t="n">
-        <v>-1.1</v>
+        <v>-1</v>
       </c>
       <c r="J19" t="n">
-        <v>18.1</v>
+        <v>17.8</v>
       </c>
       <c r="K19" t="n">
         <v>62729</v>
@@ -4902,16 +4924,16 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>53659760</v>
+        <v>53827229</v>
       </c>
       <c r="I20" t="n">
-        <v>1.5</v>
+        <v>-1.6</v>
       </c>
       <c r="J20" t="n">
-        <v>26.3</v>
+        <v>26.8</v>
       </c>
       <c r="K20" t="n">
-        <v>1217809</v>
+        <v>1237122</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -4961,16 +4983,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>17051086</v>
+        <v>17275657</v>
       </c>
       <c r="I21" t="n">
-        <v>-4.6</v>
+        <v>0.5</v>
       </c>
       <c r="J21" t="n">
-        <v>28</v>
+        <v>30.5</v>
       </c>
       <c r="K21" t="n">
-        <v>880901</v>
+        <v>884962</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -5020,16 +5042,16 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>120691</v>
+        <v>121147</v>
       </c>
       <c r="I22" t="n">
-        <v>-7.3</v>
+        <v>-6.9</v>
       </c>
       <c r="J22" t="n">
-        <v>-12.7</v>
+        <v>-12.4</v>
       </c>
       <c r="K22" t="n">
-        <v>31072</v>
+        <v>31084</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -5079,16 +5101,16 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>56395</v>
+        <v>56918</v>
       </c>
       <c r="I23" t="n">
-        <v>-2.6</v>
+        <v>-1.1</v>
       </c>
       <c r="J23" t="n">
-        <v>15.8</v>
+        <v>15.2</v>
       </c>
       <c r="K23" t="n">
-        <v>20171</v>
+        <v>20142</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -5138,16 +5160,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>340021</v>
+        <v>366758</v>
       </c>
       <c r="I24" t="n">
-        <v>219.2</v>
+        <v>100.5</v>
       </c>
       <c r="J24" t="n">
-        <v>10880.8</v>
+        <v>11744.3</v>
       </c>
       <c r="K24" t="n">
-        <v>74176</v>
+        <v>77880</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -5197,16 +5219,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>145066958</v>
+        <v>144460154</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.9</v>
+        <v>-1</v>
       </c>
       <c r="J25" t="n">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="K25" t="n">
-        <v>2416336</v>
+        <v>2405950</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -5256,16 +5278,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>379160510</v>
+        <v>380352370</v>
       </c>
       <c r="I26" t="n">
-        <v>-1.1</v>
+        <v>-0.3</v>
       </c>
       <c r="J26" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="K26" t="n">
-        <v>11427436</v>
+        <v>11428456</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -5315,16 +5337,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>598372970</v>
+        <v>586601890</v>
       </c>
       <c r="I27" t="n">
-        <v>0.3</v>
+        <v>-1.4</v>
       </c>
       <c r="J27" t="n">
-        <v>5.2</v>
+        <v>3.1</v>
       </c>
       <c r="K27" t="n">
-        <v>8804694</v>
+        <v>8749009</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -5374,16 +5396,16 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>41307631</v>
+        <v>40992995</v>
       </c>
       <c r="I28" t="n">
-        <v>-0.1</v>
+        <v>-0.2</v>
       </c>
       <c r="J28" t="n">
-        <v>-7.3</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="K28" t="n">
-        <v>2017762</v>
+        <v>2016910</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -5433,16 +5455,16 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>253063</v>
+        <v>252797</v>
       </c>
       <c r="I29" t="n">
-        <v>-9.9</v>
+        <v>-7.1</v>
       </c>
       <c r="J29" t="n">
-        <v>-21.6</v>
+        <v>-21.3</v>
       </c>
       <c r="K29" t="n">
-        <v>49747</v>
+        <v>49722</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -5492,16 +5514,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>146810</v>
+        <v>139936</v>
       </c>
       <c r="I30" t="n">
-        <v>-10.9</v>
+        <v>-10.8</v>
       </c>
       <c r="J30" t="n">
-        <v>-39.1</v>
+        <v>-42.4</v>
       </c>
       <c r="K30" t="n">
-        <v>38114</v>
+        <v>37196</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -5551,16 +5573,16 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>64185</v>
+        <v>89104</v>
       </c>
       <c r="I31" t="n">
-        <v>844.7</v>
+        <v>114.3</v>
       </c>
       <c r="J31" t="n">
-        <v>1188.2</v>
+        <v>1688.3</v>
       </c>
       <c r="K31" t="n">
-        <v>24175</v>
+        <v>28471</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -5610,16 +5632,16 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>75400413</v>
+        <v>75512134</v>
       </c>
       <c r="I32" t="n">
-        <v>-0.1</v>
+        <v>0.1</v>
       </c>
       <c r="J32" t="n">
-        <v>-0.5</v>
+        <v>0.7</v>
       </c>
       <c r="K32" t="n">
-        <v>253806</v>
+        <v>249765</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -5669,16 +5691,16 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>318645</v>
+        <v>316954</v>
       </c>
       <c r="I33" t="n">
         <v>-4.8</v>
       </c>
       <c r="J33" t="n">
-        <v>-31.1</v>
+        <v>-29.6</v>
       </c>
       <c r="K33" t="n">
-        <v>67321</v>
+        <v>67528</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -5728,16 +5750,16 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>175374</v>
+        <v>174819</v>
       </c>
       <c r="I34" t="n">
-        <v>-1.5</v>
+        <v>-1.8</v>
       </c>
       <c r="J34" t="n">
-        <v>98.5</v>
+        <v>99</v>
       </c>
       <c r="K34" t="n">
-        <v>36659</v>
+        <v>36560</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -5787,16 +5809,16 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>364175</v>
+        <v>357642</v>
       </c>
       <c r="I35" t="n">
-        <v>-11.7</v>
+        <v>-2.3</v>
       </c>
       <c r="J35" t="n">
-        <v>10589.4</v>
+        <v>10397.6</v>
       </c>
       <c r="K35" t="n">
-        <v>68212</v>
+        <v>57789</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -5846,16 +5868,16 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>98991</v>
+        <v>114154</v>
       </c>
       <c r="I36" t="n">
-        <v>-61.1</v>
+        <v>-41.8</v>
       </c>
       <c r="J36" t="n">
-        <v>2510.8</v>
+        <v>2910.7</v>
       </c>
       <c r="K36" t="n">
-        <v>26868</v>
+        <v>29017</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -5905,16 +5927,16 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>2758058</v>
+        <v>2693690</v>
       </c>
       <c r="I37" t="n">
-        <v>-0.6</v>
+        <v>-4.2</v>
       </c>
       <c r="J37" t="n">
-        <v>-55.6</v>
+        <v>-59.1</v>
       </c>
       <c r="K37" t="n">
-        <v>934715</v>
+        <v>896572</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -5964,16 +5986,16 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>145173</v>
+        <v>135054</v>
       </c>
       <c r="I38" t="n">
-        <v>5.5</v>
+        <v>-0.3</v>
       </c>
       <c r="J38" t="n">
-        <v>4157.3</v>
+        <v>3860.6</v>
       </c>
       <c r="K38" t="n">
-        <v>35381</v>
+        <v>34002</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
radar silent 10/12 20:47
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -3862,16 +3862,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>24585230</v>
+        <v>24060536</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.3</v>
+        <v>-1.8</v>
       </c>
       <c r="J2" t="n">
-        <v>-21.6</v>
+        <v>-21.1</v>
       </c>
       <c r="K2" t="n">
-        <v>862331</v>
+        <v>840644</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -3921,16 +3921,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1848785</v>
+        <v>1596474</v>
       </c>
       <c r="I3" t="n">
-        <v>17.7</v>
+        <v>3.7</v>
       </c>
       <c r="J3" t="n">
-        <v>41.9</v>
+        <v>29.9</v>
       </c>
       <c r="K3" t="n">
-        <v>190997</v>
+        <v>178443</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -3980,16 +3980,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>771925</v>
+        <v>746750</v>
       </c>
       <c r="I4" t="n">
-        <v>-7.4</v>
+        <v>-6.9</v>
       </c>
       <c r="J4" t="n">
-        <v>13.2</v>
+        <v>-13</v>
       </c>
       <c r="K4" t="n">
-        <v>103280</v>
+        <v>101738</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -4039,16 +4039,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>20690</v>
+        <v>22881</v>
       </c>
       <c r="I5" t="n">
-        <v>-1.5</v>
+        <v>10.1</v>
       </c>
       <c r="J5" t="n">
-        <v>37.7</v>
+        <v>34.9</v>
       </c>
       <c r="K5" t="n">
-        <v>13533</v>
+        <v>14172</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -4098,16 +4098,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1213732</v>
+        <v>1268385</v>
       </c>
       <c r="I6" t="n">
-        <v>11.3</v>
+        <v>20.8</v>
       </c>
       <c r="J6" t="n">
-        <v>24.1</v>
+        <v>12.3</v>
       </c>
       <c r="K6" t="n">
-        <v>108780</v>
+        <v>110511</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -4157,16 +4157,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>31853</v>
+        <v>29374</v>
       </c>
       <c r="I7" t="n">
-        <v>-1.8</v>
+        <v>-7.8</v>
       </c>
       <c r="J7" t="n">
-        <v>-60.4</v>
+        <v>-54.3</v>
       </c>
       <c r="K7" t="n">
-        <v>13800</v>
+        <v>13263</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -4216,16 +4216,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>39126</v>
+        <v>35999</v>
       </c>
       <c r="I8" t="n">
-        <v>20.4</v>
+        <v>-5.7</v>
       </c>
       <c r="J8" t="n">
-        <v>-12.7</v>
+        <v>-35.4</v>
       </c>
       <c r="K8" t="n">
-        <v>20825</v>
+        <v>20012</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -4275,16 +4275,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1415926</v>
+        <v>1434972</v>
       </c>
       <c r="I9" t="n">
-        <v>-3.3</v>
+        <v>-1.5</v>
       </c>
       <c r="J9" t="n">
-        <v>-25.7</v>
+        <v>-29.4</v>
       </c>
       <c r="K9" t="n">
-        <v>179514</v>
+        <v>166668</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -4334,16 +4334,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>41905</v>
+        <v>44972</v>
       </c>
       <c r="I10" t="n">
-        <v>0.5</v>
+        <v>10.4</v>
       </c>
       <c r="J10" t="n">
-        <v>-61.7</v>
+        <v>-38.2</v>
       </c>
       <c r="K10" t="n">
-        <v>18277</v>
+        <v>19074</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -4393,16 +4393,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>201200</v>
+        <v>178024</v>
       </c>
       <c r="I11" t="n">
-        <v>6</v>
+        <v>-5.5</v>
       </c>
       <c r="J11" t="n">
-        <v>-30.6</v>
+        <v>-50.1</v>
       </c>
       <c r="K11" t="n">
-        <v>61542</v>
+        <v>58079</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -4452,16 +4452,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3379665</v>
+        <v>3356276</v>
       </c>
       <c r="I12" t="n">
-        <v>0.4</v>
+        <v>-0.9</v>
       </c>
       <c r="J12" t="n">
-        <v>23.2</v>
+        <v>20.7</v>
       </c>
       <c r="K12" t="n">
-        <v>159946</v>
+        <v>159791</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -4511,16 +4511,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>82546</v>
+        <v>76361</v>
       </c>
       <c r="I13" t="n">
-        <v>58.9</v>
+        <v>3.7</v>
       </c>
       <c r="J13" t="n">
-        <v>1381.4</v>
+        <v>1270.4</v>
       </c>
       <c r="K13" t="n">
-        <v>31477</v>
+        <v>30312</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -4570,16 +4570,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>128100951</v>
+        <v>126787269</v>
       </c>
       <c r="I14" t="n">
-        <v>-0.5</v>
+        <v>0.1</v>
       </c>
       <c r="J14" t="n">
-        <v>14.4</v>
+        <v>13.5</v>
       </c>
       <c r="K14" t="n">
-        <v>251417</v>
+        <v>253126</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -4629,16 +4629,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>351584250</v>
+        <v>344636830</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>-2.2</v>
       </c>
       <c r="J15" t="n">
-        <v>-1.3</v>
+        <v>-4.2</v>
       </c>
       <c r="K15" t="n">
-        <v>2765335</v>
+        <v>2746603</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -4688,16 +4688,16 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>7028292</v>
+        <v>6736029</v>
       </c>
       <c r="I16" t="n">
-        <v>0.6</v>
+        <v>-3.8</v>
       </c>
       <c r="J16" t="n">
-        <v>-2.2</v>
+        <v>-5.7</v>
       </c>
       <c r="K16" t="n">
-        <v>335731</v>
+        <v>329001</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -4806,16 +4806,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>977693</v>
+        <v>990473</v>
       </c>
       <c r="I18" t="n">
-        <v>-0.1</v>
+        <v>2</v>
       </c>
       <c r="J18" t="n">
-        <v>63.4</v>
+        <v>69.5</v>
       </c>
       <c r="K18" t="n">
-        <v>117578</v>
+        <v>118457</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -4865,16 +4865,16 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>318033</v>
+        <v>314474</v>
       </c>
       <c r="I19" t="n">
-        <v>-1</v>
+        <v>-1.3</v>
       </c>
       <c r="J19" t="n">
-        <v>17.8</v>
+        <v>16.5</v>
       </c>
       <c r="K19" t="n">
-        <v>62729</v>
+        <v>61485</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -4924,16 +4924,16 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>53827229</v>
+        <v>53343439</v>
       </c>
       <c r="I20" t="n">
-        <v>-1.6</v>
+        <v>3.4</v>
       </c>
       <c r="J20" t="n">
-        <v>26.8</v>
+        <v>20.4</v>
       </c>
       <c r="K20" t="n">
-        <v>1237122</v>
+        <v>1217536</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -4983,16 +4983,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>17275657</v>
+        <v>16984017</v>
       </c>
       <c r="I21" t="n">
-        <v>0.5</v>
+        <v>-0.3</v>
       </c>
       <c r="J21" t="n">
-        <v>30.5</v>
+        <v>25.1</v>
       </c>
       <c r="K21" t="n">
-        <v>884962</v>
+        <v>862220</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -5042,16 +5042,16 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>121147</v>
+        <v>123915</v>
       </c>
       <c r="I22" t="n">
-        <v>-6.9</v>
+        <v>2.7</v>
       </c>
       <c r="J22" t="n">
-        <v>-12.4</v>
+        <v>-10.3</v>
       </c>
       <c r="K22" t="n">
-        <v>31084</v>
+        <v>31374</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -5101,16 +5101,16 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>56918</v>
+        <v>56544</v>
       </c>
       <c r="I23" t="n">
-        <v>-1.1</v>
+        <v>1.8</v>
       </c>
       <c r="J23" t="n">
-        <v>15.2</v>
+        <v>10.2</v>
       </c>
       <c r="K23" t="n">
-        <v>20142</v>
+        <v>20180</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -5160,16 +5160,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>366758</v>
+        <v>472774</v>
       </c>
       <c r="I24" t="n">
-        <v>100.5</v>
+        <v>73.7</v>
       </c>
       <c r="J24" t="n">
-        <v>11744.3</v>
+        <v>15168.1</v>
       </c>
       <c r="K24" t="n">
-        <v>77880</v>
+        <v>91367</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -5219,16 +5219,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>144460154</v>
+        <v>139540782</v>
       </c>
       <c r="I25" t="n">
-        <v>-1</v>
+        <v>-4.2</v>
       </c>
       <c r="J25" t="n">
-        <v>8.5</v>
+        <v>5</v>
       </c>
       <c r="K25" t="n">
-        <v>2405950</v>
+        <v>2360359</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -5278,16 +5278,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>380352370</v>
+        <v>377277220</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.3</v>
+        <v>-0.8</v>
       </c>
       <c r="J26" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="K26" t="n">
-        <v>11428456</v>
+        <v>11381508</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -5337,16 +5337,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>586601890</v>
+        <v>587351830</v>
       </c>
       <c r="I27" t="n">
         <v>-1.4</v>
       </c>
       <c r="J27" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="K27" t="n">
-        <v>8749009</v>
+        <v>8741285</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -5396,16 +5396,16 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>40992995</v>
+        <v>41190278</v>
       </c>
       <c r="I28" t="n">
-        <v>-0.2</v>
+        <v>0.3</v>
       </c>
       <c r="J28" t="n">
-        <v>-8.199999999999999</v>
+        <v>-8.5</v>
       </c>
       <c r="K28" t="n">
-        <v>2016910</v>
+        <v>2018738</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -5455,16 +5455,16 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>252797</v>
+        <v>252826</v>
       </c>
       <c r="I29" t="n">
-        <v>-7.1</v>
+        <v>-0.3</v>
       </c>
       <c r="J29" t="n">
-        <v>-21.3</v>
+        <v>-14</v>
       </c>
       <c r="K29" t="n">
-        <v>49722</v>
+        <v>49736</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -5514,16 +5514,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>139936</v>
+        <v>142226</v>
       </c>
       <c r="I30" t="n">
-        <v>-10.8</v>
+        <v>-3</v>
       </c>
       <c r="J30" t="n">
-        <v>-42.4</v>
+        <v>-36.5</v>
       </c>
       <c r="K30" t="n">
-        <v>37196</v>
+        <v>37441</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -5573,16 +5573,16 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>89104</v>
+        <v>95991</v>
       </c>
       <c r="I31" t="n">
-        <v>114.3</v>
+        <v>57.5</v>
       </c>
       <c r="J31" t="n">
-        <v>1688.3</v>
+        <v>1847.2</v>
       </c>
       <c r="K31" t="n">
-        <v>28471</v>
+        <v>29421</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -5632,16 +5632,16 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>75512134</v>
+        <v>75471341</v>
       </c>
       <c r="I32" t="n">
         <v>0.1</v>
       </c>
       <c r="J32" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="K32" t="n">
-        <v>249765</v>
+        <v>252553</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -5691,16 +5691,16 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>316954</v>
+        <v>360576</v>
       </c>
       <c r="I33" t="n">
-        <v>-4.8</v>
+        <v>12.4</v>
       </c>
       <c r="J33" t="n">
-        <v>-29.6</v>
+        <v>-7.4</v>
       </c>
       <c r="K33" t="n">
-        <v>67528</v>
+        <v>71661</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -5750,16 +5750,16 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>174819</v>
+        <v>177289</v>
       </c>
       <c r="I34" t="n">
-        <v>-1.8</v>
+        <v>1.1</v>
       </c>
       <c r="J34" t="n">
-        <v>99</v>
+        <v>131.8</v>
       </c>
       <c r="K34" t="n">
-        <v>36560</v>
+        <v>36405</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -5809,16 +5809,16 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>357642</v>
+        <v>396020</v>
       </c>
       <c r="I35" t="n">
-        <v>-2.3</v>
+        <v>16</v>
       </c>
       <c r="J35" t="n">
-        <v>10397.6</v>
+        <v>11524.1</v>
       </c>
       <c r="K35" t="n">
-        <v>57789</v>
+        <v>61045</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -5868,16 +5868,16 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>114154</v>
+        <v>71059</v>
       </c>
       <c r="I36" t="n">
-        <v>-41.8</v>
+        <v>-32.8</v>
       </c>
       <c r="J36" t="n">
-        <v>2910.7</v>
+        <v>1774.1</v>
       </c>
       <c r="K36" t="n">
-        <v>29017</v>
+        <v>22237</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -5927,16 +5927,16 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>2693690</v>
+        <v>3108769</v>
       </c>
       <c r="I37" t="n">
-        <v>-4.2</v>
+        <v>9.5</v>
       </c>
       <c r="J37" t="n">
-        <v>-59.1</v>
+        <v>-51.1</v>
       </c>
       <c r="K37" t="n">
-        <v>896572</v>
+        <v>945352</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -5986,16 +5986,16 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>135054</v>
+        <v>125005</v>
       </c>
       <c r="I38" t="n">
-        <v>-0.3</v>
+        <v>-13.6</v>
       </c>
       <c r="J38" t="n">
-        <v>3860.6</v>
+        <v>3565.9</v>
       </c>
       <c r="K38" t="n">
-        <v>34002</v>
+        <v>32615</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
radar silent 10/12 20:59
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -3862,16 +3862,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>24060536</v>
+        <v>24380280</v>
       </c>
       <c r="I2" t="n">
-        <v>-1.8</v>
+        <v>-0.6</v>
       </c>
       <c r="J2" t="n">
-        <v>-21.1</v>
+        <v>-20.1</v>
       </c>
       <c r="K2" t="n">
-        <v>840644</v>
+        <v>841452</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -3921,16 +3921,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1596474</v>
+        <v>1611343</v>
       </c>
       <c r="I3" t="n">
-        <v>3.7</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>29.9</v>
+        <v>31.1</v>
       </c>
       <c r="K3" t="n">
-        <v>178443</v>
+        <v>179626</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -3980,16 +3980,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>746750</v>
+        <v>768765</v>
       </c>
       <c r="I4" t="n">
-        <v>-6.9</v>
+        <v>1.5</v>
       </c>
       <c r="J4" t="n">
-        <v>-13</v>
+        <v>-10.4</v>
       </c>
       <c r="K4" t="n">
-        <v>101738</v>
+        <v>103018</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -4039,16 +4039,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>22881</v>
+        <v>22961</v>
       </c>
       <c r="I5" t="n">
-        <v>10.1</v>
+        <v>10.5</v>
       </c>
       <c r="J5" t="n">
-        <v>34.9</v>
+        <v>35.4</v>
       </c>
       <c r="K5" t="n">
-        <v>14172</v>
+        <v>14219</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -4098,16 +4098,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1268385</v>
+        <v>1249376</v>
       </c>
       <c r="I6" t="n">
-        <v>20.8</v>
+        <v>11.8</v>
       </c>
       <c r="J6" t="n">
-        <v>12.3</v>
+        <v>10.6</v>
       </c>
       <c r="K6" t="n">
-        <v>110511</v>
+        <v>110473</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -4157,16 +4157,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>29374</v>
+        <v>29220</v>
       </c>
       <c r="I7" t="n">
-        <v>-7.8</v>
+        <v>-3.4</v>
       </c>
       <c r="J7" t="n">
-        <v>-54.3</v>
+        <v>-54.6</v>
       </c>
       <c r="K7" t="n">
-        <v>13263</v>
+        <v>13224</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -4216,16 +4216,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>35999</v>
+        <v>35166</v>
       </c>
       <c r="I8" t="n">
-        <v>-5.7</v>
+        <v>2.3</v>
       </c>
       <c r="J8" t="n">
-        <v>-35.4</v>
+        <v>-36.9</v>
       </c>
       <c r="K8" t="n">
-        <v>20012</v>
+        <v>19797</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -4275,16 +4275,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1434972</v>
+        <v>1442601</v>
       </c>
       <c r="I9" t="n">
-        <v>-1.5</v>
+        <v>0.9</v>
       </c>
       <c r="J9" t="n">
-        <v>-29.4</v>
+        <v>-29</v>
       </c>
       <c r="K9" t="n">
-        <v>166668</v>
+        <v>167808</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -4334,16 +4334,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>44972</v>
+        <v>45692</v>
       </c>
       <c r="I10" t="n">
-        <v>10.4</v>
+        <v>8.6</v>
       </c>
       <c r="J10" t="n">
-        <v>-38.2</v>
+        <v>-37.2</v>
       </c>
       <c r="K10" t="n">
-        <v>19074</v>
+        <v>19277</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -4393,16 +4393,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>178024</v>
+        <v>180873</v>
       </c>
       <c r="I11" t="n">
-        <v>-5.5</v>
+        <v>-9.699999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>-50.1</v>
+        <v>-49.3</v>
       </c>
       <c r="K11" t="n">
-        <v>58079</v>
+        <v>58312</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -4452,16 +4452,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3356276</v>
+        <v>3378888</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.9</v>
+        <v>-0.1</v>
       </c>
       <c r="J12" t="n">
-        <v>20.7</v>
+        <v>21.5</v>
       </c>
       <c r="K12" t="n">
-        <v>159791</v>
+        <v>160737</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -4511,16 +4511,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>76361</v>
+        <v>80461</v>
       </c>
       <c r="I13" t="n">
-        <v>3.7</v>
+        <v>-8.1</v>
       </c>
       <c r="J13" t="n">
-        <v>1270.4</v>
+        <v>1344</v>
       </c>
       <c r="K13" t="n">
-        <v>30312</v>
+        <v>31079</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -4570,16 +4570,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>126787269</v>
+        <v>126273561</v>
       </c>
       <c r="I14" t="n">
-        <v>0.1</v>
+        <v>-1</v>
       </c>
       <c r="J14" t="n">
-        <v>13.5</v>
+        <v>13</v>
       </c>
       <c r="K14" t="n">
-        <v>253126</v>
+        <v>249430</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -4629,16 +4629,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>344636830</v>
+        <v>346474280</v>
       </c>
       <c r="I15" t="n">
-        <v>-2.2</v>
+        <v>-1.2</v>
       </c>
       <c r="J15" t="n">
-        <v>-4.2</v>
+        <v>-3.9</v>
       </c>
       <c r="K15" t="n">
-        <v>2746603</v>
+        <v>2751964</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -4688,16 +4688,16 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>6736029</v>
+        <v>6800742</v>
       </c>
       <c r="I16" t="n">
-        <v>-3.8</v>
+        <v>-3.3</v>
       </c>
       <c r="J16" t="n">
-        <v>-5.7</v>
+        <v>-4.8</v>
       </c>
       <c r="K16" t="n">
-        <v>329001</v>
+        <v>330362</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -4806,16 +4806,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>990473</v>
+        <v>974540</v>
       </c>
       <c r="I18" t="n">
-        <v>2</v>
+        <v>0.2</v>
       </c>
       <c r="J18" t="n">
-        <v>69.5</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>118457</v>
+        <v>118024</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -4865,16 +4865,16 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>314474</v>
+        <v>315559</v>
       </c>
       <c r="I19" t="n">
-        <v>-1.3</v>
+        <v>-1</v>
       </c>
       <c r="J19" t="n">
-        <v>16.5</v>
+        <v>12.4</v>
       </c>
       <c r="K19" t="n">
-        <v>61485</v>
+        <v>61614</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -4924,16 +4924,16 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>53343439</v>
+        <v>51864960</v>
       </c>
       <c r="I20" t="n">
-        <v>3.4</v>
+        <v>-0.1</v>
       </c>
       <c r="J20" t="n">
-        <v>20.4</v>
+        <v>21.1</v>
       </c>
       <c r="K20" t="n">
-        <v>1217536</v>
+        <v>1218333</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -4983,16 +4983,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>16984017</v>
+        <v>16940483</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.3</v>
+        <v>-2</v>
       </c>
       <c r="J21" t="n">
-        <v>25.1</v>
+        <v>24</v>
       </c>
       <c r="K21" t="n">
-        <v>862220</v>
+        <v>863777</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -5045,10 +5045,10 @@
         <v>123915</v>
       </c>
       <c r="I22" t="n">
-        <v>2.7</v>
+        <v>2.3</v>
       </c>
       <c r="J22" t="n">
-        <v>-10.3</v>
+        <v>-8.5</v>
       </c>
       <c r="K22" t="n">
         <v>31374</v>
@@ -5101,16 +5101,16 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>56544</v>
+        <v>58289</v>
       </c>
       <c r="I23" t="n">
-        <v>1.8</v>
+        <v>3.8</v>
       </c>
       <c r="J23" t="n">
-        <v>10.2</v>
+        <v>13.1</v>
       </c>
       <c r="K23" t="n">
-        <v>20180</v>
+        <v>20418</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -5160,16 +5160,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>472774</v>
+        <v>401242</v>
       </c>
       <c r="I24" t="n">
-        <v>73.7</v>
+        <v>5</v>
       </c>
       <c r="J24" t="n">
-        <v>15168.1</v>
+        <v>12857.9</v>
       </c>
       <c r="K24" t="n">
-        <v>91367</v>
+        <v>87845</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -5219,16 +5219,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>139540782</v>
+        <v>139986323</v>
       </c>
       <c r="I25" t="n">
-        <v>-4.2</v>
+        <v>-2.9</v>
       </c>
       <c r="J25" t="n">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="K25" t="n">
-        <v>2360359</v>
+        <v>2367204</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -5278,16 +5278,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>377277220</v>
+        <v>379920450</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.8</v>
+        <v>0.1</v>
       </c>
       <c r="J26" t="n">
-        <v>1.8</v>
+        <v>2.6</v>
       </c>
       <c r="K26" t="n">
-        <v>11381508</v>
+        <v>11398553</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -5337,16 +5337,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>587351830</v>
+        <v>588348600</v>
       </c>
       <c r="I27" t="n">
-        <v>-1.4</v>
+        <v>-0.5</v>
       </c>
       <c r="J27" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="K27" t="n">
-        <v>8741285</v>
+        <v>8760117</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -5396,16 +5396,16 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>41190278</v>
+        <v>41727476</v>
       </c>
       <c r="I28" t="n">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
       <c r="J28" t="n">
-        <v>-8.5</v>
+        <v>-7.3</v>
       </c>
       <c r="K28" t="n">
-        <v>2018738</v>
+        <v>2026844</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -5458,10 +5458,10 @@
         <v>252826</v>
       </c>
       <c r="I29" t="n">
-        <v>-0.3</v>
+        <v>-0.2</v>
       </c>
       <c r="J29" t="n">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="K29" t="n">
         <v>49736</v>
@@ -5514,16 +5514,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>142226</v>
+        <v>143790</v>
       </c>
       <c r="I30" t="n">
-        <v>-3</v>
+        <v>-0.4</v>
       </c>
       <c r="J30" t="n">
-        <v>-36.5</v>
+        <v>-28.7</v>
       </c>
       <c r="K30" t="n">
-        <v>37441</v>
+        <v>37701</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -5573,16 +5573,16 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>95991</v>
+        <v>90295</v>
       </c>
       <c r="I31" t="n">
-        <v>57.5</v>
+        <v>19.7</v>
       </c>
       <c r="J31" t="n">
-        <v>1847.2</v>
+        <v>1731.5</v>
       </c>
       <c r="K31" t="n">
-        <v>29421</v>
+        <v>28725</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -5632,16 +5632,16 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>75471341</v>
+        <v>75231770</v>
       </c>
       <c r="I32" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="J32" t="n">
         <v>0.1</v>
       </c>
-      <c r="J32" t="n">
-        <v>0.3</v>
-      </c>
       <c r="K32" t="n">
-        <v>252553</v>
+        <v>251981</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -5691,16 +5691,16 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>360576</v>
+        <v>339532</v>
       </c>
       <c r="I33" t="n">
-        <v>12.4</v>
+        <v>10.4</v>
       </c>
       <c r="J33" t="n">
-        <v>-7.4</v>
+        <v>-13.9</v>
       </c>
       <c r="K33" t="n">
-        <v>71661</v>
+        <v>70041</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -5750,16 +5750,16 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>177289</v>
+        <v>177215</v>
       </c>
       <c r="I34" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="J34" t="n">
-        <v>131.8</v>
+        <v>146</v>
       </c>
       <c r="K34" t="n">
-        <v>36405</v>
+        <v>36662</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -5809,16 +5809,16 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>396020</v>
+        <v>409551</v>
       </c>
       <c r="I35" t="n">
-        <v>16</v>
+        <v>16.2</v>
       </c>
       <c r="J35" t="n">
-        <v>11524.1</v>
+        <v>11921.3</v>
       </c>
       <c r="K35" t="n">
-        <v>61045</v>
+        <v>61567</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -5868,16 +5868,16 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>71059</v>
+        <v>61409</v>
       </c>
       <c r="I36" t="n">
-        <v>-32.8</v>
+        <v>-31.7</v>
       </c>
       <c r="J36" t="n">
-        <v>1774.1</v>
+        <v>1519.6</v>
       </c>
       <c r="K36" t="n">
-        <v>22237</v>
+        <v>20156</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -5927,16 +5927,16 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>3108769</v>
+        <v>3107588</v>
       </c>
       <c r="I37" t="n">
-        <v>9.5</v>
+        <v>10.7</v>
       </c>
       <c r="J37" t="n">
-        <v>-51.1</v>
+        <v>-50.1</v>
       </c>
       <c r="K37" t="n">
-        <v>945352</v>
+        <v>942136</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -5986,16 +5986,16 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>125005</v>
+        <v>124406</v>
       </c>
       <c r="I38" t="n">
         <v>-13.6</v>
       </c>
       <c r="J38" t="n">
-        <v>3565.9</v>
+        <v>3548.3</v>
       </c>
       <c r="K38" t="n">
-        <v>32615</v>
+        <v>32446</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
radar silent 10/12 21:44
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -3862,16 +3862,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>23850352</v>
+        <v>24072622</v>
       </c>
       <c r="I2" t="n">
-        <v>-3.1</v>
+        <v>-2.4</v>
       </c>
       <c r="J2" t="n">
-        <v>-20.7</v>
+        <v>-20</v>
       </c>
       <c r="K2" t="n">
-        <v>836166</v>
+        <v>835236</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -3921,16 +3921,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1655237</v>
+        <v>1751936</v>
       </c>
       <c r="I3" t="n">
-        <v>-2.8</v>
+        <v>11</v>
       </c>
       <c r="J3" t="n">
-        <v>30.2</v>
+        <v>37.8</v>
       </c>
       <c r="K3" t="n">
-        <v>180910</v>
+        <v>187389</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -3980,16 +3980,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>802088</v>
+        <v>744506</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.3</v>
+        <v>-0.1</v>
       </c>
       <c r="J4" t="n">
-        <v>-8.199999999999999</v>
+        <v>-14.8</v>
       </c>
       <c r="K4" t="n">
-        <v>105337</v>
+        <v>100872</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -4039,16 +4039,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>20029</v>
+        <v>19455</v>
       </c>
       <c r="I5" t="n">
-        <v>-12.4</v>
+        <v>-15</v>
       </c>
       <c r="J5" t="n">
-        <v>23.8</v>
+        <v>20.3</v>
       </c>
       <c r="K5" t="n">
-        <v>13297</v>
+        <v>13097</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -4098,16 +4098,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1231928</v>
+        <v>1238160</v>
       </c>
       <c r="I6" t="n">
-        <v>-2.3</v>
+        <v>-1.4</v>
       </c>
       <c r="J6" t="n">
-        <v>7.1</v>
+        <v>11.1</v>
       </c>
       <c r="K6" t="n">
-        <v>109575</v>
+        <v>109272</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -4157,16 +4157,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>24438</v>
+        <v>25186</v>
       </c>
       <c r="I7" t="n">
-        <v>-20.5</v>
+        <v>-15.6</v>
       </c>
       <c r="J7" t="n">
-        <v>-63.3</v>
+        <v>-62.3</v>
       </c>
       <c r="K7" t="n">
-        <v>11718</v>
+        <v>11900</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -4216,16 +4216,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>35821</v>
+        <v>31005</v>
       </c>
       <c r="I8" t="n">
-        <v>-13</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>-54.9</v>
+        <v>-66.7</v>
       </c>
       <c r="K8" t="n">
-        <v>19968</v>
+        <v>18586</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -4275,16 +4275,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1688817</v>
+        <v>1651337</v>
       </c>
       <c r="I9" t="n">
-        <v>13.6</v>
+        <v>13.8</v>
       </c>
       <c r="J9" t="n">
-        <v>-6.1</v>
+        <v>-9.5</v>
       </c>
       <c r="K9" t="n">
-        <v>164012</v>
+        <v>162496</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -4334,16 +4334,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>46455</v>
+        <v>46305</v>
       </c>
       <c r="I10" t="n">
-        <v>5.1</v>
+        <v>3</v>
       </c>
       <c r="J10" t="n">
-        <v>-1</v>
+        <v>5.7</v>
       </c>
       <c r="K10" t="n">
-        <v>19411</v>
+        <v>19208</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -4393,16 +4393,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>186897</v>
+        <v>198232</v>
       </c>
       <c r="I11" t="n">
-        <v>4.9</v>
+        <v>11</v>
       </c>
       <c r="J11" t="n">
-        <v>-42.6</v>
+        <v>-36.5</v>
       </c>
       <c r="K11" t="n">
-        <v>59373</v>
+        <v>61606</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -4452,16 +4452,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3394666</v>
+        <v>3455357</v>
       </c>
       <c r="I12" t="n">
-        <v>0.4</v>
+        <v>2.9</v>
       </c>
       <c r="J12" t="n">
-        <v>20.8</v>
+        <v>23</v>
       </c>
       <c r="K12" t="n">
-        <v>160888</v>
+        <v>161791</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -4511,16 +4511,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>55150</v>
+        <v>55230</v>
       </c>
       <c r="I13" t="n">
-        <v>-25.7</v>
+        <v>-22.5</v>
       </c>
       <c r="J13" t="n">
-        <v>889.7</v>
+        <v>891.2</v>
       </c>
       <c r="K13" t="n">
-        <v>25885</v>
+        <v>25524</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -4570,16 +4570,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>126266068</v>
+        <v>131131213</v>
       </c>
       <c r="I14" t="n">
-        <v>-2.9</v>
+        <v>2.7</v>
       </c>
       <c r="J14" t="n">
-        <v>15.1</v>
+        <v>22.7</v>
       </c>
       <c r="K14" t="n">
-        <v>247862</v>
+        <v>258190</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -4629,16 +4629,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>341947180</v>
+        <v>338844370</v>
       </c>
       <c r="I15" t="n">
-        <v>-1.9</v>
+        <v>-2.2</v>
       </c>
       <c r="J15" t="n">
-        <v>-4.7</v>
+        <v>-4.8</v>
       </c>
       <c r="K15" t="n">
-        <v>2681395</v>
+        <v>2668000</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -4688,16 +4688,16 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>6815816</v>
+        <v>6779526</v>
       </c>
       <c r="I16" t="n">
-        <v>-0.6</v>
+        <v>1.5</v>
       </c>
       <c r="J16" t="n">
-        <v>-5</v>
+        <v>-5.5</v>
       </c>
       <c r="K16" t="n">
-        <v>331027</v>
+        <v>328597</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -4806,16 +4806,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>971522</v>
+        <v>971720</v>
       </c>
       <c r="I18" t="n">
-        <v>-1.9</v>
+        <v>0.2</v>
       </c>
       <c r="J18" t="n">
         <v>64.90000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>117925</v>
+        <v>117695</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -4865,16 +4865,16 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>318516</v>
+        <v>313388</v>
       </c>
       <c r="I19" t="n">
-        <v>1.3</v>
+        <v>-0.3</v>
       </c>
       <c r="J19" t="n">
-        <v>11.3</v>
+        <v>6.3</v>
       </c>
       <c r="K19" t="n">
-        <v>61614</v>
+        <v>61477</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -4924,16 +4924,16 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>52195549</v>
+        <v>52284445</v>
       </c>
       <c r="I20" t="n">
-        <v>-2.4</v>
+        <v>-2.1</v>
       </c>
       <c r="J20" t="n">
-        <v>19.5</v>
+        <v>29.8</v>
       </c>
       <c r="K20" t="n">
-        <v>1207683</v>
+        <v>1238859</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -4983,16 +4983,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>16405611</v>
+        <v>16624645</v>
       </c>
       <c r="I21" t="n">
-        <v>-5.4</v>
+        <v>-2.5</v>
       </c>
       <c r="J21" t="n">
-        <v>10.8</v>
+        <v>17.7</v>
       </c>
       <c r="K21" t="n">
-        <v>857034</v>
+        <v>860599</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -5045,7 +5045,7 @@
         <v>131780</v>
       </c>
       <c r="I22" t="n">
-        <v>2.2</v>
+        <v>6.3</v>
       </c>
       <c r="J22" t="n">
         <v>-8.4</v>
@@ -5101,16 +5101,16 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>56755</v>
+        <v>54096</v>
       </c>
       <c r="I23" t="n">
-        <v>-0.5</v>
+        <v>-6.1</v>
       </c>
       <c r="J23" t="n">
-        <v>11.9</v>
+        <v>-5.7</v>
       </c>
       <c r="K23" t="n">
-        <v>20080</v>
+        <v>19522</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -5160,16 +5160,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>605929</v>
+        <v>509346</v>
       </c>
       <c r="I24" t="n">
-        <v>25.3</v>
+        <v>16.9</v>
       </c>
       <c r="J24" t="n">
-        <v>19468.3</v>
+        <v>16349.1</v>
       </c>
       <c r="K24" t="n">
-        <v>109705</v>
+        <v>100621</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -5219,16 +5219,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>140543209</v>
+        <v>139989195</v>
       </c>
       <c r="I25" t="n">
-        <v>-2</v>
+        <v>-2.5</v>
       </c>
       <c r="J25" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="K25" t="n">
-        <v>2368230</v>
+        <v>2372232</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -5281,10 +5281,10 @@
         <v>377762630</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.3</v>
+        <v>-0.5</v>
       </c>
       <c r="J26" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="K26" t="n">
         <v>11408915</v>
@@ -5337,16 +5337,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>590284530</v>
+        <v>590781190</v>
       </c>
       <c r="I27" t="n">
         <v>0.5</v>
       </c>
       <c r="J27" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
       <c r="K27" t="n">
-        <v>8767802</v>
+        <v>8776728</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -5396,16 +5396,16 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>41439041</v>
+        <v>41521532</v>
       </c>
       <c r="I28" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="J28" t="n">
-        <v>-7.3</v>
+        <v>-6.3</v>
       </c>
       <c r="K28" t="n">
-        <v>2018694</v>
+        <v>2021098</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -5455,16 +5455,16 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>256060</v>
+        <v>255489</v>
       </c>
       <c r="I29" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="J29" t="n">
-        <v>-13.2</v>
+        <v>-15.2</v>
       </c>
       <c r="K29" t="n">
-        <v>50009</v>
+        <v>49801</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -5514,16 +5514,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>137327</v>
+        <v>138840</v>
       </c>
       <c r="I30" t="n">
-        <v>-4.2</v>
+        <v>-2.5</v>
       </c>
       <c r="J30" t="n">
-        <v>-29</v>
+        <v>-27.1</v>
       </c>
       <c r="K30" t="n">
-        <v>36817</v>
+        <v>37044</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -5573,16 +5573,16 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>81643</v>
+        <v>76349</v>
       </c>
       <c r="I31" t="n">
-        <v>-12.2</v>
+        <v>-11.4</v>
       </c>
       <c r="J31" t="n">
-        <v>1556</v>
+        <v>1448.6</v>
       </c>
       <c r="K31" t="n">
-        <v>27366</v>
+        <v>26462</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -5632,16 +5632,16 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>75532544</v>
+        <v>75571268</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="J32" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="K32" t="n">
-        <v>249676</v>
+        <v>248104</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -5691,16 +5691,16 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>497815</v>
+        <v>538809</v>
       </c>
       <c r="I33" t="n">
-        <v>47.9</v>
+        <v>46.7</v>
       </c>
       <c r="J33" t="n">
-        <v>32.6</v>
+        <v>22.5</v>
       </c>
       <c r="K33" t="n">
-        <v>85515</v>
+        <v>89590</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -5750,16 +5750,16 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>211024</v>
+        <v>194636</v>
       </c>
       <c r="I34" t="n">
-        <v>19.1</v>
+        <v>11.8</v>
       </c>
       <c r="J34" t="n">
-        <v>192.5</v>
+        <v>182.5</v>
       </c>
       <c r="K34" t="n">
-        <v>40775</v>
+        <v>38326</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -5809,16 +5809,16 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>276047</v>
+        <v>277499</v>
       </c>
       <c r="I35" t="n">
-        <v>-26.2</v>
+        <v>-28</v>
       </c>
       <c r="J35" t="n">
-        <v>8002.6</v>
+        <v>8045.2</v>
       </c>
       <c r="K35" t="n">
-        <v>50358</v>
+        <v>50928</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -5868,16 +5868,16 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>48406</v>
+        <v>43126</v>
       </c>
       <c r="I36" t="n">
-        <v>-49.7</v>
+        <v>-41.9</v>
       </c>
       <c r="J36" t="n">
-        <v>1176.7</v>
+        <v>1037.4</v>
       </c>
       <c r="K36" t="n">
-        <v>17460</v>
+        <v>16215</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -5927,16 +5927,16 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>2975604</v>
+        <v>2836104</v>
       </c>
       <c r="I37" t="n">
-        <v>-2.6</v>
+        <v>-8.4</v>
       </c>
       <c r="J37" t="n">
-        <v>-56.7</v>
+        <v>-65</v>
       </c>
       <c r="K37" t="n">
-        <v>881162</v>
+        <v>835640</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -5986,16 +5986,16 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>134591</v>
+        <v>144563</v>
       </c>
       <c r="I38" t="n">
-        <v>4.3</v>
+        <v>17</v>
       </c>
       <c r="J38" t="n">
-        <v>3847</v>
+        <v>4139.4</v>
       </c>
       <c r="K38" t="n">
-        <v>34098</v>
+        <v>35429</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
radar silent 10/12 22:01
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -3862,16 +3862,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>24072622</v>
+        <v>23814811</v>
       </c>
       <c r="I2" t="n">
         <v>-2.4</v>
       </c>
       <c r="J2" t="n">
-        <v>-20</v>
+        <v>-19.8</v>
       </c>
       <c r="K2" t="n">
-        <v>835236</v>
+        <v>838621</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -3921,16 +3921,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1751936</v>
+        <v>1580021</v>
       </c>
       <c r="I3" t="n">
-        <v>11</v>
+        <v>-1.9</v>
       </c>
       <c r="J3" t="n">
-        <v>37.8</v>
+        <v>28.3</v>
       </c>
       <c r="K3" t="n">
-        <v>187389</v>
+        <v>176730</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -3980,16 +3980,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>744506</v>
+        <v>736556</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.1</v>
+        <v>-4.2</v>
       </c>
       <c r="J4" t="n">
-        <v>-14.8</v>
+        <v>-13.3</v>
       </c>
       <c r="K4" t="n">
-        <v>100872</v>
+        <v>100935</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -4039,16 +4039,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>19455</v>
+        <v>19500</v>
       </c>
       <c r="I5" t="n">
-        <v>-15</v>
+        <v>-15.1</v>
       </c>
       <c r="J5" t="n">
-        <v>20.3</v>
+        <v>16.3</v>
       </c>
       <c r="K5" t="n">
-        <v>13097</v>
+        <v>13110</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -4098,16 +4098,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1238160</v>
+        <v>1215332</v>
       </c>
       <c r="I6" t="n">
-        <v>-1.4</v>
+        <v>-5.1</v>
       </c>
       <c r="J6" t="n">
-        <v>11.1</v>
+        <v>10.5</v>
       </c>
       <c r="K6" t="n">
-        <v>109272</v>
+        <v>108858</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -4157,16 +4157,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>25186</v>
+        <v>24965</v>
       </c>
       <c r="I7" t="n">
-        <v>-15.6</v>
+        <v>-14.6</v>
       </c>
       <c r="J7" t="n">
-        <v>-62.3</v>
+        <v>-66.59999999999999</v>
       </c>
       <c r="K7" t="n">
-        <v>11900</v>
+        <v>11815</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -4216,16 +4216,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>31005</v>
+        <v>32780</v>
       </c>
       <c r="I8" t="n">
-        <v>-8.199999999999999</v>
+        <v>-7.8</v>
       </c>
       <c r="J8" t="n">
-        <v>-66.7</v>
+        <v>-73.40000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>18586</v>
+        <v>19136</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -4275,16 +4275,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1651337</v>
+        <v>1585467</v>
       </c>
       <c r="I9" t="n">
-        <v>13.8</v>
+        <v>10</v>
       </c>
       <c r="J9" t="n">
-        <v>-9.5</v>
+        <v>-17.5</v>
       </c>
       <c r="K9" t="n">
-        <v>162496</v>
+        <v>163420</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -4334,16 +4334,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>46305</v>
+        <v>45291</v>
       </c>
       <c r="I10" t="n">
-        <v>3</v>
+        <v>-2.1</v>
       </c>
       <c r="J10" t="n">
-        <v>5.7</v>
+        <v>3.5</v>
       </c>
       <c r="K10" t="n">
-        <v>19208</v>
+        <v>19124</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -4393,16 +4393,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>198232</v>
+        <v>185440</v>
       </c>
       <c r="I11" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="J11" t="n">
-        <v>-36.5</v>
+        <v>-40.2</v>
       </c>
       <c r="K11" t="n">
-        <v>61606</v>
+        <v>59419</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -4452,16 +4452,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3455357</v>
+        <v>3426203</v>
       </c>
       <c r="I12" t="n">
-        <v>2.9</v>
+        <v>0.5</v>
       </c>
       <c r="J12" t="n">
-        <v>23</v>
+        <v>21.9</v>
       </c>
       <c r="K12" t="n">
-        <v>161791</v>
+        <v>161821</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -4511,16 +4511,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>55230</v>
+        <v>60642</v>
       </c>
       <c r="I13" t="n">
-        <v>-22.5</v>
+        <v>-24.7</v>
       </c>
       <c r="J13" t="n">
-        <v>891.2</v>
+        <v>988.3</v>
       </c>
       <c r="K13" t="n">
-        <v>25524</v>
+        <v>27142</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -4570,16 +4570,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>131131213</v>
+        <v>126847295</v>
       </c>
       <c r="I14" t="n">
-        <v>2.7</v>
+        <v>0.3</v>
       </c>
       <c r="J14" t="n">
-        <v>22.7</v>
+        <v>17.7</v>
       </c>
       <c r="K14" t="n">
-        <v>258190</v>
+        <v>255338</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -4629,16 +4629,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>338844370</v>
+        <v>336644870</v>
       </c>
       <c r="I15" t="n">
-        <v>-2.2</v>
+        <v>-2.8</v>
       </c>
       <c r="J15" t="n">
-        <v>-4.8</v>
+        <v>-6.3</v>
       </c>
       <c r="K15" t="n">
-        <v>2668000</v>
+        <v>2650192</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -4688,16 +4688,16 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>6779526</v>
+        <v>6693874</v>
       </c>
       <c r="I16" t="n">
-        <v>1.5</v>
+        <v>-1.5</v>
       </c>
       <c r="J16" t="n">
-        <v>-5.5</v>
+        <v>-6.2</v>
       </c>
       <c r="K16" t="n">
-        <v>328597</v>
+        <v>329346</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -4747,16 +4747,16 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>1213089</v>
+        <v>1213360</v>
       </c>
       <c r="I17" t="n">
-        <v>-3.1</v>
+        <v>-3</v>
       </c>
       <c r="J17" t="n">
         <v>-1.5</v>
       </c>
       <c r="K17" t="n">
-        <v>265756</v>
+        <v>265502</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -4806,16 +4806,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>971720</v>
+        <v>1010207</v>
       </c>
       <c r="I18" t="n">
-        <v>0.2</v>
+        <v>3.7</v>
       </c>
       <c r="J18" t="n">
-        <v>64.90000000000001</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>117695</v>
+        <v>119770</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -4865,16 +4865,16 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>313388</v>
+        <v>311035</v>
       </c>
       <c r="I19" t="n">
-        <v>-0.3</v>
+        <v>-1.4</v>
       </c>
       <c r="J19" t="n">
-        <v>6.3</v>
+        <v>3.2</v>
       </c>
       <c r="K19" t="n">
-        <v>61477</v>
+        <v>61422</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -4924,16 +4924,16 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>52284445</v>
+        <v>51261746</v>
       </c>
       <c r="I20" t="n">
-        <v>-2.1</v>
+        <v>-1.1</v>
       </c>
       <c r="J20" t="n">
-        <v>29.8</v>
+        <v>27.2</v>
       </c>
       <c r="K20" t="n">
-        <v>1238859</v>
+        <v>1215148</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -4983,16 +4983,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>16624645</v>
+        <v>16650067</v>
       </c>
       <c r="I21" t="n">
-        <v>-2.5</v>
+        <v>-0.9</v>
       </c>
       <c r="J21" t="n">
-        <v>17.7</v>
+        <v>19</v>
       </c>
       <c r="K21" t="n">
-        <v>860599</v>
+        <v>862616</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -5042,16 +5042,16 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>131780</v>
+        <v>133835</v>
       </c>
       <c r="I22" t="n">
-        <v>6.3</v>
+        <v>8</v>
       </c>
       <c r="J22" t="n">
-        <v>-8.4</v>
+        <v>-7</v>
       </c>
       <c r="K22" t="n">
-        <v>32957</v>
+        <v>33154</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -5101,16 +5101,16 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>54096</v>
+        <v>49660</v>
       </c>
       <c r="I23" t="n">
-        <v>-6.1</v>
+        <v>-14.8</v>
       </c>
       <c r="J23" t="n">
-        <v>-5.7</v>
+        <v>-8.1</v>
       </c>
       <c r="K23" t="n">
-        <v>19522</v>
+        <v>18569</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -5160,16 +5160,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>509346</v>
+        <v>508629</v>
       </c>
       <c r="I24" t="n">
-        <v>16.9</v>
+        <v>21</v>
       </c>
       <c r="J24" t="n">
-        <v>16349.1</v>
+        <v>16326</v>
       </c>
       <c r="K24" t="n">
-        <v>100621</v>
+        <v>103833</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -5219,16 +5219,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>139989195</v>
+        <v>139859458</v>
       </c>
       <c r="I25" t="n">
-        <v>-2.5</v>
+        <v>-0.4</v>
       </c>
       <c r="J25" t="n">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
       <c r="K25" t="n">
-        <v>2372232</v>
+        <v>2367718</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -5278,16 +5278,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>377762630</v>
+        <v>379158990</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.5</v>
+        <v>-0.2</v>
       </c>
       <c r="J26" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="K26" t="n">
-        <v>11408915</v>
+        <v>11411977</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -5337,16 +5337,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>590781190</v>
+        <v>590050840</v>
       </c>
       <c r="I27" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="J27" t="n">
-        <v>3.3</v>
+        <v>3.1</v>
       </c>
       <c r="K27" t="n">
-        <v>8776728</v>
+        <v>8766937</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -5396,16 +5396,16 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>41521532</v>
+        <v>41704208</v>
       </c>
       <c r="I28" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="J28" t="n">
-        <v>-6.3</v>
+        <v>-5</v>
       </c>
       <c r="K28" t="n">
-        <v>2021098</v>
+        <v>2024909</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -5455,16 +5455,16 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>255489</v>
+        <v>249426</v>
       </c>
       <c r="I29" t="n">
-        <v>1.1</v>
+        <v>-1.3</v>
       </c>
       <c r="J29" t="n">
-        <v>-15.2</v>
+        <v>-22.2</v>
       </c>
       <c r="K29" t="n">
-        <v>49801</v>
+        <v>49419</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -5514,16 +5514,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>138840</v>
+        <v>141196</v>
       </c>
       <c r="I30" t="n">
-        <v>-2.5</v>
+        <v>-1.8</v>
       </c>
       <c r="J30" t="n">
-        <v>-27.1</v>
+        <v>-26.4</v>
       </c>
       <c r="K30" t="n">
-        <v>37044</v>
+        <v>37343</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -5573,16 +5573,16 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>76349</v>
+        <v>62518</v>
       </c>
       <c r="I31" t="n">
-        <v>-11.4</v>
+        <v>-31.1</v>
       </c>
       <c r="J31" t="n">
-        <v>1448.6</v>
+        <v>1168.1</v>
       </c>
       <c r="K31" t="n">
-        <v>26462</v>
+        <v>23956</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -5632,16 +5632,16 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>75571268</v>
+        <v>75391596</v>
       </c>
       <c r="I32" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="J32" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="K32" t="n">
-        <v>248104</v>
+        <v>248234</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -5691,16 +5691,16 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>538809</v>
+        <v>519967</v>
       </c>
       <c r="I33" t="n">
-        <v>46.7</v>
+        <v>54.4</v>
       </c>
       <c r="J33" t="n">
-        <v>22.5</v>
+        <v>17.1</v>
       </c>
       <c r="K33" t="n">
-        <v>89590</v>
+        <v>88129</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -5750,16 +5750,16 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>194636</v>
+        <v>195226</v>
       </c>
       <c r="I34" t="n">
-        <v>11.8</v>
+        <v>10.2</v>
       </c>
       <c r="J34" t="n">
-        <v>182.5</v>
+        <v>179</v>
       </c>
       <c r="K34" t="n">
-        <v>38326</v>
+        <v>38428</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -5809,16 +5809,16 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>277499</v>
+        <v>227832</v>
       </c>
       <c r="I35" t="n">
-        <v>-28</v>
+        <v>-41.7</v>
       </c>
       <c r="J35" t="n">
-        <v>8045.2</v>
+        <v>6587.4</v>
       </c>
       <c r="K35" t="n">
-        <v>50928</v>
+        <v>45593</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -5868,16 +5868,16 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>43126</v>
+        <v>47486</v>
       </c>
       <c r="I36" t="n">
-        <v>-41.9</v>
+        <v>-21.7</v>
       </c>
       <c r="J36" t="n">
-        <v>1037.4</v>
+        <v>1152.4</v>
       </c>
       <c r="K36" t="n">
-        <v>16215</v>
+        <v>17174</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -5927,16 +5927,16 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>2836104</v>
+        <v>2684835</v>
       </c>
       <c r="I37" t="n">
-        <v>-8.4</v>
+        <v>-13.1</v>
       </c>
       <c r="J37" t="n">
-        <v>-65</v>
+        <v>-65.90000000000001</v>
       </c>
       <c r="K37" t="n">
-        <v>835640</v>
+        <v>784085</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -5986,16 +5986,16 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>144563</v>
+        <v>141979</v>
       </c>
       <c r="I38" t="n">
-        <v>17</v>
+        <v>13.9</v>
       </c>
       <c r="J38" t="n">
-        <v>4139.4</v>
+        <v>4063.6</v>
       </c>
       <c r="K38" t="n">
-        <v>35429</v>
+        <v>35093</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
radar silent 10/12 22:16
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -3862,16 +3862,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>23814811</v>
+        <v>23903157</v>
       </c>
       <c r="I2" t="n">
-        <v>-2.4</v>
+        <v>-0.4</v>
       </c>
       <c r="J2" t="n">
-        <v>-19.8</v>
+        <v>-19.1</v>
       </c>
       <c r="K2" t="n">
-        <v>838621</v>
+        <v>836878</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -3921,16 +3921,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1580021</v>
+        <v>1576535</v>
       </c>
       <c r="I3" t="n">
-        <v>-1.9</v>
+        <v>-1.1</v>
       </c>
       <c r="J3" t="n">
-        <v>28.3</v>
+        <v>28.5</v>
       </c>
       <c r="K3" t="n">
-        <v>176730</v>
+        <v>176337</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -3980,16 +3980,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>736556</v>
+        <v>738697</v>
       </c>
       <c r="I4" t="n">
-        <v>-4.2</v>
+        <v>-1.9</v>
       </c>
       <c r="J4" t="n">
-        <v>-13.3</v>
+        <v>-10.5</v>
       </c>
       <c r="K4" t="n">
-        <v>100935</v>
+        <v>101000</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -4039,16 +4039,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>19500</v>
+        <v>18690</v>
       </c>
       <c r="I5" t="n">
-        <v>-15.1</v>
+        <v>-8.6</v>
       </c>
       <c r="J5" t="n">
-        <v>16.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>13110</v>
+        <v>12625</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -4098,16 +4098,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1215332</v>
+        <v>1199922</v>
       </c>
       <c r="I6" t="n">
-        <v>-5.1</v>
+        <v>-3.3</v>
       </c>
       <c r="J6" t="n">
-        <v>10.5</v>
+        <v>11.3</v>
       </c>
       <c r="K6" t="n">
-        <v>108858</v>
+        <v>107965</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -4157,16 +4157,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>24965</v>
+        <v>18976</v>
       </c>
       <c r="I7" t="n">
-        <v>-14.6</v>
+        <v>-35.3</v>
       </c>
       <c r="J7" t="n">
-        <v>-66.59999999999999</v>
+        <v>-71.7</v>
       </c>
       <c r="K7" t="n">
-        <v>11815</v>
+        <v>9835</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -4216,16 +4216,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>32780</v>
+        <v>38223</v>
       </c>
       <c r="I8" t="n">
-        <v>-7.8</v>
+        <v>1.5</v>
       </c>
       <c r="J8" t="n">
-        <v>-73.40000000000001</v>
+        <v>-80.40000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>19136</v>
+        <v>20612</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -4275,16 +4275,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1585467</v>
+        <v>1892744</v>
       </c>
       <c r="I9" t="n">
-        <v>10</v>
+        <v>13.6</v>
       </c>
       <c r="J9" t="n">
-        <v>-17.5</v>
+        <v>-4.3</v>
       </c>
       <c r="K9" t="n">
-        <v>163420</v>
+        <v>181225</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -4334,16 +4334,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>45291</v>
+        <v>37050</v>
       </c>
       <c r="I10" t="n">
-        <v>-2.1</v>
+        <v>-20.4</v>
       </c>
       <c r="J10" t="n">
-        <v>3.5</v>
+        <v>-13.6</v>
       </c>
       <c r="K10" t="n">
-        <v>19124</v>
+        <v>16828</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -4393,16 +4393,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>185440</v>
+        <v>184336</v>
       </c>
       <c r="I11" t="n">
-        <v>2</v>
+        <v>4.3</v>
       </c>
       <c r="J11" t="n">
-        <v>-40.2</v>
+        <v>-39.9</v>
       </c>
       <c r="K11" t="n">
-        <v>59419</v>
+        <v>59052</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -4452,16 +4452,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3426203</v>
+        <v>3475593</v>
       </c>
       <c r="I12" t="n">
-        <v>0.5</v>
+        <v>2.8</v>
       </c>
       <c r="J12" t="n">
-        <v>21.9</v>
+        <v>24.3</v>
       </c>
       <c r="K12" t="n">
-        <v>161821</v>
+        <v>161911</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -4511,16 +4511,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>60642</v>
+        <v>57429</v>
       </c>
       <c r="I13" t="n">
-        <v>-24.7</v>
+        <v>-8.6</v>
       </c>
       <c r="J13" t="n">
-        <v>988.3</v>
+        <v>930.7</v>
       </c>
       <c r="K13" t="n">
-        <v>27142</v>
+        <v>26279</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -4570,16 +4570,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>126847295</v>
+        <v>123732828</v>
       </c>
       <c r="I14" t="n">
-        <v>0.3</v>
+        <v>-2</v>
       </c>
       <c r="J14" t="n">
-        <v>17.7</v>
+        <v>15.4</v>
       </c>
       <c r="K14" t="n">
-        <v>255338</v>
+        <v>248351</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -4629,16 +4629,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>336644870</v>
+        <v>322800630</v>
       </c>
       <c r="I15" t="n">
-        <v>-2.8</v>
+        <v>-5</v>
       </c>
       <c r="J15" t="n">
-        <v>-6.3</v>
+        <v>-9.300000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>2650192</v>
+        <v>2538881</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -4688,13 +4688,13 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>6693874</v>
+        <v>6716739</v>
       </c>
       <c r="I16" t="n">
-        <v>-1.5</v>
+        <v>-0.7</v>
       </c>
       <c r="J16" t="n">
-        <v>-6.2</v>
+        <v>-5.7</v>
       </c>
       <c r="K16" t="n">
         <v>329346</v>
@@ -4747,16 +4747,16 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>1213360</v>
+        <v>1216574</v>
       </c>
       <c r="I17" t="n">
-        <v>-3</v>
+        <v>-2.8</v>
       </c>
       <c r="J17" t="n">
-        <v>-1.5</v>
+        <v>-1.1</v>
       </c>
       <c r="K17" t="n">
-        <v>265502</v>
+        <v>265982</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -4806,16 +4806,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>1010207</v>
+        <v>1016661</v>
       </c>
       <c r="I18" t="n">
-        <v>3.7</v>
+        <v>4.9</v>
       </c>
       <c r="J18" t="n">
-        <v>71.90000000000001</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="K18" t="n">
-        <v>119770</v>
+        <v>119634</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -4865,16 +4865,16 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>311035</v>
+        <v>309329</v>
       </c>
       <c r="I19" t="n">
-        <v>-1.4</v>
+        <v>-2</v>
       </c>
       <c r="J19" t="n">
-        <v>3.2</v>
+        <v>2.6</v>
       </c>
       <c r="K19" t="n">
-        <v>61422</v>
+        <v>61321</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -4924,16 +4924,16 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>51261746</v>
+        <v>53002500</v>
       </c>
       <c r="I20" t="n">
-        <v>-1.1</v>
+        <v>2.4</v>
       </c>
       <c r="J20" t="n">
-        <v>27.2</v>
+        <v>31.6</v>
       </c>
       <c r="K20" t="n">
-        <v>1215148</v>
+        <v>1231358</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -4983,16 +4983,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>16650067</v>
+        <v>16768437</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.9</v>
+        <v>-0.3</v>
       </c>
       <c r="J21" t="n">
-        <v>19</v>
+        <v>19.9</v>
       </c>
       <c r="K21" t="n">
-        <v>862616</v>
+        <v>861555</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -5042,16 +5042,16 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>133835</v>
+        <v>135731</v>
       </c>
       <c r="I22" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J22" t="n">
-        <v>-7</v>
+        <v>-5.6</v>
       </c>
       <c r="K22" t="n">
-        <v>33154</v>
+        <v>33241</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -5101,16 +5101,16 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>49660</v>
+        <v>55121</v>
       </c>
       <c r="I23" t="n">
-        <v>-14.8</v>
+        <v>-5.3</v>
       </c>
       <c r="J23" t="n">
-        <v>-8.1</v>
+        <v>-7.1</v>
       </c>
       <c r="K23" t="n">
-        <v>18569</v>
+        <v>19725</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -5160,16 +5160,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>508629</v>
+        <v>459833</v>
       </c>
       <c r="I24" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="J24" t="n">
-        <v>16326</v>
+        <v>14750.1</v>
       </c>
       <c r="K24" t="n">
-        <v>103833</v>
+        <v>96668</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -5219,16 +5219,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>139859458</v>
+        <v>140137802</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.4</v>
+        <v>0.1</v>
       </c>
       <c r="J25" t="n">
-        <v>5.4</v>
+        <v>7.4</v>
       </c>
       <c r="K25" t="n">
-        <v>2367718</v>
+        <v>2364624</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -5278,16 +5278,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>379158990</v>
+        <v>378169750</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J26" t="n">
-        <v>2.5</v>
+        <v>1.7</v>
       </c>
       <c r="K26" t="n">
-        <v>11411977</v>
+        <v>11387385</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -5337,16 +5337,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>590050840</v>
+        <v>589220950</v>
       </c>
       <c r="I27" t="n">
-        <v>0.3</v>
+        <v>-0.9</v>
       </c>
       <c r="J27" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="K27" t="n">
-        <v>8766937</v>
+        <v>8759185</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -5396,16 +5396,16 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>41704208</v>
+        <v>41645293</v>
       </c>
       <c r="I28" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="J28" t="n">
-        <v>-5</v>
+        <v>-5.5</v>
       </c>
       <c r="K28" t="n">
-        <v>2024909</v>
+        <v>2022568</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -5455,7 +5455,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>249426</v>
+        <v>249440</v>
       </c>
       <c r="I29" t="n">
         <v>-1.3</v>
@@ -5464,7 +5464,7 @@
         <v>-22.2</v>
       </c>
       <c r="K29" t="n">
-        <v>49419</v>
+        <v>49334</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -5514,16 +5514,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>141196</v>
+        <v>142529</v>
       </c>
       <c r="I30" t="n">
-        <v>-1.8</v>
+        <v>0.4</v>
       </c>
       <c r="J30" t="n">
-        <v>-26.4</v>
+        <v>-26.3</v>
       </c>
       <c r="K30" t="n">
-        <v>37343</v>
+        <v>37224</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -5573,16 +5573,16 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>62518</v>
+        <v>77391</v>
       </c>
       <c r="I31" t="n">
-        <v>-31.1</v>
+        <v>-0.8</v>
       </c>
       <c r="J31" t="n">
-        <v>1168.1</v>
+        <v>1469.7</v>
       </c>
       <c r="K31" t="n">
-        <v>23956</v>
+        <v>26647</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -5632,16 +5632,16 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>75391596</v>
+        <v>75687509</v>
       </c>
       <c r="I32" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="J32" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="K32" t="n">
-        <v>248234</v>
+        <v>250622</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -5691,16 +5691,16 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>519967</v>
+        <v>511864</v>
       </c>
       <c r="I33" t="n">
-        <v>54.4</v>
+        <v>-4.5</v>
       </c>
       <c r="J33" t="n">
-        <v>17.1</v>
+        <v>2</v>
       </c>
       <c r="K33" t="n">
-        <v>88129</v>
+        <v>87098</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -5750,16 +5750,16 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>195226</v>
+        <v>197258</v>
       </c>
       <c r="I34" t="n">
-        <v>10.2</v>
+        <v>-5.1</v>
       </c>
       <c r="J34" t="n">
-        <v>179</v>
+        <v>131.8</v>
       </c>
       <c r="K34" t="n">
-        <v>38428</v>
+        <v>38878</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -5809,16 +5809,16 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>227832</v>
+        <v>248483</v>
       </c>
       <c r="I35" t="n">
-        <v>-41.7</v>
+        <v>-35.5</v>
       </c>
       <c r="J35" t="n">
-        <v>6587.4</v>
+        <v>7193.5</v>
       </c>
       <c r="K35" t="n">
-        <v>45593</v>
+        <v>47310</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -5868,16 +5868,16 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>47486</v>
+        <v>38678</v>
       </c>
       <c r="I36" t="n">
-        <v>-21.7</v>
+        <v>-14.9</v>
       </c>
       <c r="J36" t="n">
-        <v>1152.4</v>
+        <v>920.1</v>
       </c>
       <c r="K36" t="n">
-        <v>17174</v>
+        <v>15165</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -5927,16 +5927,16 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>2684835</v>
+        <v>2446990</v>
       </c>
       <c r="I37" t="n">
-        <v>-13.1</v>
+        <v>-18.6</v>
       </c>
       <c r="J37" t="n">
-        <v>-65.90000000000001</v>
+        <v>-62.3</v>
       </c>
       <c r="K37" t="n">
-        <v>784085</v>
+        <v>741699</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -5986,16 +5986,16 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>141979</v>
+        <v>129593</v>
       </c>
       <c r="I38" t="n">
-        <v>13.9</v>
+        <v>5.8</v>
       </c>
       <c r="J38" t="n">
-        <v>4063.6</v>
+        <v>3700.4</v>
       </c>
       <c r="K38" t="n">
-        <v>35093</v>
+        <v>33367</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
radar silent 10/12 22:19
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1604,12 +1604,12 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>马斯克：No more AI, SI</t>
+          <t>Robinhood CEO Vlad Tenev 10/12 14:12 悉尼：AI 研究员开始抽烟，superintelligence is near（约 30 万浏览，已核实原帖；讨论量低，每小时不到 10 帖）</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/elonmusk/status/2106665679361618173</t>
+          <t>https://x.com/vladtenev/status/2109482209858167175</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1625,12 +1625,12 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>马斯克：It always was（猫头鹰封面）</t>
+          <t>马斯克：No more AI, SI</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/elonmusk/status/2106672522771272121</t>
+          <t>https://x.com/elonmusk/status/2106665679361618173</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1646,12 +1646,12 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>blockchainbob：OWL 是 10M+ runner</t>
+          <t>马斯克：It always was（猫头鹰封面）</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/blockchainbob/status/2108158782010540282</t>
+          <t>https://x.com/elonmusk/status/2106672522771272121</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1667,12 +1667,12 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Super Inu 回撤 &gt;70%</t>
+          <t>blockchainbob：OWL 是 10M+ runner</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/LEEJETJET/status/2107363707663851645</t>
+          <t>https://x.com/blockchainbob/status/2108158782010540282</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1688,12 +1688,12 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>OWL 聪明钱买入 · $1.3M</t>
+          <t>Super Inu 回撤 &gt;70%</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/PeepRadars/status/2108201749873869220</t>
+          <t>https://x.com/LEEJETJET/status/2107363707663851645</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1709,12 +1709,12 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>复制盘墓地：Owl -74.6%</t>
+          <t>OWL 聪明钱买入 · $1.3M</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Ldger_Logic/status/2107864245903688129</t>
+          <t>https://x.com/PeepRadars/status/2108201749873869220</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1730,12 +1730,12 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Benioff 原帖：AIForce 改名 SIForce</t>
+          <t>复制盘墓地：Owl -74.6%</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Benioff/status/2108658674118111442</t>
+          <t>https://x.com/Ldger_Logic/status/2107864245903688129</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1751,12 +1751,12 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Polymarket 转报</t>
+          <t>Benioff 原帖：AIForce 改名 SIForce</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Polymarket/status/2108684882561937750</t>
+          <t>https://x.com/Benioff/status/2108658674118111442</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1772,17 +1772,17 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>pqc.market：回购销毁上线（60% 收入回购 PQC）</t>
+          <t>Polymarket 转报</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/pqcmarket/status/2108496833928421857</t>
+          <t>https://x.com/Polymarket/status/2108684882561937750</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>量子 / AI 破解私钥</t>
+          <t>超级智能 SI · 🦉猫头鹰</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -1793,12 +1793,12 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>新闻：MemeBitcoin 量子破解游戏</t>
+          <t>pqc.market：回购销毁上线（60% 收入回购 PQC）</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2107444605931122925</t>
+          <t>https://x.com/pqcmarket/status/2108496833928421857</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1814,17 +1814,17 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>新闻：Pollak 在 Token2049 讲 memestocks</t>
+          <t>新闻：MemeBitcoin 量子破解游戏</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2107892114243670355</t>
+          <t>https://x.com/i/trending/2107444605931122925</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>股票 meme · 代币化美股</t>
+          <t>量子 / AI 破解私钥</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -1835,12 +1835,12 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>STONK 快照 $150M</t>
+          <t>新闻：Pollak 在 Token2049 讲 memestocks</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/LordWinty/status/2107833485301785000</t>
+          <t>https://x.com/i/trending/2107892114243670355</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1856,12 +1856,12 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>STONK vs PUMP 收入对比</t>
+          <t>STONK 快照 $150M</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/merccuu/status/2107708461966369176</t>
+          <t>https://x.com/LordWinty/status/2107833485301785000</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1877,12 +1877,12 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>新闻：Murad 预测 meme 超越比特币</t>
+          <t>STONK vs PUMP 收入对比</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2108211927600300533</t>
+          <t>https://x.com/merccuu/status/2107708461966369176</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -1898,17 +1898,17 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ZCAT 快照 $49.68M</t>
+          <t>新闻：Murad 预测 meme 超越比特币</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/LordWinty/status/2108331717727584352</t>
+          <t>https://x.com/i/trending/2108211927600300533</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>持币分红盘 · ZCAT/BATON</t>
+          <t>股票 meme · 代币化美股</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -1919,12 +1919,12 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>BATON 第二腿</t>
+          <t>ZCAT 快照 $49.68M</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/uncsnipes/status/2108289033051005224</t>
+          <t>https://x.com/LordWinty/status/2108331717727584352</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -1940,12 +1940,12 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>新闻：Cake Wallet 创始人买 MCAT</t>
+          <t>BATON 第二腿</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2107557735109713954</t>
+          <t>https://x.com/uncsnipes/status/2108289033051005224</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -1961,12 +1961,12 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>新闻：ZEC 回调与 ZCAT</t>
+          <t>新闻：Cake Wallet 创始人买 MCAT</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2107332169756712972</t>
+          <t>https://x.com/i/trending/2107557735109713954</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -1982,17 +1982,17 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ANSEM 第 90 天：$142.3M</t>
+          <t>新闻：ZEC 回调与 ZCAT</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/folashade_aduke/status/2108306839230357742</t>
+          <t>https://x.com/i/trending/2107332169756712972</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ANSEM · SOL 老龙头</t>
+          <t>持币分红盘 · ZCAT/BATON</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
@@ -2003,12 +2003,12 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>新闻：ANSEM 社区分歧</t>
+          <t>ANSEM 第 90 天：$142.3M</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2107375013032792464</t>
+          <t>https://x.com/folashade_aduke/status/2108306839230357742</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2024,17 +2024,17 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>新闻：首笔原子 L1→L2</t>
+          <t>新闻：ANSEM 社区分歧</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2107378801793445978</t>
+          <t>https://x.com/i/trending/2107375013032792464</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>以太坊近况 · Glamsterdam</t>
+          <t>ANSEM · SOL 老龙头</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
@@ -2045,12 +2045,12 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>新闻：BEARISH 迁回以太坊</t>
+          <t>新闻：首笔原子 L1→L2</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2108295762803302646</t>
+          <t>https://x.com/i/trending/2107378801793445978</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2066,12 +2066,12 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>新闻：Tom Lee 预测</t>
+          <t>新闻：BEARISH 迁回以太坊</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2107515726969856078</t>
+          <t>https://x.com/i/trending/2108295762803302646</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2087,12 +2087,12 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>EtherWorld：Glamsterdam 上 Sepolia</t>
+          <t>新闻：Tom Lee 预测</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/ether_world/status/2107510399436538071</t>
+          <t>https://x.com/i/trending/2107515726969856078</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2108,17 +2108,17 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>币安人生：致 CZ</t>
+          <t>EtherWorld：Glamsterdam 上 Sepolia</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/digishahed/status/2108101740809904251</t>
+          <t>https://x.com/ether_world/status/2107510399436538071</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>BSC 中文盘 · 币安人生</t>
+          <t>以太坊近况 · Glamsterdam</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
@@ -2129,12 +2129,12 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>币安人生 ATH $900M / 龙虾 $310M</t>
+          <t>币安人生：致 CZ</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/0xkitty69/status/2107177206199865466</t>
+          <t>https://x.com/digishahed/status/2108101740809904251</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2150,17 +2150,17 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>新闻：LAPTOP 崩盘报告</t>
+          <t>币安人生 ATH $900M / 龙虾 $310M</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2107922838963335273</t>
+          <t>https://x.com/0xkitty69/status/2107177206199865466</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>LAPTOP · 亨特·拜登盘</t>
+          <t>BSC 中文盘 · 币安人生</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
@@ -2171,17 +2171,17 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>pqc.market：$BNKR 首个后量子证明 meme（1.1 万浏览）</t>
+          <t>新闻：LAPTOP 崩盘报告</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/pqcmarket/status/2108382929487552537</t>
+          <t>https://x.com/i/trending/2107922838963335273</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>后量子地堡 · BNKR/PQC</t>
+          <t>LAPTOP · 亨特·拜登盘</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
@@ -2192,12 +2192,12 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>pqc.market：哈希签名后量子证明解释</t>
+          <t>pqc.market：$BNKR 首个后量子证明 meme（1.1 万浏览）</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/pqcmarket/status/2108392049032450165</t>
+          <t>https://x.com/pqcmarket/status/2108382929487552537</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2213,12 +2213,12 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>pqc.market：The "bunker" effect</t>
+          <t>pqc.market：哈希签名后量子证明解释</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/pqcmarket/status/2108233460800503947</t>
+          <t>https://x.com/pqcmarket/status/2108392049032450165</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2234,12 +2234,12 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>toly 2024：If you are into mainstream adoption, pivot to bunkers（37.7 万浏览）</t>
+          <t>pqc.market：The "bunker" effect</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/toly/status/1774794089818689699</t>
+          <t>https://x.com/pqcmarket/status/2108233460800503947</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2255,12 +2255,12 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>BNKR 上线 1h41m 从 $18K 到 $278K（catchtherunners）</t>
+          <t>toly 2024：If you are into mainstream adoption, pivot to bunkers（37.7 万浏览）</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/catchtherunners/status/2108407383995056355</t>
+          <t>https://x.com/toly/status/1774794089818689699</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2276,17 +2276,17 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Solana 官网指南 Part 2（护照插画）</t>
+          <t>BNKR 上线 1h41m 从 $18K 到 $278K（catchtherunners）</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>https://solana.com/news/breakpoint-guide-part2</t>
+          <t>https://x.com/catchtherunners/status/2108407383995056355</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Solamians · Solana 官方插画里的“国籍”</t>
+          <t>后量子地堡 · BNKR/PQC</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
@@ -2297,12 +2297,12 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>@SolanaEvents 9/29 首发原帖</t>
+          <t>Solana 官网指南 Part 2（护照插画）</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/SolanaEvents/status/2104997362653638798</t>
+          <t>https://solana.com/news/breakpoint-guide-part2</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2318,12 +2318,12 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10/12 重新挖出的首帖</t>
+          <t>@SolanaEvents 9/29 首发原帖</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/TakakoBeilo4ky/status/2109465807960871067</t>
+          <t>https://x.com/SolanaEvents/status/2104997362653638798</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2339,12 +2339,12 @@
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
-          <t>@river100x 喊出 CA</t>
+          <t>10/12 重新挖出的首帖</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/river100x/status/2109469298070892878</t>
+          <t>https://x.com/TakakoBeilo4ky/status/2109465807960871067</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2360,12 +2360,12 @@
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
-          <t>X 趋势新闻卡</t>
+          <t>@river100x 喊出 CA</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2109535488168071330</t>
+          <t>https://x.com/river100x/status/2109469298070892878</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2381,17 +2381,17 @@
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
-          <t>@Devon8zzh 原视频帖</t>
+          <t>X 趋势新闻卡</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Devon8zzh/status/2109507158790545903</t>
+          <t>https://x.com/i/trending/2109535488168071330</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+          <t>Solamians · Solana 官方插画里的“国籍”</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -2402,12 +2402,12 @@
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
-          <t>@pmarca 转发记录</t>
+          <t>@Devon8zzh 原视频帖</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/pmarca/status/2109527802194342355</t>
+          <t>https://x.com/Devon8zzh/status/2109507158790545903</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -2423,12 +2423,12 @@
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
-          <t>@pmarca 10/11 转发 Devon 前作</t>
+          <t>@pmarca 转发记录</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/pmarca/status/2109398097285861513</t>
+          <t>https://x.com/pmarca/status/2109527802194342355</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -2444,12 +2444,12 @@
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
-          <t>社区告知 Devon 手续费已划给他</t>
+          <t>@pmarca 10/11 转发 Devon 前作</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/solanashaka/status/2109532284848373933</t>
+          <t>https://x.com/pmarca/status/2109398097285861513</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -2465,12 +2465,12 @@
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Devon：还在研究怎么领</t>
+          <t>社区告知 Devon 手续费已划给他</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Devon8zzh/status/2109548421078233180</t>
+          <t>https://x.com/solanashaka/status/2109532284848373933</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -2486,12 +2486,12 @@
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Devon：比我一年存的还多（引用 1.2 万手续费帖）</t>
+          <t>Devon：还在研究怎么领</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Devon8zzh/status/2109555248457228716</t>
+          <t>https://x.com/Devon8zzh/status/2109548421078233180</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -2507,12 +2507,12 @@
       <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
-          <t>社区帖：CAESAR 手续费约 1.2 万美元待领（未核实）</t>
+          <t>Devon：比我一年存的还多（引用 1.2 万手续费帖）</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/TheRealM0nkii/status/2109555562946150806</t>
+          <t>https://x.com/Devon8zzh/status/2109555248457228716</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -2528,12 +2528,12 @@
       <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Devon 贴出 CA（19:24）</t>
+          <t>社区帖：CAESAR 手续费约 1.2 万美元待领（未核实）</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Devon8zzh/status/2109560849610522736</t>
+          <t>https://x.com/TheRealM0nkii/status/2109555562946150806</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -2549,12 +2549,12 @@
       <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Devon：108.07 SOL（19:26）</t>
+          <t>Devon 贴出 CA（19:24）</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Devon8zzh/status/2109561327723458614</t>
+          <t>https://x.com/Devon8zzh/status/2109560849610522736</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -2570,12 +2570,12 @@
       <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Devon 截图 I found the button</t>
+          <t>Devon：108.07 SOL（19:26）</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Devon8zzh/status/2109561610268553597</t>
+          <t>https://x.com/Devon8zzh/status/2109561327723458614</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -2591,12 +2591,12 @@
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Devon 确认领取手续费 19:59</t>
+          <t>Devon 截图 I found the button</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Devon8zzh/status/2109569560009679193</t>
+          <t>https://x.com/Devon8zzh/status/2109561610268553597</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -2612,17 +2612,17 @@
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Kotaku：泄露者 3000 万市值威胁（引用 10/10 原文）</t>
+          <t>Devon 确认领取手续费 19:59</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>https://kotaku.com/gta-6-leaker-threatens-rockstar-with-doomsday-scenario-if-meme-coin-hits-30-million-2000743779</t>
+          <t>https://x.com/Devon8zzh/status/2109569560009679193</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -2633,12 +2633,12 @@
       <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Yahoo Finance：CYBERLEEK 24h 涨 273%</t>
+          <t>Kotaku：泄露者 3000 万市值威胁（引用 10/10 原文）</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>https://finance.yahoo.com/markets/crypto/articles/solana-meme-coin-tied-gta-150454094.html</t>
+          <t>https://kotaku.com/gta-6-leaker-threatens-rockstar-with-doomsday-scenario-if-meme-coin-hits-30-million-2000743779</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -2654,12 +2654,12 @@
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Dotesports：8 月提走约 25 万美元手续费</t>
+          <t>Yahoo Finance：CYBERLEEK 24h 涨 273%</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>https://dotesports.com/gta/news/cyberleek-gta-6-full-build-ultimatum</t>
+          <t>https://finance.yahoo.com/markets/crypto/articles/solana-meme-coin-tied-gta-150454094.html</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -2675,12 +2675,12 @@
       <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Seeking Alpha 推文</t>
+          <t>Dotesports：8 月提走约 25 万美元手续费</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/SeekingAlpha/status/2109436393017807208</t>
+          <t>https://dotesports.com/gta/news/cyberleek-gta-6-full-build-ultimatum</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -2696,12 +2696,12 @@
       <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
-          <t>@robtmb1：泄露视频里的 Dacity Coin（未核实）</t>
+          <t>Seeking Alpha 推文</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/robtmb1/status/2109241600002118071</t>
+          <t>https://x.com/SeekingAlpha/status/2109436393017807208</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -2711,6 +2711,27 @@
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr"/>
+      <c r="B87" t="inlineStr"/>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>@robtmb1：泄露视频里的 Dacity Coin（未核实）</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/robtmb1/status/2109241600002118071</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2799,6 +2820,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
binancians: add Binance identity meme topic + heat render
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G87"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1604,17 +1604,17 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Robinhood CEO Vlad Tenev 10/12 14:12 悉尼：AI 研究员开始抽烟，superintelligence is near（约 30 万浏览，已核实原帖；讨论量低，每小时不到 10 帖）</t>
+          <t>Binance 官推原文</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/vladtenev/status/2109482209858167175</t>
+          <t>https://x.com/binance/status/2109947862998007825</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>超级智能 SI · 🦉猫头鹰</t>
+          <t>Binancians · 币安人身份梗</t>
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
@@ -1625,17 +1625,17 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>马斯克：No more AI, SI</t>
+          <t>DexScreener 主盘</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/elonmusk/status/2106665679361618173</t>
+          <t>https://dexscreener.com/bsc/0x29c3bee092954d1aa17729279a3f829f140e64d7</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>超级智能 SI · 🦉猫头鹰</t>
+          <t>Binancians · 币安人身份梗</t>
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
@@ -1646,12 +1646,12 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>马斯克：It always was（猫头鹰封面）</t>
+          <t>Robinhood CEO Vlad Tenev 10/12 14:12 悉尼：AI 研究员开始抽烟，superintelligence is near（约 30 万浏览，已核实原帖；讨论量低，每小时不到 10 帖）</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/elonmusk/status/2106672522771272121</t>
+          <t>https://x.com/vladtenev/status/2109482209858167175</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1667,12 +1667,12 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>blockchainbob：OWL 是 10M+ runner</t>
+          <t>马斯克：No more AI, SI</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/blockchainbob/status/2108158782010540282</t>
+          <t>https://x.com/elonmusk/status/2106665679361618173</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1688,12 +1688,12 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Super Inu 回撤 &gt;70%</t>
+          <t>马斯克：It always was（猫头鹰封面）</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/LEEJETJET/status/2107363707663851645</t>
+          <t>https://x.com/elonmusk/status/2106672522771272121</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1709,12 +1709,12 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>OWL 聪明钱买入 · $1.3M</t>
+          <t>blockchainbob：OWL 是 10M+ runner</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/PeepRadars/status/2108201749873869220</t>
+          <t>https://x.com/blockchainbob/status/2108158782010540282</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1730,12 +1730,12 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>复制盘墓地：Owl -74.6%</t>
+          <t>Super Inu 回撤 &gt;70%</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Ldger_Logic/status/2107864245903688129</t>
+          <t>https://x.com/LEEJETJET/status/2107363707663851645</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1751,12 +1751,12 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Benioff 原帖：AIForce 改名 SIForce</t>
+          <t>OWL 聪明钱买入 · $1.3M</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Benioff/status/2108658674118111442</t>
+          <t>https://x.com/PeepRadars/status/2108201749873869220</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1772,12 +1772,12 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Polymarket 转报</t>
+          <t>复制盘墓地：Owl -74.6%</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Polymarket/status/2108684882561937750</t>
+          <t>https://x.com/Ldger_Logic/status/2107864245903688129</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1793,17 +1793,17 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>pqc.market：回购销毁上线（60% 收入回购 PQC）</t>
+          <t>Benioff 原帖：AIForce 改名 SIForce</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/pqcmarket/status/2108496833928421857</t>
+          <t>https://x.com/Benioff/status/2108658674118111442</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>量子 / AI 破解私钥</t>
+          <t>超级智能 SI · 🦉猫头鹰</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -1814,17 +1814,17 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>新闻：MemeBitcoin 量子破解游戏</t>
+          <t>Polymarket 转报</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2107444605931122925</t>
+          <t>https://x.com/Polymarket/status/2108684882561937750</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>量子 / AI 破解私钥</t>
+          <t>超级智能 SI · 🦉猫头鹰</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -1835,17 +1835,17 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>新闻：Pollak 在 Token2049 讲 memestocks</t>
+          <t>pqc.market：回购销毁上线（60% 收入回购 PQC）</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2107892114243670355</t>
+          <t>https://x.com/pqcmarket/status/2108496833928421857</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>股票 meme · 代币化美股</t>
+          <t>量子 / AI 破解私钥</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -1856,17 +1856,17 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>STONK 快照 $150M</t>
+          <t>新闻：MemeBitcoin 量子破解游戏</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/LordWinty/status/2107833485301785000</t>
+          <t>https://x.com/i/trending/2107444605931122925</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>股票 meme · 代币化美股</t>
+          <t>量子 / AI 破解私钥</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -1877,12 +1877,12 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>STONK vs PUMP 收入对比</t>
+          <t>新闻：Pollak 在 Token2049 讲 memestocks</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/merccuu/status/2107708461966369176</t>
+          <t>https://x.com/i/trending/2107892114243670355</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -1898,12 +1898,12 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>新闻：Murad 预测 meme 超越比特币</t>
+          <t>STONK 快照 $150M</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2108211927600300533</t>
+          <t>https://x.com/LordWinty/status/2107833485301785000</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -1919,17 +1919,17 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ZCAT 快照 $49.68M</t>
+          <t>STONK vs PUMP 收入对比</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/LordWinty/status/2108331717727584352</t>
+          <t>https://x.com/merccuu/status/2107708461966369176</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>持币分红盘 · ZCAT/BATON</t>
+          <t>股票 meme · 代币化美股</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -1940,17 +1940,17 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>BATON 第二腿</t>
+          <t>新闻：Murad 预测 meme 超越比特币</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/uncsnipes/status/2108289033051005224</t>
+          <t>https://x.com/i/trending/2108211927600300533</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>持币分红盘 · ZCAT/BATON</t>
+          <t>股票 meme · 代币化美股</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -1961,12 +1961,12 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>新闻：Cake Wallet 创始人买 MCAT</t>
+          <t>ZCAT 快照 $49.68M</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2107557735109713954</t>
+          <t>https://x.com/LordWinty/status/2108331717727584352</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -1982,12 +1982,12 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>新闻：ZEC 回调与 ZCAT</t>
+          <t>BATON 第二腿</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2107332169756712972</t>
+          <t>https://x.com/uncsnipes/status/2108289033051005224</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2003,17 +2003,17 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ANSEM 第 90 天：$142.3M</t>
+          <t>新闻：Cake Wallet 创始人买 MCAT</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/folashade_aduke/status/2108306839230357742</t>
+          <t>https://x.com/i/trending/2107557735109713954</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ANSEM · SOL 老龙头</t>
+          <t>持币分红盘 · ZCAT/BATON</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
@@ -2024,17 +2024,17 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>新闻：ANSEM 社区分歧</t>
+          <t>新闻：ZEC 回调与 ZCAT</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2107375013032792464</t>
+          <t>https://x.com/i/trending/2107332169756712972</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ANSEM · SOL 老龙头</t>
+          <t>持币分红盘 · ZCAT/BATON</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
@@ -2045,17 +2045,17 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>新闻：首笔原子 L1→L2</t>
+          <t>ANSEM 第 90 天：$142.3M</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2107378801793445978</t>
+          <t>https://x.com/folashade_aduke/status/2108306839230357742</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>以太坊近况 · Glamsterdam</t>
+          <t>ANSEM · SOL 老龙头</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -2066,17 +2066,17 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>新闻：BEARISH 迁回以太坊</t>
+          <t>新闻：ANSEM 社区分歧</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2108295762803302646</t>
+          <t>https://x.com/i/trending/2107375013032792464</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>以太坊近况 · Glamsterdam</t>
+          <t>ANSEM · SOL 老龙头</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -2087,12 +2087,12 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>新闻：Tom Lee 预测</t>
+          <t>新闻：首笔原子 L1→L2</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2107515726969856078</t>
+          <t>https://x.com/i/trending/2107378801793445978</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2108,12 +2108,12 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>EtherWorld：Glamsterdam 上 Sepolia</t>
+          <t>新闻：BEARISH 迁回以太坊</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/ether_world/status/2107510399436538071</t>
+          <t>https://x.com/i/trending/2108295762803302646</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2129,17 +2129,17 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>币安人生：致 CZ</t>
+          <t>新闻：Tom Lee 预测</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/digishahed/status/2108101740809904251</t>
+          <t>https://x.com/i/trending/2107515726969856078</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>BSC 中文盘 · 币安人生</t>
+          <t>以太坊近况 · Glamsterdam</t>
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
@@ -2150,17 +2150,17 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>币安人生 ATH $900M / 龙虾 $310M</t>
+          <t>EtherWorld：Glamsterdam 上 Sepolia</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/0xkitty69/status/2107177206199865466</t>
+          <t>https://x.com/ether_world/status/2107510399436538071</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>BSC 中文盘 · 币安人生</t>
+          <t>以太坊近况 · Glamsterdam</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
@@ -2171,17 +2171,17 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>新闻：LAPTOP 崩盘报告</t>
+          <t>币安人生：致 CZ</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2107922838963335273</t>
+          <t>https://x.com/digishahed/status/2108101740809904251</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>LAPTOP · 亨特·拜登盘</t>
+          <t>BSC 中文盘 · 币安人生</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
@@ -2192,17 +2192,17 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>pqc.market：$BNKR 首个后量子证明 meme（1.1 万浏览）</t>
+          <t>币安人生 ATH $900M / 龙虾 $310M</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/pqcmarket/status/2108382929487552537</t>
+          <t>https://x.com/0xkitty69/status/2107177206199865466</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>后量子地堡 · BNKR/PQC</t>
+          <t>BSC 中文盘 · 币安人生</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2213,17 +2213,17 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>pqc.market：哈希签名后量子证明解释</t>
+          <t>新闻：LAPTOP 崩盘报告</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/pqcmarket/status/2108392049032450165</t>
+          <t>https://x.com/i/trending/2107922838963335273</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>后量子地堡 · BNKR/PQC</t>
+          <t>LAPTOP · 亨特·拜登盘</t>
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
@@ -2234,12 +2234,12 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>pqc.market：The "bunker" effect</t>
+          <t>pqc.market：$BNKR 首个后量子证明 meme（1.1 万浏览）</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/pqcmarket/status/2108233460800503947</t>
+          <t>https://x.com/pqcmarket/status/2108382929487552537</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2255,12 +2255,12 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>toly 2024：If you are into mainstream adoption, pivot to bunkers（37.7 万浏览）</t>
+          <t>pqc.market：哈希签名后量子证明解释</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/toly/status/1774794089818689699</t>
+          <t>https://x.com/pqcmarket/status/2108392049032450165</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2276,12 +2276,12 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>BNKR 上线 1h41m 从 $18K 到 $278K（catchtherunners）</t>
+          <t>pqc.market：The "bunker" effect</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/catchtherunners/status/2108407383995056355</t>
+          <t>https://x.com/pqcmarket/status/2108233460800503947</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2297,17 +2297,17 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Solana 官网指南 Part 2（护照插画）</t>
+          <t>toly 2024：If you are into mainstream adoption, pivot to bunkers（37.7 万浏览）</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>https://solana.com/news/breakpoint-guide-part2</t>
+          <t>https://x.com/toly/status/1774794089818689699</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Solamians · Solana 官方插画里的“国籍”</t>
+          <t>后量子地堡 · BNKR/PQC</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -2318,17 +2318,17 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>@SolanaEvents 9/29 首发原帖</t>
+          <t>BNKR 上线 1h41m 从 $18K 到 $278K（catchtherunners）</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/SolanaEvents/status/2104997362653638798</t>
+          <t>https://x.com/catchtherunners/status/2108407383995056355</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Solamians · Solana 官方插画里的“国籍”</t>
+          <t>后量子地堡 · BNKR/PQC</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -2339,12 +2339,12 @@
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
-          <t>10/12 重新挖出的首帖</t>
+          <t>Solana 官网指南 Part 2（护照插画）</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/TakakoBeilo4ky/status/2109465807960871067</t>
+          <t>https://solana.com/news/breakpoint-guide-part2</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2360,12 +2360,12 @@
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
-          <t>@river100x 喊出 CA</t>
+          <t>@SolanaEvents 9/29 首发原帖</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/river100x/status/2109469298070892878</t>
+          <t>https://x.com/SolanaEvents/status/2104997362653638798</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2381,12 +2381,12 @@
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
-          <t>X 趋势新闻卡</t>
+          <t>10/12 重新挖出的首帖</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/i/trending/2109535488168071330</t>
+          <t>https://x.com/TakakoBeilo4ky/status/2109465807960871067</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2402,17 +2402,17 @@
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
-          <t>@Devon8zzh 原视频帖</t>
+          <t>@river100x 喊出 CA</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Devon8zzh/status/2109507158790545903</t>
+          <t>https://x.com/river100x/status/2109469298070892878</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+          <t>Solamians · Solana 官方插画里的“国籍”</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
@@ -2423,17 +2423,17 @@
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
-          <t>@pmarca 转发记录</t>
+          <t>X 趋势新闻卡</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/pmarca/status/2109527802194342355</t>
+          <t>https://x.com/i/trending/2109535488168071330</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+          <t>Solamians · Solana 官方插画里的“国籍”</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -2444,12 +2444,12 @@
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
-          <t>@pmarca 10/11 转发 Devon 前作</t>
+          <t>@Devon8zzh 原视频帖</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/pmarca/status/2109398097285861513</t>
+          <t>https://x.com/Devon8zzh/status/2109507158790545903</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -2465,12 +2465,12 @@
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
-          <t>社区告知 Devon 手续费已划给他</t>
+          <t>@pmarca 转发记录</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/solanashaka/status/2109532284848373933</t>
+          <t>https://x.com/pmarca/status/2109527802194342355</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -2486,12 +2486,12 @@
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Devon：还在研究怎么领</t>
+          <t>@pmarca 10/11 转发 Devon 前作</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Devon8zzh/status/2109548421078233180</t>
+          <t>https://x.com/pmarca/status/2109398097285861513</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -2507,12 +2507,12 @@
       <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Devon：比我一年存的还多（引用 1.2 万手续费帖）</t>
+          <t>社区告知 Devon 手续费已划给他</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Devon8zzh/status/2109555248457228716</t>
+          <t>https://x.com/solanashaka/status/2109532284848373933</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -2528,12 +2528,12 @@
       <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr">
         <is>
-          <t>社区帖：CAESAR 手续费约 1.2 万美元待领（未核实）</t>
+          <t>Devon：还在研究怎么领</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/TheRealM0nkii/status/2109555562946150806</t>
+          <t>https://x.com/Devon8zzh/status/2109548421078233180</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -2549,12 +2549,12 @@
       <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Devon 贴出 CA（19:24）</t>
+          <t>Devon：比我一年存的还多（引用 1.2 万手续费帖）</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Devon8zzh/status/2109560849610522736</t>
+          <t>https://x.com/Devon8zzh/status/2109555248457228716</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -2570,12 +2570,12 @@
       <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Devon：108.07 SOL（19:26）</t>
+          <t>社区帖：CAESAR 手续费约 1.2 万美元待领（未核实）</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Devon8zzh/status/2109561327723458614</t>
+          <t>https://x.com/TheRealM0nkii/status/2109555562946150806</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -2591,12 +2591,12 @@
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Devon 截图 I found the button</t>
+          <t>Devon 贴出 CA（19:24）</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Devon8zzh/status/2109561610268553597</t>
+          <t>https://x.com/Devon8zzh/status/2109560849610522736</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -2612,12 +2612,12 @@
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Devon 确认领取手续费 19:59</t>
+          <t>Devon：108.07 SOL（19:26）</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/Devon8zzh/status/2109569560009679193</t>
+          <t>https://x.com/Devon8zzh/status/2109561327723458614</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -2633,17 +2633,17 @@
       <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Kotaku：泄露者 3000 万市值威胁（引用 10/10 原文）</t>
+          <t>Devon 截图 I found the button</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>https://kotaku.com/gta-6-leaker-threatens-rockstar-with-doomsday-scenario-if-meme-coin-hits-30-million-2000743779</t>
+          <t>https://x.com/Devon8zzh/status/2109561610268553597</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -2654,17 +2654,17 @@
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Yahoo Finance：CYBERLEEK 24h 涨 273%</t>
+          <t>Devon 确认领取手续费 19:59</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>https://finance.yahoo.com/markets/crypto/articles/solana-meme-coin-tied-gta-150454094.html</t>
+          <t>https://x.com/Devon8zzh/status/2109569560009679193</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -2675,12 +2675,12 @@
       <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Dotesports：8 月提走约 25 万美元手续费</t>
+          <t>Kotaku：泄露者 3000 万市值威胁（引用 10/10 原文）</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>https://dotesports.com/gta/news/cyberleek-gta-6-full-build-ultimatum</t>
+          <t>https://kotaku.com/gta-6-leaker-threatens-rockstar-with-doomsday-scenario-if-meme-coin-hits-30-million-2000743779</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -2696,12 +2696,12 @@
       <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Seeking Alpha 推文</t>
+          <t>Yahoo Finance：CYBERLEEK 24h 涨 273%</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/SeekingAlpha/status/2109436393017807208</t>
+          <t>https://finance.yahoo.com/markets/crypto/articles/solana-meme-coin-tied-gta-150454094.html</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -2717,12 +2717,12 @@
       <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr">
         <is>
-          <t>@robtmb1：泄露视频里的 Dacity Coin（未核实）</t>
+          <t>Dotesports：8 月提走约 25 万美元手续费</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/robtmb1/status/2109241600002118071</t>
+          <t>https://dotesports.com/gta/news/cyberleek-gta-6-full-build-ultimatum</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -2732,6 +2732,48 @@
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr"/>
+      <c r="B88" t="inlineStr"/>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Seeking Alpha 推文</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/SeekingAlpha/status/2109436393017807208</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr"/>
+      <c r="B89" t="inlineStr"/>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>@robtmb1：泄露视频里的 Dacity Coin（未核实）</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/robtmb1/status/2109241600002118071</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2821,6 +2863,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId88"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2832,7 +2876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2852,6 +2896,7 @@
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2940,6 +2985,11 @@
           <t>10-12 帖数</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>10-13 帖数</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -2997,6 +3047,7 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -3054,6 +3105,7 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -3117,6 +3169,7 @@
       <c r="Q4" t="n">
         <v>18931</v>
       </c>
+      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -3174,6 +3227,7 @@
       <c r="Q5" t="n">
         <v>6205</v>
       </c>
+      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -3231,6 +3285,7 @@
       <c r="Q6" t="n">
         <v>854</v>
       </c>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -3288,6 +3343,7 @@
       <c r="Q7" t="n">
         <v>424</v>
       </c>
+      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -3345,6 +3401,7 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -3402,6 +3459,7 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -3459,6 +3517,7 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -3516,6 +3575,7 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -3573,6 +3633,7 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -3580,7 +3641,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>以太坊近况 · Glamsterdam</t>
+          <t>Binancians · 币安人身份梗</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3589,47 +3650,36 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>→</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>binancians</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>技术/宏观新闻多（Glamsterdam 测试网、首笔原子 L1→L2、Abstract 关停），ETH ~$2,700 横盘，meme 热度低 → 只看 BURR 迁移</t>
-        </is>
-      </c>
-      <c r="H13" t="n">
-        <v>462</v>
-      </c>
-      <c r="I13" t="n">
-        <v>623</v>
-      </c>
-      <c r="J13" t="n">
-        <v>944</v>
-      </c>
-      <c r="K13" t="n">
-        <v>1721</v>
-      </c>
-      <c r="L13" t="n">
-        <v>1734</v>
-      </c>
-      <c r="M13" t="n">
-        <v>1117</v>
-      </c>
-      <c r="N13" t="n">
-        <v>1123</v>
-      </c>
+          <t>10/13 21:02 悉尼 @binance 官推 “the best part of binance is the binancians”（~147k views，已核实原文）。社区立刻上同名盘；讨论量从近零飙到 ~159/hr。币安/CZ 均未点名任何 CA。龙头按成交与引用暂认 0x8Dce…7777（BNCB 对，~27万美元市值），同名盘极多。</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="n">
+        <v>510</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -3637,7 +3687,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>LAPTOP · 亨特·拜登盘</t>
+          <t>以太坊近况 · Glamsterdam</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -3646,47 +3696,48 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>↑</t>
+          <t>↓</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>LAPTOP</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>政治名人盘，曾 1 小时 -98%，10/7 报告后小反弹，但讨论多为刷票机器人 → 回避</t>
+          <t>技术/宏观新闻多（Glamsterdam 测试网、首笔原子 L1→L2、Abstract 关停），ETH ~$2,700 横盘，meme 热度低 → 只看 BURR 迁移</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>51</v>
+        <v>462</v>
       </c>
       <c r="I14" t="n">
-        <v>35</v>
+        <v>623</v>
       </c>
       <c r="J14" t="n">
-        <v>34</v>
+        <v>944</v>
       </c>
       <c r="K14" t="n">
-        <v>64</v>
+        <v>1721</v>
       </c>
       <c r="L14" t="n">
-        <v>595</v>
+        <v>1734</v>
       </c>
       <c r="M14" t="n">
-        <v>448</v>
+        <v>1117</v>
       </c>
       <c r="N14" t="n">
-        <v>384</v>
+        <v>1123</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -3694,7 +3745,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>后量子地堡 · BNKR/PQC</t>
+          <t>LAPTOP · 亨特·拜登盘</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3707,49 +3758,108 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t>↑</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>LAPTOP</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>政治名人盘，曾 1 小时 -98%，10/7 报告后小反弹，但讨论多为刷票机器人 → 回避</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>51</v>
+      </c>
+      <c r="I15" t="n">
+        <v>35</v>
+      </c>
+      <c r="J15" t="n">
+        <v>34</v>
+      </c>
+      <c r="K15" t="n">
+        <v>64</v>
+      </c>
+      <c r="L15" t="n">
+        <v>595</v>
+      </c>
+      <c r="M15" t="n">
+        <v>448</v>
+      </c>
+      <c r="N15" t="n">
+        <v>384</v>
+      </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>后量子地堡 · BNKR/PQC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>25</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
           <t>↓</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>PQC</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>量子恐慌的第一个“产品化”玩法：pqc.market 发射台 + 官方 BNKR。X 讨论 2 天翻 4 倍，但 BNKR 已从 $420K 回撤到 ~$180K，PQC 是母盘</t>
         </is>
       </c>
-      <c r="H15" t="n">
+      <c r="H16" t="n">
         <v>392</v>
       </c>
-      <c r="I15" t="n">
+      <c r="I16" t="n">
         <v>243</v>
       </c>
-      <c r="J15" t="n">
+      <c r="J16" t="n">
         <v>303</v>
       </c>
-      <c r="K15" t="n">
+      <c r="K16" t="n">
         <v>282</v>
       </c>
-      <c r="L15" t="n">
+      <c r="L16" t="n">
         <v>564</v>
       </c>
-      <c r="M15" t="n">
+      <c r="M16" t="n">
         <v>1588</v>
       </c>
-      <c r="N15" t="n">
+      <c r="N16" t="n">
         <v>1463</v>
       </c>
-      <c r="O15" t="n">
+      <c r="O16" t="n">
         <v>728</v>
       </c>
-      <c r="P15" t="n">
+      <c r="P16" t="n">
         <v>587</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="Q16" t="n">
         <v>590</v>
       </c>
+      <c r="R16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3762,7 +3872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3850,12 +3960,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>超级智能 SI · 🦉猫头鹰</t>
+          <t>Binancians · 币安人身份梗</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>大周期</t>
+          <t>24小时</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3865,17 +3975,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>binancians</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>DEW9dSN6QpWyNthphCpMmAbZP1Q4cEKR9xQXAri98WDP</t>
+          <t>0x8DcefF98285b93013Ab708D65E0206880C167777</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -3884,37 +3994,37 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>16291150</v>
+        <v>356075</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>59.4</v>
       </c>
       <c r="J2" t="n">
-        <v>-31.4</v>
+        <v>9087.1</v>
       </c>
       <c r="K2" t="n">
-        <v>718525</v>
+        <v>58303</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Super Inu：马斯克“SI 超级智能”梗龙头，ATH ~$69M，现在 ~$25M 横盘。</t>
+          <t>跟 @binance 官推同句热度最高的 BSC 盘（BNCB 对），非官方发行。</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/DEW9dSN6QpWyNthphCpMmAbZP1Q4cEKR9xQXAri98WDP</t>
+          <t>https://gmgn.ai/bsc/token/0x8DcefF98285b93013Ab708D65E0206880C167777</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>超级智能 SI · 🦉猫头鹰</t>
+          <t>Binancians · 币安人身份梗</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>大周期</t>
+          <t>24小时</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3924,17 +4034,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>Binancians</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>9aqmJjCnnMQv42TXLk921ceUkN35nea2QP969n1caqjj</t>
+          <t>0xf197e06dAb32B3C1Cd8c055598bea0AF11b44444</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -3943,37 +4053,37 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1317788</v>
+        <v>90035</v>
       </c>
       <c r="I3" t="n">
-        <v>6.3</v>
+        <v>23.7</v>
       </c>
       <c r="J3" t="n">
-        <v>-19.1</v>
+        <v>53.3</v>
       </c>
       <c r="K3" t="n">
-        <v>157848</v>
+        <v>55081</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Super Intelligence：同名二号 SI，9/30 上线，百万级市值。</t>
+          <t>更早的同名盘（binanciansbnb.com），有人自称 real one，成交弱于主盘。</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/9aqmJjCnnMQv42TXLk921ceUkN35nea2QP969n1caqjj</t>
+          <t>https://gmgn.ai/bsc/token/0xf197e06dAb32B3C1Cd8c055598bea0AF11b44444</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>超级智能 SI · 🦉猫头鹰</t>
+          <t>Binancians · 币安人身份梗</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>大周期</t>
+          <t>24小时</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3983,17 +4093,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>OWL</t>
+          <t>币安人</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>68AGsjomsgTtiTaDhF6XGCeVJDnFeh415ngYYgVxGzns</t>
+          <t>0xdea10d102fa1ce9f21194a01664848ac82ba7777</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -4002,37 +4112,37 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>554009</v>
+        <v>3380664</v>
       </c>
       <c r="I4" t="n">
-        <v>1.6</v>
+        <v>26952.1</v>
       </c>
       <c r="J4" t="n">
-        <v>-23.7</v>
+        <v>26952.1</v>
       </c>
       <c r="K4" t="n">
-        <v>87601</v>
+        <v>164778</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Superintelligence Owl：马斯克“It always was”猫头鹰封面吉祥物盘，24h 反弹 +170%。</t>
+          <t>🆕 GMGN 自动发现：币安人（10/13 22:33 悉尼上线），名字命中「Binancians」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/68AGsjomsgTtiTaDhF6XGCeVJDnFeh415ngYYgVxGzns</t>
+          <t>https://gmgn.ai/bsc/token/0xdea10d102fa1ce9f21194a01664848ac82ba7777</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>超级智能 SI · 🦉猫头鹰</t>
+          <t>Binancians · 币安人身份梗</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>大周期</t>
+          <t>24小时</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4042,17 +4152,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>binancians</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Ap7R5jTGxFCZEbkFc3WNMiN3ru6nkPkn3Co5p6tbpump</t>
+          <t>0x8dceff98285b93013ab708d65e0206880c167777</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -4061,25 +4171,25 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>13776</v>
+        <v>376989</v>
       </c>
       <c r="I5" t="n">
-        <v>-10.2</v>
+        <v>65.3</v>
       </c>
       <c r="J5" t="n">
-        <v>-30.8</v>
+        <v>9626.700000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>10803</v>
+        <v>60918</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Superintelligence（2024 老盘复活）：小市值同名盘，流动性薄。</t>
+          <t>🆕 GMGN 自动发现：binancians（10/13 21:03 悉尼上线），名字命中「Binancians」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/Ap7R5jTGxFCZEbkFc3WNMiN3ru6nkPkn3Co5p6tbpump</t>
+          <t>https://gmgn.ai/bsc/token/0x8dceff98285b93013ab708d65e0206880c167777</t>
         </is>
       </c>
     </row>
@@ -4096,12 +4206,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SI276</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -4111,7 +4221,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>HMYd9tosnUXuNHmq7pXmoePRVBLBBjA3JBfydq6upump</t>
+          <t>DEW9dSN6QpWyNthphCpMmAbZP1Q4cEKR9xQXAri98WDP</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -4120,25 +4230,25 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>985049</v>
+        <v>16107600</v>
       </c>
       <c r="I6" t="n">
-        <v>1.9</v>
+        <v>-1.9</v>
       </c>
       <c r="J6" t="n">
-        <v>-14.9</v>
+        <v>-32.2</v>
       </c>
       <c r="K6" t="n">
-        <v>96207</v>
+        <v>717488</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Super Intelligence SI276：GMGN 自动发现的新 SI 同名盘（&lt;72h），~$1.8M，叙事待人工核实。</t>
+          <t>Super Inu：马斯克“SI 超级智能”梗龙头，ATH ~$69M，现在 ~$25M 横盘。</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/HMYd9tosnUXuNHmq7pXmoePRVBLBBjA3JBfydq6upump</t>
+          <t>https://gmgn.ai/sol/token/DEW9dSN6QpWyNthphCpMmAbZP1Q4cEKR9xQXAri98WDP</t>
         </is>
       </c>
     </row>
@@ -4160,7 +4270,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>SPACEXSI</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -4170,7 +4280,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>87aemjYj3JPEu8YnmLXSK6D1v9SurhaXNmQ2Xtdzpump</t>
+          <t>9aqmJjCnnMQv42TXLk921ceUkN35nea2QP969n1caqjj</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4179,25 +4289,25 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>17191</v>
+        <v>1328596</v>
       </c>
       <c r="I7" t="n">
-        <v>-8.699999999999999</v>
+        <v>3.9</v>
       </c>
       <c r="J7" t="n">
-        <v>-16.6</v>
+        <v>-18.4</v>
       </c>
       <c r="K7" t="n">
-        <v>9136</v>
+        <v>158318</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：SpaceX Super Intelligence（10/11 06:17 悉尼上线），名字命中「超级智能」关键词；叙事待人工核实。</t>
+          <t>Super Intelligence：同名二号 SI，9/30 上线，百万级市值。</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/87aemjYj3JPEu8YnmLXSK6D1v9SurhaXNmQ2Xtdzpump</t>
+          <t>https://gmgn.ai/sol/token/9aqmJjCnnMQv42TXLk921ceUkN35nea2QP969n1caqjj</t>
         </is>
       </c>
     </row>
@@ -4219,17 +4329,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>TeslaSI</t>
+          <t>OWL</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>bsc</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0xaf3c2e121372eaf5458b827abe21393665d97777</t>
+          <t>68AGsjomsgTtiTaDhF6XGCeVJDnFeh415ngYYgVxGzns</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -4238,32 +4348,32 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>15721</v>
+        <v>532774</v>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>-1.6</v>
       </c>
       <c r="J8" t="n">
-        <v>-58.9</v>
+        <v>-26.7</v>
       </c>
       <c r="K8" t="n">
-        <v>13089</v>
+        <v>86053</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Tesla Super Intelligence（10/11 19:35 悉尼上线），名字命中「超级智能」关键词；叙事待人工核实。</t>
+          <t>Superintelligence Owl：马斯克“It always was”猫头鹰封面吉祥物盘，24h 反弹 +170%。</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0xaf3c2e121372eaf5458b827abe21393665d97777</t>
+          <t>https://gmgn.ai/sol/token/68AGsjomsgTtiTaDhF6XGCeVJDnFeh415ngYYgVxGzns</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>量子 / AI 破解私钥</t>
+          <t>超级智能 SI · 🦉猫头鹰</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4273,12 +4383,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>QI</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -4288,7 +4398,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>8TiMkgvsrat9tM2esko8zVTt99LZLpefUM4SnZaziXaQ</t>
+          <t>Ap7R5jTGxFCZEbkFc3WNMiN3ru6nkPkn3Co5p6tbpump</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -4297,32 +4407,32 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>986640</v>
+        <v>13776</v>
       </c>
       <c r="I9" t="n">
-        <v>-13.9</v>
+        <v>-10.2</v>
       </c>
       <c r="J9" t="n">
-        <v>-48.6</v>
+        <v>-30.8</v>
       </c>
       <c r="K9" t="n">
-        <v>139767</v>
+        <v>10803</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Quantum Inu：10/09 新盘，量子狗，量子赛道当前市值最大的纯 meme，24h 涨幅上万 %。</t>
+          <t>Superintelligence（2024 老盘复活）：小市值同名盘，流动性薄。</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/8TiMkgvsrat9tM2esko8zVTt99LZLpefUM4SnZaziXaQ</t>
+          <t>https://gmgn.ai/sol/token/Ap7R5jTGxFCZEbkFc3WNMiN3ru6nkPkn3Co5p6tbpump</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>量子 / AI 破解私钥</t>
+          <t>超级智能 SI · 🦉猫头鹰</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4337,7 +4447,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>QCAT</t>
+          <t>SI276</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -4347,7 +4457,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>7vMkPxLwaH26qSZ2CgHhzvrgz9wUWMvT256vbUWfarm</t>
+          <t>HMYd9tosnUXuNHmq7pXmoePRVBLBBjA3JBfydq6upump</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -4356,32 +4466,32 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>75205</v>
+        <v>975677</v>
       </c>
       <c r="I10" t="n">
-        <v>13.6</v>
+        <v>3.8</v>
       </c>
       <c r="J10" t="n">
-        <v>-57.5</v>
+        <v>-15.7</v>
       </c>
       <c r="K10" t="n">
-        <v>35873</v>
+        <v>96424</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Quantum Cat（10/10 02:08 悉尼上线），名字命中「量子」关键词；叙事待人工核实。</t>
+          <t>Super Intelligence SI276：GMGN 自动发现的新 SI 同名盘（&lt;72h），~$1.8M，叙事待人工核实。</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/7vMkPxLwaH26qSZ2CgHhzvrgz9wUWMvT256vbUWfarm</t>
+          <t>https://gmgn.ai/sol/token/HMYd9tosnUXuNHmq7pXmoePRVBLBBjA3JBfydq6upump</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>量子 / AI 破解私钥</t>
+          <t>超级智能 SI · 🦉猫头鹰</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4396,7 +4506,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>QI</t>
+          <t>SPACEXSI</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -4406,7 +4516,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>eFBwUbyopvmxYHEwXZRbsTkSJHsz7WqawqKMxbqpump</t>
+          <t>87aemjYj3JPEu8YnmLXSK6D1v9SurhaXNmQ2Xtdzpump</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4415,32 +4525,32 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>3833044</v>
+        <v>17191</v>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>-10.3</v>
       </c>
       <c r="J11" t="n">
-        <v>10</v>
+        <v>-16.6</v>
       </c>
       <c r="K11" t="n">
-        <v>168184</v>
+        <v>9136</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Quantum Inu（10/10 21:41 悉尼上线），名字命中「量子」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：SpaceX Super Intelligence（10/11 06:17 悉尼上线），名字命中「超级智能」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/eFBwUbyopvmxYHEwXZRbsTkSJHsz7WqawqKMxbqpump</t>
+          <t>https://gmgn.ai/sol/token/87aemjYj3JPEu8YnmLXSK6D1v9SurhaXNmQ2Xtdzpump</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Grok Bot · 整家公司由 AI 组成</t>
+          <t>超级智能 SI · 🦉猫头鹰</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4450,12 +4560,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Grok Bot</t>
+          <t>TeslaSI</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -4465,7 +4575,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0x7aede49f29bf7bc643853c1136854ea8e4da7777</t>
+          <t>0xaf3c2e121372eaf5458b827abe21393665d97777</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4474,32 +4584,32 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>45557</v>
+        <v>15374</v>
       </c>
       <c r="I12" t="n">
-        <v>-20.8</v>
+        <v>0.5</v>
       </c>
       <c r="J12" t="n">
-        <v>-15.1</v>
+        <v>-59.8</v>
       </c>
       <c r="K12" t="n">
-        <v>23522</v>
+        <v>12963</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：AI Agent（10/12 11:45 悉尼上线），名字命中「Grok」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：Tesla Super Intelligence（10/11 19:35 悉尼上线），名字命中「超级智能」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x7aede49f29bf7bc643853c1136854ea8e4da7777</t>
+          <t>https://gmgn.ai/bsc/token/0xaf3c2e121372eaf5458b827abe21393665d97777</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>股票 meme · 代币化美股</t>
+          <t>量子 / AI 破解私钥</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -4514,7 +4624,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>STONK</t>
+          <t>QI</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -4524,7 +4634,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>6GmAFSYs4gk3FDao5FzzySQpPZaWsa4rUJHacpMpUNgx</t>
+          <t>8TiMkgvsrat9tM2esko8zVTt99LZLpefUM4SnZaziXaQ</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4533,32 +4643,32 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>94084333</v>
+        <v>1015343</v>
       </c>
       <c r="I13" t="n">
-        <v>-3.5</v>
+        <v>-9.800000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>-23.5</v>
+        <v>-47.1</v>
       </c>
       <c r="K13" t="n">
-        <v>68699</v>
+        <v>137415</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>StonkFun 发射台币：股票 meme 龙头，30 天收入 ~$28–31M，市值 ~$1.2 亿。</t>
+          <t>Quantum Inu：10/09 新盘，量子狗，量子赛道当前市值最大的纯 meme，24h 涨幅上万 %。</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/6GmAFSYs4gk3FDao5FzzySQpPZaWsa4rUJHacpMpUNgx</t>
+          <t>https://gmgn.ai/sol/token/8TiMkgvsrat9tM2esko8zVTt99LZLpefUM4SnZaziXaQ</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>股票 meme · 代币化美股</t>
+          <t>量子 / AI 破解私钥</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -4573,17 +4683,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>PONS</t>
+          <t>QCAT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>robinhood</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0x39dbed3a2bd333467115de45665cc57f813c4571</t>
+          <t>7vMkPxLwaH26qSZ2CgHhzvrgz9wUWMvT256vbUWfarm</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -4592,32 +4702,32 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>281852550</v>
+        <v>77387</v>
       </c>
       <c r="I14" t="n">
-        <v>-1.1</v>
+        <v>18.1</v>
       </c>
       <c r="J14" t="n">
-        <v>-12.6</v>
+        <v>-56.2</v>
       </c>
       <c r="K14" t="n">
-        <v>2662427</v>
+        <v>36285</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Robinhood Chain 发射台币 Pons：10 万持有人，股票链 meme 的庄家盘。</t>
+          <t>🆕 GMGN 自动发现：Quantum Cat（10/10 02:08 悉尼上线），名字命中「量子」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/robinhood/token/0x39dbed3a2bd333467115de45665cc57f813c4571</t>
+          <t>https://gmgn.ai/sol/token/7vMkPxLwaH26qSZ2CgHhzvrgz9wUWMvT256vbUWfarm</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>股票 meme · 代币化美股</t>
+          <t>量子 / AI 破解私钥</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -4632,17 +4742,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>BLUECHIP</t>
+          <t>QI</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0xb200000000000000000000cfbdf64a8706a94a01</t>
+          <t>eFBwUbyopvmxYHEwXZRbsTkSJHsz7WqawqKMxbqpump</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -4651,32 +4761,32 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>5796707</v>
+        <v>3888854</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.7</v>
+        <v>2.6</v>
       </c>
       <c r="J15" t="n">
-        <v>-13.1</v>
+        <v>11.6</v>
       </c>
       <c r="K15" t="n">
-        <v>301914</v>
+        <v>168513</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Base 股票 meme：Jesse Pollak Token2049 幻灯片点名。</t>
+          <t>🆕 GMGN 自动发现：Quantum Inu（10/10 21:41 悉尼上线），名字命中「量子」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/base/token/0xb200000000000000000000cfbdf64a8706a94a01</t>
+          <t>https://gmgn.ai/sol/token/eFBwUbyopvmxYHEwXZRbsTkSJHsz7WqawqKMxbqpump</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>股票 meme · 代币化美股</t>
+          <t>Grok Bot · 整家公司由 AI 组成</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -4686,22 +4796,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>IPOD</t>
+          <t>Grok Bot</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0xa6af0cea8fbc93e1eccc00f1fdd9a0bba251fee1</t>
+          <t>0x7aede49f29bf7bc643853c1136854ea8e4da7777</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -4710,25 +4820,25 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>1066099</v>
+        <v>46241</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>-18.2</v>
       </c>
       <c r="J16" t="n">
-        <v>-12.4</v>
+        <v>-13.8</v>
       </c>
       <c r="K16" t="n">
-        <v>256409</v>
+        <v>23749</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Base 苹果股票梗 iPod，Jesse 幻灯片点名。</t>
+          <t>🆕 GMGN 自动发现：AI Agent（10/12 11:45 悉尼上线），名字命中「Grok」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/base/token/0xa6af0cea8fbc93e1eccc00f1fdd9a0bba251fee1</t>
+          <t>https://gmgn.ai/bsc/token/0x7aede49f29bf7bc643853c1136854ea8e4da7777</t>
         </is>
       </c>
     </row>
@@ -4745,22 +4855,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>DGUY</t>
+          <t>STONK</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0xe34356dcd3d7bb991248f322e4ec31b5d60bc54e</t>
+          <t>6GmAFSYs4gk3FDao5FzzySQpPZaWsa4rUJHacpMpUNgx</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -4769,25 +4879,25 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>915528</v>
+        <v>95126432</v>
       </c>
       <c r="I17" t="n">
-        <v>13.1</v>
+        <v>2.5</v>
       </c>
       <c r="J17" t="n">
-        <v>-3</v>
+        <v>-22.6</v>
       </c>
       <c r="K17" t="n">
-        <v>112915</v>
+        <v>69636</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Delivery Guy：Base 股票 meme，Jesse 幻灯片点名。</t>
+          <t>StonkFun 发射台币：股票 meme 龙头，30 天收入 ~$28–31M，市值 ~$1.2 亿。</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/base/token/0xe34356dcd3d7bb991248f322e4ec31b5d60bc54e</t>
+          <t>https://gmgn.ai/sol/token/6GmAFSYs4gk3FDao5FzzySQpPZaWsa4rUJHacpMpUNgx</t>
         </is>
       </c>
     </row>
@@ -4809,17 +4919,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>TEMU</t>
+          <t>PONS</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>robinhood</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0x3c573bdd88008c94f025e5023212f28e5f39744c</t>
+          <t>0x39dbed3a2bd333467115de45665cc57f813c4571</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -4828,32 +4938,32 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>261622</v>
+        <v>281409610</v>
       </c>
       <c r="I18" t="n">
-        <v>2</v>
+        <v>-1.1</v>
       </c>
       <c r="J18" t="n">
-        <v>-15.4</v>
+        <v>-12.8</v>
       </c>
       <c r="K18" t="n">
-        <v>54162</v>
+        <v>2648888</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>TEMU on Base：Jesse 幻灯片点名的拼多多梗。</t>
+          <t>Robinhood Chain 发射台币 Pons：10 万持有人，股票链 meme 的庄家盘。</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/base/token/0x3c573bdd88008c94f025e5023212f28e5f39744c</t>
+          <t>https://gmgn.ai/robinhood/token/0x39dbed3a2bd333467115de45665cc57f813c4571</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>持币分红盘 · ZCAT/BATON</t>
+          <t>股票 meme · 代币化美股</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -4863,22 +4973,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>ZCAT</t>
+          <t>BLUECHIP</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>base</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
+          <t>0xb200000000000000000000cfbdf64a8706a94a01</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -4887,32 +4997,32 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>42327381</v>
+        <v>5798743</v>
       </c>
       <c r="I19" t="n">
-        <v>3.1</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>-16.1</v>
+        <v>-13.1</v>
       </c>
       <c r="K19" t="n">
-        <v>1068688</v>
+        <v>302254</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Anonymous Cat：3% 交易税自动换 ZEC 分红给持有人，分红盘龙头。</t>
+          <t>Base 股票 meme：Jesse Pollak Token2049 幻灯片点名。</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
+          <t>https://gmgn.ai/base/token/0xb200000000000000000000cfbdf64a8706a94a01</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>持币分红盘 · ZCAT/BATON</t>
+          <t>股票 meme · 代币化美股</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -4927,17 +5037,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>BATON</t>
+          <t>IPOD</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>base</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
+          <t>0xa6af0cea8fbc93e1eccc00f1fdd9a0bba251fee1</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -4946,32 +5056,32 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>12904938</v>
+        <v>1066099</v>
       </c>
       <c r="I20" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J20" t="n">
-        <v>-23.4</v>
+        <v>-12.4</v>
       </c>
       <c r="K20" t="n">
-        <v>709111</v>
+        <v>256409</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>baton：分红 PUMP 的分红盘，ATH ~$19M，回调后第二腿。</t>
+          <t>Base 苹果股票梗 iPod，Jesse 幻灯片点名。</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
+          <t>https://gmgn.ai/base/token/0xa6af0cea8fbc93e1eccc00f1fdd9a0bba251fee1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>持币分红盘 · ZCAT/BATON</t>
+          <t>股票 meme · 代币化美股</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -4986,17 +5096,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>MCAT</t>
+          <t>DGUY</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>base</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
+          <t>0xe34356dcd3d7bb991248f322e4ec31b5d60bc54e</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -5005,32 +5115,32 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>155118</v>
+        <v>914129</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.9</v>
+        <v>12.2</v>
       </c>
       <c r="J21" t="n">
-        <v>21.4</v>
+        <v>-3.1</v>
       </c>
       <c r="K21" t="n">
-        <v>35883</v>
+        <v>112757</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Addicted Cat：分红门罗币 XMR，Cake Wallet 创始人买入。</t>
+          <t>Delivery Guy：Base 股票 meme，Jesse 幻灯片点名。</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
+          <t>https://gmgn.ai/base/token/0xe34356dcd3d7bb991248f322e4ec31b5d60bc54e</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>持币分红盘 · ZCAT/BATON</t>
+          <t>股票 meme · 代币化美股</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -5045,17 +5155,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>FACTORY</t>
+          <t>TEMU</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>base</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>7536qC4LEs3W2GtSKbhVGNJSiRfuXJhKVthxsgfkpump</t>
+          <t>0x3c573bdd88008c94f025e5023212f28e5f39744c</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -5064,25 +5174,25 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>39933</v>
+        <v>265334</v>
       </c>
       <c r="I22" t="n">
-        <v>9.1</v>
+        <v>4.5</v>
       </c>
       <c r="J22" t="n">
-        <v>-24.6</v>
+        <v>-10.2</v>
       </c>
       <c r="K22" t="n">
-        <v>16109</v>
+        <v>54852</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Baton Factory（10/10 22:26 悉尼上线），名字命中「持币分红盘」关键词；叙事待人工核实。</t>
+          <t>TEMU on Base：Jesse 幻灯片点名的拼多多梗。</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/7536qC4LEs3W2GtSKbhVGNJSiRfuXJhKVthxsgfkpump</t>
+          <t>https://gmgn.ai/base/token/0x3c573bdd88008c94f025e5023212f28e5f39744c</t>
         </is>
       </c>
     </row>
@@ -5099,22 +5209,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>上等羊</t>
+          <t>ZCAT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>bsc</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0x26c4829616644144b1dcec6c6c62828c9a717777</t>
+          <t>HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -5123,32 +5233,32 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>46565</v>
+        <v>42558923</v>
       </c>
       <c r="I23" t="n">
-        <v>-22.9</v>
+        <v>4.1</v>
       </c>
       <c r="J23" t="n">
-        <v>737.4</v>
+        <v>-18.1</v>
       </c>
       <c r="K23" t="n">
-        <v>21349</v>
+        <v>1085952</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：首创锁仓拖底回购分红协议（10/13 19:17 悉尼上线），名字命中「持币分红盘」关键词；叙事待人工核实。</t>
+          <t>Anonymous Cat：3% 交易税自动换 ZEC 分红给持有人，分红盘龙头。</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x26c4829616644144b1dcec6c6c62828c9a717777</t>
+          <t>https://gmgn.ai/sol/token/HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ANSEM · SOL 老龙头</t>
+          <t>持币分红盘 · ZCAT/BATON</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5158,12 +5268,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ANSEM</t>
+          <t>BATON</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -5173,7 +5283,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
+          <t>Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -5182,32 +5292,32 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>131430684</v>
+        <v>13019742</v>
       </c>
       <c r="I24" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="J24" t="n">
-        <v>-6.2</v>
+        <v>-24.9</v>
       </c>
       <c r="K24" t="n">
-        <v>2246319</v>
+        <v>712647</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>The Black Bull：Ansem 本人梗的 SOL 老龙头，15 万持有人，前十持仓 ~65% 偏集中。</t>
+          <t>baton：分红 PUMP 的分红盘，ATH ~$19M，回调后第二腿。</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
+          <t>https://gmgn.ai/sol/token/Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>以太坊近况 · Glamsterdam</t>
+          <t>持币分红盘 · ZCAT/BATON</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -5217,22 +5327,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>MCAT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>eth</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
+          <t>H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -5241,32 +5351,32 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>361880830</v>
+        <v>148137</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.1</v>
+        <v>-5.4</v>
       </c>
       <c r="J25" t="n">
-        <v>-4.3</v>
+        <v>15.9</v>
       </c>
       <c r="K25" t="n">
-        <v>11096311</v>
+        <v>34415</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>SPX6900：Murad 舞台喊“meme 将超越比特币”的 ETH 主网 meme 龙头。</t>
+          <t>Addicted Cat：分红门罗币 XMR，Cake Wallet 创始人买入。</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/eth/token/0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
+          <t>https://gmgn.ai/sol/token/H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BSC 中文盘 · 币安人生</t>
+          <t>持币分红盘 · ZCAT/BATON</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5276,22 +5386,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>币安人生</t>
+          <t>FACTORY</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>bsc</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
+          <t>7536qC4LEs3W2GtSKbhVGNJSiRfuXJhKVthxsgfkpump</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -5300,32 +5410,32 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>525477110</v>
+        <v>40003</v>
       </c>
       <c r="I26" t="n">
-        <v>0.7</v>
+        <v>12.1</v>
       </c>
       <c r="J26" t="n">
-        <v>-11.1</v>
+        <v>-23</v>
       </c>
       <c r="K26" t="n">
-        <v>8218276</v>
+        <v>16149</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>币安人生：何一推文带火的 BSC 中文 meme 龙头，ATH ~$9 亿，现 ~$5.5 亿。</t>
+          <t>🆕 GMGN 自动发现：Baton Factory（10/10 22:26 悉尼上线），名字命中「持币分红盘」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
+          <t>https://gmgn.ai/sol/token/7536qC4LEs3W2GtSKbhVGNJSiRfuXJhKVthxsgfkpump</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>BSC 中文盘 · 币安人生</t>
+          <t>持币分红盘 · ZCAT/BATON</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5340,7 +5450,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>龙虾</t>
+          <t>上等羊</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -5350,7 +5460,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0xeccbb861c0dda7efd964010085488b69317e4444</t>
+          <t>0x26c4829616644144b1dcec6c6c62828c9a717777</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -5359,32 +5469,32 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>44319292</v>
+        <v>47407</v>
       </c>
       <c r="I27" t="n">
-        <v>1.9</v>
+        <v>-5.7</v>
       </c>
       <c r="J27" t="n">
-        <v>6.5</v>
+        <v>752.5</v>
       </c>
       <c r="K27" t="n">
-        <v>2077050</v>
+        <v>21528</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>龙虾：币安中文号推文出圈的中文盘，ATH ~$3.1 亿，现 ~$4300 万。注意今天有同名高仿盘。</t>
+          <t>🆕 GMGN 自动发现：首创锁仓拖底回购分红协议（10/13 19:17 悉尼上线），名字命中「持币分红盘」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0xeccbb861c0dda7efd964010085488b69317e4444</t>
+          <t>https://gmgn.ai/bsc/token/0x26c4829616644144b1dcec6c6c62828c9a717777</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BSC 中文盘 · 币安人生</t>
+          <t>ANSEM · SOL 老龙头</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5394,22 +5504,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>币安圣羊</t>
+          <t>ANSEM</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>bsc</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0xcc4cc7ebaab40aa19317027b63e584333f697777</t>
+          <t>9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -5418,32 +5528,32 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>215841</v>
+        <v>131755155</v>
       </c>
       <c r="I28" t="n">
-        <v>2</v>
+        <v>0.8</v>
       </c>
       <c r="J28" t="n">
-        <v>-13.5</v>
+        <v>-5.6</v>
       </c>
       <c r="K28" t="n">
-        <v>45999</v>
+        <v>2244186</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：币安圣羊（10/10 04:20 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
+          <t>The Black Bull：Ansem 本人梗的 SOL 老龙头，15 万持有人，前十持仓 ~65% 偏集中。</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0xcc4cc7ebaab40aa19317027b63e584333f697777</t>
+          <t>https://gmgn.ai/sol/token/9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>BSC 中文盘 · 币安人生</t>
+          <t>以太坊近况 · Glamsterdam</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5453,22 +5563,22 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>币安人</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>bsc</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0x2c2d4298548ae585c224714555f18abde7367777</t>
+          <t>0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -5477,25 +5587,25 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>131482</v>
+        <v>361347680</v>
       </c>
       <c r="I29" t="n">
-        <v>557</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>-8.9</v>
+        <v>-3.9</v>
       </c>
       <c r="K29" t="n">
-        <v>36020</v>
+        <v>11056669</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Binance Man（10/10 22:33 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
+          <t>SPX6900：Murad 舞台喊“meme 将超越比特币”的 ETH 主网 meme 龙头。</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x2c2d4298548ae585c224714555f18abde7367777</t>
+          <t>https://gmgn.ai/eth/token/0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
         </is>
       </c>
     </row>
@@ -5512,12 +5622,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Binance Angels</t>
+          <t>币安人生</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -5527,7 +5637,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>0x62bb38c83afeb82e8f468d122b1b9051b6167777</t>
+          <t>0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -5536,32 +5646,32 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>80524</v>
+        <v>527720700</v>
       </c>
       <c r="I30" t="n">
-        <v>-7.1</v>
+        <v>0.5</v>
       </c>
       <c r="J30" t="n">
-        <v>3.1</v>
+        <v>-9.4</v>
       </c>
       <c r="K30" t="n">
-        <v>27302</v>
+        <v>8239275</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：QQ:945497833（10/12 19:12 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
+          <t>币安人生：何一推文带火的 BSC 中文 meme 龙头，ATH ~$9 亿，现 ~$5.5 亿。</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x62bb38c83afeb82e8f468d122b1b9051b6167777</t>
+          <t>https://gmgn.ai/bsc/token/0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>LAPTOP · 亨特·拜登盘</t>
+          <t>BSC 中文盘 · 币安人生</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5571,22 +5681,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>LAPTOP</t>
+          <t>龙虾</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0xb095274743941e953c746f9c228da9c18bb6ec29</t>
+          <t>0xeccbb861c0dda7efd964010085488b69317e4444</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -5595,32 +5705,32 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>76404992</v>
+        <v>44383942</v>
       </c>
       <c r="I31" t="n">
-        <v>-0.1</v>
+        <v>2.5</v>
       </c>
       <c r="J31" t="n">
-        <v>1</v>
+        <v>6.7</v>
       </c>
       <c r="K31" t="n">
-        <v>517701</v>
+        <v>2079497</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Hunter Biden 本人发的“笔记本电脑”梗币，前十持仓 ~91% 极度集中。</t>
+          <t>龙虾：币安中文号推文出圈的中文盘，ATH ~$3.1 亿，现 ~$4300 万。注意今天有同名高仿盘。</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/base/token/0xb095274743941e953c746f9c228da9c18bb6ec29</t>
+          <t>https://gmgn.ai/bsc/token/0xeccbb861c0dda7efd964010085488b69317e4444</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>后量子地堡 · BNKR/PQC</t>
+          <t>BSC 中文盘 · 币安人生</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5630,22 +5740,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>PQC</t>
+          <t>币安圣羊</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
+          <t>0xcc4cc7ebaab40aa19317027b63e584333f697777</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -5654,32 +5764,32 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>319865</v>
+        <v>215841</v>
       </c>
       <c r="I32" t="n">
-        <v>-8.300000000000001</v>
+        <v>-3.4</v>
       </c>
       <c r="J32" t="n">
-        <v>-38.2</v>
+        <v>-12.6</v>
       </c>
       <c r="K32" t="n">
-        <v>67675</v>
+        <v>45999</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>pqc.market 平台币：后量子发射台，10/08 上线，24h 成交 ~$7.7M，BNKR 的母盘。</t>
+          <t>🆕 GMGN 自动发现：币安圣羊（10/10 04:20 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
+          <t>https://gmgn.ai/bsc/token/0xcc4cc7ebaab40aa19317027b63e584333f697777</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>后量子地堡 · BNKR/PQC</t>
+          <t>BSC 中文盘 · 币安人生</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5694,17 +5804,17 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>BUNKER</t>
+          <t>币安人</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
+          <t>0x2c2d4298548ae585c224714555f18abde7367777</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -5713,57 +5823,57 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>122549</v>
+        <v>162558</v>
       </c>
       <c r="I33" t="n">
-        <v>1.6</v>
+        <v>153.4</v>
       </c>
       <c r="J33" t="n">
-        <v>-34</v>
+        <v>25.5</v>
       </c>
       <c r="K33" t="n">
-        <v>29246</v>
+        <v>39935</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Bunker Mode（10/10 10:14 悉尼上线），名字命中「后量子地堡」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：Binance Man（10/10 22:33 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
+          <t>https://gmgn.ai/bsc/token/0x2c2d4298548ae585c224714555f18abde7367777</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Solamians · Solana 官方插画里的“国籍”</t>
+          <t>BSC 中文盘 · 币安人生</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>24小时</t>
+          <t>大周期</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Solamians</t>
+          <t>Binance Angels</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>8ZP5CzbPL1fmP8dn1GEmLd8xw1JdudUF5Dk7EpLxpump</t>
+          <t>0x62bb38c83afeb82e8f468d122b1b9051b6167777</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -5772,37 +5882,37 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>137954</v>
+        <v>76860</v>
       </c>
       <c r="I34" t="n">
-        <v>24</v>
+        <v>-4.5</v>
       </c>
       <c r="J34" t="n">
-        <v>-44.9</v>
+        <v>-10.3</v>
       </c>
       <c r="K34" t="n">
-        <v>35458</v>
+        <v>26569</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Solana 官方 Breakpoint 指南护照插画写着 Nationality: Solamian（已核实原图）。10/12 13:09 创建，ATH ~$910K，机器人成交约 57%。</t>
+          <t>🆕 GMGN 自动发现：QQ:945497833（10/12 19:12 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/8ZP5CzbPL1fmP8dn1GEmLd8xw1JdudUF5Dk7EpLxpump</t>
+          <t>https://gmgn.ai/bsc/token/0x62bb38c83afeb82e8f468d122b1b9051b6167777</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+          <t>LAPTOP · 亨特·拜登盘</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>24小时</t>
+          <t>大周期</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -5812,17 +5922,17 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>CAESAR</t>
+          <t>LAPTOP</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>base</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
+          <t>0xb095274743941e953c746f9c228da9c18bb6ec29</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -5831,37 +5941,37 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>74511</v>
+        <v>76457778</v>
       </c>
       <c r="I35" t="n">
-        <v>-19.9</v>
+        <v>0.2</v>
       </c>
       <c r="J35" t="n">
-        <v>126.3</v>
+        <v>0.9</v>
       </c>
       <c r="K35" t="n">
-        <v>22432</v>
+        <v>517911</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>pmarca 转发的《Slop Caesar》社区盘。19:24 Devon 本人贴出此 CA，自称已领约 108 SOL 手续费（GMGN：分成 100% 给 devonmvfisher，已领取）。原开发者已清仓、批量发币地址；机器人约 62%。</t>
+          <t>Hunter Biden 本人发的“笔记本电脑”梗币，前十持仓 ~91% 极度集中。</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
+          <t>https://gmgn.ai/base/token/0xb095274743941e953c746f9c228da9c18bb6ec29</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+          <t>后量子地堡 · BNKR/PQC</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>24小时</t>
+          <t>大周期</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -5871,7 +5981,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>CYBERLEEK</t>
+          <t>PQC</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -5881,7 +5991,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>ApZuxdpzMrbEYTGEzeY9afh5pj9d6qPRJCTgQYiipbKg</t>
+          <t>7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -5890,37 +6000,37 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>1755072</v>
+        <v>303113</v>
       </c>
       <c r="I36" t="n">
-        <v>-2.5</v>
+        <v>-11.6</v>
       </c>
       <c r="J36" t="n">
-        <v>-24.6</v>
+        <v>-39.1</v>
       </c>
       <c r="K36" t="n">
-        <v>561164</v>
+        <v>65598</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>GTA 6 泄露者的币，10/10 喊出 3000 万市值放完整版。8 月曾提款后崩盘，24h -53%。</t>
+          <t>pqc.market 平台币：后量子发射台，10/08 上线，24h 成交 ~$7.7M，BNKR 的母盘。</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/ApZuxdpzMrbEYTGEzeY9afh5pj9d6qPRJCTgQYiipbKg</t>
+          <t>https://gmgn.ai/sol/token/7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+          <t>后量子地堡 · BNKR/PQC</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>24小时</t>
+          <t>大周期</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -5930,7 +6040,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Dacity</t>
+          <t>BUNKER</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -5940,7 +6050,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>nxPqZ4F7ux8Vph5NFu25rEP6Kx9Gr1U6Fmj36Rjpump</t>
+          <t>BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -5949,32 +6059,32 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>138196</v>
+        <v>120400</v>
       </c>
       <c r="I37" t="n">
-        <v>-3.6</v>
+        <v>-0.2</v>
       </c>
       <c r="J37" t="n">
-        <v>8.699999999999999</v>
+        <v>-33.2</v>
       </c>
       <c r="K37" t="n">
-        <v>34543</v>
+        <v>29256</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>据称出现在泄露视频里的游戏内币（未核实），ATH 回撤 88%，机器人多。</t>
+          <t>🆕 GMGN 自动发现：Bunker Mode（10/10 10:14 悉尼上线），名字命中「后量子地堡」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/nxPqZ4F7ux8Vph5NFu25rEP6Kx9Gr1U6Fmj36Rjpump</t>
+          <t>https://gmgn.ai/sol/token/BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+          <t>Solamians · Solana 官方插画里的“国籍”</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -5984,12 +6094,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>CYBERLEEK</t>
+          <t>Solamians</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -5999,7 +6109,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>J62sjKAAk16afQssxNJS8G2RU9azmCip6VPjMcNcpump</t>
+          <t>8ZP5CzbPL1fmP8dn1GEmLd8xw1JdudUF5Dk7EpLxpump</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -6008,82 +6118,318 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>311662031</v>
+        <v>157445</v>
       </c>
       <c r="I38" t="n">
-        <v>2.8</v>
+        <v>25.9</v>
       </c>
       <c r="J38" t="n">
-        <v>2654251.6</v>
+        <v>-49.5</v>
       </c>
       <c r="K38" t="n">
-        <v>1526781</v>
+        <v>37991</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：CYBERLEEK（10/13 01:26 悉尼上线），名字命中「GTA」关键词；叙事待人工核实。</t>
+          <t>Solana 官方 Breakpoint 指南护照插画写着 Nationality: Solamian（已核实原图）。10/12 13:09 创建，ATH ~$910K，机器人成交约 57%。</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/J62sjKAAk16afQssxNJS8G2RU9azmCip6VPjMcNcpump</t>
+          <t>https://gmgn.ai/sol/token/8ZP5CzbPL1fmP8dn1GEmLd8xw1JdudUF5Dk7EpLxpump</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>龙头</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>CAESAR</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>72528</v>
+      </c>
+      <c r="I39" t="n">
+        <v>-20.1</v>
+      </c>
+      <c r="J39" t="n">
+        <v>134.7</v>
+      </c>
+      <c r="K39" t="n">
+        <v>22199</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>pmarca 转发的《Slop Caesar》社区盘。19:24 Devon 本人贴出此 CA，自称已领约 108 SOL 手续费（GMGN：分成 100% 给 devonmvfisher，已领取）。原开发者已清仓、批量发币地址；机器人约 62%。</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>24小时</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>龙头</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>CYBERLEEK</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>ApZuxdpzMrbEYTGEzeY9afh5pj9d6qPRJCTgQYiipbKg</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>1758779</v>
+      </c>
+      <c r="I40" t="n">
+        <v>-2.1</v>
+      </c>
+      <c r="J40" t="n">
+        <v>-30.8</v>
+      </c>
+      <c r="K40" t="n">
+        <v>561997</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>GTA 6 泄露者的币，10/10 喊出 3000 万市值放完整版。8 月曾提款后崩盘，24h -53%。</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/ApZuxdpzMrbEYTGEzeY9afh5pj9d6qPRJCTgQYiipbKg</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
         <is>
           <t>beta</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Dacity</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>nxPqZ4F7ux8Vph5NFu25rEP6Kx9Gr1U6Fmj36Rjpump</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>138196</v>
+      </c>
+      <c r="I41" t="n">
+        <v>-7.8</v>
+      </c>
+      <c r="J41" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="K41" t="n">
+        <v>34543</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>据称出现在泄露视频里的游戏内币（未核实），ATH 回撤 88%，机器人多。</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/nxPqZ4F7ux8Vph5NFu25rEP6Kx9Gr1U6Fmj36Rjpump</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
         <is>
           <t>CYBERLEEK</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>sol</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>J62sjKAAk16afQssxNJS8G2RU9azmCip6VPjMcNcpump</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>313045194</v>
+      </c>
+      <c r="I42" t="n">
+        <v>3</v>
+      </c>
+      <c r="J42" t="n">
+        <v>2666031.7</v>
+      </c>
+      <c r="K42" t="n">
+        <v>1530575</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>🆕 GMGN 自动发现：CYBERLEEK（10/13 01:26 悉尼上线），名字命中「GTA」关键词；叙事待人工核实。</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/J62sjKAAk16afQssxNJS8G2RU9azmCip6VPjMcNcpump</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>CYBERLEEK</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
         <is>
           <t>GkgVK2duAV9Rjbt43prMiZscuMVQ9XR1RihSYsT6tjjE</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>alive</t>
         </is>
       </c>
-      <c r="H39" t="n">
-        <v>73663</v>
-      </c>
-      <c r="I39" t="n">
-        <v>-1.1</v>
-      </c>
-      <c r="J39" t="n">
-        <v>-80.59999999999999</v>
-      </c>
-      <c r="K39" t="n">
-        <v>23016</v>
-      </c>
-      <c r="L39" t="inlineStr">
+      <c r="H43" t="n">
+        <v>73736</v>
+      </c>
+      <c r="I43" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J43" t="n">
+        <v>-80.5</v>
+      </c>
+      <c r="K43" t="n">
+        <v>23053</v>
+      </c>
+      <c r="L43" t="inlineStr">
         <is>
           <t>🆕 GMGN 自动发现：CyberLeek（10/13 07:40 悉尼上线），名字命中「GTA」关键词；叙事待人工核实。</t>
         </is>
       </c>
-      <c r="M39" s="2" t="inlineStr">
+      <c r="M43" s="2" t="inlineStr">
         <is>
           <t>https://gmgn.ai/sol/token/GkgVK2duAV9Rjbt43prMiZscuMVQ9XR1RihSYsT6tjjE</t>
         </is>
@@ -6129,6 +6475,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
binancians leader flip 10/13 23:05
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -3659,12 +3659,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>binancians</t>
+          <t>币安人</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10/13 21:02 悉尼 @binance 官推 “the best part of binance is the binancians”（~147k views，已核实原文）。社区立刻上同名盘；讨论量从近零飙到 ~159/hr。币安/CZ 均未点名任何 CA。龙头按成交与引用暂认 0x8Dce…7777（BNCB 对，~27万美元市值），同名盘极多。</t>
+          <t>10/13 23:07 悉尼：同叙事第二腿——中文「币安人」0xDEA1…7777 约 22:33 上线后市值冲到约 $3M+，超过首轮英文 binancians（0x8Dce…7777 ~$0.45M）。@binance 官推原文已核实；币安/CZ 仍未点名任何 CA。同名盘极多、image_dup 高，注意分流与砸盘。</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -3975,7 +3975,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>binancians</t>
+          <t>币安人</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -3985,7 +3985,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0x8DcefF98285b93013Ab708D65E0206880C167777</t>
+          <t>0xdea10d102fa1ce9f21194a01664848ac82ba7777</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -3994,25 +3994,25 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>452013</v>
+        <v>2785612</v>
       </c>
       <c r="I2" t="n">
-        <v>25.8</v>
+        <v>22190.5</v>
       </c>
       <c r="J2" t="n">
-        <v>11562.4</v>
+        <v>22190.5</v>
       </c>
       <c r="K2" t="n">
-        <v>67202</v>
+        <v>149974</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>跟 @binance 官推同句热度最高的 BSC 盘（BNCB 对），非官方发行。</t>
+          <t>中文名「币安人」盘，约 22:33 悉尼上线，现市值明显高于英文 binancians；币安/CZ 未点名任何 CA。image_dup=15，同名 7777 尾地址很多。</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x8DcefF98285b93013Ab708D65E0206880C167777</t>
+          <t>https://gmgn.ai/bsc/token/0xdea10d102fa1ce9f21194a01664848ac82ba7777</t>
         </is>
       </c>
     </row>
@@ -4034,7 +4034,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Binancians</t>
+          <t>binancians</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0xf197e06dAb32B3C1Cd8c055598bea0AF11b44444</t>
+          <t>0x8DcefF98285b93013Ab708D65E0206880C167777</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -4053,25 +4053,25 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>80438</v>
+        <v>452013</v>
       </c>
       <c r="I3" t="n">
-        <v>0.3</v>
+        <v>25.8</v>
       </c>
       <c r="J3" t="n">
-        <v>36.9</v>
+        <v>11562.4</v>
       </c>
       <c r="K3" t="n">
-        <v>51918</v>
+        <v>67202</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>更早的同名盘（binanciansbnb.com），有人自称 real one，成交弱于主盘。</t>
+          <t>英文名 binancians（BNCB 对），首轮讨论龙头，现市值落后于中文「币安人」。非官方。</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0xf197e06dAb32B3C1Cd8c055598bea0AF11b44444</t>
+          <t>https://gmgn.ai/bsc/token/0x8DcefF98285b93013Ab708D65E0206880C167777</t>
         </is>
       </c>
     </row>
@@ -4093,7 +4093,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>币安人</t>
+          <t>Binancians</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0xdea10d102fa1ce9f21194a01664848ac82ba7777</t>
+          <t>0xf197e06dAb32B3C1Cd8c055598bea0AF11b44444</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -4112,25 +4112,25 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2785612</v>
+        <v>80438</v>
       </c>
       <c r="I4" t="n">
-        <v>22190.5</v>
+        <v>0.3</v>
       </c>
       <c r="J4" t="n">
-        <v>22190.5</v>
+        <v>36.9</v>
       </c>
       <c r="K4" t="n">
-        <v>149974</v>
+        <v>51918</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：币安人（10/13 22:33 悉尼上线），名字命中「Binancians」关键词；叙事待人工核实。</t>
+          <t>更早的同名盘（binanciansbnb.com），有人自称 real one，成交弱于主盘。</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0xdea10d102fa1ce9f21194a01664848ac82ba7777</t>
+          <t>https://gmgn.ai/bsc/token/0xf197e06dAb32B3C1Cd8c055598bea0AF11b44444</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tokens 10/13 23:20 radar-silent
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -3872,7 +3872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M44"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3994,16 +3994,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>2785612</v>
+        <v>3210588</v>
       </c>
       <c r="I2" t="n">
-        <v>22190.5</v>
+        <v>25591.1</v>
       </c>
       <c r="J2" t="n">
-        <v>22190.5</v>
+        <v>25591.1</v>
       </c>
       <c r="K2" t="n">
-        <v>149974</v>
+        <v>160937</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -4053,16 +4053,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>452013</v>
+        <v>411807</v>
       </c>
       <c r="I3" t="n">
-        <v>25.8</v>
+        <v>16.4</v>
       </c>
       <c r="J3" t="n">
-        <v>11562.4</v>
+        <v>10525.1</v>
       </c>
       <c r="K3" t="n">
-        <v>67202</v>
+        <v>64872</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -4112,16 +4112,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>80438</v>
+        <v>76280</v>
       </c>
       <c r="I4" t="n">
-        <v>0.3</v>
+        <v>-3.3</v>
       </c>
       <c r="J4" t="n">
-        <v>36.9</v>
+        <v>29.9</v>
       </c>
       <c r="K4" t="n">
-        <v>51918</v>
+        <v>50590</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -4171,16 +4171,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>466988</v>
+        <v>410611</v>
       </c>
       <c r="I5" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="J5" t="n">
-        <v>11948.8</v>
+        <v>10494.2</v>
       </c>
       <c r="K5" t="n">
-        <v>68946</v>
+        <v>64762</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -4196,32 +4196,32 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Binancians · 币安人身份梗</t>
+          <t>超级智能 SI · 🦉猫头鹰</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>24小时</t>
+          <t>大周期</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>binancians</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>bsc</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0x78dff969d2883488766e6d99f23eb8f72a467777</t>
+          <t>DEW9dSN6QpWyNthphCpMmAbZP1Q4cEKR9xQXAri98WDP</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -4230,25 +4230,25 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>126035</v>
+        <v>16166423</v>
       </c>
       <c r="I6" t="n">
-        <v>88.7</v>
+        <v>-1.2</v>
       </c>
       <c r="J6" t="n">
-        <v>88.7</v>
+        <v>-26.9</v>
       </c>
       <c r="K6" t="n">
-        <v>36617</v>
+        <v>710345</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：binancians（10/13 23:00 悉尼上线），名字命中「Binancians」关键词；叙事待人工核实。</t>
+          <t>Super Inu：马斯克“SI 超级智能”梗龙头，ATH ~$69M，现在 ~$25M 横盘。</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x78dff969d2883488766e6d99f23eb8f72a467777</t>
+          <t>https://gmgn.ai/sol/token/DEW9dSN6QpWyNthphCpMmAbZP1Q4cEKR9xQXAri98WDP</t>
         </is>
       </c>
     </row>
@@ -4265,7 +4265,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -4280,7 +4280,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>DEW9dSN6QpWyNthphCpMmAbZP1Q4cEKR9xQXAri98WDP</t>
+          <t>9aqmJjCnnMQv42TXLk921ceUkN35nea2QP969n1caqjj</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4289,25 +4289,25 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>16176899</v>
+        <v>1259698</v>
       </c>
       <c r="I7" t="n">
-        <v>-1.4</v>
+        <v>-6.7</v>
       </c>
       <c r="J7" t="n">
-        <v>-28.7</v>
+        <v>-28.9</v>
       </c>
       <c r="K7" t="n">
-        <v>713578</v>
+        <v>154967</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Super Inu：马斯克“SI 超级智能”梗龙头，ATH ~$69M，现在 ~$25M 横盘。</t>
+          <t>Super Intelligence：同名二号 SI，9/30 上线，百万级市值。</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/DEW9dSN6QpWyNthphCpMmAbZP1Q4cEKR9xQXAri98WDP</t>
+          <t>https://gmgn.ai/sol/token/9aqmJjCnnMQv42TXLk921ceUkN35nea2QP969n1caqjj</t>
         </is>
       </c>
     </row>
@@ -4329,7 +4329,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>OWL</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9aqmJjCnnMQv42TXLk921ceUkN35nea2QP969n1caqjj</t>
+          <t>68AGsjomsgTtiTaDhF6XGCeVJDnFeh415ngYYgVxGzns</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -4348,25 +4348,25 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>1296396</v>
+        <v>496821</v>
       </c>
       <c r="I8" t="n">
-        <v>-4.2</v>
+        <v>-6.9</v>
       </c>
       <c r="J8" t="n">
-        <v>-27.1</v>
+        <v>-37</v>
       </c>
       <c r="K8" t="n">
-        <v>157577</v>
+        <v>82866</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Super Intelligence：同名二号 SI，9/30 上线，百万级市值。</t>
+          <t>Superintelligence Owl：马斯克“It always was”猫头鹰封面吉祥物盘，24h 反弹 +170%。</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/9aqmJjCnnMQv42TXLk921ceUkN35nea2QP969n1caqjj</t>
+          <t>https://gmgn.ai/sol/token/68AGsjomsgTtiTaDhF6XGCeVJDnFeh415ngYYgVxGzns</t>
         </is>
       </c>
     </row>
@@ -4388,7 +4388,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>OWL</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -4398,7 +4398,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>68AGsjomsgTtiTaDhF6XGCeVJDnFeh415ngYYgVxGzns</t>
+          <t>Ap7R5jTGxFCZEbkFc3WNMiN3ru6nkPkn3Co5p6tbpump</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -4407,25 +4407,25 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>468020</v>
+        <v>13792</v>
       </c>
       <c r="I9" t="n">
-        <v>-20.1</v>
+        <v>-7.7</v>
       </c>
       <c r="J9" t="n">
-        <v>-39.5</v>
+        <v>-40.3</v>
       </c>
       <c r="K9" t="n">
-        <v>80628</v>
+        <v>10765</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Superintelligence Owl：马斯克“It always was”猫头鹰封面吉祥物盘，24h 反弹 +170%。</t>
+          <t>Superintelligence（2024 老盘复活）：小市值同名盘，流动性薄。</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/68AGsjomsgTtiTaDhF6XGCeVJDnFeh415ngYYgVxGzns</t>
+          <t>https://gmgn.ai/sol/token/Ap7R5jTGxFCZEbkFc3WNMiN3ru6nkPkn3Co5p6tbpump</t>
         </is>
       </c>
     </row>
@@ -4447,7 +4447,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SI276</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -4457,7 +4457,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Ap7R5jTGxFCZEbkFc3WNMiN3ru6nkPkn3Co5p6tbpump</t>
+          <t>HMYd9tosnUXuNHmq7pXmoePRVBLBBjA3JBfydq6upump</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -4466,25 +4466,25 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>13792</v>
+        <v>1151646</v>
       </c>
       <c r="I10" t="n">
-        <v>-7.7</v>
+        <v>21.9</v>
       </c>
       <c r="J10" t="n">
-        <v>-39.8</v>
+        <v>-2</v>
       </c>
       <c r="K10" t="n">
-        <v>10803</v>
+        <v>104688</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Superintelligence（2024 老盘复活）：小市值同名盘，流动性薄。</t>
+          <t>Super Intelligence SI276：GMGN 自动发现的新 SI 同名盘（&lt;72h），~$1.8M，叙事待人工核实。</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/Ap7R5jTGxFCZEbkFc3WNMiN3ru6nkPkn3Co5p6tbpump</t>
+          <t>https://gmgn.ai/sol/token/HMYd9tosnUXuNHmq7pXmoePRVBLBBjA3JBfydq6upump</t>
         </is>
       </c>
     </row>
@@ -4506,7 +4506,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SI276</t>
+          <t>SPACEXSI</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>HMYd9tosnUXuNHmq7pXmoePRVBLBBjA3JBfydq6upump</t>
+          <t>87aemjYj3JPEu8YnmLXSK6D1v9SurhaXNmQ2Xtdzpump</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4525,25 +4525,25 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>1202675</v>
+        <v>14083</v>
       </c>
       <c r="I11" t="n">
-        <v>28.9</v>
+        <v>-19.1</v>
       </c>
       <c r="J11" t="n">
-        <v>4.2</v>
+        <v>-45</v>
       </c>
       <c r="K11" t="n">
-        <v>106013</v>
+        <v>7923</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Super Intelligence SI276：GMGN 自动发现的新 SI 同名盘（&lt;72h），~$1.8M，叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：SpaceX Super Intelligence（10/11 06:17 悉尼上线），名字命中「超级智能」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/HMYd9tosnUXuNHmq7pXmoePRVBLBBjA3JBfydq6upump</t>
+          <t>https://gmgn.ai/sol/token/87aemjYj3JPEu8YnmLXSK6D1v9SurhaXNmQ2Xtdzpump</t>
         </is>
       </c>
     </row>
@@ -4565,17 +4565,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>SPACEXSI</t>
+          <t>TeslaSI</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>87aemjYj3JPEu8YnmLXSK6D1v9SurhaXNmQ2Xtdzpump</t>
+          <t>0xaf3c2e121372eaf5458b827abe21393665d97777</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4584,32 +4584,32 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>14774</v>
+        <v>15201</v>
       </c>
       <c r="I12" t="n">
-        <v>-20.1</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>-38.8</v>
+        <v>-55.7</v>
       </c>
       <c r="K12" t="n">
-        <v>8346</v>
+        <v>12899</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：SpaceX Super Intelligence（10/11 06:17 悉尼上线），名字命中「超级智能」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：Tesla Super Intelligence（10/11 19:35 悉尼上线），名字命中「超级智能」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/87aemjYj3JPEu8YnmLXSK6D1v9SurhaXNmQ2Xtdzpump</t>
+          <t>https://gmgn.ai/bsc/token/0xaf3c2e121372eaf5458b827abe21393665d97777</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>超级智能 SI · 🦉猫头鹰</t>
+          <t>量子 / AI 破解私钥</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -4619,22 +4619,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>TeslaSI</t>
+          <t>QI</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>bsc</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0xaf3c2e121372eaf5458b827abe21393665d97777</t>
+          <t>8TiMkgvsrat9tM2esko8zVTt99LZLpefUM4SnZaziXaQ</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4643,25 +4643,25 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>15437</v>
+        <v>974725</v>
       </c>
       <c r="I13" t="n">
-        <v>-9.9</v>
+        <v>0.8</v>
       </c>
       <c r="J13" t="n">
-        <v>-57.4</v>
+        <v>-44.9</v>
       </c>
       <c r="K13" t="n">
-        <v>12975</v>
+        <v>124929</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Tesla Super Intelligence（10/11 19:35 悉尼上线），名字命中「超级智能」关键词；叙事待人工核实。</t>
+          <t>Quantum Inu：10/09 新盘，量子狗，量子赛道当前市值最大的纯 meme，24h 涨幅上万 %。</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0xaf3c2e121372eaf5458b827abe21393665d97777</t>
+          <t>https://gmgn.ai/sol/token/8TiMkgvsrat9tM2esko8zVTt99LZLpefUM4SnZaziXaQ</t>
         </is>
       </c>
     </row>
@@ -4678,12 +4678,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>QI</t>
+          <t>QCAT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -4693,7 +4693,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>8TiMkgvsrat9tM2esko8zVTt99LZLpefUM4SnZaziXaQ</t>
+          <t>7vMkPxLwaH26qSZ2CgHhzvrgz9wUWMvT256vbUWfarm</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -4702,25 +4702,25 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1006097</v>
+        <v>83957</v>
       </c>
       <c r="I14" t="n">
-        <v>-2.9</v>
+        <v>26</v>
       </c>
       <c r="J14" t="n">
-        <v>-48.7</v>
+        <v>-54</v>
       </c>
       <c r="K14" t="n">
-        <v>126215</v>
+        <v>37347</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Quantum Inu：10/09 新盘，量子狗，量子赛道当前市值最大的纯 meme，24h 涨幅上万 %。</t>
+          <t>🆕 GMGN 自动发现：Quantum Cat（10/10 02:08 悉尼上线），名字命中「量子」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/8TiMkgvsrat9tM2esko8zVTt99LZLpefUM4SnZaziXaQ</t>
+          <t>https://gmgn.ai/sol/token/7vMkPxLwaH26qSZ2CgHhzvrgz9wUWMvT256vbUWfarm</t>
         </is>
       </c>
     </row>
@@ -4742,7 +4742,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>QCAT</t>
+          <t>QI</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>7vMkPxLwaH26qSZ2CgHhzvrgz9wUWMvT256vbUWfarm</t>
+          <t>eFBwUbyopvmxYHEwXZRbsTkSJHsz7WqawqKMxbqpump</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -4761,32 +4761,32 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>86672</v>
+        <v>3866075</v>
       </c>
       <c r="I15" t="n">
-        <v>29.4</v>
+        <v>0.9</v>
       </c>
       <c r="J15" t="n">
-        <v>-50.6</v>
+        <v>12.4</v>
       </c>
       <c r="K15" t="n">
-        <v>38150</v>
+        <v>167324</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Quantum Cat（10/10 02:08 悉尼上线），名字命中「量子」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：Quantum Inu（10/10 21:41 悉尼上线），名字命中「量子」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/7vMkPxLwaH26qSZ2CgHhzvrgz9wUWMvT256vbUWfarm</t>
+          <t>https://gmgn.ai/sol/token/eFBwUbyopvmxYHEwXZRbsTkSJHsz7WqawqKMxbqpump</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>量子 / AI 破解私钥</t>
+          <t>Grok Bot · 整家公司由 AI 组成</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -4796,22 +4796,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>QI</t>
+          <t>Grok Bot</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>eFBwUbyopvmxYHEwXZRbsTkSJHsz7WqawqKMxbqpump</t>
+          <t>0x7aede49f29bf7bc643853c1136854ea8e4da7777</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -4820,32 +4820,32 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>3867929</v>
+        <v>46294</v>
       </c>
       <c r="I16" t="n">
-        <v>0.6</v>
+        <v>2.9</v>
       </c>
       <c r="J16" t="n">
-        <v>12.6</v>
+        <v>-5.5</v>
       </c>
       <c r="K16" t="n">
-        <v>167509</v>
+        <v>23784</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Quantum Inu（10/10 21:41 悉尼上线），名字命中「量子」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：AI Agent（10/12 11:45 悉尼上线），名字命中「Grok」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/eFBwUbyopvmxYHEwXZRbsTkSJHsz7WqawqKMxbqpump</t>
+          <t>https://gmgn.ai/bsc/token/0x7aede49f29bf7bc643853c1136854ea8e4da7777</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Grok Bot · 整家公司由 AI 组成</t>
+          <t>股票 meme · 代币化美股</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -4860,17 +4860,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Grok Bot</t>
+          <t>STONK</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>bsc</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0x7aede49f29bf7bc643853c1136854ea8e4da7777</t>
+          <t>6GmAFSYs4gk3FDao5FzzySQpPZaWsa4rUJHacpMpUNgx</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -4879,25 +4879,25 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>40663</v>
+        <v>93809944</v>
       </c>
       <c r="I17" t="n">
-        <v>-23.6</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>-17.5</v>
+        <v>-23.4</v>
       </c>
       <c r="K17" t="n">
-        <v>22271</v>
+        <v>69568</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：AI Agent（10/12 11:45 悉尼上线），名字命中「Grok」关键词；叙事待人工核实。</t>
+          <t>StonkFun 发射台币：股票 meme 龙头，30 天收入 ~$28–31M，市值 ~$1.2 亿。</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x7aede49f29bf7bc643853c1136854ea8e4da7777</t>
+          <t>https://gmgn.ai/sol/token/6GmAFSYs4gk3FDao5FzzySQpPZaWsa4rUJHacpMpUNgx</t>
         </is>
       </c>
     </row>
@@ -4914,22 +4914,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>STONK</t>
+          <t>PONS</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>robinhood</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>6GmAFSYs4gk3FDao5FzzySQpPZaWsa4rUJHacpMpUNgx</t>
+          <t>0x39dbed3a2bd333467115de45665cc57f813c4571</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -4938,25 +4938,25 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>94421900</v>
+        <v>282082430</v>
       </c>
       <c r="I18" t="n">
-        <v>2</v>
+        <v>0.6</v>
       </c>
       <c r="J18" t="n">
-        <v>-22.4</v>
+        <v>-10.8</v>
       </c>
       <c r="K18" t="n">
-        <v>70138</v>
+        <v>2634771</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>StonkFun 发射台币：股票 meme 龙头，30 天收入 ~$28–31M，市值 ~$1.2 亿。</t>
+          <t>Robinhood Chain 发射台币 Pons：10 万持有人，股票链 meme 的庄家盘。</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/6GmAFSYs4gk3FDao5FzzySQpPZaWsa4rUJHacpMpUNgx</t>
+          <t>https://gmgn.ai/robinhood/token/0x39dbed3a2bd333467115de45665cc57f813c4571</t>
         </is>
       </c>
     </row>
@@ -4978,17 +4978,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>PONS</t>
+          <t>BLUECHIP</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>robinhood</t>
+          <t>base</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0x39dbed3a2bd333467115de45665cc57f813c4571</t>
+          <t>0xb200000000000000000000cfbdf64a8706a94a01</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -4997,25 +4997,25 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>282839740</v>
+        <v>5794970</v>
       </c>
       <c r="I19" t="n">
-        <v>-0.7</v>
+        <v>-0.5</v>
       </c>
       <c r="J19" t="n">
-        <v>-10.3</v>
+        <v>-13.5</v>
       </c>
       <c r="K19" t="n">
-        <v>2637428</v>
+        <v>301373</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Robinhood Chain 发射台币 Pons：10 万持有人，股票链 meme 的庄家盘。</t>
+          <t>Base 股票 meme：Jesse Pollak Token2049 幻灯片点名。</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/robinhood/token/0x39dbed3a2bd333467115de45665cc57f813c4571</t>
+          <t>https://gmgn.ai/base/token/0xb200000000000000000000cfbdf64a8706a94a01</t>
         </is>
       </c>
     </row>
@@ -5037,7 +5037,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>BLUECHIP</t>
+          <t>IPOD</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -5047,7 +5047,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0xb200000000000000000000cfbdf64a8706a94a01</t>
+          <t>0xa6af0cea8fbc93e1eccc00f1fdd9a0bba251fee1</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -5056,25 +5056,25 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>5768684</v>
+        <v>1091244</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.3</v>
+        <v>2.4</v>
       </c>
       <c r="J20" t="n">
-        <v>-13.8</v>
+        <v>-10.3</v>
       </c>
       <c r="K20" t="n">
-        <v>301373</v>
+        <v>261963</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Base 股票 meme：Jesse Pollak Token2049 幻灯片点名。</t>
+          <t>Base 苹果股票梗 iPod，Jesse 幻灯片点名。</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/base/token/0xb200000000000000000000cfbdf64a8706a94a01</t>
+          <t>https://gmgn.ai/base/token/0xa6af0cea8fbc93e1eccc00f1fdd9a0bba251fee1</t>
         </is>
       </c>
     </row>
@@ -5096,7 +5096,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>IPOD</t>
+          <t>DGUY</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -5106,7 +5106,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0xa6af0cea8fbc93e1eccc00f1fdd9a0bba251fee1</t>
+          <t>0xe34356dcd3d7bb991248f322e4ec31b5d60bc54e</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -5115,25 +5115,25 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>1063660</v>
+        <v>988140</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.2</v>
+        <v>8</v>
       </c>
       <c r="J21" t="n">
-        <v>-12.6</v>
+        <v>3.7</v>
       </c>
       <c r="K21" t="n">
-        <v>254805</v>
+        <v>117456</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Base 苹果股票梗 iPod，Jesse 幻灯片点名。</t>
+          <t>Delivery Guy：Base 股票 meme，Jesse 幻灯片点名。</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/base/token/0xa6af0cea8fbc93e1eccc00f1fdd9a0bba251fee1</t>
+          <t>https://gmgn.ai/base/token/0xe34356dcd3d7bb991248f322e4ec31b5d60bc54e</t>
         </is>
       </c>
     </row>
@@ -5155,7 +5155,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>DGUY</t>
+          <t>TEMU</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -5165,7 +5165,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0xe34356dcd3d7bb991248f322e4ec31b5d60bc54e</t>
+          <t>0x3c573bdd88008c94f025e5023212f28e5f39744c</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -5174,32 +5174,32 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>978415</v>
+        <v>266718</v>
       </c>
       <c r="I22" t="n">
-        <v>19.6</v>
+        <v>3.5</v>
       </c>
       <c r="J22" t="n">
-        <v>2.5</v>
+        <v>-9.800000000000001</v>
       </c>
       <c r="K22" t="n">
-        <v>117530</v>
+        <v>54717</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Delivery Guy：Base 股票 meme，Jesse 幻灯片点名。</t>
+          <t>TEMU on Base：Jesse 幻灯片点名的拼多多梗。</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/base/token/0xe34356dcd3d7bb991248f322e4ec31b5d60bc54e</t>
+          <t>https://gmgn.ai/base/token/0x3c573bdd88008c94f025e5023212f28e5f39744c</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>股票 meme · 代币化美股</t>
+          <t>持币分红盘 · ZCAT/BATON</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5209,22 +5209,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>TEMU</t>
+          <t>ZCAT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0x3c573bdd88008c94f025e5023212f28e5f39744c</t>
+          <t>HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -5233,25 +5233,25 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>267149</v>
+        <v>40422914</v>
       </c>
       <c r="I23" t="n">
-        <v>3.8</v>
+        <v>-3.3</v>
       </c>
       <c r="J23" t="n">
-        <v>-9.1</v>
+        <v>-18.4</v>
       </c>
       <c r="K23" t="n">
-        <v>54691</v>
+        <v>1052092</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>TEMU on Base：Jesse 幻灯片点名的拼多多梗。</t>
+          <t>Anonymous Cat：3% 交易税自动换 ZEC 分红给持有人，分红盘龙头。</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/base/token/0x3c573bdd88008c94f025e5023212f28e5f39744c</t>
+          <t>https://gmgn.ai/sol/token/HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
         </is>
       </c>
     </row>
@@ -5268,12 +5268,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ZCAT</t>
+          <t>BATON</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -5283,7 +5283,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
+          <t>Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -5292,25 +5292,25 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>42660745</v>
+        <v>12454644</v>
       </c>
       <c r="I24" t="n">
-        <v>4.5</v>
+        <v>-1.4</v>
       </c>
       <c r="J24" t="n">
-        <v>-11.2</v>
+        <v>-27</v>
       </c>
       <c r="K24" t="n">
-        <v>1082438</v>
+        <v>686115</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Anonymous Cat：3% 交易税自动换 ZEC 分红给持有人，分红盘龙头。</t>
+          <t>baton：分红 PUMP 的分红盘，ATH ~$19M，回调后第二腿。</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
+          <t>https://gmgn.ai/sol/token/Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
         </is>
       </c>
     </row>
@@ -5332,7 +5332,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>BATON</t>
+          <t>MCAT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
+          <t>H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -5351,25 +5351,25 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>13006022</v>
+        <v>148137</v>
       </c>
       <c r="I25" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="J25" t="n">
-        <v>-24.6</v>
+        <v>16.2</v>
       </c>
       <c r="K25" t="n">
-        <v>709083</v>
+        <v>34415</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>baton：分红 PUMP 的分红盘，ATH ~$19M，回调后第二腿。</t>
+          <t>Addicted Cat：分红门罗币 XMR，Cake Wallet 创始人买入。</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
+          <t>https://gmgn.ai/sol/token/H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
         </is>
       </c>
     </row>
@@ -5391,7 +5391,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>MCAT</t>
+          <t>FACTORY</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -5401,7 +5401,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
+          <t>7536qC4LEs3W2GtSKbhVGNJSiRfuXJhKVthxsgfkpump</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -5410,25 +5410,25 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>148137</v>
+        <v>40434</v>
       </c>
       <c r="I26" t="n">
-        <v>1.2</v>
+        <v>0.1</v>
       </c>
       <c r="J26" t="n">
-        <v>15.9</v>
+        <v>-19.2</v>
       </c>
       <c r="K26" t="n">
-        <v>34415</v>
+        <v>16001</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Addicted Cat：分红门罗币 XMR，Cake Wallet 创始人买入。</t>
+          <t>🆕 GMGN 自动发现：Baton Factory（10/10 22:26 悉尼上线），名字命中「持币分红盘」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
+          <t>https://gmgn.ai/sol/token/7536qC4LEs3W2GtSKbhVGNJSiRfuXJhKVthxsgfkpump</t>
         </is>
       </c>
     </row>
@@ -5450,17 +5450,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>FACTORY</t>
+          <t>上等羊</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>7536qC4LEs3W2GtSKbhVGNJSiRfuXJhKVthxsgfkpump</t>
+          <t>0x26c4829616644144b1dcec6c6c62828c9a717777</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -5469,32 +5469,32 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>39610</v>
+        <v>35776</v>
       </c>
       <c r="I27" t="n">
-        <v>-2</v>
+        <v>-33.1</v>
       </c>
       <c r="J27" t="n">
-        <v>-26.3</v>
+        <v>543.4</v>
       </c>
       <c r="K27" t="n">
-        <v>15999</v>
+        <v>18787</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Baton Factory（10/10 22:26 悉尼上线），名字命中「持币分红盘」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：首创锁仓拖底回购分红协议（10/13 19:17 悉尼上线），名字命中「持币分红盘」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/7536qC4LEs3W2GtSKbhVGNJSiRfuXJhKVthxsgfkpump</t>
+          <t>https://gmgn.ai/bsc/token/0x26c4829616644144b1dcec6c6c62828c9a717777</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>持币分红盘 · ZCAT/BATON</t>
+          <t>ANSEM · SOL 老龙头</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5504,22 +5504,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>上等羊</t>
+          <t>ANSEM</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>bsc</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0x26c4829616644144b1dcec6c6c62828c9a717777</t>
+          <t>9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -5528,32 +5528,32 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>38301</v>
+        <v>131268432</v>
       </c>
       <c r="I28" t="n">
-        <v>-34.8</v>
+        <v>0.8</v>
       </c>
       <c r="J28" t="n">
-        <v>588.8</v>
+        <v>-5</v>
       </c>
       <c r="K28" t="n">
-        <v>19376</v>
+        <v>2237017</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：首创锁仓拖底回购分红协议（10/13 19:17 悉尼上线），名字命中「持币分红盘」关键词；叙事待人工核实。</t>
+          <t>The Black Bull：Ansem 本人梗的 SOL 老龙头，15 万持有人，前十持仓 ~65% 偏集中。</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x26c4829616644144b1dcec6c6c62828c9a717777</t>
+          <t>https://gmgn.ai/sol/token/9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ANSEM · SOL 老龙头</t>
+          <t>以太坊近况 · Glamsterdam</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5568,17 +5568,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>ANSEM</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
+          <t>0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -5587,32 +5587,32 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>130950504</v>
+        <v>358086530</v>
       </c>
       <c r="I29" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>-5.8</v>
+        <v>-5</v>
       </c>
       <c r="K29" t="n">
-        <v>2234406</v>
+        <v>10979995</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>The Black Bull：Ansem 本人梗的 SOL 老龙头，15 万持有人，前十持仓 ~65% 偏集中。</t>
+          <t>SPX6900：Murad 舞台喊“meme 将超越比特币”的 ETH 主网 meme 龙头。</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
+          <t>https://gmgn.ai/eth/token/0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>以太坊近况 · Glamsterdam</t>
+          <t>BSC 中文盘 · 币安人生</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5627,17 +5627,17 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>币安人生</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>eth</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
+          <t>0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -5646,25 +5646,25 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>359924110</v>
+        <v>525250160</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>-4.2</v>
+        <v>-9.9</v>
       </c>
       <c r="K30" t="n">
-        <v>10995319</v>
+        <v>8210195</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SPX6900：Murad 舞台喊“meme 将超越比特币”的 ETH 主网 meme 龙头。</t>
+          <t>币安人生：何一推文带火的 BSC 中文 meme 龙头，ATH ~$9 亿，现 ~$5.5 亿。</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/eth/token/0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
+          <t>https://gmgn.ai/bsc/token/0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
         </is>
       </c>
     </row>
@@ -5681,12 +5681,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>币安人生</t>
+          <t>龙虾</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -5696,7 +5696,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
+          <t>0xeccbb861c0dda7efd964010085488b69317e4444</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -5705,25 +5705,25 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>526020160</v>
+        <v>43674286</v>
       </c>
       <c r="I31" t="n">
-        <v>0.1</v>
+        <v>1.2</v>
       </c>
       <c r="J31" t="n">
-        <v>-9.6</v>
+        <v>4.7</v>
       </c>
       <c r="K31" t="n">
-        <v>8218854</v>
+        <v>2059720</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>币安人生：何一推文带火的 BSC 中文 meme 龙头，ATH ~$9 亿，现 ~$5.5 亿。</t>
+          <t>龙虾：币安中文号推文出圈的中文盘，ATH ~$3.1 亿，现 ~$4300 万。注意今天有同名高仿盘。</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
+          <t>https://gmgn.ai/bsc/token/0xeccbb861c0dda7efd964010085488b69317e4444</t>
         </is>
       </c>
     </row>
@@ -5745,7 +5745,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>龙虾</t>
+          <t>币安圣羊</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -5755,7 +5755,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>0xeccbb861c0dda7efd964010085488b69317e4444</t>
+          <t>0xcc4cc7ebaab40aa19317027b63e584333f697777</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -5764,25 +5764,25 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>43666620</v>
+        <v>249856</v>
       </c>
       <c r="I32" t="n">
-        <v>1</v>
+        <v>16.6</v>
       </c>
       <c r="J32" t="n">
-        <v>6</v>
+        <v>-6.4</v>
       </c>
       <c r="K32" t="n">
-        <v>2061579</v>
+        <v>49050</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>龙虾：币安中文号推文出圈的中文盘，ATH ~$3.1 亿，现 ~$4300 万。注意今天有同名高仿盘。</t>
+          <t>🆕 GMGN 自动发现：币安圣羊（10/10 04:20 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0xeccbb861c0dda7efd964010085488b69317e4444</t>
+          <t>https://gmgn.ai/bsc/token/0xcc4cc7ebaab40aa19317027b63e584333f697777</t>
         </is>
       </c>
     </row>
@@ -5804,7 +5804,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>币安圣羊</t>
+          <t>币安人</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>0xcc4cc7ebaab40aa19317027b63e584333f697777</t>
+          <t>0x2c2d4298548ae585c224714555f18abde7367777</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -5823,25 +5823,25 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>217290</v>
+        <v>97851</v>
       </c>
       <c r="I33" t="n">
-        <v>0.9</v>
+        <v>10.4</v>
       </c>
       <c r="J33" t="n">
-        <v>-16.4</v>
+        <v>-20.6</v>
       </c>
       <c r="K33" t="n">
-        <v>46213</v>
+        <v>31080</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：币安圣羊（10/10 04:20 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：Binance Man（10/10 22:33 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0xcc4cc7ebaab40aa19317027b63e584333f697777</t>
+          <t>https://gmgn.ai/bsc/token/0x2c2d4298548ae585c224714555f18abde7367777</t>
         </is>
       </c>
     </row>
@@ -5863,7 +5863,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>币安人</t>
+          <t>Binance Angels</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -5873,7 +5873,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>0x2c2d4298548ae585c224714555f18abde7367777</t>
+          <t>0x62bb38c83afeb82e8f468d122b1b9051b6167777</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -5882,32 +5882,32 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>147863</v>
+        <v>80008</v>
       </c>
       <c r="I34" t="n">
-        <v>91.7</v>
+        <v>-0.9</v>
       </c>
       <c r="J34" t="n">
-        <v>18.7</v>
+        <v>19.5</v>
       </c>
       <c r="K34" t="n">
-        <v>38188</v>
+        <v>27269</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Binance Man（10/10 22:33 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：QQ:945497833（10/12 19:12 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x2c2d4298548ae585c224714555f18abde7367777</t>
+          <t>https://gmgn.ai/bsc/token/0x62bb38c83afeb82e8f468d122b1b9051b6167777</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BSC 中文盘 · 币安人生</t>
+          <t>LAPTOP · 亨特·拜登盘</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -5917,22 +5917,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Binance Angels</t>
+          <t>LAPTOP</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>bsc</t>
+          <t>base</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>0x62bb38c83afeb82e8f468d122b1b9051b6167777</t>
+          <t>0xb095274743941e953c746f9c228da9c18bb6ec29</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -5941,32 +5941,32 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>78085</v>
+        <v>76180621</v>
       </c>
       <c r="I35" t="n">
-        <v>-4.9</v>
+        <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>2.9</v>
+        <v>1.1</v>
       </c>
       <c r="K35" t="n">
-        <v>26942</v>
+        <v>472480</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：QQ:945497833（10/12 19:12 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
+          <t>Hunter Biden 本人发的“笔记本电脑”梗币，前十持仓 ~91% 极度集中。</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x62bb38c83afeb82e8f468d122b1b9051b6167777</t>
+          <t>https://gmgn.ai/base/token/0xb095274743941e953c746f9c228da9c18bb6ec29</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LAPTOP · 亨特·拜登盘</t>
+          <t>后量子地堡 · BNKR/PQC</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5981,17 +5981,17 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>LAPTOP</t>
+          <t>PQC</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>0xb095274743941e953c746f9c228da9c18bb6ec29</t>
+          <t>7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -6000,25 +6000,25 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>76307528</v>
+        <v>277974</v>
       </c>
       <c r="I36" t="n">
-        <v>0.1</v>
+        <v>-11.7</v>
       </c>
       <c r="J36" t="n">
-        <v>1.2</v>
+        <v>-39.3</v>
       </c>
       <c r="K36" t="n">
-        <v>517788</v>
+        <v>61701</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Hunter Biden 本人发的“笔记本电脑”梗币，前十持仓 ~91% 极度集中。</t>
+          <t>pqc.market 平台币：后量子发射台，10/08 上线，24h 成交 ~$7.7M，BNKR 的母盘。</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/base/token/0xb095274743941e953c746f9c228da9c18bb6ec29</t>
+          <t>https://gmgn.ai/sol/token/7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
         </is>
       </c>
     </row>
@@ -6035,12 +6035,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>PQC</t>
+          <t>BUNKER</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -6050,7 +6050,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
+          <t>BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -6059,47 +6059,47 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>307295</v>
+        <v>116129</v>
       </c>
       <c r="I37" t="n">
-        <v>-6.6</v>
+        <v>-3.7</v>
       </c>
       <c r="J37" t="n">
-        <v>-36.5</v>
+        <v>-29.2</v>
       </c>
       <c r="K37" t="n">
-        <v>65757</v>
+        <v>28541</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>pqc.market 平台币：后量子发射台，10/08 上线，24h 成交 ~$7.7M，BNKR 的母盘。</t>
+          <t>🆕 GMGN 自动发现：Bunker Mode（10/10 10:14 悉尼上线），名字命中「后量子地堡」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
+          <t>https://gmgn.ai/sol/token/BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>后量子地堡 · BNKR/PQC</t>
+          <t>Solamians · Solana 官方插画里的“国籍”</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>大周期</t>
+          <t>24小时</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>BUNKER</t>
+          <t>Solamians</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -6109,7 +6109,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
+          <t>8ZP5CzbPL1fmP8dn1GEmLd8xw1JdudUF5Dk7EpLxpump</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -6118,32 +6118,32 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>118844</v>
+        <v>145177</v>
       </c>
       <c r="I38" t="n">
-        <v>-1.4</v>
+        <v>1.8</v>
       </c>
       <c r="J38" t="n">
-        <v>-30.2</v>
+        <v>-54.6</v>
       </c>
       <c r="K38" t="n">
-        <v>28936</v>
+        <v>37067</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Bunker Mode（10/10 10:14 悉尼上线），名字命中「后量子地堡」关键词；叙事待人工核实。</t>
+          <t>Solana 官方 Breakpoint 指南护照插画写着 Nationality: Solamian（已核实原图）。10/12 13:09 创建，ATH ~$910K，机器人成交约 57%。</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
+          <t>https://gmgn.ai/sol/token/8ZP5CzbPL1fmP8dn1GEmLd8xw1JdudUF5Dk7EpLxpump</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Solamians · Solana 官方插画里的“国籍”</t>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6158,7 +6158,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Solamians</t>
+          <t>CAESAR</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -6168,7 +6168,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>8ZP5CzbPL1fmP8dn1GEmLd8xw1JdudUF5Dk7EpLxpump</t>
+          <t>EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -6177,32 +6177,32 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>141379</v>
+        <v>57854</v>
       </c>
       <c r="I39" t="n">
-        <v>14.1</v>
+        <v>-33.3</v>
       </c>
       <c r="J39" t="n">
-        <v>-56.5</v>
+        <v>145.4</v>
       </c>
       <c r="K39" t="n">
-        <v>35346</v>
+        <v>19402</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Solana 官方 Breakpoint 指南护照插画写着 Nationality: Solamian（已核实原图）。10/12 13:09 创建，ATH ~$910K，机器人成交约 57%。</t>
+          <t>pmarca 转发的《Slop Caesar》社区盘。19:24 Devon 本人贴出此 CA，自称已领约 108 SOL 手续费（GMGN：分成 100% 给 devonmvfisher，已领取）。原开发者已清仓、批量发币地址；机器人约 62%。</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/8ZP5CzbPL1fmP8dn1GEmLd8xw1JdudUF5Dk7EpLxpump</t>
+          <t>https://gmgn.ai/sol/token/EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -6217,7 +6217,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>CAESAR</t>
+          <t>CYBERLEEK</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -6227,7 +6227,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
+          <t>ApZuxdpzMrbEYTGEzeY9afh5pj9d6qPRJCTgQYiipbKg</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -6236,25 +6236,25 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>63518</v>
+        <v>1759015</v>
       </c>
       <c r="I40" t="n">
-        <v>-29.4</v>
+        <v>1.8</v>
       </c>
       <c r="J40" t="n">
-        <v>125.6</v>
+        <v>-25</v>
       </c>
       <c r="K40" t="n">
-        <v>20543</v>
+        <v>559622</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>pmarca 转发的《Slop Caesar》社区盘。19:24 Devon 本人贴出此 CA，自称已领约 108 SOL 手续费（GMGN：分成 100% 给 devonmvfisher，已领取）。原开发者已清仓、批量发币地址；机器人约 62%。</t>
+          <t>GTA 6 泄露者的币，10/10 喊出 3000 万市值放完整版。8 月曾提款后崩盘，24h -53%。</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
+          <t>https://gmgn.ai/sol/token/ApZuxdpzMrbEYTGEzeY9afh5pj9d6qPRJCTgQYiipbKg</t>
         </is>
       </c>
     </row>
@@ -6271,12 +6271,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>CYBERLEEK</t>
+          <t>Dacity</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -6286,7 +6286,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>ApZuxdpzMrbEYTGEzeY9afh5pj9d6qPRJCTgQYiipbKg</t>
+          <t>nxPqZ4F7ux8Vph5NFu25rEP6Kx9Gr1U6Fmj36Rjpump</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -6295,25 +6295,25 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>1690774</v>
+        <v>126609</v>
       </c>
       <c r="I41" t="n">
-        <v>-1.6</v>
+        <v>-9.199999999999999</v>
       </c>
       <c r="J41" t="n">
-        <v>-32.9</v>
+        <v>10.4</v>
       </c>
       <c r="K41" t="n">
-        <v>549389</v>
+        <v>32823</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>GTA 6 泄露者的币，10/10 喊出 3000 万市值放完整版。8 月曾提款后崩盘，24h -53%。</t>
+          <t>据称出现在泄露视频里的游戏内币（未核实），ATH 回撤 88%，机器人多。</t>
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/ApZuxdpzMrbEYTGEzeY9afh5pj9d6qPRJCTgQYiipbKg</t>
+          <t>https://gmgn.ai/sol/token/nxPqZ4F7ux8Vph5NFu25rEP6Kx9Gr1U6Fmj36Rjpump</t>
         </is>
       </c>
     </row>
@@ -6335,7 +6335,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Dacity</t>
+          <t>CYBERLEEK</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -6345,7 +6345,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>nxPqZ4F7ux8Vph5NFu25rEP6Kx9Gr1U6Fmj36Rjpump</t>
+          <t>J62sjKAAk16afQssxNJS8G2RU9azmCip6VPjMcNcpump</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -6354,25 +6354,25 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>127430</v>
+        <v>315365426</v>
       </c>
       <c r="I42" t="n">
-        <v>-10.2</v>
+        <v>2.2</v>
       </c>
       <c r="J42" t="n">
-        <v>-1.2</v>
+        <v>2685792.6</v>
       </c>
       <c r="K42" t="n">
-        <v>32951</v>
+        <v>1529705</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>据称出现在泄露视频里的游戏内币（未核实），ATH 回撤 88%，机器人多。</t>
+          <t>🆕 GMGN 自动发现：CYBERLEEK（10/13 01:26 悉尼上线），名字命中「GTA」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/nxPqZ4F7ux8Vph5NFu25rEP6Kx9Gr1U6Fmj36Rjpump</t>
+          <t>https://gmgn.ai/sol/token/J62sjKAAk16afQssxNJS8G2RU9azmCip6VPjMcNcpump</t>
         </is>
       </c>
     </row>
@@ -6404,7 +6404,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>J62sjKAAk16afQssxNJS8G2RU9azmCip6VPjMcNcpump</t>
+          <t>GkgVK2duAV9Rjbt43prMiZscuMVQ9XR1RihSYsT6tjjE</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -6413,82 +6413,23 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>313870454</v>
+        <v>73973</v>
       </c>
       <c r="I43" t="n">
-        <v>2.6</v>
+        <v>0.1</v>
       </c>
       <c r="J43" t="n">
-        <v>2673060.3</v>
+        <v>-80.5</v>
       </c>
       <c r="K43" t="n">
-        <v>1528163</v>
+        <v>23002</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：CYBERLEEK（10/13 01:26 悉尼上线），名字命中「GTA」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：CyberLeek（10/13 07:40 悉尼上线），名字命中「GTA」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M43" s="2" t="inlineStr">
-        <is>
-          <t>https://gmgn.ai/sol/token/J62sjKAAk16afQssxNJS8G2RU9azmCip6VPjMcNcpump</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>24小时</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>beta</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>CYBERLEEK</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>sol</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>GkgVK2duAV9Rjbt43prMiZscuMVQ9XR1RihSYsT6tjjE</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>alive</t>
-        </is>
-      </c>
-      <c r="H44" t="n">
-        <v>75310</v>
-      </c>
-      <c r="I44" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="J44" t="n">
-        <v>-80.09999999999999</v>
-      </c>
-      <c r="K44" t="n">
-        <v>23227</v>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>🆕 GMGN 自动发现：CyberLeek（10/13 07:40 悉尼上线），名字命中「GTA」关键词；叙事待人工核实。</t>
-        </is>
-      </c>
-      <c r="M44" s="2" t="inlineStr">
         <is>
           <t>https://gmgn.ai/sol/token/GkgVK2duAV9Rjbt43prMiZscuMVQ9XR1RihSYsT6tjjE</t>
         </is>
@@ -6538,7 +6479,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId43"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
tokens 10/14 01:41 radar-xlimit
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -3994,16 +3994,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>163810</v>
+        <v>158909</v>
       </c>
       <c r="I2" t="n">
-        <v>-37.8</v>
+        <v>-16.6</v>
       </c>
       <c r="J2" t="n">
-        <v>4126.5</v>
+        <v>4000</v>
       </c>
       <c r="K2" t="n">
-        <v>40815</v>
+        <v>40022</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -4053,16 +4053,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>71052</v>
+        <v>70687</v>
       </c>
       <c r="I3" t="n">
-        <v>-2.5</v>
+        <v>-3.8</v>
       </c>
       <c r="J3" t="n">
-        <v>21.5</v>
+        <v>20.9</v>
       </c>
       <c r="K3" t="n">
-        <v>48964</v>
+        <v>48892</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -4112,16 +4112,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>163810</v>
+        <v>158909</v>
       </c>
       <c r="I4" t="n">
-        <v>-37.8</v>
+        <v>-16.6</v>
       </c>
       <c r="J4" t="n">
-        <v>4126.5</v>
+        <v>4000</v>
       </c>
       <c r="K4" t="n">
-        <v>40415</v>
+        <v>40022</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -4171,16 +4171,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>16833809</v>
+        <v>17748507</v>
       </c>
       <c r="I5" t="n">
-        <v>-1.3</v>
+        <v>3.8</v>
       </c>
       <c r="J5" t="n">
-        <v>-24.6</v>
+        <v>-24.4</v>
       </c>
       <c r="K5" t="n">
-        <v>749239</v>
+        <v>763364</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -4230,16 +4230,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1225436</v>
+        <v>1489731</v>
       </c>
       <c r="I6" t="n">
-        <v>-5.5</v>
+        <v>20.4</v>
       </c>
       <c r="J6" t="n">
-        <v>-29.5</v>
+        <v>-15.3</v>
       </c>
       <c r="K6" t="n">
-        <v>152841</v>
+        <v>168072</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -4289,16 +4289,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>499210</v>
+        <v>437566</v>
       </c>
       <c r="I7" t="n">
-        <v>-5.3</v>
+        <v>-14</v>
       </c>
       <c r="J7" t="n">
-        <v>-25.5</v>
+        <v>-31.9</v>
       </c>
       <c r="K7" t="n">
-        <v>82356</v>
+        <v>76885</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -4348,16 +4348,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>12282</v>
+        <v>14564</v>
       </c>
       <c r="I8" t="n">
-        <v>-8.5</v>
+        <v>19.1</v>
       </c>
       <c r="J8" t="n">
-        <v>-50.8</v>
+        <v>-40.2</v>
       </c>
       <c r="K8" t="n">
-        <v>10193</v>
+        <v>10945</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -4407,16 +4407,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1084206</v>
+        <v>1060408</v>
       </c>
       <c r="I9" t="n">
-        <v>-6</v>
+        <v>-8.1</v>
       </c>
       <c r="J9" t="n">
-        <v>6.8</v>
+        <v>6.4</v>
       </c>
       <c r="K9" t="n">
-        <v>102521</v>
+        <v>100604</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -4466,16 +4466,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>13397</v>
+        <v>10095</v>
       </c>
       <c r="I10" t="n">
-        <v>-1.9</v>
+        <v>-27.3</v>
       </c>
       <c r="J10" t="n">
-        <v>-56.7</v>
+        <v>-67.59999999999999</v>
       </c>
       <c r="K10" t="n">
-        <v>7718</v>
+        <v>6160</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -4525,16 +4525,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>14961</v>
+        <v>14527</v>
       </c>
       <c r="I11" t="n">
-        <v>-26.5</v>
+        <v>17.2</v>
       </c>
       <c r="J11" t="n">
-        <v>-45.3</v>
+        <v>-48.9</v>
       </c>
       <c r="K11" t="n">
-        <v>12769</v>
+        <v>12422</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -4584,16 +4584,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>867465</v>
+        <v>838224</v>
       </c>
       <c r="I12" t="n">
-        <v>8.9</v>
+        <v>-0.1</v>
       </c>
       <c r="J12" t="n">
-        <v>-47.9</v>
+        <v>-49.1</v>
       </c>
       <c r="K12" t="n">
-        <v>124538</v>
+        <v>123119</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -4643,16 +4643,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>65746</v>
+        <v>66944</v>
       </c>
       <c r="I13" t="n">
-        <v>-11.7</v>
+        <v>5</v>
       </c>
       <c r="J13" t="n">
-        <v>-57.4</v>
+        <v>-60.4</v>
       </c>
       <c r="K13" t="n">
-        <v>32740</v>
+        <v>33059</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -4702,16 +4702,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>4037202</v>
+        <v>4031593</v>
       </c>
       <c r="I14" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="J14" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K14" t="n">
-        <v>172894</v>
+        <v>172522</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -4761,16 +4761,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>46863</v>
+        <v>50719</v>
       </c>
       <c r="I15" t="n">
-        <v>16.8</v>
+        <v>27.1</v>
       </c>
       <c r="J15" t="n">
-        <v>24.2</v>
+        <v>30</v>
       </c>
       <c r="K15" t="n">
-        <v>23530</v>
+        <v>24337</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -4820,16 +4820,16 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>94399929</v>
+        <v>94777406</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>-1.3</v>
       </c>
       <c r="J16" t="n">
-        <v>-20.6</v>
+        <v>-19.5</v>
       </c>
       <c r="K16" t="n">
-        <v>65889</v>
+        <v>66281</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -4879,16 +4879,16 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>301815620</v>
+        <v>298753040</v>
       </c>
       <c r="I17" t="n">
-        <v>1.4</v>
+        <v>-1.8</v>
       </c>
       <c r="J17" t="n">
-        <v>-0.8</v>
+        <v>-0.4</v>
       </c>
       <c r="K17" t="n">
-        <v>2868972</v>
+        <v>2866889</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -4938,16 +4938,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>5748365</v>
+        <v>5776800</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>-0.4</v>
       </c>
       <c r="J18" t="n">
         <v>-10.7</v>
       </c>
       <c r="K18" t="n">
-        <v>302363</v>
+        <v>301076</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -5000,7 +5000,7 @@
         <v>1130756</v>
       </c>
       <c r="I19" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="J19" t="n">
         <v>-8.300000000000001</v>
@@ -5056,16 +5056,16 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>1097254</v>
+        <v>1087536</v>
       </c>
       <c r="I20" t="n">
-        <v>17.6</v>
+        <v>-1.4</v>
       </c>
       <c r="J20" t="n">
-        <v>26.5</v>
+        <v>22.8</v>
       </c>
       <c r="K20" t="n">
-        <v>125144</v>
+        <v>124763</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -5115,16 +5115,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>292853</v>
+        <v>288463</v>
       </c>
       <c r="I21" t="n">
-        <v>8.6</v>
+        <v>7</v>
       </c>
       <c r="J21" t="n">
-        <v>7.1</v>
+        <v>6</v>
       </c>
       <c r="K21" t="n">
-        <v>57849</v>
+        <v>56988</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -5174,16 +5174,16 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>49841954</v>
+        <v>49270871</v>
       </c>
       <c r="I22" t="n">
-        <v>18.4</v>
+        <v>18.2</v>
       </c>
       <c r="J22" t="n">
-        <v>13.4</v>
+        <v>12.3</v>
       </c>
       <c r="K22" t="n">
-        <v>1158963</v>
+        <v>1164369</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -5233,16 +5233,16 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>12242164</v>
+        <v>11995399</v>
       </c>
       <c r="I23" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="J23" t="n">
-        <v>-24.4</v>
+        <v>-24.6</v>
       </c>
       <c r="K23" t="n">
-        <v>697817</v>
+        <v>695997</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -5292,16 +5292,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>148516</v>
+        <v>147456</v>
       </c>
       <c r="I24" t="n">
-        <v>-5.2</v>
+        <v>-5.8</v>
       </c>
       <c r="J24" t="n">
-        <v>8.199999999999999</v>
+        <v>7.3</v>
       </c>
       <c r="K24" t="n">
-        <v>34488</v>
+        <v>34242</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -5351,16 +5351,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>33837</v>
+        <v>34897</v>
       </c>
       <c r="I25" t="n">
-        <v>-14.3</v>
+        <v>4.2</v>
       </c>
       <c r="J25" t="n">
-        <v>-27.5</v>
+        <v>-6</v>
       </c>
       <c r="K25" t="n">
-        <v>14519</v>
+        <v>14642</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -5410,16 +5410,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>39897</v>
+        <v>44263</v>
       </c>
       <c r="I26" t="n">
-        <v>51.9</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="J26" t="n">
-        <v>617.5</v>
+        <v>696</v>
       </c>
       <c r="K26" t="n">
-        <v>19772</v>
+        <v>20848</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -5469,16 +5469,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>140568320</v>
+        <v>136290601</v>
       </c>
       <c r="I27" t="n">
-        <v>4.1</v>
+        <v>0.9</v>
       </c>
       <c r="J27" t="n">
-        <v>0.6</v>
+        <v>-2.1</v>
       </c>
       <c r="K27" t="n">
-        <v>2340707</v>
+        <v>2293520</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -5528,16 +5528,16 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>366371010</v>
+        <v>364211870</v>
       </c>
       <c r="I28" t="n">
-        <v>1.3</v>
+        <v>-0.4</v>
       </c>
       <c r="J28" t="n">
-        <v>-0.9</v>
+        <v>-0.7</v>
       </c>
       <c r="K28" t="n">
-        <v>11152568</v>
+        <v>11151428</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -5587,16 +5587,16 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>525920050</v>
+        <v>531572630</v>
       </c>
       <c r="I29" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="J29" t="n">
-        <v>-7.9</v>
+        <v>-9.800000000000001</v>
       </c>
       <c r="K29" t="n">
-        <v>8281617</v>
+        <v>8301640</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -5646,16 +5646,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>42951181</v>
+        <v>43217391</v>
       </c>
       <c r="I30" t="n">
-        <v>0.3</v>
+        <v>1.5</v>
       </c>
       <c r="J30" t="n">
-        <v>5.6</v>
+        <v>6.6</v>
       </c>
       <c r="K30" t="n">
-        <v>2053636</v>
+        <v>2059927</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -5705,16 +5705,16 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>331068</v>
+        <v>296531</v>
       </c>
       <c r="I31" t="n">
-        <v>-7.5</v>
+        <v>-11.9</v>
       </c>
       <c r="J31" t="n">
-        <v>27</v>
+        <v>14.2</v>
       </c>
       <c r="K31" t="n">
-        <v>57217</v>
+        <v>54170</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -5764,16 +5764,16 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>65334</v>
+        <v>54142</v>
       </c>
       <c r="I32" t="n">
-        <v>-21.3</v>
+        <v>-33.6</v>
       </c>
       <c r="J32" t="n">
-        <v>30.2</v>
+        <v>13.5</v>
       </c>
       <c r="K32" t="n">
-        <v>25516</v>
+        <v>23254</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -5823,16 +5823,16 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>69878</v>
+        <v>73619</v>
       </c>
       <c r="I33" t="n">
-        <v>6.6</v>
+        <v>-7.6</v>
       </c>
       <c r="J33" t="n">
-        <v>5.8</v>
+        <v>27.3</v>
       </c>
       <c r="K33" t="n">
-        <v>25522</v>
+        <v>26122</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -5882,16 +5882,16 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>76031569</v>
+        <v>76175631</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J34" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="K34" t="n">
-        <v>534607</v>
+        <v>535038</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -5941,16 +5941,16 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>234958</v>
+        <v>230996</v>
       </c>
       <c r="I35" t="n">
-        <v>-16.2</v>
+        <v>-14.5</v>
       </c>
       <c r="J35" t="n">
-        <v>-56.8</v>
+        <v>-53.8</v>
       </c>
       <c r="K35" t="n">
-        <v>57575</v>
+        <v>57317</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -6000,16 +6000,16 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>108903</v>
+        <v>111543</v>
       </c>
       <c r="I36" t="n">
-        <v>-6.9</v>
+        <v>-3.9</v>
       </c>
       <c r="J36" t="n">
-        <v>-42.4</v>
+        <v>-42.5</v>
       </c>
       <c r="K36" t="n">
-        <v>27773</v>
+        <v>27979</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -6059,16 +6059,16 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>139706</v>
+        <v>129935</v>
       </c>
       <c r="I37" t="n">
-        <v>0.4</v>
+        <v>1.9</v>
       </c>
       <c r="J37" t="n">
-        <v>-58.7</v>
+        <v>-55.4</v>
       </c>
       <c r="K37" t="n">
-        <v>35483</v>
+        <v>34524</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -6118,16 +6118,16 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>63170</v>
+        <v>64538</v>
       </c>
       <c r="I38" t="n">
-        <v>7.8</v>
+        <v>-6.1</v>
       </c>
       <c r="J38" t="n">
-        <v>322.1</v>
+        <v>289.4</v>
       </c>
       <c r="K38" t="n">
-        <v>20602</v>
+        <v>20589</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -6177,16 +6177,16 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>1829058</v>
+        <v>1902833</v>
       </c>
       <c r="I39" t="n">
-        <v>7.3</v>
+        <v>10.1</v>
       </c>
       <c r="J39" t="n">
-        <v>-29.2</v>
+        <v>-21.5</v>
       </c>
       <c r="K39" t="n">
-        <v>577713</v>
+        <v>588011</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -6236,16 +6236,16 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>140842</v>
+        <v>127175</v>
       </c>
       <c r="I40" t="n">
-        <v>12.5</v>
+        <v>-13.7</v>
       </c>
       <c r="J40" t="n">
-        <v>39.3</v>
+        <v>29</v>
       </c>
       <c r="K40" t="n">
-        <v>34311</v>
+        <v>32524</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -6295,16 +6295,16 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>339622151</v>
+        <v>342519266</v>
       </c>
       <c r="I41" t="n">
-        <v>4.6</v>
+        <v>3.6</v>
       </c>
       <c r="J41" t="n">
-        <v>2892381.3</v>
+        <v>115</v>
       </c>
       <c r="K41" t="n">
-        <v>1605377</v>
+        <v>1610725</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -6354,16 +6354,16 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>20342</v>
+        <v>20215</v>
       </c>
       <c r="I42" t="n">
-        <v>2.7</v>
+        <v>0.2</v>
       </c>
       <c r="J42" t="n">
-        <v>-94.59999999999999</v>
+        <v>-94.7</v>
       </c>
       <c r="K42" t="n">
-        <v>12223</v>
+        <v>12161</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
tokens 10/14 02:33 radar-xlimit
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -3994,16 +3994,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>158909</v>
+        <v>166499</v>
       </c>
       <c r="I2" t="n">
-        <v>-16.6</v>
+        <v>15.2</v>
       </c>
       <c r="J2" t="n">
-        <v>4000</v>
+        <v>4195.8</v>
       </c>
       <c r="K2" t="n">
-        <v>40022</v>
+        <v>41289</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -4053,16 +4053,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>70687</v>
+        <v>69184</v>
       </c>
       <c r="I3" t="n">
-        <v>-3.8</v>
+        <v>-2.6</v>
       </c>
       <c r="J3" t="n">
-        <v>20.9</v>
+        <v>18.4</v>
       </c>
       <c r="K3" t="n">
-        <v>48892</v>
+        <v>48139</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -4112,16 +4112,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>158909</v>
+        <v>169300</v>
       </c>
       <c r="I4" t="n">
-        <v>-16.6</v>
+        <v>17.1</v>
       </c>
       <c r="J4" t="n">
-        <v>4000</v>
+        <v>4268.1</v>
       </c>
       <c r="K4" t="n">
-        <v>40022</v>
+        <v>41832</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -4171,16 +4171,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>17748507</v>
+        <v>16733392</v>
       </c>
       <c r="I5" t="n">
-        <v>3.8</v>
+        <v>-5.5</v>
       </c>
       <c r="J5" t="n">
-        <v>-24.4</v>
+        <v>-26.7</v>
       </c>
       <c r="K5" t="n">
-        <v>763364</v>
+        <v>749942</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -4230,16 +4230,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1489731</v>
+        <v>1323660</v>
       </c>
       <c r="I6" t="n">
-        <v>20.4</v>
+        <v>-7.9</v>
       </c>
       <c r="J6" t="n">
-        <v>-15.3</v>
+        <v>-23.8</v>
       </c>
       <c r="K6" t="n">
-        <v>168072</v>
+        <v>160463</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -4289,16 +4289,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>437566</v>
+        <v>460556</v>
       </c>
       <c r="I7" t="n">
-        <v>-14</v>
+        <v>-6.9</v>
       </c>
       <c r="J7" t="n">
-        <v>-31.9</v>
+        <v>-32.4</v>
       </c>
       <c r="K7" t="n">
-        <v>76885</v>
+        <v>78768</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -4348,16 +4348,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>14564</v>
+        <v>13939</v>
       </c>
       <c r="I8" t="n">
-        <v>19.1</v>
+        <v>3.5</v>
       </c>
       <c r="J8" t="n">
-        <v>-40.2</v>
+        <v>-42.5</v>
       </c>
       <c r="K8" t="n">
-        <v>10945</v>
+        <v>10890</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -4407,16 +4407,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1060408</v>
+        <v>1012075</v>
       </c>
       <c r="I9" t="n">
-        <v>-8.1</v>
+        <v>-7</v>
       </c>
       <c r="J9" t="n">
-        <v>6.4</v>
+        <v>1.8</v>
       </c>
       <c r="K9" t="n">
-        <v>100604</v>
+        <v>98575</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -4466,16 +4466,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>10095</v>
+        <v>10560</v>
       </c>
       <c r="I10" t="n">
-        <v>-27.3</v>
+        <v>-10.1</v>
       </c>
       <c r="J10" t="n">
-        <v>-67.59999999999999</v>
+        <v>-61.1</v>
       </c>
       <c r="K10" t="n">
-        <v>6160</v>
+        <v>6299</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -4525,16 +4525,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>14527</v>
+        <v>12957</v>
       </c>
       <c r="I11" t="n">
-        <v>17.2</v>
+        <v>-13.3</v>
       </c>
       <c r="J11" t="n">
-        <v>-48.9</v>
+        <v>-56.8</v>
       </c>
       <c r="K11" t="n">
-        <v>12422</v>
+        <v>11914</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -4584,16 +4584,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>838224</v>
+        <v>904980</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.1</v>
+        <v>5</v>
       </c>
       <c r="J12" t="n">
-        <v>-49.1</v>
+        <v>-41.4</v>
       </c>
       <c r="K12" t="n">
-        <v>123119</v>
+        <v>122094</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -4643,16 +4643,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>66944</v>
+        <v>67858</v>
       </c>
       <c r="I13" t="n">
-        <v>5</v>
+        <v>2.2</v>
       </c>
       <c r="J13" t="n">
-        <v>-60.4</v>
+        <v>-53.3</v>
       </c>
       <c r="K13" t="n">
-        <v>33059</v>
+        <v>33085</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -4702,16 +4702,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>4031593</v>
+        <v>4068503</v>
       </c>
       <c r="I14" t="n">
-        <v>2.5</v>
+        <v>0.8</v>
       </c>
       <c r="J14" t="n">
-        <v>17</v>
+        <v>17.3</v>
       </c>
       <c r="K14" t="n">
-        <v>172522</v>
+        <v>173039</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -4761,16 +4761,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>50719</v>
+        <v>50984</v>
       </c>
       <c r="I15" t="n">
-        <v>27.1</v>
+        <v>0.6</v>
       </c>
       <c r="J15" t="n">
-        <v>30</v>
+        <v>43.5</v>
       </c>
       <c r="K15" t="n">
-        <v>24337</v>
+        <v>24385</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -4820,16 +4820,16 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>94777406</v>
+        <v>93579822</v>
       </c>
       <c r="I16" t="n">
-        <v>-1.3</v>
+        <v>-1.2</v>
       </c>
       <c r="J16" t="n">
-        <v>-19.5</v>
+        <v>-20.2</v>
       </c>
       <c r="K16" t="n">
-        <v>66281</v>
+        <v>65513</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -4879,16 +4879,16 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>298753040</v>
+        <v>302166020</v>
       </c>
       <c r="I17" t="n">
-        <v>-1.8</v>
+        <v>0.2</v>
       </c>
       <c r="J17" t="n">
-        <v>-0.4</v>
+        <v>3.5</v>
       </c>
       <c r="K17" t="n">
-        <v>2866889</v>
+        <v>2859163</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -4938,16 +4938,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>5776800</v>
+        <v>5899848</v>
       </c>
       <c r="I18" t="n">
-        <v>-0.4</v>
+        <v>2.3</v>
       </c>
       <c r="J18" t="n">
-        <v>-10.7</v>
+        <v>-7.4</v>
       </c>
       <c r="K18" t="n">
-        <v>301076</v>
+        <v>304041</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -4997,16 +4997,16 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>1130756</v>
+        <v>1099444</v>
       </c>
       <c r="I19" t="n">
-        <v>2.8</v>
+        <v>-2.8</v>
       </c>
       <c r="J19" t="n">
-        <v>-8.300000000000001</v>
+        <v>-10.8</v>
       </c>
       <c r="K19" t="n">
-        <v>265620</v>
+        <v>263400</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -5056,16 +5056,16 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>1087536</v>
+        <v>1040997</v>
       </c>
       <c r="I20" t="n">
-        <v>-1.4</v>
+        <v>-5.4</v>
       </c>
       <c r="J20" t="n">
-        <v>22.8</v>
+        <v>16</v>
       </c>
       <c r="K20" t="n">
-        <v>124763</v>
+        <v>121368</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -5115,16 +5115,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>288463</v>
+        <v>295869</v>
       </c>
       <c r="I21" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="J21" t="n">
-        <v>6</v>
+        <v>6.7</v>
       </c>
       <c r="K21" t="n">
-        <v>56988</v>
+        <v>57902</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -5174,16 +5174,16 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>49270871</v>
+        <v>47402587</v>
       </c>
       <c r="I22" t="n">
-        <v>18.2</v>
+        <v>-3.5</v>
       </c>
       <c r="J22" t="n">
-        <v>12.3</v>
+        <v>6.7</v>
       </c>
       <c r="K22" t="n">
-        <v>1164369</v>
+        <v>1146358</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -5233,16 +5233,16 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>11995399</v>
+        <v>12350150</v>
       </c>
       <c r="I23" t="n">
-        <v>2.9</v>
+        <v>1.1</v>
       </c>
       <c r="J23" t="n">
-        <v>-24.6</v>
+        <v>-17.4</v>
       </c>
       <c r="K23" t="n">
-        <v>695997</v>
+        <v>698267</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -5292,16 +5292,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>147456</v>
+        <v>154303</v>
       </c>
       <c r="I24" t="n">
-        <v>-5.8</v>
+        <v>4.6</v>
       </c>
       <c r="J24" t="n">
-        <v>7.3</v>
+        <v>16</v>
       </c>
       <c r="K24" t="n">
-        <v>34242</v>
+        <v>35566</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -5351,16 +5351,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>34897</v>
+        <v>33608</v>
       </c>
       <c r="I25" t="n">
-        <v>4.2</v>
+        <v>-3.4</v>
       </c>
       <c r="J25" t="n">
-        <v>-6</v>
+        <v>-7.5</v>
       </c>
       <c r="K25" t="n">
-        <v>14642</v>
+        <v>14515</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -5410,16 +5410,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>44263</v>
+        <v>61709</v>
       </c>
       <c r="I26" t="n">
-        <v>67.59999999999999</v>
+        <v>38.5</v>
       </c>
       <c r="J26" t="n">
-        <v>696</v>
+        <v>1009.7</v>
       </c>
       <c r="K26" t="n">
-        <v>20848</v>
+        <v>24643</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -5469,16 +5469,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>136290601</v>
+        <v>135646705</v>
       </c>
       <c r="I27" t="n">
-        <v>0.9</v>
+        <v>-0.5</v>
       </c>
       <c r="J27" t="n">
-        <v>-2.1</v>
+        <v>2</v>
       </c>
       <c r="K27" t="n">
-        <v>2293520</v>
+        <v>2287511</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -5528,16 +5528,16 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>364211870</v>
+        <v>364126880</v>
       </c>
       <c r="I28" t="n">
-        <v>-0.4</v>
+        <v>-0.7</v>
       </c>
       <c r="J28" t="n">
-        <v>-0.7</v>
+        <v>-2.6</v>
       </c>
       <c r="K28" t="n">
-        <v>11151428</v>
+        <v>11102512</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -5587,16 +5587,16 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>531572630</v>
+        <v>530188510</v>
       </c>
       <c r="I29" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>-9.800000000000001</v>
+        <v>-8.9</v>
       </c>
       <c r="K29" t="n">
-        <v>8301640</v>
+        <v>8284858</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -5646,16 +5646,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>43217391</v>
+        <v>45160785</v>
       </c>
       <c r="I30" t="n">
-        <v>1.5</v>
+        <v>5.3</v>
       </c>
       <c r="J30" t="n">
-        <v>6.6</v>
+        <v>9.9</v>
       </c>
       <c r="K30" t="n">
-        <v>2059927</v>
+        <v>2105268</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -5705,16 +5705,16 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>296531</v>
+        <v>284595</v>
       </c>
       <c r="I31" t="n">
-        <v>-11.9</v>
+        <v>-13.2</v>
       </c>
       <c r="J31" t="n">
-        <v>14.2</v>
+        <v>31.6</v>
       </c>
       <c r="K31" t="n">
-        <v>54170</v>
+        <v>53023</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -5764,16 +5764,16 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>54142</v>
+        <v>59268</v>
       </c>
       <c r="I32" t="n">
-        <v>-33.6</v>
+        <v>-1.4</v>
       </c>
       <c r="J32" t="n">
-        <v>13.5</v>
+        <v>50.6</v>
       </c>
       <c r="K32" t="n">
-        <v>23254</v>
+        <v>24309</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -5823,16 +5823,16 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>73619</v>
+        <v>74383</v>
       </c>
       <c r="I33" t="n">
-        <v>-7.6</v>
+        <v>1.5</v>
       </c>
       <c r="J33" t="n">
-        <v>27.3</v>
+        <v>4.8</v>
       </c>
       <c r="K33" t="n">
-        <v>26122</v>
+        <v>26354</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -5882,16 +5882,16 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>76175631</v>
+        <v>75721607</v>
       </c>
       <c r="I34" t="n">
-        <v>1</v>
+        <v>-0.3</v>
       </c>
       <c r="J34" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="K34" t="n">
-        <v>535038</v>
+        <v>521235</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -5941,16 +5941,16 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>230996</v>
+        <v>235511</v>
       </c>
       <c r="I35" t="n">
-        <v>-14.5</v>
+        <v>-3.7</v>
       </c>
       <c r="J35" t="n">
-        <v>-53.8</v>
+        <v>-49.5</v>
       </c>
       <c r="K35" t="n">
-        <v>57317</v>
+        <v>57168</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -6000,16 +6000,16 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>111543</v>
+        <v>109806</v>
       </c>
       <c r="I36" t="n">
-        <v>-3.9</v>
+        <v>-4.2</v>
       </c>
       <c r="J36" t="n">
-        <v>-42.5</v>
+        <v>-40.4</v>
       </c>
       <c r="K36" t="n">
-        <v>27979</v>
+        <v>27866</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -6059,16 +6059,16 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>129935</v>
+        <v>80788</v>
       </c>
       <c r="I37" t="n">
-        <v>1.9</v>
+        <v>-36.4</v>
       </c>
       <c r="J37" t="n">
-        <v>-55.4</v>
+        <v>-77.40000000000001</v>
       </c>
       <c r="K37" t="n">
-        <v>34524</v>
+        <v>26490</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -6118,16 +6118,16 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>64538</v>
+        <v>43177</v>
       </c>
       <c r="I38" t="n">
-        <v>-6.1</v>
+        <v>-32.9</v>
       </c>
       <c r="J38" t="n">
-        <v>289.4</v>
+        <v>104.3</v>
       </c>
       <c r="K38" t="n">
-        <v>20589</v>
+        <v>16366</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -6177,16 +6177,16 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>1902833</v>
+        <v>1815532</v>
       </c>
       <c r="I39" t="n">
-        <v>10.1</v>
+        <v>-3.2</v>
       </c>
       <c r="J39" t="n">
-        <v>-21.5</v>
+        <v>-25.5</v>
       </c>
       <c r="K39" t="n">
-        <v>588011</v>
+        <v>573098</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -6236,16 +6236,16 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>127175</v>
+        <v>114933</v>
       </c>
       <c r="I40" t="n">
-        <v>-13.7</v>
+        <v>-17.1</v>
       </c>
       <c r="J40" t="n">
-        <v>29</v>
+        <v>53.6</v>
       </c>
       <c r="K40" t="n">
-        <v>32524</v>
+        <v>30961</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -6295,16 +6295,16 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>342519266</v>
+        <v>349811058</v>
       </c>
       <c r="I41" t="n">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
       <c r="J41" t="n">
-        <v>115</v>
+        <v>112.5</v>
       </c>
       <c r="K41" t="n">
-        <v>1610725</v>
+        <v>1623428</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -6354,16 +6354,16 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>20215</v>
+        <v>20213</v>
       </c>
       <c r="I42" t="n">
-        <v>0.2</v>
+        <v>-0.2</v>
       </c>
       <c r="J42" t="n">
         <v>-94.7</v>
       </c>
       <c r="K42" t="n">
-        <v>12161</v>
+        <v>12132</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
radar 10/14 08:20 去除虚高市值盘
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -3938,7 +3938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6411,7 +6411,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>J62sjKAAk16afQssxNJS8G2RU9azmCip6VPjMcNcpump</t>
+          <t>GkgVK2duAV9Rjbt43prMiZscuMVQ9XR1RihSYsT6tjjE</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -6420,82 +6420,23 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>403929620</v>
+        <v>21516</v>
       </c>
       <c r="I42" t="n">
-        <v>2.3</v>
+        <v>1.9</v>
       </c>
       <c r="J42" t="n">
-        <v>101.6</v>
+        <v>-95.40000000000001</v>
       </c>
       <c r="K42" t="n">
-        <v>1742056</v>
+        <v>12495</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>GMGN 显示市值约 $3.5 亿，但流动性只有约 $160 万、持有人约 2700、24h 成交约 $50 万，市值是流动性的 200 多倍，属于账面虚高，不代表真实热度。与泄露者无已核实关联，勿当龙头。</t>
+          <t>🆕 GMGN 自动发现：CyberLeek（10/13 07:40 悉尼上线），名字命中「GTA」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
-        <is>
-          <t>https://gmgn.ai/sol/token/J62sjKAAk16afQssxNJS8G2RU9azmCip6VPjMcNcpump</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>大周期</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>beta</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>CYBERLEEK</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>sol</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>GkgVK2duAV9Rjbt43prMiZscuMVQ9XR1RihSYsT6tjjE</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>alive</t>
-        </is>
-      </c>
-      <c r="H43" t="n">
-        <v>21516</v>
-      </c>
-      <c r="I43" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="J43" t="n">
-        <v>-95.40000000000001</v>
-      </c>
-      <c r="K43" t="n">
-        <v>12495</v>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>🆕 GMGN 自动发现：CyberLeek（10/13 07:40 悉尼上线），名字命中「GTA」关键词；叙事待人工核实。</t>
-        </is>
-      </c>
-      <c r="M43" s="2" t="inlineStr">
         <is>
           <t>https://gmgn.ai/sol/token/GkgVK2duAV9Rjbt43prMiZscuMVQ9XR1RihSYsT6tjjE</t>
         </is>
@@ -6544,7 +6485,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
radar silent 10/14 11:55
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -3938,7 +3938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4060,16 +4060,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>119619</v>
+        <v>122244</v>
       </c>
       <c r="I2" t="n">
-        <v>-16.8</v>
+        <v>-7.1</v>
       </c>
       <c r="J2" t="n">
-        <v>2986.3</v>
+        <v>3054</v>
       </c>
       <c r="K2" t="n">
-        <v>35217</v>
+        <v>35531</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -4122,7 +4122,7 @@
         <v>56034</v>
       </c>
       <c r="I3" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
         <v>0.7</v>
@@ -4178,16 +4178,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>119619</v>
+        <v>122244</v>
       </c>
       <c r="I4" t="n">
-        <v>-16.8</v>
+        <v>-7.1</v>
       </c>
       <c r="J4" t="n">
-        <v>2986.3</v>
+        <v>3054</v>
       </c>
       <c r="K4" t="n">
-        <v>35217</v>
+        <v>35531</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -4203,32 +4203,32 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>超级智能 SI · 🦉猫头鹰</t>
+          <t>Binancians · 币安人身份梗</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>大周期</t>
+          <t>24小时</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>binancians</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>DEW9dSN6QpWyNthphCpMmAbZP1Q4cEKR9xQXAri98WDP</t>
+          <t>0x95315e9a9382c0b41a2d69a7afd78d0e24577777</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -4237,25 +4237,25 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>14466111</v>
+        <v>123332</v>
       </c>
       <c r="I5" t="n">
-        <v>0.3</v>
+        <v>435</v>
       </c>
       <c r="J5" t="n">
-        <v>-16.6</v>
+        <v>435</v>
       </c>
       <c r="K5" t="n">
-        <v>718883</v>
+        <v>21396</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Super Inu：马斯克“SI 超级智能”梗龙头，ATH ~$69M，现在 ~$25M 横盘。</t>
+          <t>🆕 GMGN 自动发现：binancians（10/14 11:51 悉尼上线），名字命中「Binancians」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/DEW9dSN6QpWyNthphCpMmAbZP1Q4cEKR9xQXAri98WDP</t>
+          <t>https://gmgn.ai/bsc/token/0x95315e9a9382c0b41a2d69a7afd78d0e24577777</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -4287,7 +4287,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>9aqmJjCnnMQv42TXLk921ceUkN35nea2QP969n1caqjj</t>
+          <t>DEW9dSN6QpWyNthphCpMmAbZP1Q4cEKR9xQXAri98WDP</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -4296,25 +4296,25 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1215403</v>
+        <v>14653231</v>
       </c>
       <c r="I6" t="n">
-        <v>-7.7</v>
+        <v>0.4</v>
       </c>
       <c r="J6" t="n">
-        <v>-6.6</v>
+        <v>-15.5</v>
       </c>
       <c r="K6" t="n">
-        <v>154191</v>
+        <v>724701</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Super Intelligence：同名二号 SI，9/30 上线，百万级市值。</t>
+          <t>Super Inu：马斯克“SI 超级智能”梗龙头，ATH ~$69M，现在 ~$25M 横盘。</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/9aqmJjCnnMQv42TXLk921ceUkN35nea2QP969n1caqjj</t>
+          <t>https://gmgn.ai/sol/token/DEW9dSN6QpWyNthphCpMmAbZP1Q4cEKR9xQXAri98WDP</t>
         </is>
       </c>
     </row>
@@ -4336,7 +4336,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>OWL</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -4346,7 +4346,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>68AGsjomsgTtiTaDhF6XGCeVJDnFeh415ngYYgVxGzns</t>
+          <t>9aqmJjCnnMQv42TXLk921ceUkN35nea2QP969n1caqjj</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4355,25 +4355,25 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>576707</v>
+        <v>1169288</v>
       </c>
       <c r="I7" t="n">
-        <v>9.699999999999999</v>
+        <v>-12.7</v>
       </c>
       <c r="J7" t="n">
-        <v>-7</v>
+        <v>-10.1</v>
       </c>
       <c r="K7" t="n">
-        <v>88078</v>
+        <v>151049</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Superintelligence Owl：马斯克“It always was”猫头鹰封面吉祥物盘，24h 反弹 +170%。</t>
+          <t>Super Intelligence：同名二号 SI，9/30 上线，百万级市值。</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/68AGsjomsgTtiTaDhF6XGCeVJDnFeh415ngYYgVxGzns</t>
+          <t>https://gmgn.ai/sol/token/9aqmJjCnnMQv42TXLk921ceUkN35nea2QP969n1caqjj</t>
         </is>
       </c>
     </row>
@@ -4395,7 +4395,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>OWL</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -4405,7 +4405,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Ap7R5jTGxFCZEbkFc3WNMiN3ru6nkPkn3Co5p6tbpump</t>
+          <t>68AGsjomsgTtiTaDhF6XGCeVJDnFeh415ngYYgVxGzns</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -4414,25 +4414,25 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>13216</v>
+        <v>606001</v>
       </c>
       <c r="I8" t="n">
-        <v>5.7</v>
+        <v>10.3</v>
       </c>
       <c r="J8" t="n">
-        <v>-33.4</v>
+        <v>-2.3</v>
       </c>
       <c r="K8" t="n">
-        <v>10627</v>
+        <v>90768</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Superintelligence（2024 老盘复活）：小市值同名盘，流动性薄。</t>
+          <t>Superintelligence Owl：马斯克“It always was”猫头鹰封面吉祥物盘，24h 反弹 +170%。</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/Ap7R5jTGxFCZEbkFc3WNMiN3ru6nkPkn3Co5p6tbpump</t>
+          <t>https://gmgn.ai/sol/token/68AGsjomsgTtiTaDhF6XGCeVJDnFeh415ngYYgVxGzns</t>
         </is>
       </c>
     </row>
@@ -4454,7 +4454,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>SI276</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>HMYd9tosnUXuNHmq7pXmoePRVBLBBjA3JBfydq6upump</t>
+          <t>Ap7R5jTGxFCZEbkFc3WNMiN3ru6nkPkn3Co5p6tbpump</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -4473,25 +4473,25 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>816006</v>
+        <v>13926</v>
       </c>
       <c r="I9" t="n">
-        <v>-4.1</v>
+        <v>11.4</v>
       </c>
       <c r="J9" t="n">
-        <v>-1</v>
+        <v>-29.8</v>
       </c>
       <c r="K9" t="n">
-        <v>88696</v>
+        <v>10687</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Super Intelligence SI276：GMGN 自动发现的新 SI 同名盘（&lt;72h），~$1.8M，叙事待人工核实。</t>
+          <t>Superintelligence（2024 老盘复活）：小市值同名盘，流动性薄。</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/HMYd9tosnUXuNHmq7pXmoePRVBLBBjA3JBfydq6upump</t>
+          <t>https://gmgn.ai/sol/token/Ap7R5jTGxFCZEbkFc3WNMiN3ru6nkPkn3Co5p6tbpump</t>
         </is>
       </c>
     </row>
@@ -4513,17 +4513,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>TeslaSI</t>
+          <t>SI276</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>bsc</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0xaf3c2e121372eaf5458b827abe21393665d97777</t>
+          <t>HMYd9tosnUXuNHmq7pXmoePRVBLBBjA3JBfydq6upump</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -4532,25 +4532,25 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>20664</v>
+        <v>829214</v>
       </c>
       <c r="I10" t="n">
-        <v>40.6</v>
+        <v>-8.1</v>
       </c>
       <c r="J10" t="n">
-        <v>-22.6</v>
+        <v>0.6</v>
       </c>
       <c r="K10" t="n">
-        <v>15066</v>
+        <v>88715</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Tesla Super Intelligence（10/11 19:35 悉尼上线），名字命中「超级智能」关键词；叙事待人工核实。</t>
+          <t>Super Intelligence SI276：GMGN 自动发现的新 SI 同名盘（&lt;72h），~$1.8M，叙事待人工核实。</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0xaf3c2e121372eaf5458b827abe21393665d97777</t>
+          <t>https://gmgn.ai/sol/token/HMYd9tosnUXuNHmq7pXmoePRVBLBBjA3JBfydq6upump</t>
         </is>
       </c>
     </row>
@@ -4572,7 +4572,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>XSI</t>
+          <t>TeslaSI</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -4582,7 +4582,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0xf824ffa5ba5ee03caf560b6e5b2218ccb7517777</t>
+          <t>0xaf3c2e121372eaf5458b827abe21393665d97777</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4591,32 +4591,32 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>37446</v>
+        <v>19354</v>
       </c>
       <c r="I11" t="n">
-        <v>-70.40000000000001</v>
+        <v>31.9</v>
       </c>
       <c r="J11" t="n">
-        <v>145.8</v>
+        <v>-27.5</v>
       </c>
       <c r="K11" t="n">
-        <v>20764</v>
+        <v>14594</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：推特超级智能 X Super Intelligence（10/13 21:18 悉尼上线），名字命中「超级智能」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：Tesla Super Intelligence（10/11 19:35 悉尼上线），名字命中「超级智能」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0xf824ffa5ba5ee03caf560b6e5b2218ccb7517777</t>
+          <t>https://gmgn.ai/bsc/token/0xaf3c2e121372eaf5458b827abe21393665d97777</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>量子 / AI 破解私钥</t>
+          <t>超级智能 SI · 🦉猫头鹰</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4626,22 +4626,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>QI</t>
+          <t>XSI</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>8TiMkgvsrat9tM2esko8zVTt99LZLpefUM4SnZaziXaQ</t>
+          <t>0xf824ffa5ba5ee03caf560b6e5b2218ccb7517777</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4650,25 +4650,25 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>547652</v>
+        <v>32504</v>
       </c>
       <c r="I12" t="n">
-        <v>3.1</v>
+        <v>-66.5</v>
       </c>
       <c r="J12" t="n">
-        <v>-48.8</v>
+        <v>113.3</v>
       </c>
       <c r="K12" t="n">
-        <v>83740</v>
+        <v>19447</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Quantum Inu：10/09 新盘，量子狗，量子赛道当前市值最大的纯 meme，24h 涨幅上万 %。</t>
+          <t>🆕 GMGN 自动发现：推特超级智能 X Super Intelligence（10/13 21:18 悉尼上线），名字命中「超级智能」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/8TiMkgvsrat9tM2esko8zVTt99LZLpefUM4SnZaziXaQ</t>
+          <t>https://gmgn.ai/bsc/token/0xf824ffa5ba5ee03caf560b6e5b2218ccb7517777</t>
         </is>
       </c>
     </row>
@@ -4685,12 +4685,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>QCAT</t>
+          <t>QI</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -4700,7 +4700,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>7vMkPxLwaH26qSZ2CgHhzvrgz9wUWMvT256vbUWfarm</t>
+          <t>8TiMkgvsrat9tM2esko8zVTt99LZLpefUM4SnZaziXaQ</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4709,25 +4709,25 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>51796</v>
+        <v>547192</v>
       </c>
       <c r="I13" t="n">
-        <v>4.9</v>
+        <v>2.6</v>
       </c>
       <c r="J13" t="n">
-        <v>18.4</v>
+        <v>-48.8</v>
       </c>
       <c r="K13" t="n">
-        <v>28856</v>
+        <v>82792</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Quantum Cat（10/10 02:08 悉尼上线），名字命中「量子」关键词；叙事待人工核实。</t>
+          <t>Quantum Inu：10/09 新盘，量子狗，量子赛道当前市值最大的纯 meme，24h 涨幅上万 %。</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/7vMkPxLwaH26qSZ2CgHhzvrgz9wUWMvT256vbUWfarm</t>
+          <t>https://gmgn.ai/sol/token/8TiMkgvsrat9tM2esko8zVTt99LZLpefUM4SnZaziXaQ</t>
         </is>
       </c>
     </row>
@@ -4749,7 +4749,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>QI</t>
+          <t>QCAT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -4759,7 +4759,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>eFBwUbyopvmxYHEwXZRbsTkSJHsz7WqawqKMxbqpump</t>
+          <t>7vMkPxLwaH26qSZ2CgHhzvrgz9wUWMvT256vbUWfarm</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -4768,32 +4768,32 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>4403500</v>
+        <v>49324</v>
       </c>
       <c r="I14" t="n">
-        <v>1.5</v>
+        <v>-7</v>
       </c>
       <c r="J14" t="n">
-        <v>26.9</v>
+        <v>12.7</v>
       </c>
       <c r="K14" t="n">
-        <v>180633</v>
+        <v>28142</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Quantum Inu（10/10 21:41 悉尼上线），名字命中「量子」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：Quantum Cat（10/10 02:08 悉尼上线），名字命中「量子」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/eFBwUbyopvmxYHEwXZRbsTkSJHsz7WqawqKMxbqpump</t>
+          <t>https://gmgn.ai/sol/token/7vMkPxLwaH26qSZ2CgHhzvrgz9wUWMvT256vbUWfarm</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Grok Bot · 整家公司由 AI 组成</t>
+          <t>量子 / AI 破解私钥</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -4803,22 +4803,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Grok Bot</t>
+          <t>QI</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>bsc</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0x7aede49f29bf7bc643853c1136854ea8e4da7777</t>
+          <t>eFBwUbyopvmxYHEwXZRbsTkSJHsz7WqawqKMxbqpump</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -4827,32 +4827,32 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>39235</v>
+        <v>4371450</v>
       </c>
       <c r="I15" t="n">
-        <v>-8.699999999999999</v>
+        <v>0.7</v>
       </c>
       <c r="J15" t="n">
-        <v>-68.8</v>
+        <v>26</v>
       </c>
       <c r="K15" t="n">
-        <v>21526</v>
+        <v>180549</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：AI Agent（10/12 11:45 悉尼上线），名字命中「Grok」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：Quantum Inu（10/10 21:41 悉尼上线），名字命中「量子」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x7aede49f29bf7bc643853c1136854ea8e4da7777</t>
+          <t>https://gmgn.ai/sol/token/eFBwUbyopvmxYHEwXZRbsTkSJHsz7WqawqKMxbqpump</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>股票 meme · 代币化美股</t>
+          <t>Grok Bot · 整家公司由 AI 组成</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -4867,17 +4867,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>PONS</t>
+          <t>Grok Bot</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>robinhood</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0x39dbed3a2bd333467115de45665cc57f813c4571</t>
+          <t>0x7aede49f29bf7bc643853c1136854ea8e4da7777</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -4886,25 +4886,25 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>308451550</v>
+        <v>39673</v>
       </c>
       <c r="I16" t="n">
-        <v>1.9</v>
+        <v>-8.1</v>
       </c>
       <c r="J16" t="n">
-        <v>10.3</v>
+        <v>-68.40000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>2936861</v>
+        <v>21620</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Robinhood Chain 发射台币 Pons：10 万持有人，股票链 meme 的庄家盘。</t>
+          <t>🆕 GMGN 自动发现：AI Agent（10/12 11:45 悉尼上线），名字命中「Grok」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/robinhood/token/0x39dbed3a2bd333467115de45665cc57f813c4571</t>
+          <t>https://gmgn.ai/bsc/token/0x7aede49f29bf7bc643853c1136854ea8e4da7777</t>
         </is>
       </c>
     </row>
@@ -4921,22 +4921,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>BLUECHIP</t>
+          <t>PONS</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>robinhood</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0xb200000000000000000000cfbdf64a8706a94a01</t>
+          <t>0x39dbed3a2bd333467115de45665cc57f813c4571</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -4945,25 +4945,25 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>6050908</v>
+        <v>305599400</v>
       </c>
       <c r="I17" t="n">
-        <v>-2.4</v>
+        <v>1.2</v>
       </c>
       <c r="J17" t="n">
-        <v>-2.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="K17" t="n">
-        <v>311948</v>
+        <v>2929249</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Base 股票 meme：Jesse Pollak Token2049 幻灯片点名。</t>
+          <t>Robinhood Chain 发射台币 Pons：10 万持有人，股票链 meme 的庄家盘。</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/base/token/0xb200000000000000000000cfbdf64a8706a94a01</t>
+          <t>https://gmgn.ai/robinhood/token/0x39dbed3a2bd333467115de45665cc57f813c4571</t>
         </is>
       </c>
     </row>
@@ -4985,7 +4985,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>IPOD</t>
+          <t>BLUECHIP</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -4995,7 +4995,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0xa6af0cea8fbc93e1eccc00f1fdd9a0bba251fee1</t>
+          <t>0xb200000000000000000000cfbdf64a8706a94a01</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -5004,25 +5004,25 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>1097708</v>
+        <v>6112618</v>
       </c>
       <c r="I18" t="n">
-        <v>0.8</v>
+        <v>-0.8</v>
       </c>
       <c r="J18" t="n">
-        <v>-8.300000000000001</v>
+        <v>-1.2</v>
       </c>
       <c r="K18" t="n">
-        <v>261256</v>
+        <v>311948</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Base 苹果股票梗 iPod，Jesse 幻灯片点名。</t>
+          <t>Base 股票 meme：Jesse Pollak Token2049 幻灯片点名。</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/base/token/0xa6af0cea8fbc93e1eccc00f1fdd9a0bba251fee1</t>
+          <t>https://gmgn.ai/base/token/0xb200000000000000000000cfbdf64a8706a94a01</t>
         </is>
       </c>
     </row>
@@ -5044,7 +5044,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>DGUY</t>
+          <t>IPOD</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -5054,7 +5054,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0xe34356dcd3d7bb991248f322e4ec31b5d60bc54e</t>
+          <t>0xa6af0cea8fbc93e1eccc00f1fdd9a0bba251fee1</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -5063,25 +5063,25 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>1043136</v>
+        <v>1097708</v>
       </c>
       <c r="I19" t="n">
-        <v>-1.8</v>
+        <v>0.8</v>
       </c>
       <c r="J19" t="n">
-        <v>21.1</v>
+        <v>-8.300000000000001</v>
       </c>
       <c r="K19" t="n">
-        <v>121303</v>
+        <v>261256</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Delivery Guy：Base 股票 meme，Jesse 幻灯片点名。</t>
+          <t>Base 苹果股票梗 iPod，Jesse 幻灯片点名。</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/base/token/0xe34356dcd3d7bb991248f322e4ec31b5d60bc54e</t>
+          <t>https://gmgn.ai/base/token/0xa6af0cea8fbc93e1eccc00f1fdd9a0bba251fee1</t>
         </is>
       </c>
     </row>
@@ -5103,7 +5103,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>TEMU</t>
+          <t>DGUY</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -5113,7 +5113,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0x3c573bdd88008c94f025e5023212f28e5f39744c</t>
+          <t>0xe34356dcd3d7bb991248f322e4ec31b5d60bc54e</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -5122,32 +5122,32 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>282832</v>
+        <v>1043230</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.8</v>
+        <v>-0.6</v>
       </c>
       <c r="J20" t="n">
-        <v>5.4</v>
+        <v>21.1</v>
       </c>
       <c r="K20" t="n">
-        <v>57154</v>
+        <v>121236</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>TEMU on Base：Jesse 幻灯片点名的拼多多梗。</t>
+          <t>Delivery Guy：Base 股票 meme，Jesse 幻灯片点名。</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/base/token/0x3c573bdd88008c94f025e5023212f28e5f39744c</t>
+          <t>https://gmgn.ai/base/token/0xe34356dcd3d7bb991248f322e4ec31b5d60bc54e</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>持币分红盘 · ZCAT/BATON</t>
+          <t>股票 meme · 代币化美股</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -5157,22 +5157,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ZCAT</t>
+          <t>TEMU</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>base</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
+          <t>0x3c573bdd88008c94f025e5023212f28e5f39744c</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -5181,25 +5181,25 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>54223370</v>
+        <v>282832</v>
       </c>
       <c r="I21" t="n">
-        <v>9.4</v>
+        <v>-0.8</v>
       </c>
       <c r="J21" t="n">
-        <v>41.7</v>
+        <v>5.4</v>
       </c>
       <c r="K21" t="n">
-        <v>1243181</v>
+        <v>57154</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Anonymous Cat：3% 交易税自动换 ZEC 分红给持有人，分红盘龙头。</t>
+          <t>TEMU on Base：Jesse 幻灯片点名的拼多多梗。</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
+          <t>https://gmgn.ai/base/token/0x3c573bdd88008c94f025e5023212f28e5f39744c</t>
         </is>
       </c>
     </row>
@@ -5216,12 +5216,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>BATON</t>
+          <t>ZCAT</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -5231,7 +5231,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
+          <t>HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -5240,25 +5240,25 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>12310074</v>
+        <v>52437717</v>
       </c>
       <c r="I22" t="n">
-        <v>3</v>
+        <v>2.4</v>
       </c>
       <c r="J22" t="n">
-        <v>-7.7</v>
+        <v>37.1</v>
       </c>
       <c r="K22" t="n">
-        <v>708772</v>
+        <v>1241039</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>baton：分红 PUMP 的分红盘，ATH ~$19M，回调后第二腿。</t>
+          <t>Anonymous Cat：3% 交易税自动换 ZEC 分红给持有人，分红盘龙头。</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
+          <t>https://gmgn.ai/sol/token/HcRLc9VDgjLeK154xDawfb1dmVJ98DoSqcwTHGqiDeJR</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>MCAT</t>
+          <t>BATON</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -5290,7 +5290,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
+          <t>Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -5299,25 +5299,25 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>159393</v>
+        <v>12459059</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>-1.2</v>
       </c>
       <c r="J23" t="n">
-        <v>-2.1</v>
+        <v>-6.6</v>
       </c>
       <c r="K23" t="n">
-        <v>36761</v>
+        <v>705709</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Addicted Cat：分红门罗币 XMR，Cake Wallet 创始人买入。</t>
+          <t>baton：分红 PUMP 的分红盘，ATH ~$19M，回调后第二腿。</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
+          <t>https://gmgn.ai/sol/token/Hg5Ja55T5wESq4vyFoiVCMeHXtGyVA69X2UHq8hgpump</t>
         </is>
       </c>
     </row>
@@ -5339,7 +5339,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>FACTORY</t>
+          <t>MCAT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -5349,7 +5349,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>7536qC4LEs3W2GtSKbhVGNJSiRfuXJhKVthxsgfkpump</t>
+          <t>H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -5358,25 +5358,25 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>25786</v>
+        <v>142159</v>
       </c>
       <c r="I24" t="n">
-        <v>0.3</v>
+        <v>-6</v>
       </c>
       <c r="J24" t="n">
-        <v>-31.6</v>
+        <v>-12.7</v>
       </c>
       <c r="K24" t="n">
-        <v>12159</v>
+        <v>35787</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Baton Factory（10/10 22:26 悉尼上线），名字命中「持币分红盘」关键词；叙事待人工核实。</t>
+          <t>Addicted Cat：分红门罗币 XMR，Cake Wallet 创始人买入。</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/7536qC4LEs3W2GtSKbhVGNJSiRfuXJhKVthxsgfkpump</t>
+          <t>https://gmgn.ai/sol/token/H9pPKejchJ9LCWpb1P8p4BmrjzCFARUmA7XtJK4pVhCZ</t>
         </is>
       </c>
     </row>
@@ -5398,17 +5398,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>上等羊</t>
+          <t>FACTORY</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>bsc</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0x26c4829616644144b1dcec6c6c62828c9a717777</t>
+          <t>7536qC4LEs3W2GtSKbhVGNJSiRfuXJhKVthxsgfkpump</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -5417,25 +5417,25 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>103149</v>
+        <v>25786</v>
       </c>
       <c r="I25" t="n">
-        <v>51.3</v>
+        <v>0.3</v>
       </c>
       <c r="J25" t="n">
-        <v>1754.9</v>
+        <v>-31.6</v>
       </c>
       <c r="K25" t="n">
-        <v>31991</v>
+        <v>12159</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：首创锁仓拖底回购分红协议（10/13 19:17 悉尼上线），名字命中「持币分红盘」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：Baton Factory（10/10 22:26 悉尼上线），名字命中「持币分红盘」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x26c4829616644144b1dcec6c6c62828c9a717777</t>
+          <t>https://gmgn.ai/sol/token/7536qC4LEs3W2GtSKbhVGNJSiRfuXJhKVthxsgfkpump</t>
         </is>
       </c>
     </row>
@@ -5457,7 +5457,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>币安借呗</t>
+          <t>上等羊</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -5467,7 +5467,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0x423f80ae38830ea6438bcdd38b64d7bb3ae97777</t>
+          <t>0x26c4829616644144b1dcec6c6c62828c9a717777</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -5476,32 +5476,32 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>61614</v>
+        <v>94626</v>
       </c>
       <c r="I26" t="n">
-        <v>2.9</v>
+        <v>36.8</v>
       </c>
       <c r="J26" t="n">
-        <v>1195.6</v>
+        <v>1601.7</v>
       </c>
       <c r="K26" t="n">
-        <v>24619</v>
+        <v>30523</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：币安借呗首创首款链上借BNB分红DeFi（10/14 01:32 悉尼上线），名字命中「持币分红盘」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：首创锁仓拖底回购分红协议（10/13 19:17 悉尼上线），名字命中「持币分红盘」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x423f80ae38830ea6438bcdd38b64d7bb3ae97777</t>
+          <t>https://gmgn.ai/bsc/token/0x26c4829616644144b1dcec6c6c62828c9a717777</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ANSEM · SOL 老龙头</t>
+          <t>持币分红盘 · ZCAT/BATON</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5511,22 +5511,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>ANSEM</t>
+          <t>币安借呗</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
+          <t>0x423f80ae38830ea6438bcdd38b64d7bb3ae97777</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -5535,32 +5535,32 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>133997786</v>
+        <v>63563</v>
       </c>
       <c r="I27" t="n">
-        <v>1</v>
+        <v>9.1</v>
       </c>
       <c r="J27" t="n">
-        <v>2.4</v>
+        <v>1236.6</v>
       </c>
       <c r="K27" t="n">
-        <v>2275320</v>
+        <v>24953</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>The Black Bull：Ansem 本人梗的 SOL 老龙头，15 万持有人，前十持仓 ~65% 偏集中。</t>
+          <t>🆕 GMGN 自动发现：币安借呗首创首款链上借BNB分红DeFi（10/14 01:32 悉尼上线），名字命中「持币分红盘」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
+          <t>https://gmgn.ai/bsc/token/0x423f80ae38830ea6438bcdd38b64d7bb3ae97777</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>以太坊近况 · Glamsterdam</t>
+          <t>ANSEM · SOL 老龙头</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5575,17 +5575,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>ANSEM</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>eth</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
+          <t>9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -5594,32 +5594,32 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>370153140</v>
+        <v>133471379</v>
       </c>
       <c r="I28" t="n">
         <v>1.1</v>
       </c>
       <c r="J28" t="n">
-        <v>5.4</v>
+        <v>2</v>
       </c>
       <c r="K28" t="n">
-        <v>11208663</v>
+        <v>2271540</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SPX6900：Murad 舞台喊“meme 将超越比特币”的 ETH 主网 meme 龙头。</t>
+          <t>The Black Bull：Ansem 本人梗的 SOL 老龙头，15 万持有人，前十持仓 ~65% 偏集中。</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/eth/token/0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
+          <t>https://gmgn.ai/sol/token/9cRCn9rGT8V2imeM2BaKs13yhMEais3ruM3rPvTGpump</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>BSC 中文盘 · 币安人生</t>
+          <t>以太坊近况 · Glamsterdam</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5634,17 +5634,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>币安人生</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>bsc</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
+          <t>0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -5653,25 +5653,25 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>528144330</v>
+        <v>370153140</v>
       </c>
       <c r="I29" t="n">
-        <v>-0.6</v>
+        <v>1.1</v>
       </c>
       <c r="J29" t="n">
-        <v>1.6</v>
+        <v>5.4</v>
       </c>
       <c r="K29" t="n">
-        <v>8272738</v>
+        <v>11208663</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>币安人生：何一推文带火的 BSC 中文 meme 龙头，ATH ~$9 亿，现 ~$5.5 亿。</t>
+          <t>SPX6900：Murad 舞台喊“meme 将超越比特币”的 ETH 主网 meme 龙头。</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
+          <t>https://gmgn.ai/eth/token/0xe0f63a424a4439cbe457d80e4f4b51ad25b2c56c</t>
         </is>
       </c>
     </row>
@@ -5688,12 +5688,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>龙虾</t>
+          <t>币安人生</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -5703,7 +5703,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>0xeccbb861c0dda7efd964010085488b69317e4444</t>
+          <t>0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -5712,25 +5712,25 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>46284529</v>
+        <v>526403310</v>
       </c>
       <c r="I30" t="n">
-        <v>-3.3</v>
+        <v>-1</v>
       </c>
       <c r="J30" t="n">
-        <v>19.6</v>
+        <v>1.3</v>
       </c>
       <c r="K30" t="n">
-        <v>2132938</v>
+        <v>8253935</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>龙虾：币安中文号推文出圈的中文盘，ATH ~$3.1 亿，现 ~$4300 万。注意今天有同名高仿盘。</t>
+          <t>币安人生：何一推文带火的 BSC 中文 meme 龙头，ATH ~$9 亿，现 ~$5.5 亿。</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0xeccbb861c0dda7efd964010085488b69317e4444</t>
+          <t>https://gmgn.ai/bsc/token/0x924fa68a0fc644485b8df8abfa0a41c2e7744444</t>
         </is>
       </c>
     </row>
@@ -5752,7 +5752,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>币安圣羊</t>
+          <t>龙虾</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -5762,7 +5762,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0xcc4cc7ebaab40aa19317027b63e584333f697777</t>
+          <t>0xeccbb861c0dda7efd964010085488b69317e4444</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -5771,25 +5771,25 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>273615</v>
+        <v>46320360</v>
       </c>
       <c r="I31" t="n">
-        <v>1.8</v>
+        <v>-3.6</v>
       </c>
       <c r="J31" t="n">
-        <v>23.9</v>
+        <v>19.7</v>
       </c>
       <c r="K31" t="n">
-        <v>52000</v>
+        <v>2140432</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：币安圣羊（10/10 04:20 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
+          <t>龙虾：币安中文号推文出圈的中文盘，ATH ~$3.1 亿，现 ~$4300 万。注意今天有同名高仿盘。</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0xcc4cc7ebaab40aa19317027b63e584333f697777</t>
+          <t>https://gmgn.ai/bsc/token/0xeccbb861c0dda7efd964010085488b69317e4444</t>
         </is>
       </c>
     </row>
@@ -5811,7 +5811,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>币安人</t>
+          <t>币安圣羊</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -5821,7 +5821,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>0x2c2d4298548ae585c224714555f18abde7367777</t>
+          <t>0xcc4cc7ebaab40aa19317027b63e584333f697777</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -5830,25 +5830,25 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>62204</v>
+        <v>274352</v>
       </c>
       <c r="I32" t="n">
-        <v>-8.199999999999999</v>
+        <v>2.6</v>
       </c>
       <c r="J32" t="n">
-        <v>72</v>
+        <v>24.2</v>
       </c>
       <c r="K32" t="n">
-        <v>24958</v>
+        <v>52052</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Binance Man（10/10 22:33 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：币安圣羊（10/10 04:20 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x2c2d4298548ae585c224714555f18abde7367777</t>
+          <t>https://gmgn.ai/bsc/token/0xcc4cc7ebaab40aa19317027b63e584333f697777</t>
         </is>
       </c>
     </row>
@@ -5870,7 +5870,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Binance Angels</t>
+          <t>币安人</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -5880,7 +5880,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>0x62bb38c83afeb82e8f468d122b1b9051b6167777</t>
+          <t>0x2c2d4298548ae585c224714555f18abde7367777</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -5889,32 +5889,32 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>66860</v>
+        <v>59082</v>
       </c>
       <c r="I33" t="n">
-        <v>-6.5</v>
+        <v>-12.9</v>
       </c>
       <c r="J33" t="n">
-        <v>-61.7</v>
+        <v>63.4</v>
       </c>
       <c r="K33" t="n">
-        <v>25030</v>
+        <v>24311</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：QQ:945497833（10/12 19:12 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
+          <t>🆕 GMGN 自动发现：Binance Man（10/10 22:33 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/bsc/token/0x62bb38c83afeb82e8f468d122b1b9051b6167777</t>
+          <t>https://gmgn.ai/bsc/token/0x2c2d4298548ae585c224714555f18abde7367777</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>后量子地堡 · BNKR/PQC</t>
+          <t>BSC 中文盘 · 币安人生</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5924,22 +5924,22 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>PQC</t>
+          <t>Binance Angels</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>bsc</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
+          <t>0x62bb38c83afeb82e8f468d122b1b9051b6167777</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -5948,25 +5948,25 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>151005</v>
+        <v>64822</v>
       </c>
       <c r="I34" t="n">
-        <v>-6.9</v>
+        <v>-4.9</v>
       </c>
       <c r="J34" t="n">
-        <v>-52.9</v>
+        <v>-62.8</v>
       </c>
       <c r="K34" t="n">
-        <v>45685</v>
+        <v>24593</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>pqc.market 平台币：后量子发射台，10/08 上线，24h 成交 ~$7.7M，BNKR 的母盘。</t>
+          <t>🆕 GMGN 自动发现：QQ:945497833（10/12 19:12 悉尼上线），名字命中「BSC」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
+          <t>https://gmgn.ai/bsc/token/0x62bb38c83afeb82e8f468d122b1b9051b6167777</t>
         </is>
       </c>
     </row>
@@ -5983,12 +5983,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>BUNKER</t>
+          <t>PQC</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -5998,7 +5998,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
+          <t>7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -6007,32 +6007,32 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>124809</v>
+        <v>148260</v>
       </c>
       <c r="I35" t="n">
-        <v>38</v>
+        <v>-7.5</v>
       </c>
       <c r="J35" t="n">
-        <v>3.6</v>
+        <v>-53.7</v>
       </c>
       <c r="K35" t="n">
-        <v>30215</v>
+        <v>45350</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：Bunker Mode（10/10 10:14 悉尼上线），名字命中「后量子地堡」关键词；叙事待人工核实。</t>
+          <t>pqc.market 平台币：后量子发射台，10/08 上线，24h 成交 ~$7.7M，BNKR 的母盘。</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
+          <t>https://gmgn.ai/sol/token/7K52aYQW9rWGjwZmQ7o2d1P6E7bji6hSMsqaLy5EcxLh</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Solamians · Solana 官方插画里的“国籍”</t>
+          <t>后量子地堡 · BNKR/PQC</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6042,12 +6042,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>龙头</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Solamians</t>
+          <t>BUNKER</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -6057,7 +6057,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>8ZP5CzbPL1fmP8dn1GEmLd8xw1JdudUF5Dk7EpLxpump</t>
+          <t>BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -6066,32 +6066,32 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>87822</v>
+        <v>127525</v>
       </c>
       <c r="I36" t="n">
-        <v>-8.9</v>
+        <v>41</v>
       </c>
       <c r="J36" t="n">
-        <v>-46.6</v>
+        <v>5.9</v>
       </c>
       <c r="K36" t="n">
-        <v>27771</v>
+        <v>30227</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Solana 官方 Breakpoint 指南护照插画写着 Nationality: Solamian（已核实原图）。10/12 13:09 创建，ATH ~$910K，机器人成交约 57%。</t>
+          <t>🆕 GMGN 自动发现：Bunker Mode（10/10 10:14 悉尼上线），名字命中「后量子地堡」关键词；叙事待人工核实。</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/8ZP5CzbPL1fmP8dn1GEmLd8xw1JdudUF5Dk7EpLxpump</t>
+          <t>https://gmgn.ai/sol/token/BunkeRhcyfJ7dXXNA3kDi421tLijrqudb9ARytKrVbFa</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
+          <t>Solamians · Solana 官方插画里的“国籍”</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6106,7 +6106,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>CAESAR</t>
+          <t>Solamians</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -6116,7 +6116,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
+          <t>8ZP5CzbPL1fmP8dn1GEmLd8xw1JdudUF5Dk7EpLxpump</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -6125,32 +6125,32 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>33053</v>
+        <v>91474</v>
       </c>
       <c r="I37" t="n">
-        <v>-1.9</v>
+        <v>8.4</v>
       </c>
       <c r="J37" t="n">
-        <v>364.5</v>
+        <v>-44.4</v>
       </c>
       <c r="K37" t="n">
-        <v>13822</v>
+        <v>28203</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>pmarca 转发的《Slop Caesar》社区盘。19:24 Devon 本人贴出此 CA，自称已领约 108 SOL 手续费（GMGN：分成 100% 给 devonmvfisher，已领取）。原开发者已清仓、批量发币地址；机器人约 62%。</t>
+          <t>Solana 官方 Breakpoint 指南护照插画写着 Nationality: Solamian（已核实原图）。10/12 13:09 创建，ATH ~$910K，机器人成交约 57%。</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
+          <t>https://gmgn.ai/sol/token/8ZP5CzbPL1fmP8dn1GEmLd8xw1JdudUF5Dk7EpLxpump</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+          <t>Slop Caesar · 马克·安德森转发的 AI 虾皇帝</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>CYBERLEEK</t>
+          <t>CAESAR</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>ApZuxdpzMrbEYTGEzeY9afh5pj9d6qPRJCTgQYiipbKg</t>
+          <t>EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -6184,25 +6184,25 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>1944639</v>
+        <v>33269</v>
       </c>
       <c r="I38" t="n">
-        <v>-2.4</v>
+        <v>-5.4</v>
       </c>
       <c r="J38" t="n">
-        <v>1.8</v>
+        <v>367.5</v>
       </c>
       <c r="K38" t="n">
-        <v>595721</v>
+        <v>13833</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>GTA 6 泄露者的币，10/10 喊出 3000 万市值放完整版。8 月曾提款后崩盘，24h -53%。</t>
+          <t>pmarca 转发的《Slop Caesar》社区盘。19:24 Devon 本人贴出此 CA，自称已领约 108 SOL 手续费（GMGN：分成 100% 给 devonmvfisher，已领取）。原开发者已清仓、批量发币地址；机器人约 62%。</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/ApZuxdpzMrbEYTGEzeY9afh5pj9d6qPRJCTgQYiipbKg</t>
+          <t>https://gmgn.ai/sol/token/EaqXJVr1aFPhMyTJbDCpwvTeiKc8x4gueFjFKKBvtcWY</t>
         </is>
       </c>
     </row>
@@ -6219,12 +6219,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>龙头</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Dacity</t>
+          <t>CYBERLEEK</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -6234,7 +6234,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>nxPqZ4F7ux8Vph5NFu25rEP6Kx9Gr1U6Fmj36Rjpump</t>
+          <t>ApZuxdpzMrbEYTGEzeY9afh5pj9d6qPRJCTgQYiipbKg</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -6243,25 +6243,25 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>119442</v>
+        <v>1889001</v>
       </c>
       <c r="I39" t="n">
-        <v>1.4</v>
+        <v>-0.8</v>
       </c>
       <c r="J39" t="n">
-        <v>-2.8</v>
+        <v>-1.1</v>
       </c>
       <c r="K39" t="n">
-        <v>31297</v>
+        <v>586313</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>据称出现在泄露视频里的游戏内币（未核实），ATH 回撤 88%，机器人多。</t>
+          <t>GTA 6 泄露者的币，10/10 喊出 3000 万市值放完整版。8 月曾提款后崩盘，24h -53%。</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>https://gmgn.ai/sol/token/nxPqZ4F7ux8Vph5NFu25rEP6Kx9Gr1U6Fmj36Rjpump</t>
+          <t>https://gmgn.ai/sol/token/ApZuxdpzMrbEYTGEzeY9afh5pj9d6qPRJCTgQYiipbKg</t>
         </is>
       </c>
     </row>
@@ -6283,42 +6283,101 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
+          <t>Dacity</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>nxPqZ4F7ux8Vph5NFu25rEP6Kx9Gr1U6Fmj36Rjpump</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>120570</v>
+      </c>
+      <c r="I40" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="J40" t="n">
+        <v>-1.9</v>
+      </c>
+      <c r="K40" t="n">
+        <v>31438</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>据称出现在泄露视频里的游戏内币（未核实），ATH 回撤 88%，机器人多。</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/nxPqZ4F7ux8Vph5NFu25rEP6Kx9Gr1U6Fmj36Rjpump</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>GTA 6 泄露者 Cyberleek · 3000 万市值放全作</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>大周期</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
           <t>CYBERLEEK</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>sol</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>GkgVK2duAV9Rjbt43prMiZscuMVQ9XR1RihSYsT6tjjE</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>alive</t>
         </is>
       </c>
-      <c r="H40" t="n">
+      <c r="H41" t="n">
         <v>21503</v>
       </c>
-      <c r="I40" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J40" t="n">
+      <c r="I41" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="J41" t="n">
         <v>-94.90000000000001</v>
       </c>
-      <c r="K40" t="n">
+      <c r="K41" t="n">
         <v>12477</v>
       </c>
-      <c r="L40" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>🆕 GMGN 自动发现：CyberLeek（10/13 07:40 悉尼上线），名字命中「GTA」关键词；叙事待人工核实。</t>
         </is>
       </c>
-      <c r="M40" s="2" t="inlineStr">
+      <c r="M41" s="2" t="inlineStr">
         <is>
           <t>https://gmgn.ai/sol/token/GkgVK2duAV9Rjbt43prMiZscuMVQ9XR1RihSYsT6tjjE</t>
         </is>
@@ -6365,6 +6424,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId40"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
radar 10/14 12:42 embryo unicorn
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2837,6 +2837,90 @@
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr"/>
+      <c r="B93" t="inlineStr"/>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Josie 帖：币圈一直给我打 SOL</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/josiezayner/status/2110175418565238969</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Embryo Corp · 基因编辑造独角兽</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr"/>
+      <c r="B94" t="inlineStr"/>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Josie 转发 People 采访</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/josiezayner/status/2110107308478828560</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Embryo Corp · 基因编辑造独角兽</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr"/>
+      <c r="B95" t="inlineStr"/>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>People 独家</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>https://people.com/former-nasa-scientist-says-unicorn-horn-could-be-5-to-10-years-away-exclusive-12170434</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Embryo Corp · 基因编辑造独角兽</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr"/>
+      <c r="B96" t="inlineStr"/>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>公司官网</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>https://building.life/</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Embryo Corp · 基因编辑造独角兽</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2931,6 +3015,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId95"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2942,7 +3030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R16"/>
+  <dimension ref="A1:S17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2963,6 +3051,7 @@
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3056,6 +3145,11 @@
           <t>10-13 帖数</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>10-14 帖数</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -3114,6 +3208,7 @@
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -3172,6 +3267,7 @@
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -3236,6 +3332,7 @@
         <v>18931</v>
       </c>
       <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -3294,6 +3391,7 @@
         <v>6205</v>
       </c>
       <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -3352,6 +3450,7 @@
         <v>854</v>
       </c>
       <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -3410,6 +3509,7 @@
         <v>424</v>
       </c>
       <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -3468,6 +3568,7 @@
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -3526,6 +3627,7 @@
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -3584,6 +3686,7 @@
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -3642,6 +3745,7 @@
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -3700,6 +3804,7 @@
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -3707,7 +3812,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Binancians · 币安人身份梗</t>
+          <t>Embryo Corp · 基因编辑造独角兽</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3716,21 +3821,21 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>→</t>
+          <t>↑</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>binancians</t>
+          <t>UNICORN</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10/13 23:07 悉尼：同叙事第二腿——中文「币安人」0xDEA1…7777 约 22:33 上线后市值冲到约 $3M+，超过首轮英文 binancians（0x8Dce…7777 ~$0.45M）。@binance 官推原文已核实；币安/CZ 仍未点名任何 CA。同名盘极多、image_dup 高，注意分流与砸盘。</t>
+          <t>事件已核实（官网 building.life + People 独家，创始人本人转发）；创始人 10/14 12:06 悉尼发帖“币圈的人一直在给我打 SOL”但未点名任何 CA，币与她的关联未核实</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -3738,13 +3843,26 @@
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>45</v>
+      </c>
+      <c r="N13" t="n">
+        <v>36</v>
+      </c>
+      <c r="O13" t="n">
+        <v>65</v>
+      </c>
+      <c r="P13" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>75</v>
+      </c>
       <c r="R13" t="n">
-        <v>510</v>
+        <v>77</v>
+      </c>
+      <c r="S13" t="n">
+        <v>166</v>
       </c>
     </row>
     <row r="14">
@@ -3753,7 +3871,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>以太坊近况 · Glamsterdam</t>
+          <t>Binancians · 币安人身份梗</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -3762,48 +3880,37 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>→</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>binancians</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>技术/宏观新闻多（Glamsterdam 测试网、首笔原子 L1→L2、Abstract 关停），ETH ~$2,700 横盘，meme 热度低 → 只看 BURR 迁移</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>462</v>
-      </c>
-      <c r="I14" t="n">
-        <v>623</v>
-      </c>
-      <c r="J14" t="n">
-        <v>944</v>
-      </c>
-      <c r="K14" t="n">
-        <v>1721</v>
-      </c>
-      <c r="L14" t="n">
-        <v>1734</v>
-      </c>
-      <c r="M14" t="n">
-        <v>1117</v>
-      </c>
-      <c r="N14" t="n">
-        <v>1123</v>
-      </c>
+          <t>10/13 23:07 悉尼：同叙事第二腿——中文「币安人」0xDEA1…7777 约 22:33 上线后市值冲到约 $3M+，超过首轮英文 binancians（0x8Dce…7777 ~$0.45M）。@binance 官推原文已核实；币安/CZ 仍未点名任何 CA。同名盘极多、image_dup 高，注意分流与砸盘。</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
+      <c r="R14" t="n">
+        <v>510</v>
+      </c>
+      <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -3811,7 +3918,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>LAPTOP · 亨特·拜登盘</t>
+          <t>以太坊近况 · Glamsterdam</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3820,48 +3927,49 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>↑</t>
+          <t>↓</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>政治名人盘，曾 1 小时 -98%，10/7 报告后小反弹，但讨论多为刷票机器人 → 回避</t>
+          <t>技术/宏观新闻多（Glamsterdam 测试网、首笔原子 L1→L2、Abstract 关停），ETH ~$2,700 横盘，meme 热度低 → 只看 BURR 迁移</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>51</v>
+        <v>462</v>
       </c>
       <c r="I15" t="n">
-        <v>35</v>
+        <v>623</v>
       </c>
       <c r="J15" t="n">
-        <v>34</v>
+        <v>944</v>
       </c>
       <c r="K15" t="n">
-        <v>64</v>
+        <v>1721</v>
       </c>
       <c r="L15" t="n">
-        <v>595</v>
+        <v>1734</v>
       </c>
       <c r="M15" t="n">
-        <v>448</v>
+        <v>1117</v>
       </c>
       <c r="N15" t="n">
-        <v>384</v>
+        <v>1123</v>
       </c>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -3869,7 +3977,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>后量子地堡 · BNKR/PQC</t>
+          <t>LAPTOP · 亨特·拜登盘</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3882,50 +3990,110 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>↑</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>政治名人盘，曾 1 小时 -98%，10/7 报告后小反弹，但讨论多为刷票机器人 → 回避</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>51</v>
+      </c>
+      <c r="I16" t="n">
+        <v>35</v>
+      </c>
+      <c r="J16" t="n">
+        <v>34</v>
+      </c>
+      <c r="K16" t="n">
+        <v>64</v>
+      </c>
+      <c r="L16" t="n">
+        <v>595</v>
+      </c>
+      <c r="M16" t="n">
+        <v>448</v>
+      </c>
+      <c r="N16" t="n">
+        <v>384</v>
+      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>后量子地堡 · BNKR/PQC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>25</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>↓</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>PQC</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>量子恐慌的第一个“产品化”玩法：pqc.market 发射台 + 官方 BNKR。X 讨论 2 天翻 4 倍，但 BNKR 已从 $420K 回撤到 ~$180K，PQC 是母盘</t>
         </is>
       </c>
-      <c r="H16" t="n">
+      <c r="H17" t="n">
         <v>392</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I17" t="n">
         <v>243</v>
       </c>
-      <c r="J16" t="n">
+      <c r="J17" t="n">
         <v>303</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K17" t="n">
         <v>282</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L17" t="n">
         <v>564</v>
       </c>
-      <c r="M16" t="n">
+      <c r="M17" t="n">
         <v>1588</v>
       </c>
-      <c r="N16" t="n">
+      <c r="N17" t="n">
         <v>1463</v>
       </c>
-      <c r="O16" t="n">
+      <c r="O17" t="n">
         <v>728</v>
       </c>
-      <c r="P16" t="n">
+      <c r="P17" t="n">
         <v>587</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="Q17" t="n">
         <v>590</v>
       </c>
-      <c r="R16" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3938,7 +4106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4060,16 +4228,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>115935</v>
+        <v>124035</v>
       </c>
       <c r="I2" t="n">
-        <v>-11</v>
+        <v>-2.9</v>
       </c>
       <c r="J2" t="n">
-        <v>2891.3</v>
+        <v>3100.2</v>
       </c>
       <c r="K2" t="n">
-        <v>34638</v>
+        <v>35730</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -4178,16 +4346,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>115935</v>
+        <v>124035</v>
       </c>
       <c r="I4" t="n">
-        <v>-13.1</v>
+        <v>-2.9</v>
       </c>
       <c r="J4" t="n">
-        <v>2891.3</v>
+        <v>3100.2</v>
       </c>
       <c r="K4" t="n">
-        <v>34638</v>
+        <v>35730</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -4237,16 +4405,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>14534990</v>
+        <v>14404955</v>
       </c>
       <c r="I5" t="n">
-        <v>2.2</v>
+        <v>0.9</v>
       </c>
       <c r="J5" t="n">
-        <v>-9.300000000000001</v>
+        <v>-10.1</v>
       </c>
       <c r="K5" t="n">
-        <v>722707</v>
+        <v>721020</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -4296,16 +4464,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1142816</v>
+        <v>1082043</v>
       </c>
       <c r="I6" t="n">
-        <v>-5</v>
+        <v>-11.7</v>
       </c>
       <c r="J6" t="n">
-        <v>-13.1</v>
+        <v>-17.7</v>
       </c>
       <c r="K6" t="n">
-        <v>149195</v>
+        <v>143463</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -4355,16 +4523,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>547195</v>
+        <v>549137</v>
       </c>
       <c r="I7" t="n">
-        <v>-5.2</v>
+        <v>-5.1</v>
       </c>
       <c r="J7" t="n">
-        <v>-8</v>
+        <v>-7.7</v>
       </c>
       <c r="K7" t="n">
-        <v>86189</v>
+        <v>86339</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -4473,16 +4641,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>924556</v>
+        <v>941440</v>
       </c>
       <c r="I9" t="n">
-        <v>5.4</v>
+        <v>15.2</v>
       </c>
       <c r="J9" t="n">
-        <v>9.699999999999999</v>
+        <v>11.7</v>
       </c>
       <c r="K9" t="n">
-        <v>93853</v>
+        <v>94683</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -4532,16 +4700,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>20233</v>
+        <v>20457</v>
       </c>
       <c r="I10" t="n">
-        <v>18.4</v>
+        <v>-11.6</v>
       </c>
       <c r="J10" t="n">
-        <v>-11.7</v>
+        <v>-10.7</v>
       </c>
       <c r="K10" t="n">
-        <v>14886</v>
+        <v>14956</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -4591,16 +4759,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>34582</v>
+        <v>34556</v>
       </c>
       <c r="I11" t="n">
-        <v>1.2</v>
+        <v>-9.1</v>
       </c>
       <c r="J11" t="n">
-        <v>127</v>
+        <v>126.8</v>
       </c>
       <c r="K11" t="n">
-        <v>20184</v>
+        <v>20075</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -4650,16 +4818,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>531428</v>
+        <v>524442</v>
       </c>
       <c r="I12" t="n">
-        <v>-3.9</v>
+        <v>-6</v>
       </c>
       <c r="J12" t="n">
-        <v>-53.6</v>
+        <v>-54.2</v>
       </c>
       <c r="K12" t="n">
-        <v>81704</v>
+        <v>80837</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -4709,16 +4877,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>49298</v>
+        <v>48326</v>
       </c>
       <c r="I13" t="n">
-        <v>-3.3</v>
+        <v>-6.2</v>
       </c>
       <c r="J13" t="n">
-        <v>-2.2</v>
+        <v>-4.2</v>
       </c>
       <c r="K13" t="n">
-        <v>28199</v>
+        <v>27871</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -4768,16 +4936,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>4409117</v>
+        <v>4409622</v>
       </c>
       <c r="I14" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="J14" t="n">
         <v>26.3</v>
       </c>
       <c r="K14" t="n">
-        <v>180331</v>
+        <v>180107</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -4827,16 +4995,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>39506</v>
+        <v>39321</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.1</v>
+        <v>0.7</v>
       </c>
       <c r="J15" t="n">
-        <v>-58.7</v>
+        <v>-58.9</v>
       </c>
       <c r="K15" t="n">
-        <v>21565</v>
+        <v>21477</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -4886,16 +5054,16 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>315775310</v>
+        <v>316060190</v>
       </c>
       <c r="I16" t="n">
-        <v>2.9</v>
+        <v>2.1</v>
       </c>
       <c r="J16" t="n">
-        <v>11.6</v>
+        <v>11.7</v>
       </c>
       <c r="K16" t="n">
-        <v>3047684</v>
+        <v>3035460</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -4945,13 +5113,13 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>6102010</v>
+        <v>6050318</v>
       </c>
       <c r="I17" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>0.3</v>
+        <v>-0.5</v>
       </c>
       <c r="K17" t="n">
         <v>312651</v>
@@ -5063,16 +5231,16 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>1039380</v>
+        <v>1040577</v>
       </c>
       <c r="I19" t="n">
-        <v>-1.5</v>
+        <v>-1.4</v>
       </c>
       <c r="J19" t="n">
-        <v>24.4</v>
+        <v>24.5</v>
       </c>
       <c r="K19" t="n">
-        <v>121144</v>
+        <v>121145</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -5125,7 +5293,7 @@
         <v>282832</v>
       </c>
       <c r="I20" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
         <v>-1</v>
@@ -5181,16 +5349,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>54973965</v>
+        <v>54752219</v>
       </c>
       <c r="I21" t="n">
-        <v>4.3</v>
+        <v>1.7</v>
       </c>
       <c r="J21" t="n">
-        <v>35</v>
+        <v>34.4</v>
       </c>
       <c r="K21" t="n">
-        <v>1250059</v>
+        <v>1251270</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -5240,16 +5408,16 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>11968423</v>
+        <v>11923309</v>
       </c>
       <c r="I22" t="n">
-        <v>-3.1</v>
+        <v>-5.5</v>
       </c>
       <c r="J22" t="n">
-        <v>-6.4</v>
+        <v>-6.8</v>
       </c>
       <c r="K22" t="n">
-        <v>690292</v>
+        <v>690053</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -5299,16 +5467,16 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>150041</v>
+        <v>141271</v>
       </c>
       <c r="I23" t="n">
-        <v>-5.7</v>
+        <v>-6.2</v>
       </c>
       <c r="J23" t="n">
-        <v>-9.1</v>
+        <v>-14.4</v>
       </c>
       <c r="K23" t="n">
-        <v>35585</v>
+        <v>34084</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -5358,16 +5526,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>25170</v>
+        <v>24151</v>
       </c>
       <c r="I24" t="n">
-        <v>-7.1</v>
+        <v>-5.4</v>
       </c>
       <c r="J24" t="n">
-        <v>-38.3</v>
+        <v>-40.8</v>
       </c>
       <c r="K24" t="n">
-        <v>12048</v>
+        <v>11419</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -5417,16 +5585,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>103816</v>
+        <v>102336</v>
       </c>
       <c r="I25" t="n">
-        <v>-11.7</v>
+        <v>-9.9</v>
       </c>
       <c r="J25" t="n">
-        <v>1766.9</v>
+        <v>1740.3</v>
       </c>
       <c r="K25" t="n">
-        <v>31972</v>
+        <v>31655</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -5476,16 +5644,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>75194</v>
+        <v>91276</v>
       </c>
       <c r="I26" t="n">
-        <v>7.5</v>
+        <v>45.3</v>
       </c>
       <c r="J26" t="n">
-        <v>1481.2</v>
+        <v>1819.4</v>
       </c>
       <c r="K26" t="n">
-        <v>27166</v>
+        <v>30116</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -5535,16 +5703,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>133130102</v>
+        <v>132987968</v>
       </c>
       <c r="I27" t="n">
-        <v>-0.4</v>
+        <v>-0.5</v>
       </c>
       <c r="J27" t="n">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="K27" t="n">
-        <v>2267820</v>
+        <v>2262204</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -5594,13 +5762,13 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>367964650</v>
+        <v>369169870</v>
       </c>
       <c r="I28" t="n">
-        <v>0.1</v>
+        <v>-0.3</v>
       </c>
       <c r="J28" t="n">
-        <v>2.9</v>
+        <v>3.3</v>
       </c>
       <c r="K28" t="n">
         <v>11146839</v>
@@ -5653,7 +5821,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>524129800</v>
+        <v>524171050</v>
       </c>
       <c r="I29" t="n">
         <v>-0.7</v>
@@ -5662,7 +5830,7 @@
         <v>-2.9</v>
       </c>
       <c r="K29" t="n">
-        <v>8227947</v>
+        <v>8229019</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -5712,16 +5880,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>48037346</v>
+        <v>47402202</v>
       </c>
       <c r="I30" t="n">
-        <v>2.7</v>
+        <v>1.5</v>
       </c>
       <c r="J30" t="n">
-        <v>16</v>
+        <v>14.4</v>
       </c>
       <c r="K30" t="n">
-        <v>2168567</v>
+        <v>2155657</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -5771,16 +5939,16 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>264054</v>
+        <v>256469</v>
       </c>
       <c r="I31" t="n">
-        <v>-2.1</v>
+        <v>-6.4</v>
       </c>
       <c r="J31" t="n">
-        <v>11.8</v>
+        <v>8.6</v>
       </c>
       <c r="K31" t="n">
-        <v>50917</v>
+        <v>50276</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -5830,16 +5998,16 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>55540</v>
+        <v>53429</v>
       </c>
       <c r="I32" t="n">
-        <v>-11.9</v>
+        <v>-14.6</v>
       </c>
       <c r="J32" t="n">
-        <v>44.7</v>
+        <v>39.2</v>
       </c>
       <c r="K32" t="n">
-        <v>23545</v>
+        <v>23098</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -5889,16 +6057,16 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>46728</v>
+        <v>33342</v>
       </c>
       <c r="I33" t="n">
-        <v>-23.3</v>
+        <v>-49.3</v>
       </c>
       <c r="J33" t="n">
-        <v>-69.3</v>
+        <v>-78.09999999999999</v>
       </c>
       <c r="K33" t="n">
-        <v>20892</v>
+        <v>17646</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -5948,16 +6116,16 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>139843</v>
+        <v>135732</v>
       </c>
       <c r="I34" t="n">
-        <v>-8</v>
+        <v>-9.4</v>
       </c>
       <c r="J34" t="n">
-        <v>-59.9</v>
+        <v>-61</v>
       </c>
       <c r="K34" t="n">
-        <v>43785</v>
+        <v>42859</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -6007,16 +6175,16 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>123483</v>
+        <v>146139</v>
       </c>
       <c r="I35" t="n">
-        <v>19.9</v>
+        <v>43.5</v>
       </c>
       <c r="J35" t="n">
-        <v>3.9</v>
+        <v>23</v>
       </c>
       <c r="K35" t="n">
-        <v>29116</v>
+        <v>32668</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -6066,16 +6234,16 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>93486</v>
+        <v>73361</v>
       </c>
       <c r="I36" t="n">
-        <v>5.7</v>
+        <v>-15.3</v>
       </c>
       <c r="J36" t="n">
-        <v>-32.6</v>
+        <v>-47.1</v>
       </c>
       <c r="K36" t="n">
-        <v>28684</v>
+        <v>24992</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -6125,16 +6293,16 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>31116</v>
+        <v>31025</v>
       </c>
       <c r="I37" t="n">
-        <v>-6</v>
+        <v>-4.4</v>
       </c>
       <c r="J37" t="n">
-        <v>368.8</v>
+        <v>367.4</v>
       </c>
       <c r="K37" t="n">
-        <v>13282</v>
+        <v>13286</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -6184,16 +6352,16 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>1894294</v>
+        <v>1938618</v>
       </c>
       <c r="I38" t="n">
-        <v>-2.2</v>
+        <v>-0.5</v>
       </c>
       <c r="J38" t="n">
-        <v>-4</v>
+        <v>-1.7</v>
       </c>
       <c r="K38" t="n">
-        <v>585995</v>
+        <v>593136</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -6243,16 +6411,16 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>123223</v>
+        <v>123755</v>
       </c>
       <c r="I39" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="J39" t="n">
-        <v>33.5</v>
+        <v>34.1</v>
       </c>
       <c r="K39" t="n">
-        <v>31866</v>
+        <v>31820</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -6321,6 +6489,301 @@
       <c r="M40" s="2" t="inlineStr">
         <is>
           <t>https://gmgn.ai/sol/token/GkgVK2duAV9Rjbt43prMiZscuMVQ9XR1RihSYsT6tjjE</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Embryo Corp · 基因编辑造独角兽</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>龙头</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>UNICORN</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>4dLxcTxJQnkMmCKkkVoLcKgsRjj7CpGJYuwVU1repump</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>132830</v>
+      </c>
+      <c r="I41" t="n">
+        <v>1508.6</v>
+      </c>
+      <c r="J41" t="n">
+        <v>1629.6</v>
+      </c>
+      <c r="K41" t="n">
+        <v>32151</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>最早的同名盘，网站挂 UsePaid 分成页；创始人未点名 CA，关联未核实。机器人成交约 66%，已从 ATH ~$36.5万回落。</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/4dLxcTxJQnkMmCKkkVoLcKgsRjj7CpGJYuwVU1repump</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Embryo Corp · 基因编辑造独角兽</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>UNICORN</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>DuxVrk5SQ8pCmNi9ToowSmx375hDFbtU1MnJDaBTpump</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>37515</v>
+      </c>
+      <c r="I42" t="n">
+        <v>859.7</v>
+      </c>
+      <c r="J42" t="n">
+        <v>1126.5</v>
+      </c>
+      <c r="K42" t="n">
+        <v>14395</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>第二个同名盘，dev 已清仓。</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/DuxVrk5SQ8pCmNi9ToowSmx375hDFbtU1MnJDaBTpump</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Embryo Corp · 基因编辑造独角兽</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>UNICORN</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>HMzkfMT4TqpC7X2Skc92Vn9q8R3xXnSKF4tn4Y5j2LXk</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>195582</v>
+      </c>
+      <c r="I43" t="n">
+        <v>72739493.5</v>
+      </c>
+      <c r="J43" t="n">
+        <v>72739493.5</v>
+      </c>
+      <c r="K43" t="n">
+        <v>40178</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>🆕 GMGN 自动发现：The Embryo Corporation（10/14 12:19 悉尼上线），名字命中「Embryo」关键词；叙事待人工核实。</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/HMzkfMT4TqpC7X2Skc92Vn9q8R3xXnSKF4tn4Y5j2LXk</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Embryo Corp · 基因编辑造独角兽</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>UNICORN</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Co2nDVEbPSY7JRrWSCCLWhsUGhRubPMQT5hyZVRySkAd</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>80739</v>
+      </c>
+      <c r="I44" t="n">
+        <v>30013759.2</v>
+      </c>
+      <c r="J44" t="n">
+        <v>30013759.2</v>
+      </c>
+      <c r="K44" t="n">
+        <v>27140</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>🆕 GMGN 自动发现：The Embryo Corporation（10/14 12:34 悉尼上线），名字命中「Embryo」关键词；叙事待人工核实。</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/Co2nDVEbPSY7JRrWSCCLWhsUGhRubPMQT5hyZVRySkAd</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Embryo Corp · 基因编辑造独角兽</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>UNICORN</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>38anPGKgXfFCW8ZE9F7YejoK39BvNbz2ReVWX4DTkMKs</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>72297</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>634.8</v>
+      </c>
+      <c r="K45" t="n">
+        <v>63449</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>🆕 GMGN 自动发现：The Embryo Corporation（10/14 06:47 悉尼上线），名字命中「Embryo」关键词；叙事待人工核实。</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/38anPGKgXfFCW8ZE9F7YejoK39BvNbz2ReVWX4DTkMKs</t>
         </is>
       </c>
     </row>
@@ -6365,6 +6828,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
radar 10/14 12:45 embryo fix
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -6660,7 +6660,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：The Embryo Corporation（10/14 12:19 悉尼上线），名字命中「Embryo」关键词；叙事待人工核实。</t>
+          <t>同名非 pump 后缀盘，10/14 中午新开，借用 4dLx 的社交链接，疑似蹭盘</t>
         </is>
       </c>
       <c r="M43" s="2" t="inlineStr">
@@ -6719,7 +6719,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：The Embryo Corporation（10/14 12:34 悉尼上线），名字命中「Embryo」关键词；叙事待人工核实。</t>
+          <t>同名非 pump 后缀盘，10/14 中午新开，借用 4dLx 的社交链接，疑似蹭盘</t>
         </is>
       </c>
       <c r="M44" s="2" t="inlineStr">
@@ -6778,7 +6778,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>🆕 GMGN 自动发现：The Embryo Corporation（10/14 06:47 悉尼上线），名字命中「Embryo」关键词；叙事待人工核实。</t>
+          <t>同名非 pump 后缀盘，10/14 中午新开，借用 4dLx 的社交链接，疑似蹭盘</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">

</xml_diff>

<commit_message>
floyd sahil 10/14 13:23
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G96"/>
+  <dimension ref="A1:G100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2921,6 +2921,90 @@
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr"/>
+      <c r="B97" t="inlineStr"/>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Floyd What's next</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/FloydMayweather/status/2110175346838708626</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Floyd × fomo × sahil</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr"/>
+      <c r="B98" t="inlineStr"/>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>sahil next crime</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/villainmonkey/status/2110176871757631774</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Floyd × fomo × sahil</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr"/>
+      <c r="B99" t="inlineStr"/>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>CryptoGorilla 二报</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/CryptoGorilla/status/2110117870604841020</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Floyd × fomo × sahil</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr"/>
+      <c r="B100" t="inlineStr"/>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>MrketInsider</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/MrketInsider/status/2110192247560114270</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Floyd × fomo × sahil</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3019,6 +3103,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId93"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId94"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId99"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3030,7 +3118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S17"/>
+  <dimension ref="A1:S18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3918,7 +4006,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>以太坊近况 · Glamsterdam</t>
+          <t>Floyd × fomo × sahil</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3927,49 +4015,39 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>↑</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>FLOYD</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>技术/宏观新闻多（Glamsterdam 测试网、首笔原子 L1→L2、Abstract 关停），ETH ~$2,700 横盘，meme 热度低 → 只看 BURR 迁移</t>
-        </is>
-      </c>
-      <c r="H15" t="n">
-        <v>462</v>
-      </c>
-      <c r="I15" t="n">
-        <v>623</v>
-      </c>
-      <c r="J15" t="n">
-        <v>944</v>
-      </c>
-      <c r="K15" t="n">
-        <v>1721</v>
-      </c>
-      <c r="L15" t="n">
-        <v>1734</v>
-      </c>
-      <c r="M15" t="n">
-        <v>1117</v>
-      </c>
-      <c r="N15" t="n">
-        <v>1123</v>
-      </c>
+          <t>10/14 13:23 悉尼：原 CA 帖已删（已核实 Not Found）；Floyd 现帖「What's next @villainmonkey?」已核实；sahil 预告 next crime @fomo 10/15 05:00 悉尼。本人/买推/被盗未核实。高风险名人连发盘。</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
+      <c r="R15" t="n">
+        <v>200</v>
+      </c>
+      <c r="S15" t="n">
+        <v>293</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -3977,7 +4055,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>LAPTOP · 亨特·拜登盘</t>
+          <t>以太坊近况 · Glamsterdam</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3986,43 +4064,43 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>↑</t>
+          <t>↓</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>政治名人盘，曾 1 小时 -98%，10/7 报告后小反弹，但讨论多为刷票机器人 → 回避</t>
+          <t>技术/宏观新闻多（Glamsterdam 测试网、首笔原子 L1→L2、Abstract 关停），ETH ~$2,700 横盘，meme 热度低 → 只看 BURR 迁移</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>51</v>
+        <v>462</v>
       </c>
       <c r="I16" t="n">
-        <v>35</v>
+        <v>623</v>
       </c>
       <c r="J16" t="n">
-        <v>34</v>
+        <v>944</v>
       </c>
       <c r="K16" t="n">
-        <v>64</v>
+        <v>1721</v>
       </c>
       <c r="L16" t="n">
-        <v>595</v>
+        <v>1734</v>
       </c>
       <c r="M16" t="n">
-        <v>448</v>
+        <v>1117</v>
       </c>
       <c r="N16" t="n">
-        <v>384</v>
+        <v>1123</v>
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
@@ -4036,7 +4114,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>后量子地堡 · BNKR/PQC</t>
+          <t>LAPTOP · 亨特·拜登盘</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -4049,51 +4127,110 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>↓</t>
+          <t>↑</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>PQC</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>量子恐慌的第一个“产品化”玩法：pqc.market 发射台 + 官方 BNKR。X 讨论 2 天翻 4 倍，但 BNKR 已从 $420K 回撤到 ~$180K，PQC 是母盘</t>
+          <t>政治名人盘，曾 1 小时 -98%，10/7 报告后小反弹，但讨论多为刷票机器人 → 回避</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>392</v>
+        <v>51</v>
       </c>
       <c r="I17" t="n">
-        <v>243</v>
+        <v>35</v>
       </c>
       <c r="J17" t="n">
-        <v>303</v>
+        <v>34</v>
       </c>
       <c r="K17" t="n">
-        <v>282</v>
+        <v>64</v>
       </c>
       <c r="L17" t="n">
-        <v>564</v>
+        <v>595</v>
       </c>
       <c r="M17" t="n">
-        <v>1588</v>
+        <v>448</v>
       </c>
       <c r="N17" t="n">
-        <v>1463</v>
-      </c>
-      <c r="O17" t="n">
-        <v>728</v>
-      </c>
-      <c r="P17" t="n">
-        <v>587</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>590</v>
-      </c>
+        <v>384</v>
+      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>后量子地堡 · BNKR/PQC</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>25</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>↓</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>PQC</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>量子恐慌的第一个“产品化”玩法：pqc.market 发射台 + 官方 BNKR。X 讨论 2 天翻 4 倍，但 BNKR 已从 $420K 回撤到 ~$180K，PQC 是母盘</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>392</v>
+      </c>
+      <c r="I18" t="n">
+        <v>243</v>
+      </c>
+      <c r="J18" t="n">
+        <v>303</v>
+      </c>
+      <c r="K18" t="n">
+        <v>282</v>
+      </c>
+      <c r="L18" t="n">
+        <v>564</v>
+      </c>
+      <c r="M18" t="n">
+        <v>1588</v>
+      </c>
+      <c r="N18" t="n">
+        <v>1463</v>
+      </c>
+      <c r="O18" t="n">
+        <v>728</v>
+      </c>
+      <c r="P18" t="n">
+        <v>587</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>590</v>
+      </c>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4106,7 +4243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M44"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4228,16 +4365,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>116737</v>
+        <v>117769</v>
       </c>
       <c r="I2" t="n">
-        <v>6.9</v>
+        <v>1.1</v>
       </c>
       <c r="J2" t="n">
-        <v>2911.9</v>
+        <v>2938.6</v>
       </c>
       <c r="K2" t="n">
-        <v>34725</v>
+        <v>34852</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -4346,16 +4483,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>116737</v>
+        <v>117769</v>
       </c>
       <c r="I4" t="n">
-        <v>6.9</v>
+        <v>1.1</v>
       </c>
       <c r="J4" t="n">
-        <v>2911.9</v>
+        <v>2938.6</v>
       </c>
       <c r="K4" t="n">
-        <v>34725</v>
+        <v>34852</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -4405,16 +4542,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>14548114</v>
+        <v>14732880</v>
       </c>
       <c r="I5" t="n">
-        <v>3.3</v>
+        <v>1.5</v>
       </c>
       <c r="J5" t="n">
-        <v>-14.7</v>
+        <v>-13.4</v>
       </c>
       <c r="K5" t="n">
-        <v>726684</v>
+        <v>753871</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -4464,16 +4601,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1069305</v>
+        <v>1070848</v>
       </c>
       <c r="I6" t="n">
-        <v>-8.9</v>
+        <v>-7.6</v>
       </c>
       <c r="J6" t="n">
-        <v>-20.4</v>
+        <v>-22</v>
       </c>
       <c r="K6" t="n">
-        <v>144301</v>
+        <v>144493</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -4523,16 +4660,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>547896</v>
+        <v>554667</v>
       </c>
       <c r="I7" t="n">
-        <v>-2.7</v>
+        <v>1.4</v>
       </c>
       <c r="J7" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="K7" t="n">
-        <v>86336</v>
+        <v>86899</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -4588,7 +4725,7 @@
         <v>-2.4</v>
       </c>
       <c r="J8" t="n">
-        <v>-20.8</v>
+        <v>-28.3</v>
       </c>
       <c r="K8" t="n">
         <v>10229</v>
@@ -4641,16 +4778,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>851916</v>
+        <v>851669</v>
       </c>
       <c r="I9" t="n">
-        <v>-1.9</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>-5.8</v>
+        <v>-5.9</v>
       </c>
       <c r="K9" t="n">
-        <v>90635</v>
+        <v>90659</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -4700,16 +4837,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>16729</v>
+        <v>14769</v>
       </c>
       <c r="I10" t="n">
-        <v>-19.9</v>
+        <v>-15.8</v>
       </c>
       <c r="J10" t="n">
-        <v>-39.9</v>
+        <v>-47</v>
       </c>
       <c r="K10" t="n">
-        <v>13556</v>
+        <v>12727</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -4759,16 +4896,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>28388</v>
+        <v>27601</v>
       </c>
       <c r="I11" t="n">
-        <v>-26.4</v>
+        <v>-19.3</v>
       </c>
       <c r="J11" t="n">
-        <v>86.3</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="K11" t="n">
-        <v>18212</v>
+        <v>17940</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -4818,16 +4955,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>576965</v>
+        <v>584098</v>
       </c>
       <c r="I12" t="n">
-        <v>10.6</v>
+        <v>15.2</v>
       </c>
       <c r="J12" t="n">
-        <v>-45.4</v>
+        <v>-44.7</v>
       </c>
       <c r="K12" t="n">
-        <v>85929</v>
+        <v>87052</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -4877,16 +5014,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>43115</v>
+        <v>42968</v>
       </c>
       <c r="I13" t="n">
-        <v>-13.1</v>
+        <v>-13.4</v>
       </c>
       <c r="J13" t="n">
-        <v>-22.6</v>
+        <v>-22.8</v>
       </c>
       <c r="K13" t="n">
-        <v>26132</v>
+        <v>25949</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -4936,16 +5073,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>4445679</v>
+        <v>4462907</v>
       </c>
       <c r="I14" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="J14" t="n">
-        <v>23.6</v>
+        <v>24.1</v>
       </c>
       <c r="K14" t="n">
-        <v>181255</v>
+        <v>181670</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -4995,16 +5132,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>37938</v>
+        <v>38147</v>
       </c>
       <c r="I15" t="n">
-        <v>-5.3</v>
+        <v>-3.4</v>
       </c>
       <c r="J15" t="n">
-        <v>-67.5</v>
+        <v>-67.3</v>
       </c>
       <c r="K15" t="n">
-        <v>21162</v>
+        <v>21418</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -5054,16 +5191,16 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>318409260</v>
+        <v>321432760</v>
       </c>
       <c r="I16" t="n">
-        <v>3.6</v>
+        <v>1.1</v>
       </c>
       <c r="J16" t="n">
-        <v>13.5</v>
+        <v>14.6</v>
       </c>
       <c r="K16" t="n">
-        <v>3043822</v>
+        <v>3059552</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -5113,10 +5250,10 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>6119757</v>
+        <v>6120081</v>
       </c>
       <c r="I17" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="J17" t="n">
         <v>-2.7</v>
@@ -5231,16 +5368,16 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>1019783</v>
+        <v>1028348</v>
       </c>
       <c r="I19" t="n">
-        <v>-1.9</v>
+        <v>-2.1</v>
       </c>
       <c r="J19" t="n">
-        <v>21.5</v>
+        <v>22.5</v>
       </c>
       <c r="K19" t="n">
-        <v>120474</v>
+        <v>120500</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -5349,16 +5486,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>57843845</v>
+        <v>57983136</v>
       </c>
       <c r="I21" t="n">
-        <v>9.699999999999999</v>
+        <v>11.7</v>
       </c>
       <c r="J21" t="n">
-        <v>35.7</v>
+        <v>36</v>
       </c>
       <c r="K21" t="n">
-        <v>1295478</v>
+        <v>1294749</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -5408,16 +5545,16 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>11836265</v>
+        <v>11856575</v>
       </c>
       <c r="I22" t="n">
-        <v>-2</v>
+        <v>-1.3</v>
       </c>
       <c r="J22" t="n">
-        <v>-13.5</v>
+        <v>-13.3</v>
       </c>
       <c r="K22" t="n">
-        <v>688678</v>
+        <v>689225</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -5467,16 +5604,16 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>139223</v>
+        <v>147544</v>
       </c>
       <c r="I23" t="n">
-        <v>-6.8</v>
+        <v>-1.7</v>
       </c>
       <c r="J23" t="n">
-        <v>-16.6</v>
+        <v>-11.6</v>
       </c>
       <c r="K23" t="n">
-        <v>33707</v>
+        <v>33606</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -5526,16 +5663,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>23617</v>
+        <v>24098</v>
       </c>
       <c r="I24" t="n">
-        <v>-6.2</v>
+        <v>-4.3</v>
       </c>
       <c r="J24" t="n">
-        <v>-38.6</v>
+        <v>-37.4</v>
       </c>
       <c r="K24" t="n">
-        <v>11492</v>
+        <v>11610</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -5585,16 +5722,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>166029</v>
+        <v>202895</v>
       </c>
       <c r="I25" t="n">
-        <v>82.8</v>
+        <v>96.7</v>
       </c>
       <c r="J25" t="n">
-        <v>2885.7</v>
+        <v>3548.7</v>
       </c>
       <c r="K25" t="n">
-        <v>40641</v>
+        <v>45295</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -5644,16 +5781,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>112969</v>
+        <v>145222</v>
       </c>
       <c r="I26" t="n">
-        <v>75.7</v>
+        <v>100.4</v>
       </c>
       <c r="J26" t="n">
-        <v>2275.5</v>
+        <v>2953.7</v>
       </c>
       <c r="K26" t="n">
-        <v>33489</v>
+        <v>37906</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -5703,16 +5840,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>133229299</v>
+        <v>132654989</v>
       </c>
       <c r="I27" t="n">
-        <v>0.3</v>
+        <v>-0.7</v>
       </c>
       <c r="J27" t="n">
-        <v>1.9</v>
+        <v>1.5</v>
       </c>
       <c r="K27" t="n">
-        <v>2267546</v>
+        <v>2262143</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -5821,16 +5958,16 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>523680320</v>
+        <v>524178440</v>
       </c>
       <c r="I29" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>-4.7</v>
+        <v>-4.6</v>
       </c>
       <c r="K29" t="n">
-        <v>8225681</v>
+        <v>8233467</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -5880,16 +6017,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>45785105</v>
+        <v>46015578</v>
       </c>
       <c r="I30" t="n">
-        <v>-3.2</v>
+        <v>-3.4</v>
       </c>
       <c r="J30" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="K30" t="n">
-        <v>2118566</v>
+        <v>2124971</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -5939,16 +6076,16 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>255975</v>
+        <v>258204</v>
       </c>
       <c r="I31" t="n">
-        <v>-10.5</v>
+        <v>-9.1</v>
       </c>
       <c r="J31" t="n">
-        <v>8.5</v>
+        <v>9.4</v>
       </c>
       <c r="K31" t="n">
-        <v>50206</v>
+        <v>50494</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -5998,16 +6135,16 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>47304</v>
+        <v>47272</v>
       </c>
       <c r="I32" t="n">
-        <v>-17.5</v>
+        <v>-16.7</v>
       </c>
       <c r="J32" t="n">
-        <v>48.1</v>
+        <v>48</v>
       </c>
       <c r="K32" t="n">
-        <v>21733</v>
+        <v>21739</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -6057,16 +6194,16 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>35267</v>
+        <v>38408</v>
       </c>
       <c r="I33" t="n">
-        <v>-34.5</v>
+        <v>-26.2</v>
       </c>
       <c r="J33" t="n">
-        <v>-75.5</v>
+        <v>-73.3</v>
       </c>
       <c r="K33" t="n">
-        <v>18189</v>
+        <v>18991</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -6116,16 +6253,16 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>132865</v>
+        <v>134105</v>
       </c>
       <c r="I34" t="n">
-        <v>-6.3</v>
+        <v>-7.1</v>
       </c>
       <c r="J34" t="n">
-        <v>-58.4</v>
+        <v>-58.1</v>
       </c>
       <c r="K34" t="n">
-        <v>42757</v>
+        <v>42995</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -6175,16 +6312,16 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>154672</v>
+        <v>151788</v>
       </c>
       <c r="I35" t="n">
-        <v>13.8</v>
+        <v>16.3</v>
       </c>
       <c r="J35" t="n">
-        <v>30.6</v>
+        <v>28.2</v>
       </c>
       <c r="K35" t="n">
-        <v>33857</v>
+        <v>33580</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -6234,16 +6371,16 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>63733</v>
+        <v>66069</v>
       </c>
       <c r="I36" t="n">
-        <v>-29.7</v>
+        <v>-27.1</v>
       </c>
       <c r="J36" t="n">
-        <v>-49.6</v>
+        <v>-47.8</v>
       </c>
       <c r="K36" t="n">
-        <v>23338</v>
+        <v>23772</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -6293,16 +6430,16 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>35758</v>
+        <v>35205</v>
       </c>
       <c r="I37" t="n">
-        <v>9</v>
+        <v>13.1</v>
       </c>
       <c r="J37" t="n">
-        <v>337.3</v>
+        <v>330.5</v>
       </c>
       <c r="K37" t="n">
-        <v>14534</v>
+        <v>14405</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -6352,16 +6489,16 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>1951934</v>
+        <v>1872118</v>
       </c>
       <c r="I38" t="n">
-        <v>3.8</v>
+        <v>0.1</v>
       </c>
       <c r="J38" t="n">
-        <v>-1.9</v>
+        <v>-5.9</v>
       </c>
       <c r="K38" t="n">
-        <v>595987</v>
+        <v>583962</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -6414,7 +6551,7 @@
         <v>125466</v>
       </c>
       <c r="I39" t="n">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="J39" t="n">
         <v>29.5</v>
@@ -6529,16 +6666,16 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>153706</v>
+        <v>151264</v>
       </c>
       <c r="I41" t="n">
-        <v>-11</v>
+        <v>-41.1</v>
       </c>
       <c r="J41" t="n">
-        <v>1972.9</v>
+        <v>1939.9</v>
       </c>
       <c r="K41" t="n">
-        <v>34178</v>
+        <v>35347</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -6588,16 +6725,16 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>26089</v>
+        <v>25298</v>
       </c>
       <c r="I42" t="n">
-        <v>-68.59999999999999</v>
+        <v>-67.8</v>
       </c>
       <c r="J42" t="n">
-        <v>753</v>
+        <v>727.1</v>
       </c>
       <c r="K42" t="n">
-        <v>11158</v>
+        <v>11150</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
@@ -6647,16 +6784,16 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>231938</v>
+        <v>181035</v>
       </c>
       <c r="I43" t="n">
-        <v>86220673.2</v>
+        <v>67297878</v>
       </c>
       <c r="J43" t="n">
-        <v>86220673.2</v>
+        <v>67297878</v>
       </c>
       <c r="K43" t="n">
-        <v>55028</v>
+        <v>55017</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -6725,6 +6862,124 @@
       <c r="M44" s="2" t="inlineStr">
         <is>
           <t>https://gmgn.ai/sol/token/38anPGKgXfFCW8ZE9F7YejoK39BvNbz2ReVWX4DTkMKs</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Floyd × fomo × sahil</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>龙头</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>FLOYD</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Gjd3JUbNG2C3n5Ww98SfPxyWaqvDk2BkiKongGwEpump</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>96248</v>
+      </c>
+      <c r="I45" t="n">
+        <v>186.8</v>
+      </c>
+      <c r="J45" t="n">
+        <v>3343.4</v>
+      </c>
+      <c r="K45" t="n">
+        <v>29138</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Floyd 曾发 CA 后删帖；与官方无关。ATH~$1.1M，现回落。</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/Gjd3JUbNG2C3n5Ww98SfPxyWaqvDk2BkiKongGwEpump</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Floyd × fomo × sahil</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>24小时</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>FWOYD</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>sol</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>GjMrz9j5Bt5Va1tsqfi71XpcqKAbhFoyPxw9CAzZpump</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>alive</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>53402</v>
+      </c>
+      <c r="I46" t="n">
+        <v>-51.5</v>
+      </c>
+      <c r="J46" t="n">
+        <v>1772.5</v>
+      </c>
+      <c r="K46" t="n">
+        <v>17695</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>恶搞盘，有机讨论弱。</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>https://gmgn.ai/sol/token/GjMrz9j5Bt5Va1tsqfi71XpcqKAbhFoyPxw9CAzZpump</t>
         </is>
       </c>
     </row>
@@ -6773,6 +7028,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
radar silent 10/14 14:06
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G100"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2927,17 +2927,17 @@
       <c r="B97" t="inlineStr"/>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Floyd What's next</t>
+          <t>Josie 不支持任一 token</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/FloydMayweather/status/2110175346838708626</t>
+          <t>https://x.com/josiezayner/status/2110202201939288261</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Floyd × fomo × sahil</t>
+          <t>Embryo Corp · 基因编辑造独角兽</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -2948,12 +2948,12 @@
       <c r="B98" t="inlineStr"/>
       <c r="C98" t="inlineStr">
         <is>
-          <t>sahil next crime</t>
+          <t>Floyd What's next</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/villainmonkey/status/2110176871757631774</t>
+          <t>https://x.com/FloydMayweather/status/2110175346838708626</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -2969,12 +2969,12 @@
       <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr">
         <is>
-          <t>CryptoGorilla 二报</t>
+          <t>sahil next crime</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/CryptoGorilla/status/2110117870604841020</t>
+          <t>https://x.com/villainmonkey/status/2110176871757631774</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -2990,12 +2990,12 @@
       <c r="B100" t="inlineStr"/>
       <c r="C100" t="inlineStr">
         <is>
-          <t>MrketInsider</t>
+          <t>CryptoGorilla 二报</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/MrketInsider/status/2110192247560114270</t>
+          <t>https://x.com/CryptoGorilla/status/2110117870604841020</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -3005,6 +3005,27 @@
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr"/>
+      <c r="B101" t="inlineStr"/>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>MrketInsider</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/MrketInsider/status/2110192247560114270</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Floyd × fomo × sahil</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3107,6 +3128,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId100"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3923,7 +3945,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>事件已核实（官网 building.life + People 独家，创始人本人转发）；创始人 10/14 12:06 悉尼发帖“币圈的人一直在给我打 SOL”但未点名任何 CA，币与她的关联未核实</t>
+          <t>10/14 14:06 悉尼：Josie 已核实声明「I don't support either of the tokens」（https://x.com/josiezayner/status/2110202201939288261 ~1k浏览）；同时仍感谢打 SOL。未点名任何 CA，多盘竞争。SOL 帖 2110175418565238969 ~12.6k浏览。热度约 0→13→31/hr（相对低）。龙头未确认，回避追盘。</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -4029,7 +4051,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10/14 13:23 悉尼：原 CA 帖已删（已核实 Not Found）；Floyd 现帖「What's next @villainmonkey?」已核实；sahil 预告 next crime @fomo 10/15 05:00 悉尼。本人/买推/被盗未核实。高风险名人连发盘。</t>
+          <t>10/14 14:06 悉尼：热度回落 178→62→32/hr；无 Floyd/villainmonkey/fomo 新帖。原 CA 帖仍删；盘面 FLOYD/FWOYD 各约 $63K 1h 约 -16~-23%。不重复推。</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>

</xml_diff>

<commit_message>
radar altai trump-ai 10/14 15:00
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -4387,16 +4387,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>122539</v>
+        <v>101411</v>
       </c>
       <c r="I2" t="n">
-        <v>5.1</v>
+        <v>-16.1</v>
       </c>
       <c r="J2" t="n">
-        <v>3061.6</v>
+        <v>2516.5</v>
       </c>
       <c r="K2" t="n">
-        <v>35653</v>
+        <v>32418</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -4449,7 +4449,7 @@
         <v>54680</v>
       </c>
       <c r="I3" t="n">
-        <v>-1.2</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
         <v>-1.8</v>
@@ -4505,16 +4505,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>122539</v>
+        <v>101146</v>
       </c>
       <c r="I4" t="n">
-        <v>5.1</v>
+        <v>-16.3</v>
       </c>
       <c r="J4" t="n">
-        <v>3061.6</v>
+        <v>2509.7</v>
       </c>
       <c r="K4" t="n">
-        <v>35653</v>
+        <v>32345</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -4564,16 +4564,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>15630660</v>
+        <v>15496404</v>
       </c>
       <c r="I5" t="n">
-        <v>5.4</v>
+        <v>4.1</v>
       </c>
       <c r="J5" t="n">
-        <v>-12.5</v>
+        <v>0.5</v>
       </c>
       <c r="K5" t="n">
-        <v>733820</v>
+        <v>723196</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -4623,16 +4623,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>976418</v>
+        <v>972631</v>
       </c>
       <c r="I6" t="n">
-        <v>-7.4</v>
+        <v>-1</v>
       </c>
       <c r="J6" t="n">
-        <v>-27.7</v>
+        <v>-25.7</v>
       </c>
       <c r="K6" t="n">
-        <v>136753</v>
+        <v>137775</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -4682,16 +4682,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>503754</v>
+        <v>511459</v>
       </c>
       <c r="I7" t="n">
-        <v>-9.5</v>
+        <v>-1.9</v>
       </c>
       <c r="J7" t="n">
-        <v>-12.9</v>
+        <v>-8.9</v>
       </c>
       <c r="K7" t="n">
-        <v>82769</v>
+        <v>84525</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -4741,16 +4741,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>11681</v>
+        <v>10699</v>
       </c>
       <c r="I8" t="n">
-        <v>-3.8</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>-44.3</v>
+        <v>-41.6</v>
       </c>
       <c r="K8" t="n">
-        <v>9974</v>
+        <v>9574</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -4800,16 +4800,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>979215</v>
+        <v>953531</v>
       </c>
       <c r="I9" t="n">
-        <v>13.1</v>
+        <v>2.7</v>
       </c>
       <c r="J9" t="n">
-        <v>8.6</v>
+        <v>11.6</v>
       </c>
       <c r="K9" t="n">
-        <v>97100</v>
+        <v>96339</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -4859,16 +4859,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>24490</v>
+        <v>26295</v>
       </c>
       <c r="I10" t="n">
-        <v>-13.7</v>
+        <v>-3.6</v>
       </c>
       <c r="J10" t="n">
-        <v>60.7</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="K10" t="n">
-        <v>16923</v>
+        <v>17577</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -4918,16 +4918,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>519362</v>
+        <v>530117</v>
       </c>
       <c r="I11" t="n">
-        <v>-9.6</v>
+        <v>-7.9</v>
       </c>
       <c r="J11" t="n">
-        <v>-58.5</v>
+        <v>-57.9</v>
       </c>
       <c r="K11" t="n">
-        <v>81657</v>
+        <v>82444</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -4977,16 +4977,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>44929</v>
+        <v>44566</v>
       </c>
       <c r="I12" t="n">
-        <v>4.1</v>
+        <v>3.5</v>
       </c>
       <c r="J12" t="n">
-        <v>-9.199999999999999</v>
+        <v>-11.5</v>
       </c>
       <c r="K12" t="n">
-        <v>26653</v>
+        <v>26388</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -5036,16 +5036,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>4455363</v>
+        <v>4462321</v>
       </c>
       <c r="I13" t="n">
-        <v>0.2</v>
+        <v>-0.3</v>
       </c>
       <c r="J13" t="n">
         <v>21.6</v>
       </c>
       <c r="K13" t="n">
-        <v>182560</v>
+        <v>182739</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -5095,16 +5095,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>31272</v>
+        <v>32956</v>
       </c>
       <c r="I14" t="n">
-        <v>-16.9</v>
+        <v>-12.9</v>
       </c>
       <c r="J14" t="n">
-        <v>-73</v>
+        <v>-64.7</v>
       </c>
       <c r="K14" t="n">
-        <v>19231</v>
+        <v>19744</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -5154,16 +5154,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>332946650</v>
+        <v>331451900</v>
       </c>
       <c r="I15" t="n">
-        <v>4.4</v>
+        <v>1.6</v>
       </c>
       <c r="J15" t="n">
-        <v>19.2</v>
+        <v>17.7</v>
       </c>
       <c r="K15" t="n">
-        <v>3207525</v>
+        <v>3201631</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -5213,16 +5213,16 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>6150141</v>
+        <v>6160757</v>
       </c>
       <c r="I16" t="n">
-        <v>0.4</v>
+        <v>-0.1</v>
       </c>
       <c r="J16" t="n">
         <v>-0.4</v>
       </c>
       <c r="K16" t="n">
-        <v>313386</v>
+        <v>313759</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -5331,16 +5331,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>1056564</v>
+        <v>1022043</v>
       </c>
       <c r="I18" t="n">
-        <v>1.5</v>
+        <v>-1.6</v>
       </c>
       <c r="J18" t="n">
-        <v>21.7</v>
+        <v>16</v>
       </c>
       <c r="K18" t="n">
-        <v>121794</v>
+        <v>120737</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -5390,16 +5390,16 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>283735</v>
+        <v>273294</v>
       </c>
       <c r="I19" t="n">
-        <v>0.6</v>
+        <v>-1.7</v>
       </c>
       <c r="J19" t="n">
-        <v>-1.6</v>
+        <v>-5.3</v>
       </c>
       <c r="K19" t="n">
-        <v>56707</v>
+        <v>55851</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -5449,16 +5449,16 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>56941921</v>
+        <v>55076958</v>
       </c>
       <c r="I20" t="n">
-        <v>2.2</v>
+        <v>-0.1</v>
       </c>
       <c r="J20" t="n">
-        <v>29.5</v>
+        <v>26.3</v>
       </c>
       <c r="K20" t="n">
-        <v>1259915</v>
+        <v>1264869</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -5508,16 +5508,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>12338937</v>
+        <v>12227604</v>
       </c>
       <c r="I21" t="n">
-        <v>3.9</v>
+        <v>-3.9</v>
       </c>
       <c r="J21" t="n">
-        <v>-16.7</v>
+        <v>-14.5</v>
       </c>
       <c r="K21" t="n">
-        <v>708281</v>
+        <v>702492</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -5626,16 +5626,16 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>23920</v>
+        <v>24391</v>
       </c>
       <c r="I23" t="n">
-        <v>-0.7</v>
+        <v>0.7</v>
       </c>
       <c r="J23" t="n">
-        <v>-36.1</v>
+        <v>-39</v>
       </c>
       <c r="K23" t="n">
-        <v>11508</v>
+        <v>11820</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -5685,16 +5685,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>176426</v>
+        <v>170522</v>
       </c>
       <c r="I24" t="n">
-        <v>-9.800000000000001</v>
+        <v>-0.5</v>
       </c>
       <c r="J24" t="n">
-        <v>3072.7</v>
+        <v>2966.5</v>
       </c>
       <c r="K24" t="n">
-        <v>42165</v>
+        <v>41358</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -5744,16 +5744,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>134551</v>
+        <v>131450</v>
       </c>
       <c r="I25" t="n">
-        <v>-29.9</v>
+        <v>-20.7</v>
       </c>
       <c r="J25" t="n">
-        <v>2729.3</v>
+        <v>2664.1</v>
       </c>
       <c r="K25" t="n">
-        <v>36573</v>
+        <v>36198</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -5803,16 +5803,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>132460354</v>
+        <v>132525521</v>
       </c>
       <c r="I26" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="J26" t="n">
-        <v>1.8</v>
+        <v>0.9</v>
       </c>
       <c r="K26" t="n">
-        <v>2266292</v>
+        <v>2265387</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -5862,16 +5862,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>371970850</v>
+        <v>371363640</v>
       </c>
       <c r="I27" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J27" t="n">
         <v>0.9</v>
       </c>
-      <c r="J27" t="n">
-        <v>1.9</v>
-      </c>
       <c r="K27" t="n">
-        <v>11226620</v>
+        <v>11203301</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -5921,16 +5921,16 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>525515920</v>
+        <v>523910270</v>
       </c>
       <c r="I28" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>-3.6</v>
+        <v>-4.7</v>
       </c>
       <c r="K28" t="n">
-        <v>8259090</v>
+        <v>8238867</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -5980,16 +5980,16 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>44179661</v>
+        <v>43215349</v>
       </c>
       <c r="I29" t="n">
-        <v>-4.8</v>
+        <v>-5.6</v>
       </c>
       <c r="J29" t="n">
-        <v>-0.5</v>
+        <v>-7.1</v>
       </c>
       <c r="K29" t="n">
-        <v>2085976</v>
+        <v>2061214</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -6039,16 +6039,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>231003</v>
+        <v>223069</v>
       </c>
       <c r="I30" t="n">
-        <v>-5</v>
+        <v>-11.7</v>
       </c>
       <c r="J30" t="n">
-        <v>-0.8</v>
+        <v>-4.2</v>
       </c>
       <c r="K30" t="n">
-        <v>47616</v>
+        <v>47006</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -6098,16 +6098,16 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>42050</v>
+        <v>41894</v>
       </c>
       <c r="I31" t="n">
-        <v>-8.9</v>
+        <v>-4.6</v>
       </c>
       <c r="J31" t="n">
-        <v>54.6</v>
+        <v>50.7</v>
       </c>
       <c r="K31" t="n">
-        <v>20543</v>
+        <v>20480</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -6157,16 +6157,16 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>57366</v>
+        <v>63285</v>
       </c>
       <c r="I32" t="n">
-        <v>36.7</v>
+        <v>2.8</v>
       </c>
       <c r="J32" t="n">
-        <v>-47.2</v>
+        <v>-36.4</v>
       </c>
       <c r="K32" t="n">
-        <v>23177</v>
+        <v>24360</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -6216,16 +6216,16 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>122777</v>
+        <v>132923</v>
       </c>
       <c r="I33" t="n">
-        <v>-8.800000000000001</v>
+        <v>3</v>
       </c>
       <c r="J33" t="n">
-        <v>-65.09999999999999</v>
+        <v>-59.6</v>
       </c>
       <c r="K33" t="n">
-        <v>40756</v>
+        <v>42688</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -6275,16 +6275,16 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>137217</v>
+        <v>117972</v>
       </c>
       <c r="I34" t="n">
-        <v>-9.6</v>
+        <v>-16.7</v>
       </c>
       <c r="J34" t="n">
-        <v>15.6</v>
+        <v>1.6</v>
       </c>
       <c r="K34" t="n">
-        <v>31664</v>
+        <v>29166</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -6334,16 +6334,16 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>66072</v>
+        <v>56700</v>
       </c>
       <c r="I35" t="n">
-        <v>1</v>
+        <v>-7.2</v>
       </c>
       <c r="J35" t="n">
-        <v>-54.4</v>
+        <v>-51.7</v>
       </c>
       <c r="K35" t="n">
-        <v>23653</v>
+        <v>21468</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -6393,16 +6393,16 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>33458</v>
+        <v>32932</v>
       </c>
       <c r="I36" t="n">
-        <v>-4.3</v>
+        <v>-1.1</v>
       </c>
       <c r="J36" t="n">
-        <v>260.8</v>
+        <v>338.6</v>
       </c>
       <c r="K36" t="n">
-        <v>13967</v>
+        <v>13821</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -6452,16 +6452,16 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>1882991</v>
+        <v>1871111</v>
       </c>
       <c r="I37" t="n">
-        <v>0.2</v>
+        <v>-4</v>
       </c>
       <c r="J37" t="n">
-        <v>-1.5</v>
+        <v>1.4</v>
       </c>
       <c r="K37" t="n">
-        <v>587097</v>
+        <v>584215</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -6511,16 +6511,16 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>144756</v>
+        <v>138125</v>
       </c>
       <c r="I38" t="n">
-        <v>12.2</v>
+        <v>5.6</v>
       </c>
       <c r="J38" t="n">
-        <v>53.3</v>
+        <v>44.8</v>
       </c>
       <c r="K38" t="n">
-        <v>34560</v>
+        <v>33890</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -6576,7 +6576,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>-94.8</v>
+        <v>-94.7</v>
       </c>
       <c r="K39" t="n">
         <v>12477</v>
@@ -6629,16 +6629,16 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>67462</v>
+        <v>175896</v>
       </c>
       <c r="I40" t="n">
-        <v>-60.7</v>
+        <v>97.8</v>
       </c>
       <c r="J40" t="n">
-        <v>554.4</v>
+        <v>1593.6</v>
       </c>
       <c r="K40" t="n">
-        <v>21902</v>
+        <v>40308</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -6688,16 +6688,16 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>24643</v>
+        <v>38925</v>
       </c>
       <c r="I41" t="n">
-        <v>-27</v>
+        <v>148.8</v>
       </c>
       <c r="J41" t="n">
-        <v>705.7</v>
+        <v>1172.6</v>
       </c>
       <c r="K41" t="n">
-        <v>10931</v>
+        <v>15068</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -6806,16 +6806,16 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>59296</v>
+        <v>76782</v>
       </c>
       <c r="I43" t="n">
-        <v>-28.3</v>
+        <v>22.1</v>
       </c>
       <c r="J43" t="n">
-        <v>2021.4</v>
+        <v>2647</v>
       </c>
       <c r="K43" t="n">
-        <v>22197</v>
+        <v>25465</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -6865,16 +6865,16 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>40717</v>
+        <v>21251</v>
       </c>
       <c r="I44" t="n">
-        <v>-29.8</v>
+        <v>-66.59999999999999</v>
       </c>
       <c r="J44" t="n">
-        <v>1327.7</v>
+        <v>645.2</v>
       </c>
       <c r="K44" t="n">
-        <v>15233</v>
+        <v>9932</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
radar 10/14 15:12 embryo note
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2843,12 +2843,12 @@
       <c r="B93" t="inlineStr"/>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Josie 帖：币圈一直给我打 SOL</t>
+          <t>Josie 转发 People 采访</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/josiezayner/status/2110175418565238969</t>
+          <t>https://x.com/josiezayner/status/2110107308478828560</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -2864,12 +2864,12 @@
       <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Josie 转发 People 采访</t>
+          <t>People 独家</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/josiezayner/status/2110107308478828560</t>
+          <t>https://people.com/former-nasa-scientist-says-unicorn-horn-could-be-5-to-10-years-away-exclusive-12170434</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -2885,12 +2885,12 @@
       <c r="B95" t="inlineStr"/>
       <c r="C95" t="inlineStr">
         <is>
-          <t>People 独家</t>
+          <t>公司官网</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>https://people.com/former-nasa-scientist-says-unicorn-horn-could-be-5-to-10-years-away-exclusive-12170434</t>
+          <t>https://building.life/</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -2906,12 +2906,12 @@
       <c r="B96" t="inlineStr"/>
       <c r="C96" t="inlineStr">
         <is>
-          <t>公司官网</t>
+          <t>Josie 不支持任一 token</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>https://building.life/</t>
+          <t>https://x.com/josiezayner/status/2110202201939288261</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -2927,12 +2927,12 @@
       <c r="B97" t="inlineStr"/>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Josie 不支持任一 token</t>
+          <t>Josie unfinished support</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/josiezayner/status/2110202201939288261</t>
+          <t>https://x.com/josiezayner/status/2110218359975313588</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -2948,17 +2948,17 @@
       <c r="B98" t="inlineStr"/>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Floyd What's next</t>
+          <t>Josie over my head</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/FloydMayweather/status/2110175346838708626</t>
+          <t>https://x.com/josiezayner/status/2110221628793635213</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Floyd × fomo × sahil</t>
+          <t>Embryo Corp · 基因编辑造独角兽</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -2969,12 +2969,12 @@
       <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr">
         <is>
-          <t>sahil next crime</t>
+          <t>Floyd What's next</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/villainmonkey/status/2110176871757631774</t>
+          <t>https://x.com/FloydMayweather/status/2110175346838708626</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -2990,12 +2990,12 @@
       <c r="B100" t="inlineStr"/>
       <c r="C100" t="inlineStr">
         <is>
-          <t>CryptoGorilla 二报</t>
+          <t>sahil next crime</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/CryptoGorilla/status/2110117870604841020</t>
+          <t>https://x.com/villainmonkey/status/2110176871757631774</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -3011,12 +3011,12 @@
       <c r="B101" t="inlineStr"/>
       <c r="C101" t="inlineStr">
         <is>
-          <t>MrketInsider</t>
+          <t>CryptoGorilla 二报</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>https://x.com/MrketInsider/status/2110192247560114270</t>
+          <t>https://x.com/CryptoGorilla/status/2110117870604841020</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -3026,6 +3026,27 @@
       </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr"/>
+      <c r="B102" t="inlineStr"/>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>MrketInsider</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/MrketInsider/status/2110192247560114270</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Floyd × fomo × sahil</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3129,6 +3150,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId99"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId101"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3945,7 +3967,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10/14 14:33 悉尼：Josie 已核实在回复里确认收款钱包 9D99UtHw3FjFXwURJgGrXVs4HWNC1qj3HMuYz8BTBr3h 是她的（回复 @OnchainPeasant「is this your wallet?」；本轮扫描未另存该回复 status id）。此前已核实「I don't support either of the tokens」（https://x.com/josiezayner/status/2110202201939288261）。对「Unicorn will only be sent at a billion dollar mcap」仅回「fr」，未点名 CA。持币人互撕升温（4dLx…repump vs DuxVrk…pump），属内斗非外部新注意力。龙头未确认，回避追盘。</t>
+          <t>10/14 15:12 悉尼：Josie 03:57–03:59Z 连发未写完的“The token I will/support is”后又收回（已核实原帖），04:10Z 称自己“in way over my head”、只想做科研；讨论量 95→79→181/hr 再起，但官方 CA 仍查不到，同名盘 4dLx…repump vs DuxVrk…pump 互掐，仍不推盘。</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>

</xml_diff>

<commit_message>
radar 10/14 16:00 silent
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -3430,7 +3430,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>10/12：马斯克再推 Cybercab 内 Grok @Bot（已核实，~45万浏览）；链上仍无像样龙头 → 盯叙事不追盘</t>
+          <t>10/14 16:00 悉尼：15:00–15:25 Elon 连发/转 Grok @Bot（税、awesome 等，单帖 40万+浏览）；叙事升温但链上仍无干净龙头 → 盯叙事不追盘。</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -3967,7 +3967,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10/14 15:12 悉尼：Josie 03:57–03:59Z 连发未写完的“The token I will/support is”后又收回（已核实原帖），04:10Z 称自己“in way over my head”、只想做科研；讨论量 95→79→181/hr 再起，但官方 CA 仍查不到，同名盘 4dLx…repump vs DuxVrk…pump 互掐，仍不推盘。</t>
+          <t>10/14 16:00 悉尼：继续冷却；窗口内仅刷单喊单，无 Josie 新表态。</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -4073,7 +4073,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10/14 14:06 悉尼：热度回落 178→62→32/hr；无 Floyd/villainmonkey/fomo 新帖。原 CA 帖仍删；盘面 FLOYD/FWOYD 各约 $63K 1h 约 -16~-23%。不重复推。</t>
+          <t>10/14 16:00 悉尼：热度续降 51→31→24/hr；无 Floyd/fomo 新帖；不重复推。</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -4409,16 +4409,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>75475</v>
+        <v>82992</v>
       </c>
       <c r="I2" t="n">
-        <v>-32.8</v>
+        <v>-16.5</v>
       </c>
       <c r="J2" t="n">
-        <v>1847.3</v>
+        <v>2041.3</v>
       </c>
       <c r="K2" t="n">
-        <v>28041</v>
+        <v>29349</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -4468,16 +4468,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>54486</v>
+        <v>53476</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.4</v>
+        <v>-2.2</v>
       </c>
       <c r="J3" t="n">
-        <v>-2.1</v>
+        <v>-3.9</v>
       </c>
       <c r="K3" t="n">
-        <v>42928</v>
+        <v>42165</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -4527,16 +4527,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>75475</v>
+        <v>82992</v>
       </c>
       <c r="I4" t="n">
-        <v>-31.9</v>
+        <v>-16.6</v>
       </c>
       <c r="J4" t="n">
-        <v>1847.3</v>
+        <v>2041.3</v>
       </c>
       <c r="K4" t="n">
-        <v>28041</v>
+        <v>29349</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -4586,16 +4586,16 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>15220552</v>
+        <v>14824721</v>
       </c>
       <c r="I5" t="n">
-        <v>-3</v>
+        <v>-4.2</v>
       </c>
       <c r="J5" t="n">
-        <v>-2.7</v>
+        <v>-8.300000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>758346</v>
+        <v>752312</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -4645,16 +4645,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1022652</v>
+        <v>999103</v>
       </c>
       <c r="I6" t="n">
-        <v>3.5</v>
+        <v>0.3</v>
       </c>
       <c r="J6" t="n">
-        <v>-20.1</v>
+        <v>-25.7</v>
       </c>
       <c r="K6" t="n">
-        <v>141977</v>
+        <v>139463</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -4704,16 +4704,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>527748</v>
+        <v>526339</v>
       </c>
       <c r="I7" t="n">
-        <v>0.3</v>
+        <v>3.2</v>
       </c>
       <c r="J7" t="n">
-        <v>-10.3</v>
+        <v>-13.7</v>
       </c>
       <c r="K7" t="n">
-        <v>82418</v>
+        <v>84682</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -4763,16 +4763,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>11232</v>
+        <v>11446</v>
       </c>
       <c r="I8" t="n">
-        <v>-3.8</v>
+        <v>7</v>
       </c>
       <c r="J8" t="n">
-        <v>-38.7</v>
+        <v>-45.5</v>
       </c>
       <c r="K8" t="n">
-        <v>9550</v>
+        <v>9919</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -4822,16 +4822,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>918280</v>
+        <v>917729</v>
       </c>
       <c r="I9" t="n">
-        <v>-4.6</v>
+        <v>-3.7</v>
       </c>
       <c r="J9" t="n">
-        <v>6.8</v>
+        <v>9.4</v>
       </c>
       <c r="K9" t="n">
-        <v>94339</v>
+        <v>93844</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -4881,16 +4881,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>30211</v>
+        <v>31187</v>
       </c>
       <c r="I10" t="n">
-        <v>24.9</v>
+        <v>19</v>
       </c>
       <c r="J10" t="n">
-        <v>98.3</v>
+        <v>104.7</v>
       </c>
       <c r="K10" t="n">
-        <v>18753</v>
+        <v>19112</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -4940,16 +4940,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>562311</v>
+        <v>558169</v>
       </c>
       <c r="I11" t="n">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
       <c r="J11" t="n">
-        <v>-55.2</v>
+        <v>-54.7</v>
       </c>
       <c r="K11" t="n">
-        <v>84350</v>
+        <v>84702</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -4999,16 +4999,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>45207</v>
+        <v>45388</v>
       </c>
       <c r="I12" t="n">
-        <v>0.6</v>
+        <v>1.8</v>
       </c>
       <c r="J12" t="n">
-        <v>10.7</v>
+        <v>4.6</v>
       </c>
       <c r="K12" t="n">
-        <v>26551</v>
+        <v>26984</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -5058,16 +5058,16 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>4551915</v>
+        <v>4504902</v>
       </c>
       <c r="I13" t="n">
-        <v>2</v>
+        <v>0.1</v>
       </c>
       <c r="J13" t="n">
-        <v>23.3</v>
+        <v>20.2</v>
       </c>
       <c r="K13" t="n">
-        <v>183963</v>
+        <v>183355</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -5117,16 +5117,16 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>31114</v>
+        <v>28785</v>
       </c>
       <c r="I14" t="n">
-        <v>-2.9</v>
+        <v>-11.6</v>
       </c>
       <c r="J14" t="n">
-        <v>-60.2</v>
+        <v>-71.09999999999999</v>
       </c>
       <c r="K14" t="n">
-        <v>19125</v>
+        <v>18400</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -5176,16 +5176,16 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>342308990</v>
+        <v>337171590</v>
       </c>
       <c r="I15" t="n">
-        <v>2.9</v>
+        <v>1.9</v>
       </c>
       <c r="J15" t="n">
-        <v>21.1</v>
+        <v>19.2</v>
       </c>
       <c r="K15" t="n">
-        <v>3282446</v>
+        <v>3293438</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -5235,16 +5235,16 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>6392314</v>
+        <v>6383240</v>
       </c>
       <c r="I16" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="J16" t="n">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="K16" t="n">
-        <v>320034</v>
+        <v>320431</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -5300,7 +5300,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>5.1</v>
+        <v>5.4</v>
       </c>
       <c r="K17" t="n">
         <v>261660</v>
@@ -5353,16 +5353,16 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>1040671</v>
+        <v>1028815</v>
       </c>
       <c r="I18" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J18" t="n">
-        <v>23</v>
+        <v>21.3</v>
       </c>
       <c r="K18" t="n">
-        <v>121092</v>
+        <v>121111</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -5412,16 +5412,16 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>273079</v>
+        <v>275378</v>
       </c>
       <c r="I19" t="n">
-        <v>-3.8</v>
+        <v>0.8</v>
       </c>
       <c r="J19" t="n">
-        <v>-5.3</v>
+        <v>-4.9</v>
       </c>
       <c r="K19" t="n">
-        <v>55462</v>
+        <v>56044</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -5471,16 +5471,16 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>53582129</v>
+        <v>54769860</v>
       </c>
       <c r="I20" t="n">
-        <v>-6.1</v>
+        <v>-0.5</v>
       </c>
       <c r="J20" t="n">
-        <v>18.8</v>
+        <v>19.8</v>
       </c>
       <c r="K20" t="n">
-        <v>1249148</v>
+        <v>1257574</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -5530,16 +5530,16 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>11746836</v>
+        <v>11644665</v>
       </c>
       <c r="I21" t="n">
-        <v>-5.6</v>
+        <v>-5.3</v>
       </c>
       <c r="J21" t="n">
-        <v>-16.5</v>
+        <v>-17.8</v>
       </c>
       <c r="K21" t="n">
-        <v>689816</v>
+        <v>680281</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -5595,7 +5595,7 @@
         <v>0.6</v>
       </c>
       <c r="J22" t="n">
-        <v>0.2</v>
+        <v>1.8</v>
       </c>
       <c r="K22" t="n">
         <v>35747</v>
@@ -5648,16 +5648,16 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>23776</v>
+        <v>24147</v>
       </c>
       <c r="I23" t="n">
-        <v>-0.6</v>
+        <v>-1</v>
       </c>
       <c r="J23" t="n">
-        <v>-39</v>
+        <v>-41.1</v>
       </c>
       <c r="K23" t="n">
-        <v>11479</v>
+        <v>11740</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -5707,16 +5707,16 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>169273</v>
+        <v>151861</v>
       </c>
       <c r="I24" t="n">
-        <v>0.6</v>
+        <v>-10.5</v>
       </c>
       <c r="J24" t="n">
-        <v>2944</v>
+        <v>2630.9</v>
       </c>
       <c r="K24" t="n">
-        <v>41109</v>
+        <v>38918</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -5766,16 +5766,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>95794</v>
+        <v>94128</v>
       </c>
       <c r="I25" t="n">
-        <v>-21.3</v>
+        <v>-28.6</v>
       </c>
       <c r="J25" t="n">
-        <v>1914.4</v>
+        <v>1879.3</v>
       </c>
       <c r="K25" t="n">
-        <v>30905</v>
+        <v>30611</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -5825,16 +5825,16 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>132320494</v>
+        <v>131635726</v>
       </c>
       <c r="I26" t="n">
         <v>-0.8</v>
       </c>
       <c r="J26" t="n">
-        <v>-0.2</v>
+        <v>-0.3</v>
       </c>
       <c r="K26" t="n">
-        <v>2268174</v>
+        <v>2254687</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -5884,16 +5884,16 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>372607630</v>
+        <v>372634350</v>
       </c>
       <c r="I27" t="n">
-        <v>0.1</v>
+        <v>0.6</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="K27" t="n">
-        <v>11231225</v>
+        <v>11224544</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -5943,16 +5943,16 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>527451350</v>
+        <v>521219450</v>
       </c>
       <c r="I28" t="n">
-        <v>0.4</v>
+        <v>-0.5</v>
       </c>
       <c r="J28" t="n">
-        <v>-4</v>
+        <v>-5.2</v>
       </c>
       <c r="K28" t="n">
-        <v>8238919</v>
+        <v>8212584</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -6002,16 +6002,16 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>43585403</v>
+        <v>43585232</v>
       </c>
       <c r="I29" t="n">
-        <v>-0.9</v>
+        <v>0.4</v>
       </c>
       <c r="J29" t="n">
-        <v>-6.4</v>
+        <v>-8.6</v>
       </c>
       <c r="K29" t="n">
-        <v>2071194</v>
+        <v>2069118</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -6061,16 +6061,16 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>247347</v>
+        <v>249898</v>
       </c>
       <c r="I30" t="n">
-        <v>13.3</v>
+        <v>10.1</v>
       </c>
       <c r="J30" t="n">
-        <v>6.8</v>
+        <v>7.1</v>
       </c>
       <c r="K30" t="n">
-        <v>49544</v>
+        <v>49576</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -6120,16 +6120,16 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>40153</v>
+        <v>40293</v>
       </c>
       <c r="I31" t="n">
-        <v>-4.6</v>
+        <v>-4.4</v>
       </c>
       <c r="J31" t="n">
-        <v>82.3</v>
+        <v>81.8</v>
       </c>
       <c r="K31" t="n">
-        <v>20068</v>
+        <v>20088</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -6179,16 +6179,16 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>60211</v>
+        <v>48852</v>
       </c>
       <c r="I32" t="n">
-        <v>6.4</v>
+        <v>-21.6</v>
       </c>
       <c r="J32" t="n">
-        <v>-27.2</v>
+        <v>-50.3</v>
       </c>
       <c r="K32" t="n">
-        <v>23779</v>
+        <v>21223</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -6238,16 +6238,16 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>132388</v>
+        <v>131268</v>
       </c>
       <c r="I33" t="n">
-        <v>12</v>
+        <v>-0.5</v>
       </c>
       <c r="J33" t="n">
-        <v>-59.6</v>
+        <v>-56.6</v>
       </c>
       <c r="K33" t="n">
-        <v>42826</v>
+        <v>41991</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -6297,16 +6297,16 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>111073</v>
+        <v>114048</v>
       </c>
       <c r="I34" t="n">
-        <v>-19.1</v>
+        <v>-2.8</v>
       </c>
       <c r="J34" t="n">
-        <v>-6.5</v>
+        <v>-4</v>
       </c>
       <c r="K34" t="n">
-        <v>28259</v>
+        <v>28625</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -6356,16 +6356,16 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>72629</v>
+        <v>78372</v>
       </c>
       <c r="I35" t="n">
-        <v>13.4</v>
+        <v>39.1</v>
       </c>
       <c r="J35" t="n">
-        <v>-41</v>
+        <v>-41.3</v>
       </c>
       <c r="K35" t="n">
-        <v>24934</v>
+        <v>26270</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -6415,16 +6415,16 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>32939</v>
+        <v>70486</v>
       </c>
       <c r="I36" t="n">
-        <v>-1.6</v>
+        <v>114</v>
       </c>
       <c r="J36" t="n">
-        <v>361.1</v>
+        <v>743.5</v>
       </c>
       <c r="K36" t="n">
-        <v>13847</v>
+        <v>21897</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -6474,16 +6474,16 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>1789877</v>
+        <v>1852573</v>
       </c>
       <c r="I37" t="n">
-        <v>-5.1</v>
+        <v>-0.8</v>
       </c>
       <c r="J37" t="n">
-        <v>-8.1</v>
+        <v>-6.5</v>
       </c>
       <c r="K37" t="n">
-        <v>572629</v>
+        <v>581127</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -6533,16 +6533,16 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>134008</v>
+        <v>134351</v>
       </c>
       <c r="I38" t="n">
-        <v>-6.8</v>
+        <v>-1.4</v>
       </c>
       <c r="J38" t="n">
-        <v>25.7</v>
+        <v>26.5</v>
       </c>
       <c r="K38" t="n">
-        <v>33251</v>
+        <v>33336</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -6598,7 +6598,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>-94.7</v>
+        <v>-94.90000000000001</v>
       </c>
       <c r="K39" t="n">
         <v>12477</v>
@@ -6651,16 +6651,16 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>129631</v>
+        <v>150855</v>
       </c>
       <c r="I40" t="n">
-        <v>87</v>
+        <v>1.6</v>
       </c>
       <c r="J40" t="n">
-        <v>1091.5</v>
+        <v>1282.8</v>
       </c>
       <c r="K40" t="n">
-        <v>33211</v>
+        <v>35576</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -6710,16 +6710,16 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>32824</v>
+        <v>17685</v>
       </c>
       <c r="I41" t="n">
-        <v>40.7</v>
+        <v>-52</v>
       </c>
       <c r="J41" t="n">
-        <v>973.2</v>
+        <v>478.2</v>
       </c>
       <c r="K41" t="n">
-        <v>13685</v>
+        <v>8819</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -6828,16 +6828,16 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>90184</v>
+        <v>85419</v>
       </c>
       <c r="I43" t="n">
-        <v>45.6</v>
+        <v>16</v>
       </c>
       <c r="J43" t="n">
-        <v>3126.5</v>
+        <v>2956</v>
       </c>
       <c r="K43" t="n">
-        <v>28020</v>
+        <v>27089</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -6887,16 +6887,16 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>16759</v>
+        <v>14249</v>
       </c>
       <c r="I44" t="n">
-        <v>-58.3</v>
+        <v>-33.2</v>
       </c>
       <c r="J44" t="n">
-        <v>487.7</v>
+        <v>399.6</v>
       </c>
       <c r="K44" t="n">
-        <v>8445</v>
+        <v>7564</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>

</xml_diff>